<commit_message>
Pilotage : emails de démarrage et de relance tracés, retours dans l'app mesurés (jour même ou lendemain)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AUzY5Y8Bt2KRzzte5cJgH8
</commit_message>
<xml_diff>
--- a/docs/recette/Recette_prod_decembre_2026.xlsx
+++ b/docs/recette/Recette_prod_decembre_2026.xlsx
@@ -497,7 +497,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I32"/>
+  <dimension ref="A1:I33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -1620,6 +1620,47 @@
       <c r="H32" s="6" t="n"/>
       <c r="I32" s="6" t="n"/>
     </row>
+    <row r="33">
+      <c r="A33" s="4" t="n">
+        <v>29</v>
+      </c>
+      <c r="B33" s="5" t="inlineStr">
+        <is>
+          <t>Pilotage — retours après démarrage et relances</t>
+        </is>
+      </c>
+      <c r="C33" s="4" t="inlineStr">
+        <is>
+          <t>Pilotage → Activité (carte Notifications)</t>
+        </is>
+      </c>
+      <c r="D33" s="4" t="inlineStr">
+        <is>
+          <t>Après quelques jours de prod : lire la nouvelle section « Démarrage et relances : retours dans l'app ».</t>
+        </is>
+      </c>
+      <c r="E33" s="4" t="inlineStr">
+        <is>
+          <t>Lignes « demarrage · email », « demarrage · push », « relance · … » avec envois et retours (visite le jour même ou le lendemain) ; les emails apparaissent aussi dans le total « conseils par email ».</t>
+        </is>
+      </c>
+      <c r="F33" s="4" t="inlineStr">
+        <is>
+          <t>Admin</t>
+        </is>
+      </c>
+      <c r="G33" s="6" t="inlineStr">
+        <is>
+          <t>Non testable</t>
+        </is>
+      </c>
+      <c r="H33" s="6" t="inlineStr">
+        <is>
+          <t>Données de prod : à lire quelques jours après la mise en prod.</t>
+        </is>
+      </c>
+      <c r="I33" s="6" t="n"/>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A2:I2"/>
@@ -1633,7 +1674,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="G5:G32" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="G5:G32 G33" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"À tester,OK,KO,Non testable"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Recette : suivi des retours déplacé dans les exceptions déjà en prod
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AUzY5Y8Bt2KRzzte5cJgH8
</commit_message>
<xml_diff>
--- a/docs/recette/Recette_prod_decembre_2026.xlsx
+++ b/docs/recette/Recette_prod_decembre_2026.xlsx
@@ -497,7 +497,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I33"/>
+  <dimension ref="A1:I32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -1619,47 +1619,6 @@
       </c>
       <c r="H32" s="6" t="n"/>
       <c r="I32" s="6" t="n"/>
-    </row>
-    <row r="33">
-      <c r="A33" s="4" t="n">
-        <v>29</v>
-      </c>
-      <c r="B33" s="5" t="inlineStr">
-        <is>
-          <t>Pilotage — retours après démarrage et relances</t>
-        </is>
-      </c>
-      <c r="C33" s="4" t="inlineStr">
-        <is>
-          <t>Pilotage → Activité (carte Notifications)</t>
-        </is>
-      </c>
-      <c r="D33" s="4" t="inlineStr">
-        <is>
-          <t>Après quelques jours de prod : lire la nouvelle section « Démarrage et relances : retours dans l'app ».</t>
-        </is>
-      </c>
-      <c r="E33" s="4" t="inlineStr">
-        <is>
-          <t>Lignes « demarrage · email », « demarrage · push », « relance · … » avec envois et retours (visite le jour même ou le lendemain) ; les emails apparaissent aussi dans le total « conseils par email ».</t>
-        </is>
-      </c>
-      <c r="F33" s="4" t="inlineStr">
-        <is>
-          <t>Admin</t>
-        </is>
-      </c>
-      <c r="G33" s="6" t="inlineStr">
-        <is>
-          <t>Non testable</t>
-        </is>
-      </c>
-      <c r="H33" s="6" t="inlineStr">
-        <is>
-          <t>Données de prod : à lire quelques jours après la mise en prod.</t>
-        </is>
-      </c>
-      <c r="I33" s="6" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -1688,7 +1647,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I6"/>
+  <dimension ref="A1:I7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -1845,6 +1804,47 @@
       </c>
       <c r="I6" s="6" t="n"/>
     </row>
+    <row r="7">
+      <c r="A7" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>Pilotage — retours après démarrage et relances</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>Pilotage → Activité (carte Notifications)</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>Après quelques jours de prod : lire la nouvelle section « Démarrage et relances : retours dans l'app ».</t>
+        </is>
+      </c>
+      <c r="E7" s="4" t="inlineStr">
+        <is>
+          <t>Lignes « demarrage · email », « demarrage · push », « relance · … » avec envois et retours (visite le jour même ou le lendemain) ; les emails apparaissent aussi dans le total « conseils par email ».</t>
+        </is>
+      </c>
+      <c r="F7" s="4" t="inlineStr">
+        <is>
+          <t>Admin</t>
+        </is>
+      </c>
+      <c r="G7" s="6" t="inlineStr">
+        <is>
+          <t>À tester</t>
+        </is>
+      </c>
+      <c r="H7" s="6" t="inlineStr">
+        <is>
+          <t>En prod le 07/10/2026 (exception) : lire la section quelques jours après.</t>
+        </is>
+      </c>
+      <c r="I7" s="6" t="n"/>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A2:I2"/>
@@ -1858,7 +1858,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="G5:G6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="G5:G6 G7" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"À tester,OK,KO,Non testable"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Robots Gardena SILENO : connexion, état et mode Proposition
- Connexion Gardena (objet gardena_robot) par le compte Husqvarna Group ; une connexion enregistre
  l'arrosage et le robot du compte (sans remplacer un équipement d'une autre marque)
- Jardin relu en une requête pour l'arrosage et le robot (limite Gardena de 700 requêtes/semaine)
- Jetons partagés renouvelés partout, révoqués seulement avec le dernier équipement
- Commandes MOWER_CONTROL ; repos jusqu'à demain matin relancé par la tâche du matin
- Mes équipements, Bob, confidentialité, CLAUDE.md et recette de décembre

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AUzY5Y8Bt2KRzzte5cJgH8
</commit_message>
<xml_diff>
--- a/docs/recette/Recette_prod_decembre_2026.xlsx
+++ b/docs/recette/Recette_prod_decembre_2026.xlsx
@@ -497,7 +497,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I32"/>
+  <dimension ref="A1:I37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -1515,27 +1515,27 @@
       </c>
       <c r="B30" s="5" t="inlineStr">
         <is>
-          <t>Alignement PROD / STA</t>
+          <t>Robot Gardena SILENO — connexion</t>
         </is>
       </c>
       <c r="C30" s="4" t="inlineStr">
         <is>
-          <t>Git</t>
+          <t>Mes équipements → Robot tondeuse</t>
         </is>
       </c>
       <c r="D30" s="4" t="inlineStr">
         <is>
-          <t>Après la fusion : git diff --quiet origin/main origin/Staging.</t>
+          <t>« Connecter mon robot Gardena » avec un compte GARDENA smart system qui a un SILENO.</t>
         </is>
       </c>
       <c r="E30" s="4" t="inlineStr">
         <is>
-          <t>Aucune différence.</t>
+          <t>Retour sur Mes équipements avec « Robot Gardena connecté » ; carte robot (nom, état, batterie) ; libellé « Gardena SILENO ». Si le compte a aussi un arrosage Gardena : les deux sont connectés.</t>
         </is>
       </c>
       <c r="F30" s="4" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Compte avec SILENO (testeur à trouver)</t>
         </is>
       </c>
       <c r="G30" s="6" t="inlineStr">
@@ -1552,27 +1552,27 @@
       </c>
       <c r="B31" s="5" t="inlineStr">
         <is>
-          <t>Base de données PROD</t>
+          <t>Robot Gardena SILENO — sans robot</t>
         </is>
       </c>
       <c r="C31" s="4" t="inlineStr">
         <is>
-          <t>Supabase PROD</t>
+          <t>Mes équipements → Robot tondeuse</t>
         </is>
       </c>
       <c r="D31" s="4" t="inlineStr">
         <is>
-          <t>Vérifier les tables codes et parrainages.</t>
+          <t>Même bouton avec un compte Gardena sans robot.</t>
         </is>
       </c>
       <c r="E31" s="4" t="inlineStr">
         <is>
-          <t>Tables présentes (créées le 05/10 sur les deux projets).</t>
+          <t>Message « Aucun robot Gardena trouvé sur ce compte » ; rien n'est enregistré.</t>
         </is>
       </c>
       <c r="F31" s="4" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Compte Gardena sans robot</t>
         </is>
       </c>
       <c r="G31" s="6" t="inlineStr">
@@ -1589,27 +1589,27 @@
       </c>
       <c r="B32" s="5" t="inlineStr">
         <is>
-          <t>Règle de travail de décembre</t>
+          <t>Robot Gardena SILENO — proposition</t>
         </is>
       </c>
       <c r="C32" s="4" t="inlineStr">
         <is>
-          <t>CLAUDE.md</t>
+          <t>Aujourd'hui</t>
         </is>
       </c>
       <c r="D32" s="4" t="inlineStr">
         <is>
-          <t>Après la mise en prod : retirer le paragraphe « Jusqu'à décembre 2026 ».</t>
+          <t>Jour de pluie / gel : valider « Mettre au repos jusqu'à demain matin », puis un jour sans contrainte : « Relancer son planning ».</t>
         </is>
       </c>
       <c r="E32" s="4" t="inlineStr">
         <is>
-          <t>STA redevient identique à la PROD.</t>
+          <t>Le robot rentre et reste garé (app Gardena : garé jusqu'à nouvel ordre) ; la relance remet son planning. Rien n'est envoyé sans validation.</t>
         </is>
       </c>
       <c r="F32" s="4" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Compte avec SILENO</t>
         </is>
       </c>
       <c r="G32" s="6" t="inlineStr">
@@ -1619,6 +1619,191 @@
       </c>
       <c r="H32" s="6" t="n"/>
       <c r="I32" s="6" t="n"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="n">
+        <v>29</v>
+      </c>
+      <c r="B33" s="5" t="inlineStr">
+        <is>
+          <t>Robot Gardena SILENO — reprise du matin</t>
+        </is>
+      </c>
+      <c r="C33" s="4" t="inlineStr">
+        <is>
+          <t>Tâche du matin (PROD)</t>
+        </is>
+      </c>
+      <c r="D33" s="4" t="inlineStr">
+        <is>
+          <t>Le lendemain d'un « repos jusqu'à demain matin », regarder le robot après 8 h.</t>
+        </is>
+      </c>
+      <c r="E33" s="4" t="inlineStr">
+        <is>
+          <t>Planning relancé automatiquement (journal de la tâche : robotsRelances ≥ 1). Non testable sur STA (tâches planifiées en PROD seulement).</t>
+        </is>
+      </c>
+      <c r="F33" s="4" t="inlineStr">
+        <is>
+          <t>Compte avec SILENO</t>
+        </is>
+      </c>
+      <c r="G33" s="6" t="inlineStr">
+        <is>
+          <t>À tester</t>
+        </is>
+      </c>
+      <c r="H33" s="6" t="n"/>
+      <c r="I33" s="6" t="n"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="n">
+        <v>30</v>
+      </c>
+      <c r="B34" s="5" t="inlineStr">
+        <is>
+          <t>Robot Gardena SILENO — déconnexion</t>
+        </is>
+      </c>
+      <c r="C34" s="4" t="inlineStr">
+        <is>
+          <t>Mes équipements</t>
+        </is>
+      </c>
+      <c r="D34" s="4" t="inlineStr">
+        <is>
+          <t>Avec arrosage ET robot Gardena : déconnecter le robot, puis vérifier l'arrosage.</t>
+        </is>
+      </c>
+      <c r="E34" s="4" t="inlineStr">
+        <is>
+          <t>L'arrosage reste connecté et fonctionne (la connexion commune n'est révoquée qu'avec le dernier équipement Gardena).</t>
+        </is>
+      </c>
+      <c r="F34" s="4" t="inlineStr">
+        <is>
+          <t>Compte avec SILENO + arrosage Gardena</t>
+        </is>
+      </c>
+      <c r="G34" s="6" t="inlineStr">
+        <is>
+          <t>À tester</t>
+        </is>
+      </c>
+      <c r="H34" s="6" t="n"/>
+      <c r="I34" s="6" t="n"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="n">
+        <v>31</v>
+      </c>
+      <c r="B35" s="5" t="inlineStr">
+        <is>
+          <t>Alignement PROD / STA</t>
+        </is>
+      </c>
+      <c r="C35" s="4" t="inlineStr">
+        <is>
+          <t>Git</t>
+        </is>
+      </c>
+      <c r="D35" s="4" t="inlineStr">
+        <is>
+          <t>Après la fusion : git diff --quiet origin/main origin/Staging.</t>
+        </is>
+      </c>
+      <c r="E35" s="4" t="inlineStr">
+        <is>
+          <t>Aucune différence.</t>
+        </is>
+      </c>
+      <c r="F35" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G35" s="6" t="inlineStr">
+        <is>
+          <t>À tester</t>
+        </is>
+      </c>
+      <c r="H35" s="6" t="n"/>
+      <c r="I35" s="6" t="n"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="n">
+        <v>32</v>
+      </c>
+      <c r="B36" s="5" t="inlineStr">
+        <is>
+          <t>Base de données PROD</t>
+        </is>
+      </c>
+      <c r="C36" s="4" t="inlineStr">
+        <is>
+          <t>Supabase PROD</t>
+        </is>
+      </c>
+      <c r="D36" s="4" t="inlineStr">
+        <is>
+          <t>Vérifier les tables codes et parrainages.</t>
+        </is>
+      </c>
+      <c r="E36" s="4" t="inlineStr">
+        <is>
+          <t>Tables présentes (créées le 05/10 sur les deux projets).</t>
+        </is>
+      </c>
+      <c r="F36" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G36" s="6" t="inlineStr">
+        <is>
+          <t>À tester</t>
+        </is>
+      </c>
+      <c r="H36" s="6" t="n"/>
+      <c r="I36" s="6" t="n"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="n">
+        <v>33</v>
+      </c>
+      <c r="B37" s="5" t="inlineStr">
+        <is>
+          <t>Règle de travail de décembre</t>
+        </is>
+      </c>
+      <c r="C37" s="4" t="inlineStr">
+        <is>
+          <t>CLAUDE.md</t>
+        </is>
+      </c>
+      <c r="D37" s="4" t="inlineStr">
+        <is>
+          <t>Après la mise en prod : retirer le paragraphe « Jusqu'à décembre 2026 ».</t>
+        </is>
+      </c>
+      <c r="E37" s="4" t="inlineStr">
+        <is>
+          <t>STA redevient identique à la PROD.</t>
+        </is>
+      </c>
+      <c r="F37" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G37" s="6" t="inlineStr">
+        <is>
+          <t>À tester</t>
+        </is>
+      </c>
+      <c r="H37" s="6" t="n"/>
+      <c r="I37" s="6" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -1633,7 +1818,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="G5:G32 G33" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="G5:G37" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"À tester,OK,KO,Non testable"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Recette : correctifs urgents et dernier message de démarrage ajoutés aux exceptions déjà en prod
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AUzY5Y8Bt2KRzzte5cJgH8
</commit_message>
<xml_diff>
--- a/docs/recette/Recette_prod_decembre_2026.xlsx
+++ b/docs/recette/Recette_prod_decembre_2026.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Recette décembre" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Déjà en prod (exceptions)" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Recette décembre" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Déjà en prod (exceptions)" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1832,7 +1832,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I7"/>
+  <dimension ref="A1:I10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -2030,6 +2030,129 @@
       </c>
       <c r="I7" s="6" t="n"/>
     </row>
+    <row r="8">
+      <c r="A8" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>Tonte bloquée sur herbe ou sol mouillés (correctif urgent)</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>Aujourd'hui, notifications, Bob, robot</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>Un jour de pluie, ou avec 2 mm prévus ou plus de 10 mm la veille : ouvrir « Aujourd'hui ».</t>
+        </is>
+      </c>
+      <c r="E8" s="4" t="inlineStr">
+        <is>
+          <t>Tonte non proposée, avec la raison (pluie, herbe mouillée, sol détrempé) ; pas de rappel de tonte ; robot invité au repos.</t>
+        </is>
+      </c>
+      <c r="F8" s="4" t="inlineStr">
+        <is>
+          <t>Tout compte</t>
+        </is>
+      </c>
+      <c r="G8" s="6" t="inlineStr">
+        <is>
+          <t>À tester</t>
+        </is>
+      </c>
+      <c r="H8" s="6" t="inlineStr">
+        <is>
+          <t>En prod le 07/10/2026 (correctif urgent).</t>
+        </is>
+      </c>
+      <c r="I8" s="6" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>Arrosage : pluie de la veille déduite (correctif urgent)</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>Aujourd'hui (arrosage, parcours semis), arrosage connecté</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>Le lendemain d'une pluie : ouvrir « Aujourd'hui ».</t>
+        </is>
+      </c>
+      <c r="E9" s="4" t="inlineStr">
+        <is>
+          <t>Dose réduite ou arrosage supprimé dès 8 mm cumulés (veille + jour) ; « Prévoir » affiche « Demain, selon la météo ».</t>
+        </is>
+      </c>
+      <c r="F9" s="4" t="inlineStr">
+        <is>
+          <t>Tout compte</t>
+        </is>
+      </c>
+      <c r="G9" s="6" t="inlineStr">
+        <is>
+          <t>À tester</t>
+        </is>
+      </c>
+      <c r="H9" s="6" t="inlineStr">
+        <is>
+          <t>En prod le 07/10/2026 (correctif urgent).</t>
+        </is>
+      </c>
+      <c r="I9" s="6" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>Démarrage : dernier message J+6 selon la situation</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>Email ou notification (tâche du matin)</t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="inlineStr">
+        <is>
+          <t>Suivre un inscrit jamais revenu jusqu'à J+6.</t>
+        </is>
+      </c>
+      <c r="E10" s="4" t="inlineStr">
+        <is>
+          <t>Message construit sur sa situation : zones à regarnir avec la fenêtre de semis de sa zone (ouverte ou prochaine date), autre problème du diagnostic, action du jour, ou invitation au diagnostic ; profil incomplet : plan à créer.</t>
+        </is>
+      </c>
+      <c r="F10" s="4" t="inlineStr">
+        <is>
+          <t>Nouvel inscrit</t>
+        </is>
+      </c>
+      <c r="G10" s="6" t="inlineStr">
+        <is>
+          <t>À tester</t>
+        </is>
+      </c>
+      <c r="H10" s="6" t="inlineStr">
+        <is>
+          <t>En prod le 08/10/2026 au soir (1er envoi : inscrit de Lamorlaye, le 09/10).</t>
+        </is>
+      </c>
+      <c r="I10" s="6" t="n"/>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A2:I2"/>
@@ -2043,7 +2166,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="G5:G6 G7" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="G5:G10" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"À tester,OK,KO,Non testable"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Station météo Netatmo : connexion, mesures du jardin et écran Mes équipements
- Connexion OAuth sur le site de Netatmo (lecture seule), retour par api/objets (aucun nouvel endpoint)
- Mesures du module extérieur, du pluviomètre et de l'anémomètre, ignorées au-delà de 3 h,
  appliquées à la météo du jour comme pour Ecowitt ; jeton renouvelé et réenregistré
- Retour « Connexion annulée » quand l'utilisateur refuse (Netatmo, Husqvarna, Gardena)
- Bob, confidentialité, CLAUDE.md et recette de décembre

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AUzY5Y8Bt2KRzzte5cJgH8
</commit_message>
<xml_diff>
--- a/docs/recette/Recette_prod_decembre_2026.xlsx
+++ b/docs/recette/Recette_prod_decembre_2026.xlsx
@@ -497,7 +497,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I37"/>
+  <dimension ref="A1:I42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -1700,27 +1700,27 @@
       </c>
       <c r="B35" s="5" t="inlineStr">
         <is>
-          <t>Alignement PROD / STA</t>
+          <t>Station Netatmo — connexion</t>
         </is>
       </c>
       <c r="C35" s="4" t="inlineStr">
         <is>
-          <t>Git</t>
+          <t>Mes équipements → Station météo</t>
         </is>
       </c>
       <c r="D35" s="4" t="inlineStr">
         <is>
-          <t>Après la fusion : git diff --quiet origin/main origin/Staging.</t>
+          <t>« Connecter ma station Netatmo » avec un compte Netatmo qui a un module extérieur ou un pluviomètre.</t>
         </is>
       </c>
       <c r="E35" s="4" t="inlineStr">
         <is>
-          <t>Aucune différence.</t>
+          <t>Retour sur Mes équipements avec « Station Netatmo connectée » ; carte avec température, pluie du jour et vent ; libellé « Netatmo ».</t>
         </is>
       </c>
       <c r="F35" s="4" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Compte avec station Netatmo (testeur à trouver)</t>
         </is>
       </c>
       <c r="G35" s="6" t="inlineStr">
@@ -1737,27 +1737,27 @@
       </c>
       <c r="B36" s="5" t="inlineStr">
         <is>
-          <t>Base de données PROD</t>
+          <t>Station Netatmo — mesures du jardin</t>
         </is>
       </c>
       <c r="C36" s="4" t="inlineStr">
         <is>
-          <t>Supabase PROD</t>
+          <t>Aujourd'hui, notifications, Bob</t>
         </is>
       </c>
       <c r="D36" s="4" t="inlineStr">
         <is>
-          <t>Vérifier les tables codes et parrainages.</t>
+          <t>Un jour de pluie, ouvrir « Aujourd'hui » et poser une question à Bob sur l'arrosage.</t>
         </is>
       </c>
       <c r="E36" s="4" t="inlineStr">
         <is>
-          <t>Tables présentes (créées le 05/10 sur les deux projets).</t>
+          <t>La pluie mesurée par la station est prise en compte (arrosage, tonte) ; Bob cite la mesure de la station ; relevé de moins de 10 min.</t>
         </is>
       </c>
       <c r="F36" s="4" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Compte avec station Netatmo</t>
         </is>
       </c>
       <c r="G36" s="6" t="inlineStr">
@@ -1774,27 +1774,27 @@
       </c>
       <c r="B37" s="5" t="inlineStr">
         <is>
-          <t>Règle de travail de décembre</t>
+          <t>Station Netatmo — connexion annulée</t>
         </is>
       </c>
       <c r="C37" s="4" t="inlineStr">
         <is>
-          <t>CLAUDE.md</t>
+          <t>Mes équipements</t>
         </is>
       </c>
       <c r="D37" s="4" t="inlineStr">
         <is>
-          <t>Après la mise en prod : retirer le paragraphe « Jusqu'à décembre 2026 ».</t>
+          <t>Cliquer « Connecter ma station Netatmo », puis refuser l'accès sur le site de Netatmo.</t>
         </is>
       </c>
       <c r="E37" s="4" t="inlineStr">
         <is>
-          <t>STA redevient identique à la PROD.</t>
+          <t>Message « Connexion annulée : rien n'a été enregistré » (même chose pour Husqvarna et Gardena).</t>
         </is>
       </c>
       <c r="F37" s="4" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Tout compte</t>
         </is>
       </c>
       <c r="G37" s="6" t="inlineStr">
@@ -1804,6 +1804,191 @@
       </c>
       <c r="H37" s="6" t="n"/>
       <c r="I37" s="6" t="n"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="n">
+        <v>34</v>
+      </c>
+      <c r="B38" s="5" t="inlineStr">
+        <is>
+          <t>Station Netatmo — déconnexion</t>
+        </is>
+      </c>
+      <c r="C38" s="4" t="inlineStr">
+        <is>
+          <t>Mes équipements</t>
+        </is>
+      </c>
+      <c r="D38" s="4" t="inlineStr">
+        <is>
+          <t>« Déconnecter la station ».</t>
+        </is>
+      </c>
+      <c r="E38" s="4" t="inlineStr">
+        <is>
+          <t>La station disparaît ; « Aujourd'hui » repart sur les prévisions météo.</t>
+        </is>
+      </c>
+      <c r="F38" s="4" t="inlineStr">
+        <is>
+          <t>Compte avec station Netatmo</t>
+        </is>
+      </c>
+      <c r="G38" s="6" t="inlineStr">
+        <is>
+          <t>À tester</t>
+        </is>
+      </c>
+      <c r="H38" s="6" t="n"/>
+      <c r="I38" s="6" t="n"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="n">
+        <v>35</v>
+      </c>
+      <c r="B39" s="5" t="inlineStr">
+        <is>
+          <t>Station Netatmo — réglages PROD</t>
+        </is>
+      </c>
+      <c r="C39" s="4" t="inlineStr">
+        <is>
+          <t>Application Netatmo (dev.netatmo.com) et Vercel</t>
+        </is>
+      </c>
+      <c r="D39" s="4" t="inlineStr">
+        <is>
+          <t>Vérifier l'adresse de retour déclarée dans l'application Netatmo et les variables Vercel.</t>
+        </is>
+      </c>
+      <c r="E39" s="4" t="inlineStr">
+        <is>
+          <t>Adresse de retour https://mongazon360.fr/api/objets ; NETATMO_CLIENT_ID et NETATMO_CLIENT_SECRET présentes en Production.</t>
+        </is>
+      </c>
+      <c r="F39" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G39" s="6" t="inlineStr">
+        <is>
+          <t>À tester</t>
+        </is>
+      </c>
+      <c r="H39" s="6" t="n"/>
+      <c r="I39" s="6" t="n"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="n">
+        <v>36</v>
+      </c>
+      <c r="B40" s="5" t="inlineStr">
+        <is>
+          <t>Alignement PROD / STA</t>
+        </is>
+      </c>
+      <c r="C40" s="4" t="inlineStr">
+        <is>
+          <t>Git</t>
+        </is>
+      </c>
+      <c r="D40" s="4" t="inlineStr">
+        <is>
+          <t>Après la fusion : git diff --quiet origin/main origin/Staging.</t>
+        </is>
+      </c>
+      <c r="E40" s="4" t="inlineStr">
+        <is>
+          <t>Aucune différence.</t>
+        </is>
+      </c>
+      <c r="F40" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G40" s="6" t="inlineStr">
+        <is>
+          <t>À tester</t>
+        </is>
+      </c>
+      <c r="H40" s="6" t="n"/>
+      <c r="I40" s="6" t="n"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="4" t="n">
+        <v>37</v>
+      </c>
+      <c r="B41" s="5" t="inlineStr">
+        <is>
+          <t>Base de données PROD</t>
+        </is>
+      </c>
+      <c r="C41" s="4" t="inlineStr">
+        <is>
+          <t>Supabase PROD</t>
+        </is>
+      </c>
+      <c r="D41" s="4" t="inlineStr">
+        <is>
+          <t>Vérifier les tables codes et parrainages.</t>
+        </is>
+      </c>
+      <c r="E41" s="4" t="inlineStr">
+        <is>
+          <t>Tables présentes (créées le 05/10 sur les deux projets).</t>
+        </is>
+      </c>
+      <c r="F41" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G41" s="6" t="inlineStr">
+        <is>
+          <t>À tester</t>
+        </is>
+      </c>
+      <c r="H41" s="6" t="n"/>
+      <c r="I41" s="6" t="n"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="4" t="n">
+        <v>38</v>
+      </c>
+      <c r="B42" s="5" t="inlineStr">
+        <is>
+          <t>Règle de travail de décembre</t>
+        </is>
+      </c>
+      <c r="C42" s="4" t="inlineStr">
+        <is>
+          <t>CLAUDE.md</t>
+        </is>
+      </c>
+      <c r="D42" s="4" t="inlineStr">
+        <is>
+          <t>Après la mise en prod : retirer le paragraphe « Jusqu'à décembre 2026 ».</t>
+        </is>
+      </c>
+      <c r="E42" s="4" t="inlineStr">
+        <is>
+          <t>STA redevient identique à la PROD.</t>
+        </is>
+      </c>
+      <c r="F42" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G42" s="6" t="inlineStr">
+        <is>
+          <t>À tester</t>
+        </is>
+      </c>
+      <c r="H42" s="6" t="n"/>
+      <c r="I42" s="6" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -1818,7 +2003,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="G5:G37" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="G5:G42" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"À tester,OK,KO,Non testable"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Recette : météo des comptes gratuits et textes sans « IA » validés sur STA le 09/10
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AUzY5Y8Bt2KRzzte5cJgH8
</commit_message>
<xml_diff>
--- a/docs/recette/Recette_prod_decembre_2026.xlsx
+++ b/docs/recette/Recette_prod_decembre_2026.xlsx
@@ -1173,7 +1173,11 @@
           <t>À tester</t>
         </is>
       </c>
-      <c r="H20" s="6" t="n"/>
+      <c r="H20" s="6" t="inlineStr">
+        <is>
+          <t>Validé sur STA le 09/10/2026 par Jordan ; à revérifier en prod.</t>
+        </is>
+      </c>
       <c r="I20" s="6" t="n"/>
     </row>
     <row r="21">
@@ -1210,7 +1214,11 @@
           <t>À tester</t>
         </is>
       </c>
-      <c r="H21" s="6" t="n"/>
+      <c r="H21" s="6" t="inlineStr">
+        <is>
+          <t>Validé sur STA le 09/10/2026 par Jordan ; à revérifier en prod.</t>
+        </is>
+      </c>
       <c r="I21" s="6" t="n"/>
     </row>
     <row r="22">
@@ -1247,7 +1255,11 @@
           <t>À tester</t>
         </is>
       </c>
-      <c r="H22" s="6" t="n"/>
+      <c r="H22" s="6" t="inlineStr">
+        <is>
+          <t>Validé sur STA le 09/10/2026 par Jordan ; à revérifier en prod.</t>
+        </is>
+      </c>
       <c r="I22" s="6" t="n"/>
     </row>
     <row r="23">
@@ -1284,7 +1296,11 @@
           <t>À tester</t>
         </is>
       </c>
-      <c r="H23" s="6" t="n"/>
+      <c r="H23" s="6" t="inlineStr">
+        <is>
+          <t>Validé sur STA le 09/10/2026 par Jordan ; à revérifier en prod.</t>
+        </is>
+      </c>
       <c r="I23" s="6" t="n"/>
     </row>
     <row r="24">
@@ -1321,7 +1337,11 @@
           <t>À tester</t>
         </is>
       </c>
-      <c r="H24" s="6" t="n"/>
+      <c r="H24" s="6" t="inlineStr">
+        <is>
+          <t>Validé sur STA le 09/10/2026 par Jordan ; à revérifier en prod.</t>
+        </is>
+      </c>
       <c r="I24" s="6" t="n"/>
     </row>
     <row r="25">
@@ -1358,7 +1378,11 @@
           <t>À tester</t>
         </is>
       </c>
-      <c r="H25" s="6" t="n"/>
+      <c r="H25" s="6" t="inlineStr">
+        <is>
+          <t>Validé sur STA le 09/10/2026 par Jordan ; à revérifier en prod.</t>
+        </is>
+      </c>
       <c r="I25" s="6" t="n"/>
     </row>
     <row r="26">
@@ -1395,7 +1419,11 @@
           <t>À tester</t>
         </is>
       </c>
-      <c r="H26" s="6" t="n"/>
+      <c r="H26" s="6" t="inlineStr">
+        <is>
+          <t>Validé sur STA le 09/10/2026 par Jordan ; à revérifier en prod.</t>
+        </is>
+      </c>
       <c r="I26" s="6" t="n"/>
     </row>
     <row r="27">
@@ -1432,7 +1460,11 @@
           <t>À tester</t>
         </is>
       </c>
-      <c r="H27" s="6" t="n"/>
+      <c r="H27" s="6" t="inlineStr">
+        <is>
+          <t>Validé sur STA le 09/10/2026 par Jordan ; à revérifier en prod.</t>
+        </is>
+      </c>
       <c r="I27" s="6" t="n"/>
     </row>
     <row r="28">

</xml_diff>

<commit_message>
Recette : affichage de la raison de tonte (en prod le 09/10) ajouté au correctif urgent
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AUzY5Y8Bt2KRzzte5cJgH8
</commit_message>
<xml_diff>
--- a/docs/recette/Recette_prod_decembre_2026.xlsx
+++ b/docs/recette/Recette_prod_decembre_2026.xlsx
@@ -2268,7 +2268,7 @@
       </c>
       <c r="E8" s="4" t="inlineStr">
         <is>
-          <t>Tonte non proposée, avec la raison (pluie, herbe mouillée, sol détrempé) ; pas de rappel de tonte ; robot invité au repos.</t>
+          <t>Tonte non proposée ; dans « Prévoir », étiquette courte (« Il pleut aujourd'hui », « Pluie prévue », « Sol détrempé ») et explication en dessous, sans débordement ; pas de rappel de tonte ; robot invité au repos.</t>
         </is>
       </c>
       <c r="F8" s="4" t="inlineStr">
@@ -2283,7 +2283,7 @@
       </c>
       <c r="H8" s="6" t="inlineStr">
         <is>
-          <t>En prod le 07/10/2026 (correctif urgent).</t>
+          <t>En prod le 07/10/2026 (correctif urgent) ; affichage corrigé le 09/10/2026.</t>
         </is>
       </c>
       <c r="I8" s="6" t="n"/>

</xml_diff>

<commit_message>
Automower : hauteur de coupe en cm et proposition de réglage selon la saison
- Niveau 1-9 de l'API converti en cm selon la plage du modèle (src/lib/automowerHauteurs.json)
- Les jours où la tonte est possible, proposition d'ajuster la coupe au milieu de la hauteur de la
  saison (Tonte Précise, +1 cm en objectif naturel), bornée à la plage du robot ; commande envoyée
  seulement après validation (POST mowers/{id}/settings) ; modèles manuels et SILENO exclus
- Hauteur de la saison calculée à un seul endroit (plan d'entretien, carte du robot, proposition)
- Bob, confidentialité, CLAUDE.md et recette de décembre

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AUzY5Y8Bt2KRzzte5cJgH8
</commit_message>
<xml_diff>
--- a/docs/recette/Recette_prod_decembre_2026.xlsx
+++ b/docs/recette/Recette_prod_decembre_2026.xlsx
@@ -497,7 +497,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I42"/>
+  <dimension ref="A1:I46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -1917,27 +1917,27 @@
       </c>
       <c r="B40" s="5" t="inlineStr">
         <is>
-          <t>Alignement PROD / STA</t>
+          <t>Automower — hauteur en cm</t>
         </is>
       </c>
       <c r="C40" s="4" t="inlineStr">
         <is>
-          <t>Git</t>
+          <t>Mes équipements, Aujourd'hui (carte du robot)</t>
         </is>
       </c>
       <c r="D40" s="4" t="inlineStr">
         <is>
-          <t>Après la fusion : git diff --quiet origin/main origin/Staging.</t>
+          <t>Ouvrir la carte d'un Automower à réglage électrique (ex. 430X).</t>
         </is>
       </c>
       <c r="E40" s="4" t="inlineStr">
         <is>
-          <t>Aucune différence.</t>
+          <t>« Réglage actuel du robot : X cm (niveau N) » ; hauteur conseillée de la saison affichée au-dessus.</t>
         </is>
       </c>
       <c r="F40" s="4" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Compte avec Automower (testeur à trouver)</t>
         </is>
       </c>
       <c r="G40" s="6" t="inlineStr">
@@ -1954,27 +1954,27 @@
       </c>
       <c r="B41" s="5" t="inlineStr">
         <is>
-          <t>Base de données PROD</t>
+          <t>Automower — proposition de hauteur</t>
         </is>
       </c>
       <c r="C41" s="4" t="inlineStr">
         <is>
-          <t>Supabase PROD</t>
+          <t>Aujourd'hui (carte du robot)</t>
         </is>
       </c>
       <c r="D41" s="4" t="inlineStr">
         <is>
-          <t>Vérifier les tables codes et parrainages.</t>
+          <t>Un jour où la tonte est possible, avec un robot réglé loin de la hauteur de la saison.</t>
         </is>
       </c>
       <c r="E41" s="4" t="inlineStr">
         <is>
-          <t>Tables présentes (créées le 05/10 sur les deux projets).</t>
+          <t>Proposition « 📏 Régler la coupe sur X cm » avec la raison (hauteur de la saison, réglage actuel, limite du robot) ; rien n'est envoyé sans clic.</t>
         </is>
       </c>
       <c r="F41" s="4" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Compte avec Automower</t>
         </is>
       </c>
       <c r="G41" s="6" t="inlineStr">
@@ -1991,27 +1991,27 @@
       </c>
       <c r="B42" s="5" t="inlineStr">
         <is>
-          <t>Règle de travail de décembre</t>
+          <t>Automower — réglage envoyé</t>
         </is>
       </c>
       <c r="C42" s="4" t="inlineStr">
         <is>
-          <t>CLAUDE.md</t>
+          <t>Aujourd'hui → app Automower Connect</t>
         </is>
       </c>
       <c r="D42" s="4" t="inlineStr">
         <is>
-          <t>Après la mise en prod : retirer le paragraphe « Jusqu'à décembre 2026 ».</t>
+          <t>Valider la proposition, puis regarder la hauteur dans l'app Automower Connect.</t>
         </is>
       </c>
       <c r="E42" s="4" t="inlineStr">
         <is>
-          <t>STA redevient identique à la PROD.</t>
+          <t>Hauteur changée sur le robot ; la proposition disparaît au rafraîchissement.</t>
         </is>
       </c>
       <c r="F42" s="4" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Compte avec Automower</t>
         </is>
       </c>
       <c r="G42" s="6" t="inlineStr">
@@ -2021,6 +2021,154 @@
       </c>
       <c r="H42" s="6" t="n"/>
       <c r="I42" s="6" t="n"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="4" t="n">
+        <v>39</v>
+      </c>
+      <c r="B43" s="5" t="inlineStr">
+        <is>
+          <t>Automower — priorités et modèles sans réglage</t>
+        </is>
+      </c>
+      <c r="C43" s="4" t="inlineStr">
+        <is>
+          <t>Aujourd'hui</t>
+        </is>
+      </c>
+      <c r="D43" s="4" t="inlineStr">
+        <is>
+          <t>Un jour de pluie ; puis un robot à réglage manuel (305, Mark II) ou un Gardena SILENO.</t>
+        </is>
+      </c>
+      <c r="E43" s="4" t="inlineStr">
+        <is>
+          <t>Pluie : proposition de repos, pas de hauteur ; réglage manuel ou Gardena : aucune proposition de hauteur.</t>
+        </is>
+      </c>
+      <c r="F43" s="4" t="inlineStr">
+        <is>
+          <t>Compte avec Automower ou SILENO</t>
+        </is>
+      </c>
+      <c r="G43" s="6" t="inlineStr">
+        <is>
+          <t>À tester</t>
+        </is>
+      </c>
+      <c r="H43" s="6" t="n"/>
+      <c r="I43" s="6" t="n"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="4" t="n">
+        <v>40</v>
+      </c>
+      <c r="B44" s="5" t="inlineStr">
+        <is>
+          <t>Alignement PROD / STA</t>
+        </is>
+      </c>
+      <c r="C44" s="4" t="inlineStr">
+        <is>
+          <t>Git</t>
+        </is>
+      </c>
+      <c r="D44" s="4" t="inlineStr">
+        <is>
+          <t>Après la fusion : git diff --quiet origin/main origin/Staging.</t>
+        </is>
+      </c>
+      <c r="E44" s="4" t="inlineStr">
+        <is>
+          <t>Aucune différence.</t>
+        </is>
+      </c>
+      <c r="F44" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G44" s="6" t="inlineStr">
+        <is>
+          <t>À tester</t>
+        </is>
+      </c>
+      <c r="H44" s="6" t="n"/>
+      <c r="I44" s="6" t="n"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="4" t="n">
+        <v>41</v>
+      </c>
+      <c r="B45" s="5" t="inlineStr">
+        <is>
+          <t>Base de données PROD</t>
+        </is>
+      </c>
+      <c r="C45" s="4" t="inlineStr">
+        <is>
+          <t>Supabase PROD</t>
+        </is>
+      </c>
+      <c r="D45" s="4" t="inlineStr">
+        <is>
+          <t>Vérifier les tables codes et parrainages.</t>
+        </is>
+      </c>
+      <c r="E45" s="4" t="inlineStr">
+        <is>
+          <t>Tables présentes (créées le 05/10 sur les deux projets).</t>
+        </is>
+      </c>
+      <c r="F45" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G45" s="6" t="inlineStr">
+        <is>
+          <t>À tester</t>
+        </is>
+      </c>
+      <c r="H45" s="6" t="n"/>
+      <c r="I45" s="6" t="n"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="4" t="n">
+        <v>42</v>
+      </c>
+      <c r="B46" s="5" t="inlineStr">
+        <is>
+          <t>Règle de travail de décembre</t>
+        </is>
+      </c>
+      <c r="C46" s="4" t="inlineStr">
+        <is>
+          <t>CLAUDE.md</t>
+        </is>
+      </c>
+      <c r="D46" s="4" t="inlineStr">
+        <is>
+          <t>Après la mise en prod : retirer le paragraphe « Jusqu'à décembre 2026 ».</t>
+        </is>
+      </c>
+      <c r="E46" s="4" t="inlineStr">
+        <is>
+          <t>STA redevient identique à la PROD.</t>
+        </is>
+      </c>
+      <c r="F46" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G46" s="6" t="inlineStr">
+        <is>
+          <t>À tester</t>
+        </is>
+      </c>
+      <c r="H46" s="6" t="n"/>
+      <c r="I46" s="6" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -2035,7 +2183,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="G5:G42" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="G5:G46" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"À tester,OK,KO,Non testable"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Recette : mesure des pages et des tuiles (en prod le 09/10) ajoutée aux exceptions déjà en prod
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AUzY5Y8Bt2KRzzte5cJgH8
</commit_message>
<xml_diff>
--- a/docs/recette/Recette_prod_decembre_2026.xlsx
+++ b/docs/recette/Recette_prod_decembre_2026.xlsx
@@ -2197,7 +2197,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I10"/>
+  <dimension ref="A1:I11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -2517,6 +2517,49 @@
         </is>
       </c>
       <c r="I10" s="6" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>Mesure anonyme des pages et des tuiles</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>Toute l'app (accueil, Aujourd'hui, Mon gazon, badges, Bob)</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="inlineStr">
+        <is>
+          <t>Après quelques jours : compter les lignes « page_view » et « tuile » de funnel_events (niveau visiteur, gratuit ou premium).</t>
+        </is>
+      </c>
+      <c r="E11" s="4" t="inlineStr">
+        <is>
+          <t>Une ligne par page ouverte et par tuile touchée, sans identifiant ; aucune ligne pour un compte admin.</t>
+        </is>
+      </c>
+      <c r="F11" s="4" t="inlineStr">
+        <is>
+          <t>Visiteur et compte gratuit</t>
+        </is>
+      </c>
+      <c r="G11" s="6" t="inlineStr">
+        <is>
+          <t>À tester</t>
+        </is>
+      </c>
+      <c r="H11" s="6" t="inlineStr">
+        <is>
+          <t>En prod le 09/10/2026 (exception confirmée par Jordan) ; visite de test du 09/10 enregistrée (« page_view », visiteur).</t>
+        </is>
+      </c>
+      <c r="I11" s="6" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>

<commit_message>
Recette et journal : articles Conseils mis en prod le 10/10 (exception confirmée par Jordan)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AUzY5Y8Bt2KRzzte5cJgH8
</commit_message>
<xml_diff>
--- a/docs/recette/Recette_prod_decembre_2026.xlsx
+++ b/docs/recette/Recette_prod_decembre_2026.xlsx
@@ -2197,7 +2197,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I11"/>
+  <dimension ref="A1:I12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -2560,6 +2560,47 @@
         </is>
       </c>
       <c r="I11" s="6" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>Articles Conseils retravaillés pour Google : chaulage, engrais d'automne, carottage</t>
+        </is>
+      </c>
+      <c r="C12" s="4" t="inlineStr">
+        <is>
+          <t>Site (/conseils/chaulage-ph-pelouse, /conseils/engrais-gazon-automne, /conseils/aerer-pelouse-carottage)</t>
+        </is>
+      </c>
+      <c r="D12" s="4" t="inlineStr">
+        <is>
+          <t>Ouvrir les 3 articles sur téléphone ; dans la Search Console, inspecter les 3 adresses et demander une indexation.</t>
+        </is>
+      </c>
+      <c r="E12" s="4" t="inlineStr">
+        <is>
+          <t>Nouveaux titres, encadré « En bref » en tête, questions fréquentes en fin d'article, liens entre articles, « Mis à jour le 10 octobre 2026 ».</t>
+        </is>
+      </c>
+      <c r="F12" s="4" t="inlineStr">
+        <is>
+          <t>Visiteur</t>
+        </is>
+      </c>
+      <c r="G12" s="6" t="inlineStr">
+        <is>
+          <t>À tester</t>
+        </is>
+      </c>
+      <c r="H12" s="6" t="inlineStr">
+        <is>
+          <t>En prod le 10/10/2026 (exception articles Conseils confirmée par Jordan).</t>
+        </is>
+      </c>
+      <c r="I12" s="6" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>

<commit_message>
Règles, recette et journal : accord permanent pour les articles Conseils, 4 articles mis en prod le 10/10
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AUzY5Y8Bt2KRzzte5cJgH8
</commit_message>
<xml_diff>
--- a/docs/recette/Recette_prod_decembre_2026.xlsx
+++ b/docs/recette/Recette_prod_decembre_2026.xlsx
@@ -2197,7 +2197,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I12"/>
+  <dimension ref="A1:I13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -2601,6 +2601,47 @@
         </is>
       </c>
       <c r="I12" s="6" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>Articles Conseils retravaillés pour Google : mousse, feuilles mortes, entretien d'hiver, hivernage du matériel</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="inlineStr">
+        <is>
+          <t>Site (/conseils/mousse-pelouse, /conseils/feuilles-mortes-pelouse, /conseils/preparer-gazon-hiver, /conseils/hiverner-tondeuse-robot-arrosage)</t>
+        </is>
+      </c>
+      <c r="D13" s="4" t="inlineStr">
+        <is>
+          <t>Ouvrir les 4 articles sur téléphone ; dans la Search Console, inspecter les 4 adresses et demander une indexation.</t>
+        </is>
+      </c>
+      <c r="E13" s="4" t="inlineStr">
+        <is>
+          <t>Nouveaux titres, encadré « En bref » en tête, questions fréquentes en fin d'article, liens entre articles, « Mis à jour le 10 octobre 2026 ».</t>
+        </is>
+      </c>
+      <c r="F13" s="4" t="inlineStr">
+        <is>
+          <t>Visiteur</t>
+        </is>
+      </c>
+      <c r="G13" s="6" t="inlineStr">
+        <is>
+          <t>À tester</t>
+        </is>
+      </c>
+      <c r="H13" s="6" t="inlineStr">
+        <is>
+          <t>En prod le 10/10/2026 (accord permanent de Jordan pour les articles Conseils).</t>
+        </is>
+      </c>
+      <c r="I13" s="6" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>

<commit_message>
Suivi des articles Conseils du 11/10 : journal, recette, consignes de Bob
Journal (décision de Jordan, 21 nouveaux articles et 11 retravaillés), lignes 10 et 11 de la recette
« Déjà en prod (exceptions) », et consignes de Bob sans nombre d'articles figé (la liste réelle suit).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AUzY5Y8Bt2KRzzte5cJgH8
</commit_message>
<xml_diff>
--- a/docs/recette/Recette_prod_decembre_2026.xlsx
+++ b/docs/recette/Recette_prod_decembre_2026.xlsx
@@ -2197,7 +2197,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I13"/>
+  <dimension ref="A1:I15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -2642,6 +2642,88 @@
         </is>
       </c>
       <c r="I13" s="6" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>Nouveaux articles Conseils (8) et 4 articles retravaillés : calendrier mois par mois, dernière tonte, vers blancs, maladies du gazon, taupes, engrais (4 apports), choix du gazon, dates de semis par région ; regarnissage, gel, scarification, robot tondeuse</t>
+        </is>
+      </c>
+      <c r="C14" s="4" t="inlineStr">
+        <is>
+          <t>Site (/conseils et les 12 articles)</t>
+        </is>
+      </c>
+      <c r="D14" s="4" t="inlineStr">
+        <is>
+          <t>Ouvrir la rubrique et 2 ou 3 nouveaux articles sur téléphone ; dans la Search Console, demander l'indexation des 8 nouvelles adresses ; dans Bing Webmaster Tools (menu IndexNow), vérifier les pages reçues.</t>
+        </is>
+      </c>
+      <c r="E14" s="4" t="inlineStr">
+        <is>
+          <t>Pages en ligne, tableaux lisibles sur téléphone, encadré « En bref », questions fréquentes, liens entre articles ; plan du site à jour.</t>
+        </is>
+      </c>
+      <c r="F14" s="4" t="inlineStr">
+        <is>
+          <t>Visiteur</t>
+        </is>
+      </c>
+      <c r="G14" s="6" t="inlineStr">
+        <is>
+          <t>À tester</t>
+        </is>
+      </c>
+      <c r="H14" s="6" t="inlineStr">
+        <is>
+          <t>En prod le 11/10/2026 (décision de Jordan : tous les articles utiles au référencement, accord permanent pour les articles Conseils).</t>
+        </is>
+      </c>
+      <c r="I14" s="6" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="n">
+        <v>11</v>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>Nouveaux articles Conseils (13) et 7 articles retravaillés : préparer au printemps, engrais de printemps, créer, rénover, temps de pousse, quand tondre, ombre, arrosage automatique, sulfate de fer, sol calcaire, pelouse naturelle, fourmis, biostimulant ; semis de printemps, 1re tonte, hauteur de tonte, pelouse jaune, arrosage, canicule, désherbage</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t>Site (/conseils et les 20 articles)</t>
+        </is>
+      </c>
+      <c r="D15" s="4" t="inlineStr">
+        <is>
+          <t>Ouvrir 2 ou 3 nouveaux articles sur téléphone ; dans la Search Console, demander l'indexation des 13 nouvelles adresses.</t>
+        </is>
+      </c>
+      <c r="E15" s="4" t="inlineStr">
+        <is>
+          <t>Pages en ligne, encadré « En bref », questions fréquentes, liens entre articles ; 39 articles dans la rubrique et le plan du site.</t>
+        </is>
+      </c>
+      <c r="F15" s="4" t="inlineStr">
+        <is>
+          <t>Visiteur</t>
+        </is>
+      </c>
+      <c r="G15" s="6" t="inlineStr">
+        <is>
+          <t>À tester</t>
+        </is>
+      </c>
+      <c r="H15" s="6" t="inlineStr">
+        <is>
+          <t>En prod le 11/10/2026 (même décision).</t>
+        </is>
+      </c>
+      <c r="I15" s="6" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>

<commit_message>
Recette et journal du 11/10 : réglages techniques du référencement et 3 sujets de la base
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AUzY5Y8Bt2KRzzte5cJgH8
</commit_message>
<xml_diff>
--- a/docs/recette/Recette_prod_decembre_2026.xlsx
+++ b/docs/recette/Recette_prod_decembre_2026.xlsx
@@ -2197,7 +2197,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I15"/>
+  <dimension ref="A1:I17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -2724,6 +2724,88 @@
         </is>
       </c>
       <c r="I15" s="6" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>Référencement : grand aperçu des images (max-image-preview), photos d'articles, page « Qui sommes-nous », « À lire aussi » par sujet</t>
+        </is>
+      </c>
+      <c r="C16" s="4" t="inlineStr">
+        <is>
+          <t>Site (/a-propos, /conseils/renover-pelouse, /conseils/regarnir-gazon-automne, /conseils/calendrier-entretien-pelouse, pied de page des articles)</t>
+        </is>
+      </c>
+      <c r="D16" s="4" t="inlineStr">
+        <is>
+          <t>Sur téléphone : ouvrir les 3 articles avec photo et la page « Qui sommes-nous » ; partager un article sur WhatsApp ; vérifier le lien « l'équipe Mongazon360 » sous le titre et « Qui sommes-nous » en pied de page ; lire « À lire aussi » en bas d'un article.</t>
+        </is>
+      </c>
+      <c r="E16" s="4" t="inlineStr">
+        <is>
+          <t>Photo en tête et avant/après lisibles, pas de décalage à l'affichage ; l'aperçu de partage montre la photo de l'article ; « À lire aussi » propose des articles du même sujet ; page « Qui sommes-nous » complète.</t>
+        </is>
+      </c>
+      <c r="F16" s="4" t="inlineStr">
+        <is>
+          <t>Visiteur</t>
+        </is>
+      </c>
+      <c r="G16" s="6" t="inlineStr">
+        <is>
+          <t>À tester</t>
+        </is>
+      </c>
+      <c r="H16" s="6" t="inlineStr">
+        <is>
+          <t>En prod le 11/10/2026 (go prod de Jordan : réglages techniques).</t>
+        </is>
+      </c>
+      <c r="I16" s="6" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="n">
+        <v>13</v>
+      </c>
+      <c r="B17" s="5" t="inlineStr">
+        <is>
+          <t>Base de connaissances : sujets complémentaires (champignons et ronds de sorcière, gazon en plaques, mulching) et 3 nouveaux articles</t>
+        </is>
+      </c>
+      <c r="C17" s="4" t="inlineStr">
+        <is>
+          <t>Site (/conseils/champignons-pelouse, /conseils/gazon-en-plaques, /conseils/mulching-pelouse) ; base docs/kb</t>
+        </is>
+      </c>
+      <c r="D17" s="4" t="inlineStr">
+        <is>
+          <t>Ouvrir les 3 articles sur téléphone ; relire l'onglet « Sujets complémentaires » de la base.</t>
+        </is>
+      </c>
+      <c r="E17" s="4" t="inlineStr">
+        <is>
+          <t>Articles en ligne, cohérents avec la base ; encadré « En bref », questions fréquentes, liens depuis pelouse jaune, maladies, hauteur de tonte, robot, création.</t>
+        </is>
+      </c>
+      <c r="F17" s="4" t="inlineStr">
+        <is>
+          <t>Visiteur</t>
+        </is>
+      </c>
+      <c r="G17" s="6" t="inlineStr">
+        <is>
+          <t>À tester</t>
+        </is>
+      </c>
+      <c r="H17" s="6" t="inlineStr">
+        <is>
+          <t>En prod le 11/10/2026 (sujets validés par Jordan).</t>
+        </is>
+      </c>
+      <c r="I17" s="6" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>

<commit_message>
Pilotage : position moyenne sur Google, par mois (onglet Activité)
Carte « Position moyenne sur Google — par mois » : courbe à axe inversé (1 en haut, repères 3 et 10),
valeur du dernier mois et évolution sur un mois, détail au toucher, tableau des mois avec affichages et
clics. Données de la Search Console lues par /api/stats?type=seo (admin), moyenne des positions
quotidiennes pondérée par les affichages, 16 mois au plus. Jeton et calcul dans api/searchConsole.cjs,
partagé avec scripts/gsc-stats.mjs. Clé GSC_SERVICE_ACCOUNT_JSON à ajouter dans Vercel.
Recette de décembre n° 40, CLAUDE.md et journal du 11/10.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AUzY5Y8Bt2KRzzte5cJgH8
</commit_message>
<xml_diff>
--- a/docs/recette/Recette_prod_decembre_2026.xlsx
+++ b/docs/recette/Recette_prod_decembre_2026.xlsx
@@ -497,7 +497,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I46"/>
+  <dimension ref="A1:I47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -525,6 +525,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -2065,27 +2066,27 @@
       </c>
       <c r="B44" s="5" t="inlineStr">
         <is>
-          <t>Alignement PROD / STA</t>
+          <t>Pilotage — position moyenne sur Google par mois</t>
         </is>
       </c>
       <c r="C44" s="4" t="inlineStr">
         <is>
-          <t>Git</t>
+          <t>Pilotage → Activité (carte « Position moyenne sur Google »)</t>
         </is>
       </c>
       <c r="D44" s="4" t="inlineStr">
         <is>
-          <t>Après la fusion : git diff --quiet origin/main origin/Staging.</t>
+          <t>Ouvrir Pilotage → Activité ; lire la carte, toucher un point du graphique. Prérequis : variable Vercel GSC_SERVICE_ACCOUNT_JSON (Production et Preview).</t>
         </is>
       </c>
       <c r="E44" s="4" t="inlineStr">
         <is>
-          <t>Aucune différence.</t>
+          <t>Courbe par mois (axe inversé, 1 en haut), valeur du dernier mois et évolution sur un mois, détail au toucher, tableau des mois ; mêmes chiffres que la Search Console (Performances, position moyenne par mois).</t>
         </is>
       </c>
       <c r="F44" s="4" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Admin</t>
         </is>
       </c>
       <c r="G44" s="6" t="inlineStr">
@@ -2093,7 +2094,11 @@
           <t>À tester</t>
         </is>
       </c>
-      <c r="H44" s="6" t="n"/>
+      <c r="H44" s="6" t="inlineStr">
+        <is>
+          <t>Sur STA le 11/10/2026 (demande de Jordan).</t>
+        </is>
+      </c>
       <c r="I44" s="6" t="n"/>
     </row>
     <row r="45">
@@ -2102,22 +2107,22 @@
       </c>
       <c r="B45" s="5" t="inlineStr">
         <is>
-          <t>Base de données PROD</t>
+          <t>Alignement PROD / STA</t>
         </is>
       </c>
       <c r="C45" s="4" t="inlineStr">
         <is>
-          <t>Supabase PROD</t>
+          <t>Git</t>
         </is>
       </c>
       <c r="D45" s="4" t="inlineStr">
         <is>
-          <t>Vérifier les tables codes et parrainages.</t>
+          <t>Après la fusion : git diff --quiet origin/main origin/Staging.</t>
         </is>
       </c>
       <c r="E45" s="4" t="inlineStr">
         <is>
-          <t>Tables présentes (créées le 05/10 sur les deux projets).</t>
+          <t>Aucune différence.</t>
         </is>
       </c>
       <c r="F45" s="4" t="inlineStr">
@@ -2139,22 +2144,22 @@
       </c>
       <c r="B46" s="5" t="inlineStr">
         <is>
-          <t>Règle de travail de décembre</t>
+          <t>Base de données PROD</t>
         </is>
       </c>
       <c r="C46" s="4" t="inlineStr">
         <is>
-          <t>CLAUDE.md</t>
+          <t>Supabase PROD</t>
         </is>
       </c>
       <c r="D46" s="4" t="inlineStr">
         <is>
-          <t>Après la mise en prod : retirer le paragraphe « Jusqu'à décembre 2026 ».</t>
+          <t>Vérifier les tables codes et parrainages.</t>
         </is>
       </c>
       <c r="E46" s="4" t="inlineStr">
         <is>
-          <t>STA redevient identique à la PROD.</t>
+          <t>Tables présentes (créées le 05/10 sur les deux projets).</t>
         </is>
       </c>
       <c r="F46" s="4" t="inlineStr">
@@ -2169,6 +2174,43 @@
       </c>
       <c r="H46" s="6" t="n"/>
       <c r="I46" s="6" t="n"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="4" t="n">
+        <v>43</v>
+      </c>
+      <c r="B47" s="5" t="inlineStr">
+        <is>
+          <t>Règle de travail de décembre</t>
+        </is>
+      </c>
+      <c r="C47" s="4" t="inlineStr">
+        <is>
+          <t>CLAUDE.md</t>
+        </is>
+      </c>
+      <c r="D47" s="4" t="inlineStr">
+        <is>
+          <t>Après la mise en prod : retirer le paragraphe « Jusqu'à décembre 2026 ».</t>
+        </is>
+      </c>
+      <c r="E47" s="4" t="inlineStr">
+        <is>
+          <t>STA redevient identique à la PROD.</t>
+        </is>
+      </c>
+      <c r="F47" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G47" s="6" t="inlineStr">
+        <is>
+          <t>À tester</t>
+        </is>
+      </c>
+      <c r="H47" s="6" t="n"/>
+      <c r="I47" s="6" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>

<commit_message>
Pilotage : Pinterest reconnu comme source des visites et des inscriptions ; journal et recette des épingles
Source « pinterest » (lien ?utm_source=pinterest ou arrivée depuis Pinterest) dans l'app, les pages Conseils et le
décompte des inscrits ; Pinterest proposé dans le relevé mensuel des réseaux. Recette de décembre n° 41 ; épingles
notées dans « Déjà en prod (exceptions) » (n° 14).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AUzY5Y8Bt2KRzzte5cJgH8
</commit_message>
<xml_diff>
--- a/docs/recette/Recette_prod_decembre_2026.xlsx
+++ b/docs/recette/Recette_prod_decembre_2026.xlsx
@@ -497,7 +497,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I47"/>
+  <dimension ref="A1:I48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -525,7 +525,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -2107,27 +2106,27 @@
       </c>
       <c r="B45" s="5" t="inlineStr">
         <is>
-          <t>Alignement PROD / STA</t>
+          <t>Pilotage — source Pinterest</t>
         </is>
       </c>
       <c r="C45" s="4" t="inlineStr">
         <is>
-          <t>Git</t>
+          <t>Pilotage → Activité (« Par source ») et Réseaux sociaux (relevé mensuel)</t>
         </is>
       </c>
       <c r="D45" s="4" t="inlineStr">
         <is>
-          <t>Après la fusion : git diff --quiet origin/main origin/Staging.</t>
+          <t>En navigation privée, ouvrir un article avec ?utm_source=pinterest (ex. /conseils/mousse-pelouse?utm_source=pinterest), puis regarder Pilotage → Activité ; dans le relevé mensuel des réseaux, ouvrir la liste des plateformes.</t>
         </is>
       </c>
       <c r="E45" s="4" t="inlineStr">
         <is>
-          <t>Aucune différence.</t>
+          <t>Visite comptée sous « 📌 Pinterest » (et non « autre ») ; une inscription venue de Pinterest est comptée dans Pinterest ; Pinterest proposé dans le relevé des followers.</t>
         </is>
       </c>
       <c r="F45" s="4" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Visiteur, puis Admin</t>
         </is>
       </c>
       <c r="G45" s="6" t="inlineStr">
@@ -2135,7 +2134,11 @@
           <t>À tester</t>
         </is>
       </c>
-      <c r="H45" s="6" t="n"/>
+      <c r="H45" s="6" t="inlineStr">
+        <is>
+          <t>Sur STA le 11/10/2026 (suivi des épingles Pinterest).</t>
+        </is>
+      </c>
       <c r="I45" s="6" t="n"/>
     </row>
     <row r="46">
@@ -2144,22 +2147,22 @@
       </c>
       <c r="B46" s="5" t="inlineStr">
         <is>
-          <t>Base de données PROD</t>
+          <t>Alignement PROD / STA</t>
         </is>
       </c>
       <c r="C46" s="4" t="inlineStr">
         <is>
-          <t>Supabase PROD</t>
+          <t>Git</t>
         </is>
       </c>
       <c r="D46" s="4" t="inlineStr">
         <is>
-          <t>Vérifier les tables codes et parrainages.</t>
+          <t>Après la fusion : git diff --quiet origin/main origin/Staging.</t>
         </is>
       </c>
       <c r="E46" s="4" t="inlineStr">
         <is>
-          <t>Tables présentes (créées le 05/10 sur les deux projets).</t>
+          <t>Aucune différence.</t>
         </is>
       </c>
       <c r="F46" s="4" t="inlineStr">
@@ -2181,22 +2184,22 @@
       </c>
       <c r="B47" s="5" t="inlineStr">
         <is>
-          <t>Règle de travail de décembre</t>
+          <t>Base de données PROD</t>
         </is>
       </c>
       <c r="C47" s="4" t="inlineStr">
         <is>
-          <t>CLAUDE.md</t>
+          <t>Supabase PROD</t>
         </is>
       </c>
       <c r="D47" s="4" t="inlineStr">
         <is>
-          <t>Après la mise en prod : retirer le paragraphe « Jusqu'à décembre 2026 ».</t>
+          <t>Vérifier les tables codes et parrainages.</t>
         </is>
       </c>
       <c r="E47" s="4" t="inlineStr">
         <is>
-          <t>STA redevient identique à la PROD.</t>
+          <t>Tables présentes (créées le 05/10 sur les deux projets).</t>
         </is>
       </c>
       <c r="F47" s="4" t="inlineStr">
@@ -2211,12 +2214,49 @@
       </c>
       <c r="H47" s="6" t="n"/>
       <c r="I47" s="6" t="n"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="4" t="n">
+        <v>44</v>
+      </c>
+      <c r="B48" s="5" t="inlineStr">
+        <is>
+          <t>Règle de travail de décembre</t>
+        </is>
+      </c>
+      <c r="C48" s="4" t="inlineStr">
+        <is>
+          <t>CLAUDE.md</t>
+        </is>
+      </c>
+      <c r="D48" s="4" t="inlineStr">
+        <is>
+          <t>Après la mise en prod : retirer le paragraphe « Jusqu'à décembre 2026 ».</t>
+        </is>
+      </c>
+      <c r="E48" s="4" t="inlineStr">
+        <is>
+          <t>STA redevient identique à la PROD.</t>
+        </is>
+      </c>
+      <c r="F48" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G48" s="6" t="inlineStr">
+        <is>
+          <t>À tester</t>
+        </is>
+      </c>
+      <c r="H48" s="6" t="n"/>
+      <c r="I48" s="6" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A2:I2"/>
   </mergeCells>
-  <conditionalFormatting sqref="G5:G32">
+  <conditionalFormatting sqref="G5:G48">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"OK"</formula>
     </cfRule>
@@ -2225,7 +2265,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="G5:G46" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="G5:G48" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"À tester,OK,KO,Non testable"</formula1>
     </dataValidation>
   </dataValidations>
@@ -2239,7 +2279,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I17"/>
+  <dimension ref="A1:I18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -2849,11 +2889,52 @@
       </c>
       <c r="I17" s="6" t="n"/>
     </row>
+    <row r="18">
+      <c r="A18" s="4" t="n">
+        <v>14</v>
+      </c>
+      <c r="B18" s="5" t="inlineStr">
+        <is>
+          <t>Épingles Pinterest : une image par article Conseils (42)</t>
+        </is>
+      </c>
+      <c r="C18" s="4" t="inlineStr">
+        <is>
+          <t>Site (/images/pinterest/&lt;article&gt;.jpg) ; compte Pinterest de Mongazon360</t>
+        </is>
+      </c>
+      <c r="D18" s="4" t="inlineStr">
+        <is>
+          <t>Ouvrir 2 ou 3 images sur téléphone (ex. /images/pinterest/regarnir-gazon-automne.jpg) ; après l'import, ouvrir une épingle sur Pinterest et toucher son lien.</t>
+        </is>
+      </c>
+      <c r="E18" s="4" t="inlineStr">
+        <is>
+          <t>Image 1000 × 1500 nette, titre lisible ; le lien ouvre le bon article ; visite comptée sous « pinterest » dans Pilotage → Activité.</t>
+        </is>
+      </c>
+      <c r="F18" s="4" t="inlineStr">
+        <is>
+          <t>Visiteur</t>
+        </is>
+      </c>
+      <c r="G18" s="6" t="inlineStr">
+        <is>
+          <t>À tester</t>
+        </is>
+      </c>
+      <c r="H18" s="6" t="inlineStr">
+        <is>
+          <t>En prod le 11/10/2026 (go prod de Jordan : épingles Pinterest).</t>
+        </is>
+      </c>
+      <c r="I18" s="6" t="n"/>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A2:I2"/>
   </mergeCells>
-  <conditionalFormatting sqref="G5:G6">
+  <conditionalFormatting sqref="G5:G18">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"OK"</formula>
     </cfRule>
@@ -2862,7 +2943,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="G5:G10" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="G5:G18" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"À tester,OK,KO,Non testable"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Réseaux sociaux : liens « Suivez-nous » en bas de l'accueil et des pages Conseils, profils déclarés à Google
Liste unique dans src/lib/reseaux.js (Instagram, Facebook, TikTok, YouTube), reprise dans les données structurées de
index.html (sameAs) et de la page « Qui sommes-nous ». Recette de décembre n° 42 ; journal du 11/10.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AUzY5Y8Bt2KRzzte5cJgH8
</commit_message>
<xml_diff>
--- a/docs/recette/Recette_prod_decembre_2026.xlsx
+++ b/docs/recette/Recette_prod_decembre_2026.xlsx
@@ -497,7 +497,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I48"/>
+  <dimension ref="A1:I49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -2147,27 +2147,27 @@
       </c>
       <c r="B46" s="5" t="inlineStr">
         <is>
-          <t>Alignement PROD / STA</t>
+          <t>Liens vers les réseaux sociaux (Instagram, Facebook, TikTok, YouTube)</t>
         </is>
       </c>
       <c r="C46" s="4" t="inlineStr">
         <is>
-          <t>Git</t>
+          <t>Accueil (visiteur), pages Conseils et « Qui sommes-nous » : pied de page</t>
         </is>
       </c>
       <c r="D46" s="4" t="inlineStr">
         <is>
-          <t>Après la fusion : git diff --quiet origin/main origin/Staging.</t>
+          <t>Ouvrir l'accueil sans être connecté, puis un article ; toucher chaque lien « Suivez-nous » du pied de page.</t>
         </is>
       </c>
       <c r="E46" s="4" t="inlineStr">
         <is>
-          <t>Aucune différence.</t>
+          <t>Chaque lien ouvre le bon profil Mongazon360 dans un nouvel onglet ; profils déclarés à Google (test des résultats enrichis sur l'accueil : Organization avec sameAs).</t>
         </is>
       </c>
       <c r="F46" s="4" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Visiteur</t>
         </is>
       </c>
       <c r="G46" s="6" t="inlineStr">
@@ -2175,7 +2175,11 @@
           <t>À tester</t>
         </is>
       </c>
-      <c r="H46" s="6" t="n"/>
+      <c r="H46" s="6" t="inlineStr">
+        <is>
+          <t>Sur STA le 11/10/2026 (adresses envoyées par Jordan).</t>
+        </is>
+      </c>
       <c r="I46" s="6" t="n"/>
     </row>
     <row r="47">
@@ -2184,22 +2188,22 @@
       </c>
       <c r="B47" s="5" t="inlineStr">
         <is>
-          <t>Base de données PROD</t>
+          <t>Alignement PROD / STA</t>
         </is>
       </c>
       <c r="C47" s="4" t="inlineStr">
         <is>
-          <t>Supabase PROD</t>
+          <t>Git</t>
         </is>
       </c>
       <c r="D47" s="4" t="inlineStr">
         <is>
-          <t>Vérifier les tables codes et parrainages.</t>
+          <t>Après la fusion : git diff --quiet origin/main origin/Staging.</t>
         </is>
       </c>
       <c r="E47" s="4" t="inlineStr">
         <is>
-          <t>Tables présentes (créées le 05/10 sur les deux projets).</t>
+          <t>Aucune différence.</t>
         </is>
       </c>
       <c r="F47" s="4" t="inlineStr">
@@ -2221,22 +2225,22 @@
       </c>
       <c r="B48" s="5" t="inlineStr">
         <is>
-          <t>Règle de travail de décembre</t>
+          <t>Base de données PROD</t>
         </is>
       </c>
       <c r="C48" s="4" t="inlineStr">
         <is>
-          <t>CLAUDE.md</t>
+          <t>Supabase PROD</t>
         </is>
       </c>
       <c r="D48" s="4" t="inlineStr">
         <is>
-          <t>Après la mise en prod : retirer le paragraphe « Jusqu'à décembre 2026 ».</t>
+          <t>Vérifier les tables codes et parrainages.</t>
         </is>
       </c>
       <c r="E48" s="4" t="inlineStr">
         <is>
-          <t>STA redevient identique à la PROD.</t>
+          <t>Tables présentes (créées le 05/10 sur les deux projets).</t>
         </is>
       </c>
       <c r="F48" s="4" t="inlineStr">
@@ -2251,12 +2255,49 @@
       </c>
       <c r="H48" s="6" t="n"/>
       <c r="I48" s="6" t="n"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="4" t="n">
+        <v>45</v>
+      </c>
+      <c r="B49" s="5" t="inlineStr">
+        <is>
+          <t>Règle de travail de décembre</t>
+        </is>
+      </c>
+      <c r="C49" s="4" t="inlineStr">
+        <is>
+          <t>CLAUDE.md</t>
+        </is>
+      </c>
+      <c r="D49" s="4" t="inlineStr">
+        <is>
+          <t>Après la mise en prod : retirer le paragraphe « Jusqu'à décembre 2026 ».</t>
+        </is>
+      </c>
+      <c r="E49" s="4" t="inlineStr">
+        <is>
+          <t>STA redevient identique à la PROD.</t>
+        </is>
+      </c>
+      <c r="F49" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G49" s="6" t="inlineStr">
+        <is>
+          <t>À tester</t>
+        </is>
+      </c>
+      <c r="H49" s="6" t="n"/>
+      <c r="I49" s="6" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A2:I2"/>
   </mergeCells>
-  <conditionalFormatting sqref="G5:G48">
+  <conditionalFormatting sqref="G5:G49">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"OK"</formula>
     </cfRule>
@@ -2265,7 +2306,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="G5:G48" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="G5:G49" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"À tester,OK,KO,Non testable"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Journal et recette : liens vers les réseaux passés en prod (go prod de Jordan)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AUzY5Y8Bt2KRzzte5cJgH8
</commit_message>
<xml_diff>
--- a/docs/recette/Recette_prod_decembre_2026.xlsx
+++ b/docs/recette/Recette_prod_decembre_2026.xlsx
@@ -497,7 +497,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I49"/>
+  <dimension ref="A1:I48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -2147,27 +2147,27 @@
       </c>
       <c r="B46" s="5" t="inlineStr">
         <is>
-          <t>Liens vers les réseaux sociaux (Instagram, Facebook, TikTok, YouTube)</t>
+          <t>Alignement PROD / STA</t>
         </is>
       </c>
       <c r="C46" s="4" t="inlineStr">
         <is>
-          <t>Accueil (visiteur), pages Conseils et « Qui sommes-nous » : pied de page</t>
+          <t>Git</t>
         </is>
       </c>
       <c r="D46" s="4" t="inlineStr">
         <is>
-          <t>Ouvrir l'accueil sans être connecté, puis un article ; toucher chaque lien « Suivez-nous » du pied de page.</t>
+          <t>Après la fusion : git diff --quiet origin/main origin/Staging.</t>
         </is>
       </c>
       <c r="E46" s="4" t="inlineStr">
         <is>
-          <t>Chaque lien ouvre le bon profil Mongazon360 dans un nouvel onglet ; profils déclarés à Google (test des résultats enrichis sur l'accueil : Organization avec sameAs).</t>
+          <t>Aucune différence.</t>
         </is>
       </c>
       <c r="F46" s="4" t="inlineStr">
         <is>
-          <t>Visiteur</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G46" s="6" t="inlineStr">
@@ -2175,11 +2175,7 @@
           <t>À tester</t>
         </is>
       </c>
-      <c r="H46" s="6" t="inlineStr">
-        <is>
-          <t>Sur STA le 11/10/2026 (adresses envoyées par Jordan).</t>
-        </is>
-      </c>
+      <c r="H46" s="6" t="n"/>
       <c r="I46" s="6" t="n"/>
     </row>
     <row r="47">
@@ -2188,22 +2184,22 @@
       </c>
       <c r="B47" s="5" t="inlineStr">
         <is>
-          <t>Alignement PROD / STA</t>
+          <t>Base de données PROD</t>
         </is>
       </c>
       <c r="C47" s="4" t="inlineStr">
         <is>
-          <t>Git</t>
+          <t>Supabase PROD</t>
         </is>
       </c>
       <c r="D47" s="4" t="inlineStr">
         <is>
-          <t>Après la fusion : git diff --quiet origin/main origin/Staging.</t>
+          <t>Vérifier les tables codes et parrainages.</t>
         </is>
       </c>
       <c r="E47" s="4" t="inlineStr">
         <is>
-          <t>Aucune différence.</t>
+          <t>Tables présentes (créées le 05/10 sur les deux projets).</t>
         </is>
       </c>
       <c r="F47" s="4" t="inlineStr">
@@ -2225,22 +2221,22 @@
       </c>
       <c r="B48" s="5" t="inlineStr">
         <is>
-          <t>Base de données PROD</t>
+          <t>Règle de travail de décembre</t>
         </is>
       </c>
       <c r="C48" s="4" t="inlineStr">
         <is>
-          <t>Supabase PROD</t>
+          <t>CLAUDE.md</t>
         </is>
       </c>
       <c r="D48" s="4" t="inlineStr">
         <is>
-          <t>Vérifier les tables codes et parrainages.</t>
+          <t>Après la mise en prod : retirer le paragraphe « Jusqu'à décembre 2026 ».</t>
         </is>
       </c>
       <c r="E48" s="4" t="inlineStr">
         <is>
-          <t>Tables présentes (créées le 05/10 sur les deux projets).</t>
+          <t>STA redevient identique à la PROD.</t>
         </is>
       </c>
       <c r="F48" s="4" t="inlineStr">
@@ -2255,49 +2251,12 @@
       </c>
       <c r="H48" s="6" t="n"/>
       <c r="I48" s="6" t="n"/>
-    </row>
-    <row r="49">
-      <c r="A49" s="4" t="n">
-        <v>45</v>
-      </c>
-      <c r="B49" s="5" t="inlineStr">
-        <is>
-          <t>Règle de travail de décembre</t>
-        </is>
-      </c>
-      <c r="C49" s="4" t="inlineStr">
-        <is>
-          <t>CLAUDE.md</t>
-        </is>
-      </c>
-      <c r="D49" s="4" t="inlineStr">
-        <is>
-          <t>Après la mise en prod : retirer le paragraphe « Jusqu'à décembre 2026 ».</t>
-        </is>
-      </c>
-      <c r="E49" s="4" t="inlineStr">
-        <is>
-          <t>STA redevient identique à la PROD.</t>
-        </is>
-      </c>
-      <c r="F49" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G49" s="6" t="inlineStr">
-        <is>
-          <t>À tester</t>
-        </is>
-      </c>
-      <c r="H49" s="6" t="n"/>
-      <c r="I49" s="6" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A2:I2"/>
   </mergeCells>
-  <conditionalFormatting sqref="G5:G49">
+  <conditionalFormatting sqref="G5:G48">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"OK"</formula>
     </cfRule>
@@ -2306,7 +2265,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="G5:G49" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="G5:G48" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"À tester,OK,KO,Non testable"</formula1>
     </dataValidation>
   </dataValidations>
@@ -2320,7 +2279,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I18"/>
+  <dimension ref="A1:I19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -2971,11 +2930,52 @@
       </c>
       <c r="I18" s="6" t="n"/>
     </row>
+    <row r="19">
+      <c r="A19" s="4" t="n">
+        <v>15</v>
+      </c>
+      <c r="B19" s="5" t="inlineStr">
+        <is>
+          <t>Liens vers les réseaux sociaux (Instagram, Facebook, TikTok, YouTube)</t>
+        </is>
+      </c>
+      <c r="C19" s="4" t="inlineStr">
+        <is>
+          <t>Accueil (visiteur), pages Conseils et « Qui sommes-nous » : pied de page</t>
+        </is>
+      </c>
+      <c r="D19" s="4" t="inlineStr">
+        <is>
+          <t>Ouvrir l'accueil sans être connecté, puis un article ; toucher chaque lien « Suivez-nous » du pied de page.</t>
+        </is>
+      </c>
+      <c r="E19" s="4" t="inlineStr">
+        <is>
+          <t>Chaque lien ouvre le bon profil Mongazon360 dans un nouvel onglet ; profils déclarés à Google (test des résultats enrichis sur l'accueil : Organization avec sameAs).</t>
+        </is>
+      </c>
+      <c r="F19" s="4" t="inlineStr">
+        <is>
+          <t>Visiteur</t>
+        </is>
+      </c>
+      <c r="G19" s="6" t="inlineStr">
+        <is>
+          <t>À tester</t>
+        </is>
+      </c>
+      <c r="H19" s="6" t="inlineStr">
+        <is>
+          <t>En prod le 11/10/2026 (go prod de Jordan : liens vers les réseaux sociaux).</t>
+        </is>
+      </c>
+      <c r="I19" s="6" t="n"/>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A2:I2"/>
   </mergeCells>
-  <conditionalFormatting sqref="G5:G18">
+  <conditionalFormatting sqref="G5:G19">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"OK"</formula>
     </cfRule>
@@ -2984,7 +2984,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="G5:G18" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="G5:G19" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"À tester,OK,KO,Non testable"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Journal et recette : compte Pinterest créé, site revendiqué
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AUzY5Y8Bt2KRzzte5cJgH8
</commit_message>
<xml_diff>
--- a/docs/recette/Recette_prod_decembre_2026.xlsx
+++ b/docs/recette/Recette_prod_decembre_2026.xlsx
@@ -2279,7 +2279,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I19"/>
+  <dimension ref="A1:I20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -2971,11 +2971,52 @@
       </c>
       <c r="I19" s="6" t="n"/>
     </row>
+    <row r="20">
+      <c r="A20" s="4" t="n">
+        <v>16</v>
+      </c>
+      <c r="B20" s="5" t="inlineStr">
+        <is>
+          <t>Pinterest : site revendiqué et profil ajouté aux réseaux</t>
+        </is>
+      </c>
+      <c r="C20" s="4" t="inlineStr">
+        <is>
+          <t>Accueil (balise p:domain_verify) ; pied de page « Suivez-nous » ; compte Pinterest (Paramètres → Lien vers Pinterest)</t>
+        </is>
+      </c>
+      <c r="D20" s="4" t="inlineStr">
+        <is>
+          <t>Dans Pinterest, vérifier que mongazon360.fr apparaît comme site revendiqué ; sur le site, toucher le lien Pinterest du pied de page.</t>
+        </is>
+      </c>
+      <c r="E20" s="4" t="inlineStr">
+        <is>
+          <t>Site revendiqué (coche verte) ; le lien ouvre pinterest.com/mongazon360.</t>
+        </is>
+      </c>
+      <c r="F20" s="4" t="inlineStr">
+        <is>
+          <t>Visiteur</t>
+        </is>
+      </c>
+      <c r="G20" s="6" t="inlineStr">
+        <is>
+          <t>À tester</t>
+        </is>
+      </c>
+      <c r="H20" s="6" t="inlineStr">
+        <is>
+          <t>En prod le 11/10/2026 (go prod de Jordan : épingles Pinterest et réseaux).</t>
+        </is>
+      </c>
+      <c r="I20" s="6" t="n"/>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A2:I2"/>
   </mergeCells>
-  <conditionalFormatting sqref="G5:G19">
+  <conditionalFormatting sqref="G5:G20">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"OK"</formula>
     </cfRule>
@@ -2984,7 +3025,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="G5:G19" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="G5:G20" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"À tester,OK,KO,Non testable"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Journal et recette : Pilotage et Bob passés en prod ; profil Facebook Bob Gazon en mode professionnel
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AUzY5Y8Bt2KRzzte5cJgH8
</commit_message>
<xml_diff>
--- a/docs/recette/Recette_prod_decembre_2026.xlsx
+++ b/docs/recette/Recette_prod_decembre_2026.xlsx
@@ -497,7 +497,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I48"/>
+  <dimension ref="A1:I46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -2065,27 +2065,27 @@
       </c>
       <c r="B44" s="5" t="inlineStr">
         <is>
-          <t>Pilotage — position moyenne sur Google par mois</t>
+          <t>Alignement PROD / STA</t>
         </is>
       </c>
       <c r="C44" s="4" t="inlineStr">
         <is>
-          <t>Pilotage → Activité (carte « Position moyenne sur Google »)</t>
+          <t>Git</t>
         </is>
       </c>
       <c r="D44" s="4" t="inlineStr">
         <is>
-          <t>Ouvrir Pilotage → Activité ; lire la carte, toucher un point du graphique. Prérequis : variable Vercel GSC_SERVICE_ACCOUNT_JSON (Production et Preview).</t>
+          <t>Après la fusion : git diff --quiet origin/main origin/Staging.</t>
         </is>
       </c>
       <c r="E44" s="4" t="inlineStr">
         <is>
-          <t>Courbe par mois (axe inversé, 1 en haut), valeur du dernier mois et évolution sur un mois, détail au toucher, tableau des mois ; mêmes chiffres que la Search Console (Performances, position moyenne par mois).</t>
+          <t>Aucune différence.</t>
         </is>
       </c>
       <c r="F44" s="4" t="inlineStr">
         <is>
-          <t>Admin</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G44" s="6" t="inlineStr">
@@ -2093,11 +2093,7 @@
           <t>À tester</t>
         </is>
       </c>
-      <c r="H44" s="6" t="inlineStr">
-        <is>
-          <t>Sur STA le 11/10/2026 (demande de Jordan).</t>
-        </is>
-      </c>
+      <c r="H44" s="6" t="n"/>
       <c r="I44" s="6" t="n"/>
     </row>
     <row r="45">
@@ -2106,27 +2102,27 @@
       </c>
       <c r="B45" s="5" t="inlineStr">
         <is>
-          <t>Pilotage — source Pinterest</t>
+          <t>Base de données PROD</t>
         </is>
       </c>
       <c r="C45" s="4" t="inlineStr">
         <is>
-          <t>Pilotage → Activité (« Par source ») et Réseaux sociaux (relevé mensuel)</t>
+          <t>Supabase PROD</t>
         </is>
       </c>
       <c r="D45" s="4" t="inlineStr">
         <is>
-          <t>En navigation privée, ouvrir un article avec ?utm_source=pinterest (ex. /conseils/mousse-pelouse?utm_source=pinterest), puis regarder Pilotage → Activité ; dans le relevé mensuel des réseaux, ouvrir la liste des plateformes.</t>
+          <t>Vérifier les tables codes et parrainages.</t>
         </is>
       </c>
       <c r="E45" s="4" t="inlineStr">
         <is>
-          <t>Visite comptée sous « 📌 Pinterest » (et non « autre ») ; une inscription venue de Pinterest est comptée dans Pinterest ; Pinterest proposé dans le relevé des followers.</t>
+          <t>Tables présentes (créées le 05/10 sur les deux projets).</t>
         </is>
       </c>
       <c r="F45" s="4" t="inlineStr">
         <is>
-          <t>Visiteur, puis Admin</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G45" s="6" t="inlineStr">
@@ -2134,11 +2130,7 @@
           <t>À tester</t>
         </is>
       </c>
-      <c r="H45" s="6" t="inlineStr">
-        <is>
-          <t>Sur STA le 11/10/2026 (suivi des épingles Pinterest).</t>
-        </is>
-      </c>
+      <c r="H45" s="6" t="n"/>
       <c r="I45" s="6" t="n"/>
     </row>
     <row r="46">
@@ -2147,22 +2139,22 @@
       </c>
       <c r="B46" s="5" t="inlineStr">
         <is>
-          <t>Alignement PROD / STA</t>
+          <t>Règle de travail de décembre</t>
         </is>
       </c>
       <c r="C46" s="4" t="inlineStr">
         <is>
-          <t>Git</t>
+          <t>CLAUDE.md</t>
         </is>
       </c>
       <c r="D46" s="4" t="inlineStr">
         <is>
-          <t>Après la fusion : git diff --quiet origin/main origin/Staging.</t>
+          <t>Après la mise en prod : retirer le paragraphe « Jusqu'à décembre 2026 ».</t>
         </is>
       </c>
       <c r="E46" s="4" t="inlineStr">
         <is>
-          <t>Aucune différence.</t>
+          <t>STA redevient identique à la PROD.</t>
         </is>
       </c>
       <c r="F46" s="4" t="inlineStr">
@@ -2177,86 +2169,12 @@
       </c>
       <c r="H46" s="6" t="n"/>
       <c r="I46" s="6" t="n"/>
-    </row>
-    <row r="47">
-      <c r="A47" s="4" t="n">
-        <v>43</v>
-      </c>
-      <c r="B47" s="5" t="inlineStr">
-        <is>
-          <t>Base de données PROD</t>
-        </is>
-      </c>
-      <c r="C47" s="4" t="inlineStr">
-        <is>
-          <t>Supabase PROD</t>
-        </is>
-      </c>
-      <c r="D47" s="4" t="inlineStr">
-        <is>
-          <t>Vérifier les tables codes et parrainages.</t>
-        </is>
-      </c>
-      <c r="E47" s="4" t="inlineStr">
-        <is>
-          <t>Tables présentes (créées le 05/10 sur les deux projets).</t>
-        </is>
-      </c>
-      <c r="F47" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G47" s="6" t="inlineStr">
-        <is>
-          <t>À tester</t>
-        </is>
-      </c>
-      <c r="H47" s="6" t="n"/>
-      <c r="I47" s="6" t="n"/>
-    </row>
-    <row r="48">
-      <c r="A48" s="4" t="n">
-        <v>44</v>
-      </c>
-      <c r="B48" s="5" t="inlineStr">
-        <is>
-          <t>Règle de travail de décembre</t>
-        </is>
-      </c>
-      <c r="C48" s="4" t="inlineStr">
-        <is>
-          <t>CLAUDE.md</t>
-        </is>
-      </c>
-      <c r="D48" s="4" t="inlineStr">
-        <is>
-          <t>Après la mise en prod : retirer le paragraphe « Jusqu'à décembre 2026 ».</t>
-        </is>
-      </c>
-      <c r="E48" s="4" t="inlineStr">
-        <is>
-          <t>STA redevient identique à la PROD.</t>
-        </is>
-      </c>
-      <c r="F48" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G48" s="6" t="inlineStr">
-        <is>
-          <t>À tester</t>
-        </is>
-      </c>
-      <c r="H48" s="6" t="n"/>
-      <c r="I48" s="6" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A2:I2"/>
   </mergeCells>
-  <conditionalFormatting sqref="G5:G48">
+  <conditionalFormatting sqref="G5:G46">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"OK"</formula>
     </cfRule>
@@ -2265,7 +2183,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="G5:G48" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="G5:G46" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"À tester,OK,KO,Non testable"</formula1>
     </dataValidation>
   </dataValidations>
@@ -2279,7 +2197,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I20"/>
+  <dimension ref="A1:I23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -3012,11 +2930,134 @@
       </c>
       <c r="I20" s="6" t="n"/>
     </row>
+    <row r="21">
+      <c r="A21" s="4" t="n">
+        <v>17</v>
+      </c>
+      <c r="B21" s="5" t="inlineStr">
+        <is>
+          <t>Pilotage — position moyenne sur Google par mois</t>
+        </is>
+      </c>
+      <c r="C21" s="4" t="inlineStr">
+        <is>
+          <t>Pilotage → Activité (carte « Position moyenne sur Google »)</t>
+        </is>
+      </c>
+      <c r="D21" s="4" t="inlineStr">
+        <is>
+          <t>Ouvrir Pilotage → Activité ; lire la carte, toucher un point du graphique. Prérequis : variable Vercel GSC_SERVICE_ACCOUNT_JSON (Production et Preview).</t>
+        </is>
+      </c>
+      <c r="E21" s="4" t="inlineStr">
+        <is>
+          <t>Courbe par mois (axe inversé, 1 en haut), valeur du dernier mois et évolution sur un mois, détail au toucher, tableau des mois ; mêmes chiffres que la Search Console (Performances, position moyenne par mois).</t>
+        </is>
+      </c>
+      <c r="F21" s="4" t="inlineStr">
+        <is>
+          <t>Admin</t>
+        </is>
+      </c>
+      <c r="G21" s="6" t="inlineStr">
+        <is>
+          <t>À tester</t>
+        </is>
+      </c>
+      <c r="H21" s="6" t="inlineStr">
+        <is>
+          <t>En prod le 11/10/2026 (go prod de Jordan).</t>
+        </is>
+      </c>
+      <c r="I21" s="6" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="n">
+        <v>18</v>
+      </c>
+      <c r="B22" s="5" t="inlineStr">
+        <is>
+          <t>Pilotage — source Pinterest</t>
+        </is>
+      </c>
+      <c r="C22" s="4" t="inlineStr">
+        <is>
+          <t>Pilotage → Activité (« Par source ») et Réseaux sociaux (relevé mensuel)</t>
+        </is>
+      </c>
+      <c r="D22" s="4" t="inlineStr">
+        <is>
+          <t>En navigation privée, ouvrir un article avec ?utm_source=pinterest (ex. /conseils/mousse-pelouse?utm_source=pinterest), puis regarder Pilotage → Activité ; dans le relevé mensuel des réseaux, ouvrir la liste des plateformes.</t>
+        </is>
+      </c>
+      <c r="E22" s="4" t="inlineStr">
+        <is>
+          <t>Visite comptée sous « 📌 Pinterest » (et non « autre ») ; une inscription venue de Pinterest est comptée dans Pinterest ; Pinterest proposé dans le relevé des followers.</t>
+        </is>
+      </c>
+      <c r="F22" s="4" t="inlineStr">
+        <is>
+          <t>Visiteur, puis Admin</t>
+        </is>
+      </c>
+      <c r="G22" s="6" t="inlineStr">
+        <is>
+          <t>À tester</t>
+        </is>
+      </c>
+      <c r="H22" s="6" t="inlineStr">
+        <is>
+          <t>En prod le 11/10/2026 (go prod de Jordan).</t>
+        </is>
+      </c>
+      <c r="I22" s="6" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="n">
+        <v>19</v>
+      </c>
+      <c r="B23" s="5" t="inlineStr">
+        <is>
+          <t>Bob : rubrique Conseils sans nombre de guides figé</t>
+        </is>
+      </c>
+      <c r="C23" s="4" t="inlineStr">
+        <is>
+          <t>Bob (assistant IA, compte Premium ou essai)</t>
+        </is>
+      </c>
+      <c r="D23" s="4" t="inlineStr">
+        <is>
+          <t>Demander à Bob : « Avez-vous des guides pour entretenir ma pelouse ? »</t>
+        </is>
+      </c>
+      <c r="E23" s="4" t="inlineStr">
+        <is>
+          <t>Bob renvoie vers la rubrique Conseils et les articles du sujet, sans annoncer « 18 guides ».</t>
+        </is>
+      </c>
+      <c r="F23" s="4" t="inlineStr">
+        <is>
+          <t>Premium</t>
+        </is>
+      </c>
+      <c r="G23" s="6" t="inlineStr">
+        <is>
+          <t>À tester</t>
+        </is>
+      </c>
+      <c r="H23" s="6" t="inlineStr">
+        <is>
+          <t>En prod le 11/10/2026 (go prod de Jordan).</t>
+        </is>
+      </c>
+      <c r="I23" s="6" t="n"/>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A2:I2"/>
   </mergeCells>
-  <conditionalFormatting sqref="G5:G20">
+  <conditionalFormatting sqref="G5:G23">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"OK"</formula>
     </cfRule>
@@ -3025,7 +3066,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="G5:G20" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="G5:G23" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"À tester,OK,KO,Non testable"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Bob : repères semis et regarnissage de la base de connaissances, lieu demandé, aucun produit hors catalogue
Quand la conversation parle de semis, Bob reçoit les fenêtres optimales des 7 zones (src/lib/zonesGazon.json, comme
les parcours guidés), la méthode, l'arrosage de germination, la première tonte et l'engrais de la base de connaissances.
Il répond pour le lieu demandé (pas pour la zone de son jardin) et ne cite plus de marque ni de prix hors catalogue.
Recette de décembre n° 40.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AUzY5Y8Bt2KRzzte5cJgH8
</commit_message>
<xml_diff>
--- a/docs/recette/Recette_prod_decembre_2026.xlsx
+++ b/docs/recette/Recette_prod_decembre_2026.xlsx
@@ -497,7 +497,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I46"/>
+  <dimension ref="A1:I47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -2065,27 +2065,27 @@
       </c>
       <c r="B44" s="5" t="inlineStr">
         <is>
-          <t>Alignement PROD / STA</t>
+          <t>Bob — repères semis et regarnissage (base de connaissances)</t>
         </is>
       </c>
       <c r="C44" s="4" t="inlineStr">
         <is>
-          <t>Git</t>
+          <t>Bob (compte Premium ou essai)</t>
         </is>
       </c>
       <c r="D44" s="4" t="inlineStr">
         <is>
-          <t>Après la fusion : git diff --quiet origin/main origin/Staging.</t>
+          <t>Demander à Bob : « Quand puis-je regarnir dans les Landes ? », puis « Et l'arrosage ? » et « Quand tondre ? ».</t>
         </is>
       </c>
       <c r="E44" s="4" t="inlineStr">
         <is>
-          <t>Aucune différence.</t>
+          <t>Landes = Sud-Ouest : semis jusqu'au 31/10, sinon de début mars à mi-avril ; 25 g/m² ; surface humide en permanence ~3 semaines ; 1re tonte à 8-10 cm (coupe à ~6 cm) ; aucun produit ni prix hors catalogue ; parcours « Regarnissage » cité.</t>
         </is>
       </c>
       <c r="F44" s="4" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Premium</t>
         </is>
       </c>
       <c r="G44" s="6" t="inlineStr">
@@ -2093,7 +2093,11 @@
           <t>À tester</t>
         </is>
       </c>
-      <c r="H44" s="6" t="n"/>
+      <c r="H44" s="6" t="inlineStr">
+        <is>
+          <t>Sur STA le 16/10/2026 (réponse fausse de Bob signalée par Jordan).</t>
+        </is>
+      </c>
       <c r="I44" s="6" t="n"/>
     </row>
     <row r="45">
@@ -2102,22 +2106,22 @@
       </c>
       <c r="B45" s="5" t="inlineStr">
         <is>
-          <t>Base de données PROD</t>
+          <t>Alignement PROD / STA</t>
         </is>
       </c>
       <c r="C45" s="4" t="inlineStr">
         <is>
-          <t>Supabase PROD</t>
+          <t>Git</t>
         </is>
       </c>
       <c r="D45" s="4" t="inlineStr">
         <is>
-          <t>Vérifier les tables codes et parrainages.</t>
+          <t>Après la fusion : git diff --quiet origin/main origin/Staging.</t>
         </is>
       </c>
       <c r="E45" s="4" t="inlineStr">
         <is>
-          <t>Tables présentes (créées le 05/10 sur les deux projets).</t>
+          <t>Aucune différence.</t>
         </is>
       </c>
       <c r="F45" s="4" t="inlineStr">
@@ -2139,22 +2143,22 @@
       </c>
       <c r="B46" s="5" t="inlineStr">
         <is>
-          <t>Règle de travail de décembre</t>
+          <t>Base de données PROD</t>
         </is>
       </c>
       <c r="C46" s="4" t="inlineStr">
         <is>
-          <t>CLAUDE.md</t>
+          <t>Supabase PROD</t>
         </is>
       </c>
       <c r="D46" s="4" t="inlineStr">
         <is>
-          <t>Après la mise en prod : retirer le paragraphe « Jusqu'à décembre 2026 ».</t>
+          <t>Vérifier les tables codes et parrainages.</t>
         </is>
       </c>
       <c r="E46" s="4" t="inlineStr">
         <is>
-          <t>STA redevient identique à la PROD.</t>
+          <t>Tables présentes (créées le 05/10 sur les deux projets).</t>
         </is>
       </c>
       <c r="F46" s="4" t="inlineStr">
@@ -2169,12 +2173,49 @@
       </c>
       <c r="H46" s="6" t="n"/>
       <c r="I46" s="6" t="n"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="4" t="n">
+        <v>43</v>
+      </c>
+      <c r="B47" s="5" t="inlineStr">
+        <is>
+          <t>Règle de travail de décembre</t>
+        </is>
+      </c>
+      <c r="C47" s="4" t="inlineStr">
+        <is>
+          <t>CLAUDE.md</t>
+        </is>
+      </c>
+      <c r="D47" s="4" t="inlineStr">
+        <is>
+          <t>Après la mise en prod : retirer le paragraphe « Jusqu'à décembre 2026 ».</t>
+        </is>
+      </c>
+      <c r="E47" s="4" t="inlineStr">
+        <is>
+          <t>STA redevient identique à la PROD.</t>
+        </is>
+      </c>
+      <c r="F47" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G47" s="6" t="inlineStr">
+        <is>
+          <t>À tester</t>
+        </is>
+      </c>
+      <c r="H47" s="6" t="n"/>
+      <c r="I47" s="6" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A2:I2"/>
   </mergeCells>
-  <conditionalFormatting sqref="G5:G46">
+  <conditionalFormatting sqref="G5:G47">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"OK"</formula>
     </cfRule>
@@ -2183,7 +2224,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="G5:G46" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="G5:G47" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"À tester,OK,KO,Non testable"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Bob : modèle plus puissant, message allégé, limite Groq gérée
Bob passe sur openai/gpt-oss-120b (aiModels.cjs : BOB_MODEL, gratuit lui aussi ; quota Groq par minute propre à chaque
modèle, séparé des recommandations du jour). Seuls les articles proches de la question sont joints (liens de la réponse
vérifiés), 6 derniers messages avec réponses de Bob raccourcies, 800 jetons de réponse au plus. Limite par minute
atteinte : une nouvelle tentative après l'attente indiquée par Groq, sinon message d'attente et question non décomptée
(kind « Assistant IA Bob — limite Groq atteinte »). Modèles vérifiés par la tâche du matin et Pilotage → Services.
Recette de décembre n° 41.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AUzY5Y8Bt2KRzzte5cJgH8
</commit_message>
<xml_diff>
--- a/docs/recette/Recette_prod_decembre_2026.xlsx
+++ b/docs/recette/Recette_prod_decembre_2026.xlsx
@@ -497,7 +497,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I47"/>
+  <dimension ref="A1:I48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -2106,27 +2106,27 @@
       </c>
       <c r="B45" s="5" t="inlineStr">
         <is>
-          <t>Alignement PROD / STA</t>
+          <t>Bob — modèle plus puissant, message allégé, limite Groq gérée</t>
         </is>
       </c>
       <c r="C45" s="4" t="inlineStr">
         <is>
-          <t>Git</t>
+          <t>Bob (compte Premium ou essai) ; Pilotage → Services ; Pilotage → Bugs</t>
         </is>
       </c>
       <c r="D45" s="4" t="inlineStr">
         <is>
-          <t>Après la fusion : git diff --quiet origin/main origin/Staging.</t>
+          <t>Poser 3 ou 4 questions variées à Bob (semis, tonte, maladie, achat) ; puis 3 questions en moins d'une minute.</t>
         </is>
       </c>
       <c r="E45" s="4" t="inlineStr">
         <is>
-          <t>Aucune différence.</t>
+          <t>Réponses justes et liens d'articles valides ; Pilotage → Services affiche « Bob : openai/gpt-oss-120b » ; si la limite est atteinte, message « repose-moi ta question dans une minute » et question non décomptée (kind « limite Groq atteinte »).</t>
         </is>
       </c>
       <c r="F45" s="4" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Premium, puis Admin</t>
         </is>
       </c>
       <c r="G45" s="6" t="inlineStr">
@@ -2134,7 +2134,11 @@
           <t>À tester</t>
         </is>
       </c>
-      <c r="H45" s="6" t="n"/>
+      <c r="H45" s="6" t="inlineStr">
+        <is>
+          <t>Sur STA le 16/10/2026 (go de Jordan pour les 3 changements).</t>
+        </is>
+      </c>
       <c r="I45" s="6" t="n"/>
     </row>
     <row r="46">
@@ -2143,22 +2147,22 @@
       </c>
       <c r="B46" s="5" t="inlineStr">
         <is>
-          <t>Base de données PROD</t>
+          <t>Alignement PROD / STA</t>
         </is>
       </c>
       <c r="C46" s="4" t="inlineStr">
         <is>
-          <t>Supabase PROD</t>
+          <t>Git</t>
         </is>
       </c>
       <c r="D46" s="4" t="inlineStr">
         <is>
-          <t>Vérifier les tables codes et parrainages.</t>
+          <t>Après la fusion : git diff --quiet origin/main origin/Staging.</t>
         </is>
       </c>
       <c r="E46" s="4" t="inlineStr">
         <is>
-          <t>Tables présentes (créées le 05/10 sur les deux projets).</t>
+          <t>Aucune différence.</t>
         </is>
       </c>
       <c r="F46" s="4" t="inlineStr">
@@ -2180,22 +2184,22 @@
       </c>
       <c r="B47" s="5" t="inlineStr">
         <is>
-          <t>Règle de travail de décembre</t>
+          <t>Base de données PROD</t>
         </is>
       </c>
       <c r="C47" s="4" t="inlineStr">
         <is>
-          <t>CLAUDE.md</t>
+          <t>Supabase PROD</t>
         </is>
       </c>
       <c r="D47" s="4" t="inlineStr">
         <is>
-          <t>Après la mise en prod : retirer le paragraphe « Jusqu'à décembre 2026 ».</t>
+          <t>Vérifier les tables codes et parrainages.</t>
         </is>
       </c>
       <c r="E47" s="4" t="inlineStr">
         <is>
-          <t>STA redevient identique à la PROD.</t>
+          <t>Tables présentes (créées le 05/10 sur les deux projets).</t>
         </is>
       </c>
       <c r="F47" s="4" t="inlineStr">
@@ -2210,12 +2214,49 @@
       </c>
       <c r="H47" s="6" t="n"/>
       <c r="I47" s="6" t="n"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="4" t="n">
+        <v>44</v>
+      </c>
+      <c r="B48" s="5" t="inlineStr">
+        <is>
+          <t>Règle de travail de décembre</t>
+        </is>
+      </c>
+      <c r="C48" s="4" t="inlineStr">
+        <is>
+          <t>CLAUDE.md</t>
+        </is>
+      </c>
+      <c r="D48" s="4" t="inlineStr">
+        <is>
+          <t>Après la mise en prod : retirer le paragraphe « Jusqu'à décembre 2026 ».</t>
+        </is>
+      </c>
+      <c r="E48" s="4" t="inlineStr">
+        <is>
+          <t>STA redevient identique à la PROD.</t>
+        </is>
+      </c>
+      <c r="F48" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G48" s="6" t="inlineStr">
+        <is>
+          <t>À tester</t>
+        </is>
+      </c>
+      <c r="H48" s="6" t="n"/>
+      <c r="I48" s="6" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A2:I2"/>
   </mergeCells>
-  <conditionalFormatting sqref="G5:G47">
+  <conditionalFormatting sqref="G5:G48">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"OK"</formula>
     </cfRule>
@@ -2224,7 +2265,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="G5:G47" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="G5:G48" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"À tester,OK,KO,Non testable"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Pilotage : taux de clic dans la carte Position moyenne sur Google
Le taux de clic (clics ÷ affichages) est affiché sous la position du dernier
mois, dans la bulle au toucher et sur chaque ligne du tableau des mois.
Calcul côté app : clics et affichages sont déjà renvoyés par l'API Search
Console, aucune donnée nouvelle à récupérer.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UtDc7rX7uUQP7enmdn118M
</commit_message>
<xml_diff>
--- a/docs/recette/Recette_prod_decembre_2026.xlsx
+++ b/docs/recette/Recette_prod_decembre_2026.xlsx
@@ -497,7 +497,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I48"/>
+  <dimension ref="A1:I49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -2251,6 +2251,47 @@
       </c>
       <c r="H48" s="6" t="n"/>
       <c r="I48" s="6" t="n"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="4" t="n">
+        <v>45</v>
+      </c>
+      <c r="B49" s="5" t="inlineStr">
+        <is>
+          <t>Pilotage — taux de clic dans la carte Google</t>
+        </is>
+      </c>
+      <c r="C49" s="4" t="inlineStr">
+        <is>
+          <t>Pilotage → Activité (carte « Position moyenne sur Google »)</t>
+        </is>
+      </c>
+      <c r="D49" s="4" t="inlineStr">
+        <is>
+          <t>Ouvrir Pilotage → Activité ; lire la ligne sous la position, toucher un point du graphique, parcourir le tableau des mois.</t>
+        </is>
+      </c>
+      <c r="E49" s="4" t="inlineStr">
+        <is>
+          <t>Taux de clic du dernier mois affiché sous la position (clics ÷ affichages, une décimale) ; le taux apparaît aussi dans la bulle au toucher et sur chaque ligne du tableau ; mêmes valeurs que la Search Console (Performances, CTR par mois).</t>
+        </is>
+      </c>
+      <c r="F49" s="4" t="inlineStr">
+        <is>
+          <t>Admin</t>
+        </is>
+      </c>
+      <c r="G49" s="6" t="inlineStr">
+        <is>
+          <t>À tester</t>
+        </is>
+      </c>
+      <c r="H49" s="6" t="inlineStr">
+        <is>
+          <t>Sur STA le 16/10/2026.</t>
+        </is>
+      </c>
+      <c r="I49" s="6" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>

<commit_message>
Suivi : go prod des corrections de Bob (journal et recette)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AUzY5Y8Bt2KRzzte5cJgH8
</commit_message>
<xml_diff>
--- a/docs/recette/Recette_prod_decembre_2026.xlsx
+++ b/docs/recette/Recette_prod_decembre_2026.xlsx
@@ -497,7 +497,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I49"/>
+  <dimension ref="A1:I47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -2065,27 +2065,27 @@
       </c>
       <c r="B44" s="5" t="inlineStr">
         <is>
-          <t>Bob — repères semis et regarnissage (base de connaissances)</t>
+          <t>Pilotage — taux de clic dans la carte Google</t>
         </is>
       </c>
       <c r="C44" s="4" t="inlineStr">
         <is>
-          <t>Bob (compte Premium ou essai)</t>
+          <t>Pilotage → Activité (carte « Position moyenne sur Google »)</t>
         </is>
       </c>
       <c r="D44" s="4" t="inlineStr">
         <is>
-          <t>Demander à Bob : « Quand puis-je regarnir dans les Landes ? », puis « Et l'arrosage ? » et « Quand tondre ? ».</t>
+          <t>Ouvrir Pilotage → Activité ; lire la ligne sous la position, toucher un point du graphique, parcourir le tableau des mois.</t>
         </is>
       </c>
       <c r="E44" s="4" t="inlineStr">
         <is>
-          <t>Landes = Sud-Ouest : semis jusqu'au 31/10, sinon de début mars à mi-avril ; 25 g/m² ; surface humide en permanence ~3 semaines ; 1re tonte à 8-10 cm (coupe à ~6 cm) ; aucun produit ni prix hors catalogue ; parcours « Regarnissage » cité.</t>
+          <t>Taux de clic du dernier mois affiché sous la position (clics ÷ affichages, une décimale) ; le taux apparaît aussi dans la bulle au toucher et sur chaque ligne du tableau ; mêmes valeurs que la Search Console (Performances, CTR par mois).</t>
         </is>
       </c>
       <c r="F44" s="4" t="inlineStr">
         <is>
-          <t>Premium</t>
+          <t>Admin</t>
         </is>
       </c>
       <c r="G44" s="6" t="inlineStr">
@@ -2095,7 +2095,7 @@
       </c>
       <c r="H44" s="6" t="inlineStr">
         <is>
-          <t>Sur STA le 16/10/2026 (réponse fausse de Bob signalée par Jordan).</t>
+          <t>Sur STA le 16/10/2026.</t>
         </is>
       </c>
       <c r="I44" s="6" t="n"/>
@@ -2106,27 +2106,27 @@
       </c>
       <c r="B45" s="5" t="inlineStr">
         <is>
-          <t>Bob — modèle plus puissant, message allégé, limite Groq gérée</t>
+          <t>Alignement PROD / STA</t>
         </is>
       </c>
       <c r="C45" s="4" t="inlineStr">
         <is>
-          <t>Bob (compte Premium ou essai) ; Pilotage → Services ; Pilotage → Bugs</t>
+          <t>Git</t>
         </is>
       </c>
       <c r="D45" s="4" t="inlineStr">
         <is>
-          <t>Poser 3 ou 4 questions variées à Bob (semis, tonte, maladie, achat) ; puis 3 questions en moins d'une minute.</t>
+          <t>Après la fusion : git diff --quiet origin/main origin/Staging.</t>
         </is>
       </c>
       <c r="E45" s="4" t="inlineStr">
         <is>
-          <t>Réponses justes et liens d'articles valides ; Pilotage → Services affiche « Bob : openai/gpt-oss-120b » ; si la limite est atteinte, message « repose-moi ta question dans une minute » et question non décomptée (kind « limite Groq atteinte »).</t>
+          <t>Aucune différence.</t>
         </is>
       </c>
       <c r="F45" s="4" t="inlineStr">
         <is>
-          <t>Premium, puis Admin</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G45" s="6" t="inlineStr">
@@ -2134,11 +2134,7 @@
           <t>À tester</t>
         </is>
       </c>
-      <c r="H45" s="6" t="inlineStr">
-        <is>
-          <t>Sur STA le 16/10/2026 (go de Jordan pour les 3 changements).</t>
-        </is>
-      </c>
+      <c r="H45" s="6" t="n"/>
       <c r="I45" s="6" t="n"/>
     </row>
     <row r="46">
@@ -2147,27 +2143,27 @@
       </c>
       <c r="B46" s="5" t="inlineStr">
         <is>
-          <t>Pilotage — taux de clic dans la carte Google</t>
+          <t>Base de données PROD</t>
         </is>
       </c>
       <c r="C46" s="4" t="inlineStr">
         <is>
-          <t>Pilotage → Activité (carte « Position moyenne sur Google »)</t>
+          <t>Supabase PROD</t>
         </is>
       </c>
       <c r="D46" s="4" t="inlineStr">
         <is>
-          <t>Ouvrir Pilotage → Activité ; lire la ligne sous la position, toucher un point du graphique, parcourir le tableau des mois.</t>
+          <t>Vérifier les tables codes et parrainages.</t>
         </is>
       </c>
       <c r="E46" s="4" t="inlineStr">
         <is>
-          <t>Taux de clic du dernier mois affiché sous la position (clics ÷ affichages, une décimale) ; le taux apparaît aussi dans la bulle au toucher et sur chaque ligne du tableau ; mêmes valeurs que la Search Console (Performances, CTR par mois).</t>
+          <t>Tables présentes (créées le 05/10 sur les deux projets).</t>
         </is>
       </c>
       <c r="F46" s="4" t="inlineStr">
         <is>
-          <t>Admin</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G46" s="6" t="inlineStr">
@@ -2175,11 +2171,7 @@
           <t>À tester</t>
         </is>
       </c>
-      <c r="H46" s="6" t="inlineStr">
-        <is>
-          <t>Sur STA le 16/10/2026.</t>
-        </is>
-      </c>
+      <c r="H46" s="6" t="n"/>
       <c r="I46" s="6" t="n"/>
     </row>
     <row r="47">
@@ -2188,22 +2180,22 @@
       </c>
       <c r="B47" s="5" t="inlineStr">
         <is>
-          <t>Alignement PROD / STA</t>
+          <t>Règle de travail de décembre</t>
         </is>
       </c>
       <c r="C47" s="4" t="inlineStr">
         <is>
-          <t>Git</t>
+          <t>CLAUDE.md</t>
         </is>
       </c>
       <c r="D47" s="4" t="inlineStr">
         <is>
-          <t>Après la fusion : git diff --quiet origin/main origin/Staging.</t>
+          <t>Après la mise en prod : retirer le paragraphe « Jusqu'à décembre 2026 ».</t>
         </is>
       </c>
       <c r="E47" s="4" t="inlineStr">
         <is>
-          <t>Aucune différence.</t>
+          <t>STA redevient identique à la PROD.</t>
         </is>
       </c>
       <c r="F47" s="4" t="inlineStr">
@@ -2218,86 +2210,12 @@
       </c>
       <c r="H47" s="6" t="n"/>
       <c r="I47" s="6" t="n"/>
-    </row>
-    <row r="48">
-      <c r="A48" s="4" t="n">
-        <v>44</v>
-      </c>
-      <c r="B48" s="5" t="inlineStr">
-        <is>
-          <t>Base de données PROD</t>
-        </is>
-      </c>
-      <c r="C48" s="4" t="inlineStr">
-        <is>
-          <t>Supabase PROD</t>
-        </is>
-      </c>
-      <c r="D48" s="4" t="inlineStr">
-        <is>
-          <t>Vérifier les tables codes et parrainages.</t>
-        </is>
-      </c>
-      <c r="E48" s="4" t="inlineStr">
-        <is>
-          <t>Tables présentes (créées le 05/10 sur les deux projets).</t>
-        </is>
-      </c>
-      <c r="F48" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G48" s="6" t="inlineStr">
-        <is>
-          <t>À tester</t>
-        </is>
-      </c>
-      <c r="H48" s="6" t="n"/>
-      <c r="I48" s="6" t="n"/>
-    </row>
-    <row r="49">
-      <c r="A49" s="4" t="n">
-        <v>45</v>
-      </c>
-      <c r="B49" s="5" t="inlineStr">
-        <is>
-          <t>Règle de travail de décembre</t>
-        </is>
-      </c>
-      <c r="C49" s="4" t="inlineStr">
-        <is>
-          <t>CLAUDE.md</t>
-        </is>
-      </c>
-      <c r="D49" s="4" t="inlineStr">
-        <is>
-          <t>Après la mise en prod : retirer le paragraphe « Jusqu'à décembre 2026 ».</t>
-        </is>
-      </c>
-      <c r="E49" s="4" t="inlineStr">
-        <is>
-          <t>STA redevient identique à la PROD.</t>
-        </is>
-      </c>
-      <c r="F49" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G49" s="6" t="inlineStr">
-        <is>
-          <t>À tester</t>
-        </is>
-      </c>
-      <c r="H49" s="6" t="n"/>
-      <c r="I49" s="6" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A2:I2"/>
   </mergeCells>
-  <conditionalFormatting sqref="G5:G48">
+  <conditionalFormatting sqref="G5:G47">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"OK"</formula>
     </cfRule>
@@ -2306,7 +2224,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="G5:G48" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="G5:G47" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"À tester,OK,KO,Non testable"</formula1>
     </dataValidation>
   </dataValidations>
@@ -2320,7 +2238,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I23"/>
+  <dimension ref="A1:I25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -3176,11 +3094,93 @@
       </c>
       <c r="I23" s="6" t="n"/>
     </row>
+    <row r="24">
+      <c r="A24" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="B24" s="5" t="inlineStr">
+        <is>
+          <t>Bob — repères semis et regarnissage (base de connaissances)</t>
+        </is>
+      </c>
+      <c r="C24" s="4" t="inlineStr">
+        <is>
+          <t>Bob (compte Premium ou essai)</t>
+        </is>
+      </c>
+      <c r="D24" s="4" t="inlineStr">
+        <is>
+          <t>Demander à Bob : « Quand puis-je regarnir dans les Landes ? », puis « Et l'arrosage ? » et « Quand tondre ? ».</t>
+        </is>
+      </c>
+      <c r="E24" s="4" t="inlineStr">
+        <is>
+          <t>Landes = Sud-Ouest : semis jusqu'au 31/10, sinon de début mars à mi-avril ; 25 g/m² ; surface humide en permanence ~3 semaines ; 1re tonte à 8-10 cm (coupe à ~6 cm) ; aucun produit ni prix hors catalogue ; parcours « Regarnissage » cité.</t>
+        </is>
+      </c>
+      <c r="F24" s="4" t="inlineStr">
+        <is>
+          <t>Premium</t>
+        </is>
+      </c>
+      <c r="G24" s="6" t="inlineStr">
+        <is>
+          <t>À tester</t>
+        </is>
+      </c>
+      <c r="H24" s="6" t="inlineStr">
+        <is>
+          <t>Sur STA le 16/10/2026, testé par Jordan ; en prod le 17/10/2026 (go prod de Jordan : corrections de Bob).</t>
+        </is>
+      </c>
+      <c r="I24" s="6" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="n">
+        <v>21</v>
+      </c>
+      <c r="B25" s="5" t="inlineStr">
+        <is>
+          <t>Bob — modèle plus puissant, message allégé, limite Groq gérée</t>
+        </is>
+      </c>
+      <c r="C25" s="4" t="inlineStr">
+        <is>
+          <t>Bob (compte Premium ou essai) ; Pilotage → Services ; Pilotage → Bugs</t>
+        </is>
+      </c>
+      <c r="D25" s="4" t="inlineStr">
+        <is>
+          <t>Poser 3 ou 4 questions variées à Bob (semis, tonte, maladie, achat) ; puis 3 questions en moins d'une minute.</t>
+        </is>
+      </c>
+      <c r="E25" s="4" t="inlineStr">
+        <is>
+          <t>Réponses justes et liens d'articles valides ; Pilotage → Services affiche « Bob : openai/gpt-oss-120b » ; si la limite est atteinte, message « repose-moi ta question dans une minute » et question non décomptée (kind « limite Groq atteinte »).</t>
+        </is>
+      </c>
+      <c r="F25" s="4" t="inlineStr">
+        <is>
+          <t>Premium, puis Admin</t>
+        </is>
+      </c>
+      <c r="G25" s="6" t="inlineStr">
+        <is>
+          <t>À tester</t>
+        </is>
+      </c>
+      <c r="H25" s="6" t="inlineStr">
+        <is>
+          <t>Sur STA le 16/10/2026, testé par Jordan ; en prod le 17/10/2026 (go prod de Jordan : corrections de Bob).</t>
+        </is>
+      </c>
+      <c r="I25" s="6" t="n"/>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A2:I2"/>
   </mergeCells>
-  <conditionalFormatting sqref="G5:G23">
+  <conditionalFormatting sqref="G5:G25">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"OK"</formula>
     </cfRule>
@@ -3189,7 +3189,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="G5:G23" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="G5:G25" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"À tester,OK,KO,Non testable"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Suivi : test de Bob en prod validé, go prod du taux de clic de Pilotage (journal et recette)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AUzY5Y8Bt2KRzzte5cJgH8
</commit_message>
<xml_diff>
--- a/docs/recette/Recette_prod_decembre_2026.xlsx
+++ b/docs/recette/Recette_prod_decembre_2026.xlsx
@@ -17,7 +17,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
+  <numFmts count="2">
+    <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
+    <numFmt numFmtId="165" formatCode="DD/MM/YYYY"/>
+  </numFmts>
   <fonts count="6">
     <font>
       <name val="Calibri"/>
@@ -98,7 +101,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -114,6 +117,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -497,7 +503,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I47"/>
+  <dimension ref="A1:I46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -2065,27 +2071,27 @@
       </c>
       <c r="B44" s="5" t="inlineStr">
         <is>
-          <t>Pilotage — taux de clic dans la carte Google</t>
+          <t>Alignement PROD / STA</t>
         </is>
       </c>
       <c r="C44" s="4" t="inlineStr">
         <is>
-          <t>Pilotage → Activité (carte « Position moyenne sur Google »)</t>
+          <t>Git</t>
         </is>
       </c>
       <c r="D44" s="4" t="inlineStr">
         <is>
-          <t>Ouvrir Pilotage → Activité ; lire la ligne sous la position, toucher un point du graphique, parcourir le tableau des mois.</t>
+          <t>Après la fusion : git diff --quiet origin/main origin/Staging.</t>
         </is>
       </c>
       <c r="E44" s="4" t="inlineStr">
         <is>
-          <t>Taux de clic du dernier mois affiché sous la position (clics ÷ affichages, une décimale) ; le taux apparaît aussi dans la bulle au toucher et sur chaque ligne du tableau ; mêmes valeurs que la Search Console (Performances, CTR par mois).</t>
+          <t>Aucune différence.</t>
         </is>
       </c>
       <c r="F44" s="4" t="inlineStr">
         <is>
-          <t>Admin</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G44" s="6" t="inlineStr">
@@ -2093,11 +2099,7 @@
           <t>À tester</t>
         </is>
       </c>
-      <c r="H44" s="6" t="inlineStr">
-        <is>
-          <t>Sur STA le 16/10/2026.</t>
-        </is>
-      </c>
+      <c r="H44" s="6" t="n"/>
       <c r="I44" s="6" t="n"/>
     </row>
     <row r="45">
@@ -2106,22 +2108,22 @@
       </c>
       <c r="B45" s="5" t="inlineStr">
         <is>
-          <t>Alignement PROD / STA</t>
+          <t>Base de données PROD</t>
         </is>
       </c>
       <c r="C45" s="4" t="inlineStr">
         <is>
-          <t>Git</t>
+          <t>Supabase PROD</t>
         </is>
       </c>
       <c r="D45" s="4" t="inlineStr">
         <is>
-          <t>Après la fusion : git diff --quiet origin/main origin/Staging.</t>
+          <t>Vérifier les tables codes et parrainages.</t>
         </is>
       </c>
       <c r="E45" s="4" t="inlineStr">
         <is>
-          <t>Aucune différence.</t>
+          <t>Tables présentes (créées le 05/10 sur les deux projets).</t>
         </is>
       </c>
       <c r="F45" s="4" t="inlineStr">
@@ -2143,22 +2145,22 @@
       </c>
       <c r="B46" s="5" t="inlineStr">
         <is>
-          <t>Base de données PROD</t>
+          <t>Règle de travail de décembre</t>
         </is>
       </c>
       <c r="C46" s="4" t="inlineStr">
         <is>
-          <t>Supabase PROD</t>
+          <t>CLAUDE.md</t>
         </is>
       </c>
       <c r="D46" s="4" t="inlineStr">
         <is>
-          <t>Vérifier les tables codes et parrainages.</t>
+          <t>Après la mise en prod : retirer le paragraphe « Jusqu'à décembre 2026 ».</t>
         </is>
       </c>
       <c r="E46" s="4" t="inlineStr">
         <is>
-          <t>Tables présentes (créées le 05/10 sur les deux projets).</t>
+          <t>STA redevient identique à la PROD.</t>
         </is>
       </c>
       <c r="F46" s="4" t="inlineStr">
@@ -2173,49 +2175,12 @@
       </c>
       <c r="H46" s="6" t="n"/>
       <c r="I46" s="6" t="n"/>
-    </row>
-    <row r="47">
-      <c r="A47" s="4" t="n">
-        <v>43</v>
-      </c>
-      <c r="B47" s="5" t="inlineStr">
-        <is>
-          <t>Règle de travail de décembre</t>
-        </is>
-      </c>
-      <c r="C47" s="4" t="inlineStr">
-        <is>
-          <t>CLAUDE.md</t>
-        </is>
-      </c>
-      <c r="D47" s="4" t="inlineStr">
-        <is>
-          <t>Après la mise en prod : retirer le paragraphe « Jusqu'à décembre 2026 ».</t>
-        </is>
-      </c>
-      <c r="E47" s="4" t="inlineStr">
-        <is>
-          <t>STA redevient identique à la PROD.</t>
-        </is>
-      </c>
-      <c r="F47" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G47" s="6" t="inlineStr">
-        <is>
-          <t>À tester</t>
-        </is>
-      </c>
-      <c r="H47" s="6" t="n"/>
-      <c r="I47" s="6" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A2:I2"/>
   </mergeCells>
-  <conditionalFormatting sqref="G5:G47">
+  <conditionalFormatting sqref="G5:G46">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"OK"</formula>
     </cfRule>
@@ -2224,7 +2189,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="G5:G47" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="G5:G46" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"À tester,OK,KO,Non testable"</formula1>
     </dataValidation>
   </dataValidations>
@@ -2238,7 +2203,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I25"/>
+  <dimension ref="A1:I26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -3125,15 +3090,17 @@
       </c>
       <c r="G24" s="6" t="inlineStr">
         <is>
-          <t>À tester</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="H24" s="6" t="inlineStr">
         <is>
-          <t>Sur STA le 16/10/2026, testé par Jordan ; en prod le 17/10/2026 (go prod de Jordan : corrections de Bob).</t>
-        </is>
-      </c>
-      <c r="I24" s="6" t="n"/>
+          <t>Sur STA le 16/10/2026, testé par Jordan ; en prod le 17/10/2026 (go prod de Jordan : corrections de Bob). Test en prod OK (Jordan).</t>
+        </is>
+      </c>
+      <c r="I24" s="7" t="n">
+        <v>46312</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="4" t="n">
@@ -3166,21 +3133,64 @@
       </c>
       <c r="G25" s="6" t="inlineStr">
         <is>
-          <t>À tester</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="H25" s="6" t="inlineStr">
         <is>
-          <t>Sur STA le 16/10/2026, testé par Jordan ; en prod le 17/10/2026 (go prod de Jordan : corrections de Bob).</t>
-        </is>
-      </c>
-      <c r="I25" s="6" t="n"/>
+          <t>Sur STA le 16/10/2026, testé par Jordan ; en prod le 17/10/2026 (go prod de Jordan : corrections de Bob). Test en prod OK (Jordan) ; Groq OK dans Pilotage → Services.</t>
+        </is>
+      </c>
+      <c r="I25" s="7" t="n">
+        <v>46312</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="n">
+        <v>22</v>
+      </c>
+      <c r="B26" s="5" t="inlineStr">
+        <is>
+          <t>Pilotage — taux de clic dans la carte Google</t>
+        </is>
+      </c>
+      <c r="C26" s="4" t="inlineStr">
+        <is>
+          <t>Pilotage → Activité (carte « Position moyenne sur Google »)</t>
+        </is>
+      </c>
+      <c r="D26" s="4" t="inlineStr">
+        <is>
+          <t>Ouvrir Pilotage → Activité ; lire la ligne sous la position, toucher un point du graphique, parcourir le tableau des mois.</t>
+        </is>
+      </c>
+      <c r="E26" s="4" t="inlineStr">
+        <is>
+          <t>Taux de clic du dernier mois affiché sous la position (clics ÷ affichages, une décimale) ; le taux apparaît aussi dans la bulle au toucher et sur chaque ligne du tableau ; mêmes valeurs que la Search Console (Performances, CTR par mois).</t>
+        </is>
+      </c>
+      <c r="F26" s="4" t="inlineStr">
+        <is>
+          <t>Admin</t>
+        </is>
+      </c>
+      <c r="G26" s="6" t="inlineStr">
+        <is>
+          <t>À tester</t>
+        </is>
+      </c>
+      <c r="H26" s="6" t="inlineStr">
+        <is>
+          <t>Sur STA le 16/10/2026 ; en prod le 17/10/2026 (go prod de Jordan).</t>
+        </is>
+      </c>
+      <c r="I26" s="6" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A2:I2"/>
   </mergeCells>
-  <conditionalFormatting sqref="G5:G25">
+  <conditionalFormatting sqref="G5:G26">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"OK"</formula>
     </cfRule>
@@ -3189,7 +3199,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="G5:G25" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="G5:G26" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"À tester,OK,KO,Non testable"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Suivi : taux de clic de Pilotage validé en prod par Jordan (journal et recette)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AUzY5Y8Bt2KRzzte5cJgH8
</commit_message>
<xml_diff>
--- a/docs/recette/Recette_prod_decembre_2026.xlsx
+++ b/docs/recette/Recette_prod_decembre_2026.xlsx
@@ -18,8 +18,8 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
-    <numFmt numFmtId="165" formatCode="DD/MM/YYYY"/>
+    <numFmt numFmtId="164" formatCode="DD/MM/YYYY"/>
+    <numFmt numFmtId="165" formatCode="yyyy-mm-dd"/>
   </numFmts>
   <fonts count="6">
     <font>
@@ -101,7 +101,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -119,7 +119,10 @@
     <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -3098,7 +3101,7 @@
           <t>Sur STA le 16/10/2026, testé par Jordan ; en prod le 17/10/2026 (go prod de Jordan : corrections de Bob). Test en prod OK (Jordan).</t>
         </is>
       </c>
-      <c r="I24" s="7" t="n">
+      <c r="I24" s="8" t="n">
         <v>46312</v>
       </c>
     </row>
@@ -3141,7 +3144,7 @@
           <t>Sur STA le 16/10/2026, testé par Jordan ; en prod le 17/10/2026 (go prod de Jordan : corrections de Bob). Test en prod OK (Jordan) ; Groq OK dans Pilotage → Services.</t>
         </is>
       </c>
-      <c r="I25" s="7" t="n">
+      <c r="I25" s="8" t="n">
         <v>46312</v>
       </c>
     </row>
@@ -3176,15 +3179,17 @@
       </c>
       <c r="G26" s="6" t="inlineStr">
         <is>
-          <t>À tester</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="H26" s="6" t="inlineStr">
         <is>
-          <t>Sur STA le 16/10/2026 ; en prod le 17/10/2026 (go prod de Jordan).</t>
-        </is>
-      </c>
-      <c r="I26" s="6" t="n"/>
+          <t>Sur STA le 16/10/2026 ; en prod le 17/10/2026 (go prod de Jordan). Test en prod OK (Jordan).</t>
+        </is>
+      </c>
+      <c r="I26" s="8" t="n">
+        <v>46312</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>

<commit_message>
Équipements : robot Mammotion et station météo Davis connectables (STA)
- Mammotion (modèles sortis à partir de 2025) : identifiants personnels créés par
  l'utilisateur sur developer.mammotion.com, chiffrés ; état, batterie et charge du
  robot ; dans « Aujourd'hui », proposition de le faire rentrer à sa base quand la tonte
  est déconseillée, ou de reprendre une tonte en pause (l'API ne sait pas mettre au
  repos pour une durée ni suspendre les tâches programmées).
- Davis (Vantage Pro2 ou Vue avec WeatherLink Live ou console) : clé et secret créés
  sur weatherlink.com ; pluie du jour, température, humidité et vent du jardin
  remplacent les prévisions de la journée, comme Ecowitt et Netatmo.
- Écran « Mes équipements », consignes et contexte de Bob, politique de confidentialité
  (article 6.3) et CLAUDE.md à jour ; recette de décembre n° 40 à 43.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AUzY5Y8Bt2KRzzte5cJgH8
</commit_message>
<xml_diff>
--- a/docs/recette/Recette_prod_decembre_2026.xlsx
+++ b/docs/recette/Recette_prod_decembre_2026.xlsx
@@ -17,9 +17,8 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="1">
     <numFmt numFmtId="164" formatCode="DD/MM/YYYY"/>
-    <numFmt numFmtId="165" formatCode="yyyy-mm-dd"/>
   </numFmts>
   <fonts count="6">
     <font>
@@ -506,7 +505,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I46"/>
+  <dimension ref="A1:I50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -2074,27 +2073,27 @@
       </c>
       <c r="B44" s="5" t="inlineStr">
         <is>
-          <t>Alignement PROD / STA</t>
+          <t>Robot Mammotion — connexion</t>
         </is>
       </c>
       <c r="C44" s="4" t="inlineStr">
         <is>
-          <t>Git</t>
+          <t>Mes équipements → Robot tondeuse</t>
         </is>
       </c>
       <c r="D44" s="4" t="inlineStr">
         <is>
-          <t>Après la fusion : git diff --quiet origin/main origin/Staging.</t>
+          <t>Sur developer.mammotion.com, créer des identifiants (« Create Credentials ») avec un compte Mammotion qui a un robot sorti à partir de 2025, les coller puis « Connecter mon robot Mammotion » ; recommencer avec un compte sans robot compatible.</t>
         </is>
       </c>
       <c r="E44" s="4" t="inlineStr">
         <is>
-          <t>Aucune différence.</t>
+          <t>Robot « ✓ connecté » avec son nom, son état et sa batterie ; compte sans robot compatible : message « Aucun robot sur ce compte Mammotion » ; faux identifiants : « Identifiants Mammotion refusés ».</t>
         </is>
       </c>
       <c r="F44" s="4" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Compte avec robot Mammotion</t>
         </is>
       </c>
       <c r="G44" s="6" t="inlineStr">
@@ -2102,7 +2101,11 @@
           <t>À tester</t>
         </is>
       </c>
-      <c r="H44" s="6" t="n"/>
+      <c r="H44" s="6" t="inlineStr">
+        <is>
+          <t>Sur STA le 17/10/2026. Avant la prod : accord écrit de Mammotion pour une app payante (ou connexion OAuth fournie par Mammotion).</t>
+        </is>
+      </c>
       <c r="I44" s="6" t="n"/>
     </row>
     <row r="45">
@@ -2111,27 +2114,27 @@
       </c>
       <c r="B45" s="5" t="inlineStr">
         <is>
-          <t>Base de données PROD</t>
+          <t>Robot Mammotion — propositions</t>
         </is>
       </c>
       <c r="C45" s="4" t="inlineStr">
         <is>
-          <t>Supabase PROD</t>
+          <t>Aujourd'hui (carte du robot)</t>
         </is>
       </c>
       <c r="D45" s="4" t="inlineStr">
         <is>
-          <t>Vérifier les tables codes et parrainages.</t>
+          <t>Un jour de pluie ou de gel pendant que le robot tond : valider « Le faire rentrer à sa base » ; un jour sans contre-indication avec le robot en pause : « Reprendre la tonte ».</t>
         </is>
       </c>
       <c r="E45" s="4" t="inlineStr">
         <is>
-          <t>Tables présentes (créées le 05/10 sur les deux projets).</t>
+          <t>Le robot rentre à sa base, ou reprend la tonte ; hors saison ou pendant un semis, la raison rappelle de suspendre ses tâches programmées dans l'app Mammotion ; aucune proposition quand le robot est à l'arrêt.</t>
         </is>
       </c>
       <c r="F45" s="4" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Compte avec robot Mammotion</t>
         </is>
       </c>
       <c r="G45" s="6" t="inlineStr">
@@ -2139,7 +2142,11 @@
           <t>À tester</t>
         </is>
       </c>
-      <c r="H45" s="6" t="n"/>
+      <c r="H45" s="6" t="inlineStr">
+        <is>
+          <t>Sur STA le 17/10/2026.</t>
+        </is>
+      </c>
       <c r="I45" s="6" t="n"/>
     </row>
     <row r="46">
@@ -2148,42 +2155,198 @@
       </c>
       <c r="B46" s="5" t="inlineStr">
         <is>
+          <t>Station Davis — connexion et mesures</t>
+        </is>
+      </c>
+      <c r="C46" s="4" t="inlineStr">
+        <is>
+          <t>Mes équipements → Station météo ; Aujourd'hui ; Bob</t>
+        </is>
+      </c>
+      <c r="D46" s="4" t="inlineStr">
+        <is>
+          <t>Sur weatherlink.com, « Generate v2 Key », coller l'API Key v2 et l'API Secret, « Trouver ma station Davis » puis la choisir ; un jour de pluie, ouvrir « Aujourd'hui » et demander à Bob s'il faut arroser.</t>
+        </is>
+      </c>
+      <c r="E46" s="4" t="inlineStr">
+        <is>
+          <t>Température en °C, pluie du jour en mm, humidité et vent en km/h affichés ; l'arrosage et Bob tiennent compte de la pluie mesurée ; fausses clés : « Clé ou secret WeatherLink refusés ».</t>
+        </is>
+      </c>
+      <c r="F46" s="4" t="inlineStr">
+        <is>
+          <t>Compte avec station Davis (WeatherLink Live ou console)</t>
+        </is>
+      </c>
+      <c r="G46" s="6" t="inlineStr">
+        <is>
+          <t>À tester</t>
+        </is>
+      </c>
+      <c r="H46" s="6" t="inlineStr">
+        <is>
+          <t>Sur STA le 17/10/2026.</t>
+        </is>
+      </c>
+      <c r="I46" s="6" t="n"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="4" t="n">
+        <v>43</v>
+      </c>
+      <c r="B47" s="5" t="inlineStr">
+        <is>
+          <t>Équipements — textes et Bob</t>
+        </is>
+      </c>
+      <c r="C47" s="4" t="inlineStr">
+        <is>
+          <t>Politique de confidentialité (6.3) ; Bob</t>
+        </is>
+      </c>
+      <c r="D47" s="4" t="inlineStr">
+        <is>
+          <t>Lire l'article 6.3 de la politique de confidentialité ; demander à Bob quelles marques l'app peut connecter.</t>
+        </is>
+      </c>
+      <c r="E47" s="4" t="inlineStr">
+        <is>
+          <t>Davis et Mammotion cités dans l'article 6.3 (date du 17 octobre) ; Bob cite Netatmo, Ecowitt, Davis, Husqvarna, Gardena, Mammotion et Rachio, sans autre marque.</t>
+        </is>
+      </c>
+      <c r="F47" s="4" t="inlineStr">
+        <is>
+          <t>Premium</t>
+        </is>
+      </c>
+      <c r="G47" s="6" t="inlineStr">
+        <is>
+          <t>À tester</t>
+        </is>
+      </c>
+      <c r="H47" s="6" t="inlineStr">
+        <is>
+          <t>Sur STA le 17/10/2026.</t>
+        </is>
+      </c>
+      <c r="I47" s="6" t="n"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="4" t="n">
+        <v>44</v>
+      </c>
+      <c r="B48" s="5" t="inlineStr">
+        <is>
+          <t>Alignement PROD / STA</t>
+        </is>
+      </c>
+      <c r="C48" s="4" t="inlineStr">
+        <is>
+          <t>Git</t>
+        </is>
+      </c>
+      <c r="D48" s="4" t="inlineStr">
+        <is>
+          <t>Après la fusion : git diff --quiet origin/main origin/Staging.</t>
+        </is>
+      </c>
+      <c r="E48" s="4" t="inlineStr">
+        <is>
+          <t>Aucune différence.</t>
+        </is>
+      </c>
+      <c r="F48" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G48" s="6" t="inlineStr">
+        <is>
+          <t>À tester</t>
+        </is>
+      </c>
+      <c r="H48" s="6" t="n"/>
+      <c r="I48" s="6" t="n"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="4" t="n">
+        <v>45</v>
+      </c>
+      <c r="B49" s="5" t="inlineStr">
+        <is>
+          <t>Base de données PROD</t>
+        </is>
+      </c>
+      <c r="C49" s="4" t="inlineStr">
+        <is>
+          <t>Supabase PROD</t>
+        </is>
+      </c>
+      <c r="D49" s="4" t="inlineStr">
+        <is>
+          <t>Vérifier les tables codes et parrainages.</t>
+        </is>
+      </c>
+      <c r="E49" s="4" t="inlineStr">
+        <is>
+          <t>Tables présentes (créées le 05/10 sur les deux projets).</t>
+        </is>
+      </c>
+      <c r="F49" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G49" s="6" t="inlineStr">
+        <is>
+          <t>À tester</t>
+        </is>
+      </c>
+      <c r="H49" s="6" t="n"/>
+      <c r="I49" s="6" t="n"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="4" t="n">
+        <v>46</v>
+      </c>
+      <c r="B50" s="5" t="inlineStr">
+        <is>
           <t>Règle de travail de décembre</t>
         </is>
       </c>
-      <c r="C46" s="4" t="inlineStr">
+      <c r="C50" s="4" t="inlineStr">
         <is>
           <t>CLAUDE.md</t>
         </is>
       </c>
-      <c r="D46" s="4" t="inlineStr">
+      <c r="D50" s="4" t="inlineStr">
         <is>
           <t>Après la mise en prod : retirer le paragraphe « Jusqu'à décembre 2026 ».</t>
         </is>
       </c>
-      <c r="E46" s="4" t="inlineStr">
+      <c r="E50" s="4" t="inlineStr">
         <is>
           <t>STA redevient identique à la PROD.</t>
         </is>
       </c>
-      <c r="F46" s="4" t="inlineStr">
+      <c r="F50" s="4" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G46" s="6" t="inlineStr">
-        <is>
-          <t>À tester</t>
-        </is>
-      </c>
-      <c r="H46" s="6" t="n"/>
-      <c r="I46" s="6" t="n"/>
+      <c r="G50" s="6" t="inlineStr">
+        <is>
+          <t>À tester</t>
+        </is>
+      </c>
+      <c r="H50" s="6" t="n"/>
+      <c r="I50" s="6" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A2:I2"/>
   </mergeCells>
-  <conditionalFormatting sqref="G5:G46">
+  <conditionalFormatting sqref="G5:G50">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"OK"</formula>
     </cfRule>
@@ -2192,7 +2355,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="G5:G46" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="G5:G50" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"À tester,OK,KO,Non testable"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Suivi : publication automatique en prod, horaires précis (journal, recette « Déjà en prod » n° 23 à 26)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AUzY5Y8Bt2KRzzte5cJgH8
</commit_message>
<xml_diff>
--- a/docs/recette/Recette_prod_decembre_2026.xlsx
+++ b/docs/recette/Recette_prod_decembre_2026.xlsx
@@ -505,7 +505,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I58"/>
+  <dimension ref="A1:I54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -2402,27 +2402,27 @@
       </c>
       <c r="B52" s="5" t="inlineStr">
         <is>
-          <t>Publications réseaux — connexion Meta</t>
+          <t>Alignement PROD / STA</t>
         </is>
       </c>
       <c r="C52" s="4" t="inlineStr">
         <is>
-          <t>Pilotage → Réseaux ; Pilotage → Services</t>
+          <t>Git</t>
         </is>
       </c>
       <c r="D52" s="4" t="inlineStr">
         <is>
-          <t>Après la saisie de META_PAGE_TOKEN dans Vercel : toucher « Tester la connexion Meta » ; regarder la ligne « Meta (publications) » des Services.</t>
+          <t>Après la fusion : git diff --quiet origin/main origin/Staging.</t>
         </is>
       </c>
       <c r="E52" s="4" t="inlineStr">
         <is>
-          <t>« ✅ Connexion Meta valide : page Mongazon360 et Instagram @… » ; rien de publié sur la page ni sur Instagram ; Services : ligne verte avec la page et le compte Instagram.</t>
+          <t>Aucune différence.</t>
         </is>
       </c>
       <c r="F52" s="4" t="inlineStr">
         <is>
-          <t>Admin</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G52" s="6" t="inlineStr">
@@ -2430,11 +2430,7 @@
           <t>À tester</t>
         </is>
       </c>
-      <c r="H52" s="6" t="inlineStr">
-        <is>
-          <t>Validé sur STA le 18/10/2026 par Jordan (page Mongazon360 et Instagram @mongazon360) ; à revérifier en prod.</t>
-        </is>
-      </c>
+      <c r="H52" s="6" t="n"/>
       <c r="I52" s="6" t="n"/>
     </row>
     <row r="53">
@@ -2443,27 +2439,27 @@
       </c>
       <c r="B53" s="5" t="inlineStr">
         <is>
-          <t>Publications réseaux — validation du lot</t>
+          <t>Base de données PROD</t>
         </is>
       </c>
       <c r="C53" s="4" t="inlineStr">
         <is>
-          <t>Pilotage → Réseaux</t>
+          <t>Supabase PROD</t>
         </is>
       </c>
       <c r="D53" s="4" t="inlineStr">
         <is>
-          <t>Ouvrir le lot de la semaine : « Voir les textes », valider une publication, en refuser une, « Remettre à valider », puis « Tout valider ».</t>
+          <t>Vérifier les tables codes et parrainages.</t>
         </is>
       </c>
       <c r="E53" s="4" t="inlineStr">
         <is>
-          <t>Statuts à jour (À valider, Validée, Refusée) et compteur « à valider » juste ; jour passé : plus de bouton, publication pas validée écartée (« Pas validée avant le jour prévu »).</t>
+          <t>Tables présentes (créées le 05/10 sur les deux projets).</t>
         </is>
       </c>
       <c r="F53" s="4" t="inlineStr">
         <is>
-          <t>Admin</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G53" s="6" t="inlineStr">
@@ -2471,11 +2467,7 @@
           <t>À tester</t>
         </is>
       </c>
-      <c r="H53" s="6" t="inlineStr">
-        <is>
-          <t>Sur STA le 17/10/2026.</t>
-        </is>
-      </c>
+      <c r="H53" s="6" t="n"/>
       <c r="I53" s="6" t="n"/>
     </row>
     <row r="54">
@@ -2484,198 +2476,42 @@
       </c>
       <c r="B54" s="5" t="inlineStr">
         <is>
-          <t>Publications réseaux — publication au créneau</t>
+          <t>Règle de travail de décembre</t>
         </is>
       </c>
       <c r="C54" s="4" t="inlineStr">
         <is>
-          <t>Tâches du matin et du soir (PROD uniquement) ; page Facebook et Instagram</t>
+          <t>CLAUDE.md</t>
         </is>
       </c>
       <c r="D54" s="4" t="inlineStr">
         <is>
-          <t>Une publication validée pour aujourd'hui : regarder la page Facebook et le compte Instagram après le créneau (dimanche vers 7-8 h, lundi, mercredi et vendredi vers 16-17 h).</t>
+          <t>Après la mise en prod : retirer le paragraphe « Jusqu'à décembre 2026 ».</t>
         </is>
       </c>
       <c r="E54" s="4" t="inlineStr">
         <is>
-          <t>Publiée sur les deux réseaux avec le visuel et le bon texte (lien suivi sur Facebook, hashtags sur Instagram) ; statut « Publiée » dans Pilotage.</t>
+          <t>STA redevient identique à la PROD.</t>
         </is>
       </c>
       <c r="F54" s="4" t="inlineStr">
         <is>
-          <t>Admin</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G54" s="6" t="inlineStr">
         <is>
-          <t>Non testable</t>
-        </is>
-      </c>
-      <c r="H54" s="6" t="inlineStr">
-        <is>
-          <t>Les tâches planifiées ne tournent qu'en prod : à vérifier à la première publication.</t>
-        </is>
-      </c>
+          <t>À tester</t>
+        </is>
+      </c>
+      <c r="H54" s="6" t="n"/>
       <c r="I54" s="6" t="n"/>
-    </row>
-    <row r="55">
-      <c r="A55" s="4" t="n">
-        <v>51</v>
-      </c>
-      <c r="B55" s="5" t="inlineStr">
-        <is>
-          <t>Publications réseaux — échec et nouvel essai</t>
-        </is>
-      </c>
-      <c r="C55" s="4" t="inlineStr">
-        <is>
-          <t>Pilotage → Réseaux ; email d'alerte ; Pilotage → Bugs</t>
-        </is>
-      </c>
-      <c r="D55" s="4" t="inlineStr">
-        <is>
-          <t>En cas d'échec (ex. Instagram refuse le visuel) : lire le message de la publication, toucher « Réessayer » le jour même.</t>
-        </is>
-      </c>
-      <c r="E55" s="4" t="inlineStr">
-        <is>
-          <t>Alerte par email et dans Bugs ; le réseau déjà publié n'est pas republié ; « Publiée » après le nouvel essai.</t>
-        </is>
-      </c>
-      <c r="F55" s="4" t="inlineStr">
-        <is>
-          <t>Admin</t>
-        </is>
-      </c>
-      <c r="G55" s="6" t="inlineStr">
-        <is>
-          <t>Non testable</t>
-        </is>
-      </c>
-      <c r="H55" s="6" t="inlineStr">
-        <is>
-          <t>Au premier cas réel.</t>
-        </is>
-      </c>
-      <c r="I55" s="6" t="n"/>
-    </row>
-    <row r="56">
-      <c r="A56" s="4" t="n">
-        <v>52</v>
-      </c>
-      <c r="B56" s="5" t="inlineStr">
-        <is>
-          <t>Alignement PROD / STA</t>
-        </is>
-      </c>
-      <c r="C56" s="4" t="inlineStr">
-        <is>
-          <t>Git</t>
-        </is>
-      </c>
-      <c r="D56" s="4" t="inlineStr">
-        <is>
-          <t>Après la fusion : git diff --quiet origin/main origin/Staging.</t>
-        </is>
-      </c>
-      <c r="E56" s="4" t="inlineStr">
-        <is>
-          <t>Aucune différence.</t>
-        </is>
-      </c>
-      <c r="F56" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G56" s="6" t="inlineStr">
-        <is>
-          <t>À tester</t>
-        </is>
-      </c>
-      <c r="H56" s="6" t="n"/>
-      <c r="I56" s="6" t="n"/>
-    </row>
-    <row r="57">
-      <c r="A57" s="4" t="n">
-        <v>53</v>
-      </c>
-      <c r="B57" s="5" t="inlineStr">
-        <is>
-          <t>Base de données PROD</t>
-        </is>
-      </c>
-      <c r="C57" s="4" t="inlineStr">
-        <is>
-          <t>Supabase PROD</t>
-        </is>
-      </c>
-      <c r="D57" s="4" t="inlineStr">
-        <is>
-          <t>Vérifier les tables codes et parrainages.</t>
-        </is>
-      </c>
-      <c r="E57" s="4" t="inlineStr">
-        <is>
-          <t>Tables présentes (créées le 05/10 sur les deux projets).</t>
-        </is>
-      </c>
-      <c r="F57" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G57" s="6" t="inlineStr">
-        <is>
-          <t>À tester</t>
-        </is>
-      </c>
-      <c r="H57" s="6" t="n"/>
-      <c r="I57" s="6" t="n"/>
-    </row>
-    <row r="58">
-      <c r="A58" s="4" t="n">
-        <v>54</v>
-      </c>
-      <c r="B58" s="5" t="inlineStr">
-        <is>
-          <t>Règle de travail de décembre</t>
-        </is>
-      </c>
-      <c r="C58" s="4" t="inlineStr">
-        <is>
-          <t>CLAUDE.md</t>
-        </is>
-      </c>
-      <c r="D58" s="4" t="inlineStr">
-        <is>
-          <t>Après la mise en prod : retirer le paragraphe « Jusqu'à décembre 2026 ».</t>
-        </is>
-      </c>
-      <c r="E58" s="4" t="inlineStr">
-        <is>
-          <t>STA redevient identique à la PROD.</t>
-        </is>
-      </c>
-      <c r="F58" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G58" s="6" t="inlineStr">
-        <is>
-          <t>À tester</t>
-        </is>
-      </c>
-      <c r="H58" s="6" t="n"/>
-      <c r="I58" s="6" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A2:I2"/>
   </mergeCells>
-  <conditionalFormatting sqref="G5:G58">
+  <conditionalFormatting sqref="G5:G54">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"OK"</formula>
     </cfRule>
@@ -2684,7 +2520,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="G5:G58" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="G5:G54" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"À tester,OK,KO,Non testable"</formula1>
     </dataValidation>
   </dataValidations>
@@ -2698,7 +2534,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I26"/>
+  <dimension ref="A1:I30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -3683,11 +3519,175 @@
         <v>46312</v>
       </c>
     </row>
+    <row r="27">
+      <c r="A27" s="4" t="n">
+        <v>23</v>
+      </c>
+      <c r="B27" s="5" t="inlineStr">
+        <is>
+          <t>Publications réseaux — connexion Meta</t>
+        </is>
+      </c>
+      <c r="C27" s="4" t="inlineStr">
+        <is>
+          <t>Pilotage → Réseaux ; Pilotage → Services</t>
+        </is>
+      </c>
+      <c r="D27" s="4" t="inlineStr">
+        <is>
+          <t>Sur mongazon360.fr : toucher « Tester la connexion Meta » ; regarder la ligne « Meta (publications) » des Services.</t>
+        </is>
+      </c>
+      <c r="E27" s="4" t="inlineStr">
+        <is>
+          <t>« ✅ Connexion Meta valide : page Mongazon360 et Instagram @mongazon360 » ; rien de publié ; Services : ligne verte.</t>
+        </is>
+      </c>
+      <c r="F27" s="4" t="inlineStr">
+        <is>
+          <t>Admin</t>
+        </is>
+      </c>
+      <c r="G27" s="6" t="inlineStr">
+        <is>
+          <t>À tester</t>
+        </is>
+      </c>
+      <c r="H27" s="6" t="inlineStr">
+        <is>
+          <t>Validé sur STA le 18/10/2026 par Jordan ; en prod le 18/10/2026 (go prod de Jordan).</t>
+        </is>
+      </c>
+      <c r="I27" s="8" t="n"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="n">
+        <v>24</v>
+      </c>
+      <c r="B28" s="5" t="inlineStr">
+        <is>
+          <t>Publications réseaux — validation du lot</t>
+        </is>
+      </c>
+      <c r="C28" s="4" t="inlineStr">
+        <is>
+          <t>Pilotage → Réseaux</t>
+        </is>
+      </c>
+      <c r="D28" s="4" t="inlineStr">
+        <is>
+          <t>Samedi 24/10 : ouvrir le lot du 1er au 7 novembre, « Voir les textes », valider une par une ou « Tout valider », en refuser une si besoin.</t>
+        </is>
+      </c>
+      <c r="E28" s="4" t="inlineStr">
+        <is>
+          <t>Statuts à jour (À valider, Validée, Refusée) et compteur « à valider » juste ; jour passé : plus de bouton.</t>
+        </is>
+      </c>
+      <c r="F28" s="4" t="inlineStr">
+        <is>
+          <t>Admin</t>
+        </is>
+      </c>
+      <c r="G28" s="6" t="inlineStr">
+        <is>
+          <t>À tester</t>
+        </is>
+      </c>
+      <c r="H28" s="6" t="inlineStr">
+        <is>
+          <t>Premier lot inséré par la tâche du samedi 24/10/2026.</t>
+        </is>
+      </c>
+      <c r="I28" s="8" t="n"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="n">
+        <v>25</v>
+      </c>
+      <c r="B29" s="5" t="inlineStr">
+        <is>
+          <t>Publications réseaux — publication à l'heure</t>
+        </is>
+      </c>
+      <c r="C29" s="4" t="inlineStr">
+        <is>
+          <t>Page Facebook et compte Instagram de Mongazon360</t>
+        </is>
+      </c>
+      <c r="D29" s="4" t="inlineStr">
+        <is>
+          <t>Dimanche 1er novembre après 8 h, puis lundi 2 après 16 h 30 : regarder la page Facebook et le compte Instagram.</t>
+        </is>
+      </c>
+      <c r="E29" s="4" t="inlineStr">
+        <is>
+          <t>Publication en ligne sur les deux réseaux à l'heure prévue (à quelques minutes près), avec le visuel et le bon texte ; « Publiée » dans Pilotage.</t>
+        </is>
+      </c>
+      <c r="F29" s="4" t="inlineStr">
+        <is>
+          <t>Admin</t>
+        </is>
+      </c>
+      <c r="G29" s="6" t="inlineStr">
+        <is>
+          <t>À tester</t>
+        </is>
+      </c>
+      <c r="H29" s="6" t="inlineStr">
+        <is>
+          <t>Déclencheur pg_cron toutes les 15 min (Supabase PROD), tâches planifiées de Vercel en secours.</t>
+        </is>
+      </c>
+      <c r="I29" s="8" t="n"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="n">
+        <v>26</v>
+      </c>
+      <c r="B30" s="5" t="inlineStr">
+        <is>
+          <t>Publications réseaux — échec et nouvel essai</t>
+        </is>
+      </c>
+      <c r="C30" s="4" t="inlineStr">
+        <is>
+          <t>Pilotage → Réseaux ; email d'alerte ; Pilotage → Bugs</t>
+        </is>
+      </c>
+      <c r="D30" s="4" t="inlineStr">
+        <is>
+          <t>En cas d'échec (ex. Instagram refuse le visuel) : lire le message de la publication, toucher « Réessayer » le jour même.</t>
+        </is>
+      </c>
+      <c r="E30" s="4" t="inlineStr">
+        <is>
+          <t>Alerte par email et dans Bugs ; le réseau déjà publié n'est pas republié ; « Publiée » après le nouvel essai.</t>
+        </is>
+      </c>
+      <c r="F30" s="4" t="inlineStr">
+        <is>
+          <t>Admin</t>
+        </is>
+      </c>
+      <c r="G30" s="6" t="inlineStr">
+        <is>
+          <t>Non testable</t>
+        </is>
+      </c>
+      <c r="H30" s="6" t="inlineStr">
+        <is>
+          <t>Au premier cas réel.</t>
+        </is>
+      </c>
+      <c r="I30" s="8" t="n"/>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A2:I2"/>
   </mergeCells>
-  <conditionalFormatting sqref="G5:G26">
+  <conditionalFormatting sqref="G5:G30">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"OK"</formula>
     </cfRule>
@@ -3696,7 +3696,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="G5:G26" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="G5:G30" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"À tester,OK,KO,Non testable"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Suivi : connexion Meta validée en prod, app Meta publiée (journal, recette n° 23)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AUzY5Y8Bt2KRzzte5cJgH8
</commit_message>
<xml_diff>
--- a/docs/recette/Recette_prod_decembre_2026.xlsx
+++ b/docs/recette/Recette_prod_decembre_2026.xlsx
@@ -533,7 +533,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -2562,6 +2561,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -3550,15 +3550,17 @@
       </c>
       <c r="G27" s="6" t="inlineStr">
         <is>
-          <t>À tester</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="H27" s="6" t="inlineStr">
         <is>
-          <t>Validé sur STA le 18/10/2026 par Jordan ; en prod le 18/10/2026 (go prod de Jordan).</t>
-        </is>
-      </c>
-      <c r="I27" s="8" t="n"/>
+          <t>Validé sur STA le 18/10/2026 par Jordan ; en prod le 18/10/2026 (go prod de Jordan) ; testé en prod par Jordan le 18/10/2026 : OK.</t>
+        </is>
+      </c>
+      <c r="I27" s="8" t="n">
+        <v>46313</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="4" t="n">

</xml_diff>

<commit_message>
Équipements : stations météo de toutes marques par Weather Underground (STA)
Une station qui publie sur Weather Underground (Froggit, Bresser, Ambient Weather…) se connecte avec son identifiant et
la clé API créée par son propriétaire sur wunderground.com (clé chiffrée, jamais de mot de passe). Température, pluie du
jour, humidité et vent remplacent les prévisions de la journée, comme pour Netatmo, Ecowitt et Davis. Politique de
confidentialité (6.3), consignes de Bob, CLAUDE.md, journal, recette de décembre n° 48.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AUzY5Y8Bt2KRzzte5cJgH8
</commit_message>
<xml_diff>
--- a/docs/recette/Recette_prod_decembre_2026.xlsx
+++ b/docs/recette/Recette_prod_decembre_2026.xlsx
@@ -505,7 +505,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I54"/>
+  <dimension ref="A1:I55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -533,6 +533,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -2401,27 +2402,27 @@
       </c>
       <c r="B52" s="5" t="inlineStr">
         <is>
-          <t>Alignement PROD / STA</t>
+          <t>Station Weather Underground — connexion et mesures</t>
         </is>
       </c>
       <c r="C52" s="4" t="inlineStr">
         <is>
-          <t>Git</t>
+          <t>Mes équipements → Station météo ; Aujourd'hui ; Bob</t>
         </is>
       </c>
       <c r="D52" s="4" t="inlineStr">
         <is>
-          <t>Après la fusion : git diff --quiet origin/main origin/Staging.</t>
+          <t>Avec une station qui publie sur Weather Underground (Froggit, Bresser, Ambient Weather…) : créer une clé sur wunderground.com (API Keys), saisir l'identifiant de la station et la clé, connecter ; puis ouvrir « Aujourd'hui ».</t>
         </is>
       </c>
       <c r="E52" s="4" t="inlineStr">
         <is>
-          <t>Aucune différence.</t>
+          <t>Station « ✓ connectée » avec son nom (quartier déclaré) ; température en °C, pluie du jour en mm, vent en km/h ; pluie mesurée prise en compte pour l'arrosage ; identifiant faux : message clair.</t>
         </is>
       </c>
       <c r="F52" s="4" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Compte avec station publiant sur Weather Underground</t>
         </is>
       </c>
       <c r="G52" s="6" t="inlineStr">
@@ -2429,7 +2430,11 @@
           <t>À tester</t>
         </is>
       </c>
-      <c r="H52" s="6" t="n"/>
+      <c r="H52" s="6" t="inlineStr">
+        <is>
+          <t>Sur STA le 18/10/2026.</t>
+        </is>
+      </c>
       <c r="I52" s="6" t="n"/>
     </row>
     <row r="53">
@@ -2438,22 +2443,22 @@
       </c>
       <c r="B53" s="5" t="inlineStr">
         <is>
-          <t>Base de données PROD</t>
+          <t>Alignement PROD / STA</t>
         </is>
       </c>
       <c r="C53" s="4" t="inlineStr">
         <is>
-          <t>Supabase PROD</t>
+          <t>Git</t>
         </is>
       </c>
       <c r="D53" s="4" t="inlineStr">
         <is>
-          <t>Vérifier les tables codes et parrainages.</t>
+          <t>Après la fusion : git diff --quiet origin/main origin/Staging.</t>
         </is>
       </c>
       <c r="E53" s="4" t="inlineStr">
         <is>
-          <t>Tables présentes (créées le 05/10 sur les deux projets).</t>
+          <t>Aucune différence.</t>
         </is>
       </c>
       <c r="F53" s="4" t="inlineStr">
@@ -2475,22 +2480,22 @@
       </c>
       <c r="B54" s="5" t="inlineStr">
         <is>
-          <t>Règle de travail de décembre</t>
+          <t>Base de données PROD</t>
         </is>
       </c>
       <c r="C54" s="4" t="inlineStr">
         <is>
-          <t>CLAUDE.md</t>
+          <t>Supabase PROD</t>
         </is>
       </c>
       <c r="D54" s="4" t="inlineStr">
         <is>
-          <t>Après la mise en prod : retirer le paragraphe « Jusqu'à décembre 2026 ».</t>
+          <t>Vérifier les tables codes et parrainages.</t>
         </is>
       </c>
       <c r="E54" s="4" t="inlineStr">
         <is>
-          <t>STA redevient identique à la PROD.</t>
+          <t>Tables présentes (créées le 05/10 sur les deux projets).</t>
         </is>
       </c>
       <c r="F54" s="4" t="inlineStr">
@@ -2505,12 +2510,49 @@
       </c>
       <c r="H54" s="6" t="n"/>
       <c r="I54" s="6" t="n"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="4" t="n">
+        <v>51</v>
+      </c>
+      <c r="B55" s="5" t="inlineStr">
+        <is>
+          <t>Règle de travail de décembre</t>
+        </is>
+      </c>
+      <c r="C55" s="4" t="inlineStr">
+        <is>
+          <t>CLAUDE.md</t>
+        </is>
+      </c>
+      <c r="D55" s="4" t="inlineStr">
+        <is>
+          <t>Après la mise en prod : retirer le paragraphe « Jusqu'à décembre 2026 ».</t>
+        </is>
+      </c>
+      <c r="E55" s="4" t="inlineStr">
+        <is>
+          <t>STA redevient identique à la PROD.</t>
+        </is>
+      </c>
+      <c r="F55" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G55" s="6" t="inlineStr">
+        <is>
+          <t>À tester</t>
+        </is>
+      </c>
+      <c r="H55" s="6" t="n"/>
+      <c r="I55" s="6" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A2:I2"/>
   </mergeCells>
-  <conditionalFormatting sqref="G5:G54">
+  <conditionalFormatting sqref="G5:G55">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"OK"</formula>
     </cfRule>
@@ -2519,7 +2561,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="G5:G54" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="G5:G55" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"À tester,OK,KO,Non testable"</formula1>
     </dataValidation>
   </dataValidations>
@@ -2561,7 +2603,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Équipements : « Ton équipement n'est pas dans la liste ? » et équipements demandés dans Pilotage (STA)
En bas de « Mes équipements », l'utilisateur indique le type, la marque et le modèle d'un équipement à connecter (envoi
anonyme, table equipements_demandes). Pilotage → Activité regroupe les demandes par type et marque, de la plus demandée
à la moins demandée : choix des prochains connecteurs et chiffres pour les marques. Consignes de Bob, CLAUDE.md, journal,
recette de décembre n° 49 et 50.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AUzY5Y8Bt2KRzzte5cJgH8
</commit_message>
<xml_diff>
--- a/docs/recette/Recette_prod_decembre_2026.xlsx
+++ b/docs/recette/Recette_prod_decembre_2026.xlsx
@@ -505,7 +505,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I55"/>
+  <dimension ref="A1:I57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -2443,27 +2443,27 @@
       </c>
       <c r="B53" s="5" t="inlineStr">
         <is>
-          <t>Alignement PROD / STA</t>
+          <t>Équipement non listé — envoi</t>
         </is>
       </c>
       <c r="C53" s="4" t="inlineStr">
         <is>
-          <t>Git</t>
+          <t>Mes équipements (en bas de page)</t>
         </is>
       </c>
       <c r="D53" s="4" t="inlineStr">
         <is>
-          <t>Après la fusion : git diff --quiet origin/main origin/Staging.</t>
+          <t>Dans « Ton équipement n'est pas dans la liste ? » : choisir un type, saisir une marque (et un modèle), toucher « Envoyer ».</t>
         </is>
       </c>
       <c r="E53" s="4" t="inlineStr">
         <is>
-          <t>Aucune différence.</t>
+          <t>« ✅ Merci, c'est noté » ; bouton grisé sans marque ; rien de personnel enregistré (demande anonyme).</t>
         </is>
       </c>
       <c r="F53" s="4" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Tous</t>
         </is>
       </c>
       <c r="G53" s="6" t="inlineStr">
@@ -2471,7 +2471,11 @@
           <t>À tester</t>
         </is>
       </c>
-      <c r="H53" s="6" t="n"/>
+      <c r="H53" s="6" t="inlineStr">
+        <is>
+          <t>Sur STA le 18/10/2026.</t>
+        </is>
+      </c>
       <c r="I53" s="6" t="n"/>
     </row>
     <row r="54">
@@ -2480,27 +2484,27 @@
       </c>
       <c r="B54" s="5" t="inlineStr">
         <is>
-          <t>Base de données PROD</t>
+          <t>Pilotage — équipements demandés</t>
         </is>
       </c>
       <c r="C54" s="4" t="inlineStr">
         <is>
-          <t>Supabase PROD</t>
+          <t>Pilotage → Activité (carte « Équipements demandés »)</t>
         </is>
       </c>
       <c r="D54" s="4" t="inlineStr">
         <is>
-          <t>Vérifier les tables codes et parrainages.</t>
+          <t>Après une ou deux demandes de test : ouvrir Pilotage → Activité.</t>
         </is>
       </c>
       <c r="E54" s="4" t="inlineStr">
         <is>
-          <t>Tables présentes (créées le 05/10 sur les deux projets).</t>
+          <t>Demandes regroupées par type et marque (casse ignorée), du plus demandé au moins demandé, avec les modèles cités.</t>
         </is>
       </c>
       <c r="F54" s="4" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Admin</t>
         </is>
       </c>
       <c r="G54" s="6" t="inlineStr">
@@ -2508,7 +2512,11 @@
           <t>À tester</t>
         </is>
       </c>
-      <c r="H54" s="6" t="n"/>
+      <c r="H54" s="6" t="inlineStr">
+        <is>
+          <t>Sur STA le 18/10/2026.</t>
+        </is>
+      </c>
       <c r="I54" s="6" t="n"/>
     </row>
     <row r="55">
@@ -2517,22 +2525,22 @@
       </c>
       <c r="B55" s="5" t="inlineStr">
         <is>
-          <t>Règle de travail de décembre</t>
+          <t>Alignement PROD / STA</t>
         </is>
       </c>
       <c r="C55" s="4" t="inlineStr">
         <is>
-          <t>CLAUDE.md</t>
+          <t>Git</t>
         </is>
       </c>
       <c r="D55" s="4" t="inlineStr">
         <is>
-          <t>Après la mise en prod : retirer le paragraphe « Jusqu'à décembre 2026 ».</t>
+          <t>Après la fusion : git diff --quiet origin/main origin/Staging.</t>
         </is>
       </c>
       <c r="E55" s="4" t="inlineStr">
         <is>
-          <t>STA redevient identique à la PROD.</t>
+          <t>Aucune différence.</t>
         </is>
       </c>
       <c r="F55" s="4" t="inlineStr">
@@ -2547,12 +2555,86 @@
       </c>
       <c r="H55" s="6" t="n"/>
       <c r="I55" s="6" t="n"/>
+    </row>
+    <row r="56">
+      <c r="A56" s="4" t="n">
+        <v>52</v>
+      </c>
+      <c r="B56" s="5" t="inlineStr">
+        <is>
+          <t>Base de données PROD</t>
+        </is>
+      </c>
+      <c r="C56" s="4" t="inlineStr">
+        <is>
+          <t>Supabase PROD</t>
+        </is>
+      </c>
+      <c r="D56" s="4" t="inlineStr">
+        <is>
+          <t>Vérifier les tables codes et parrainages.</t>
+        </is>
+      </c>
+      <c r="E56" s="4" t="inlineStr">
+        <is>
+          <t>Tables présentes (créées le 05/10 sur les deux projets).</t>
+        </is>
+      </c>
+      <c r="F56" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G56" s="6" t="inlineStr">
+        <is>
+          <t>À tester</t>
+        </is>
+      </c>
+      <c r="H56" s="6" t="n"/>
+      <c r="I56" s="6" t="n"/>
+    </row>
+    <row r="57">
+      <c r="A57" s="4" t="n">
+        <v>53</v>
+      </c>
+      <c r="B57" s="5" t="inlineStr">
+        <is>
+          <t>Règle de travail de décembre</t>
+        </is>
+      </c>
+      <c r="C57" s="4" t="inlineStr">
+        <is>
+          <t>CLAUDE.md</t>
+        </is>
+      </c>
+      <c r="D57" s="4" t="inlineStr">
+        <is>
+          <t>Après la mise en prod : retirer le paragraphe « Jusqu'à décembre 2026 ».</t>
+        </is>
+      </c>
+      <c r="E57" s="4" t="inlineStr">
+        <is>
+          <t>STA redevient identique à la PROD.</t>
+        </is>
+      </c>
+      <c r="F57" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G57" s="6" t="inlineStr">
+        <is>
+          <t>À tester</t>
+        </is>
+      </c>
+      <c r="H57" s="6" t="n"/>
+      <c r="I57" s="6" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A2:I2"/>
   </mergeCells>
-  <conditionalFormatting sqref="G5:G55">
+  <conditionalFormatting sqref="G5:G57">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"OK"</formula>
     </cfRule>
@@ -2561,7 +2643,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="G5:G55" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="G5:G57" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"À tester,OK,KO,Non testable"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Suivi : sécurité de la tâche planifiée en prod (journal, recette « Déjà en prod » n° 27 et 28)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AUzY5Y8Bt2KRzzte5cJgH8
</commit_message>
<xml_diff>
--- a/docs/recette/Recette_prod_decembre_2026.xlsx
+++ b/docs/recette/Recette_prod_decembre_2026.xlsx
@@ -533,7 +533,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -2657,7 +2656,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I30"/>
+  <dimension ref="A1:I32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -3808,6 +3807,90 @@
       </c>
       <c r="I30" s="8" t="n"/>
     </row>
+    <row r="31">
+      <c r="A31" s="4" t="n">
+        <v>27</v>
+      </c>
+      <c r="B31" s="5" t="inlineStr">
+        <is>
+          <t>Tâche planifiée — clé CRON_SECRET</t>
+        </is>
+      </c>
+      <c r="C31" s="4" t="inlineStr">
+        <is>
+          <t>Tâches planifiées de Vercel (matin et soir) ; Pilotage → Bugs</t>
+        </is>
+      </c>
+      <c r="D31" s="4" t="inlineStr">
+        <is>
+          <t>Lendemain de la mise en prod : vérifier que la tâche du matin (8 h) et celle du soir (17 h) sont passées (conseils du jour reçus) ; regarder Pilotage → Bugs.</t>
+        </is>
+      </c>
+      <c r="E31" s="4" t="inlineStr">
+        <is>
+          <t>Tâches passées, aucune erreur « Tâche planifiée refusée » ; un appel sans la clé ou avec une mauvaise clé est refusé (401).</t>
+        </is>
+      </c>
+      <c r="F31" s="4" t="inlineStr">
+        <is>
+          <t>Admin</t>
+        </is>
+      </c>
+      <c r="G31" s="6" t="inlineStr">
+        <is>
+          <t>À tester</t>
+        </is>
+      </c>
+      <c r="H31" s="6" t="inlineStr">
+        <is>
+          <t>En prod le 18/10/2026 (go prod de Jordan) ; clé remplacée par Jordan en prod et sur STA (l'ancienne figurait dans l'historique public du dépôt). Appels sans clé ou avec une mauvaise clé refusés : vérifié le 18/10/2026.</t>
+        </is>
+      </c>
+      <c r="I31" s="8" t="n"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="n">
+        <v>28</v>
+      </c>
+      <c r="B32" s="5" t="inlineStr">
+        <is>
+          <t>Publications réseaux — déclencheur réservé à pg_cron</t>
+        </is>
+      </c>
+      <c r="C32" s="4" t="inlineStr">
+        <is>
+          <t>Supabase PROD (tâche mongazon360-publications-reseaux)</t>
+        </is>
+      </c>
+      <c r="D32" s="4" t="inlineStr">
+        <is>
+          <t>Appeler POST /api/send?type=publications sans clé ; regarder les derniers passages de la tâche pg_cron.</t>
+        </is>
+      </c>
+      <c r="E32" s="4" t="inlineStr">
+        <is>
+          <t>Appel sans clé refusé (401) ; passages de la tâche pg_cron acceptés (200), toutes les 15 min.</t>
+        </is>
+      </c>
+      <c r="F32" s="4" t="inlineStr">
+        <is>
+          <t>Admin</t>
+        </is>
+      </c>
+      <c r="G32" s="6" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="H32" s="6" t="inlineStr">
+        <is>
+          <t>En prod le 18/10/2026 (go prod de Jordan) ; vérifié le 18/10/2026 : appel sans clé refusé, passage pg_cron de 18 h 45 accepté.</t>
+        </is>
+      </c>
+      <c r="I32" s="8" t="n">
+        <v>46313</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A2:I2"/>
@@ -3821,7 +3904,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="G5:G30" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="G5:G32" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"À tester,OK,KO,Non testable"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Diagnostic : niveau de confiance, ce que Bob a vu et photo à reprendre (STA)
Le diagnostic photo indique sa confiance (élevée, moyenne, faible) et les éléments réellement observés sur la photo.
Une photo qui ne permet pas de conclure (floue, sombre, sans gazon) n'a plus de score inventé : écran « Photo à
reprendre » avec le conseil de Bob, rien d'enregistré ; à l'essai sans compte, elle ne consomme pas le diagnostic
gratuit. Colonnes confiance et observations (diagnostics, diagnostics_anon) ; confiance dans le contexte et les consignes
de Bob ; recette de décembre n° 51 à 53.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AUzY5Y8Bt2KRzzte5cJgH8
</commit_message>
<xml_diff>
--- a/docs/recette/Recette_prod_decembre_2026.xlsx
+++ b/docs/recette/Recette_prod_decembre_2026.xlsx
@@ -505,7 +505,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I57"/>
+  <dimension ref="A1:I60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -2524,27 +2524,27 @@
       </c>
       <c r="B55" s="5" t="inlineStr">
         <is>
-          <t>Alignement PROD / STA</t>
+          <t>Diagnostic — niveau de confiance</t>
         </is>
       </c>
       <c r="C55" s="4" t="inlineStr">
         <is>
-          <t>Git</t>
+          <t>Diagnostic (résultat et historique)</t>
         </is>
       </c>
       <c r="D55" s="4" t="inlineStr">
         <is>
-          <t>Après la fusion : git diff --quiet origin/main origin/Staging.</t>
+          <t>Faire un diagnostic avec une photo nette, en plein jour, à 1 m du sol ; puis rouvrir ce diagnostic dans l'historique.</t>
         </is>
       </c>
       <c r="E55" s="4" t="inlineStr">
         <is>
-          <t>Aucune différence.</t>
+          <t>Sous le score : « 🎯 Confiance élevée, moyenne ou faible » avec une phrase d'explication, et « 👀 Ce que Bob a vu » (2 à 4 éléments réellement visibles sur la photo) ; mêmes informations dans l'historique. Confiance faible : conseil pour reprendre la photo et bouton « Reprendre une photo ».</t>
         </is>
       </c>
       <c r="F55" s="4" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Premium</t>
         </is>
       </c>
       <c r="G55" s="6" t="inlineStr">
@@ -2552,7 +2552,11 @@
           <t>À tester</t>
         </is>
       </c>
-      <c r="H55" s="6" t="n"/>
+      <c r="H55" s="6" t="inlineStr">
+        <is>
+          <t>Sur STA le 18/10/2026.</t>
+        </is>
+      </c>
       <c r="I55" s="6" t="n"/>
     </row>
     <row r="56">
@@ -2561,27 +2565,27 @@
       </c>
       <c r="B56" s="5" t="inlineStr">
         <is>
-          <t>Base de données PROD</t>
+          <t>Diagnostic — photo à reprendre</t>
         </is>
       </c>
       <c r="C56" s="4" t="inlineStr">
         <is>
-          <t>Supabase PROD</t>
+          <t>Diagnostic</t>
         </is>
       </c>
       <c r="D56" s="4" t="inlineStr">
         <is>
-          <t>Vérifier les tables codes et parrainages.</t>
+          <t>Lancer un diagnostic avec une photo floue, très sombre ou sans gazon (ex. un mur).</t>
         </is>
       </c>
       <c r="E56" s="4" t="inlineStr">
         <is>
-          <t>Tables présentes (créées le 05/10 sur les deux projets).</t>
+          <t>Écran « 📷 Photo à reprendre » : explication de Bob, conseil pour la reprendre et boutons photo ; aucun score, rien dans l'historique ni dans Bob.</t>
         </is>
       </c>
       <c r="F56" s="4" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Premium</t>
         </is>
       </c>
       <c r="G56" s="6" t="inlineStr">
@@ -2589,7 +2593,11 @@
           <t>À tester</t>
         </is>
       </c>
-      <c r="H56" s="6" t="n"/>
+      <c r="H56" s="6" t="inlineStr">
+        <is>
+          <t>Sur STA le 18/10/2026.</t>
+        </is>
+      </c>
       <c r="I56" s="6" t="n"/>
     </row>
     <row r="57">
@@ -2598,42 +2606,157 @@
       </c>
       <c r="B57" s="5" t="inlineStr">
         <is>
+          <t>Essai sans compte — photo à reprendre</t>
+        </is>
+      </c>
+      <c r="C57" s="4" t="inlineStr">
+        <is>
+          <t>Essai du diagnostic (sans compte)</t>
+        </is>
+      </c>
+      <c r="D57" s="4" t="inlineStr">
+        <is>
+          <t>Non connecté : essai du diagnostic avec une photo sans gazon, puis avec une vraie photo de pelouse.</t>
+        </is>
+      </c>
+      <c r="E57" s="4" t="inlineStr">
+        <is>
+          <t>1re photo : « Bob ne peut pas conclure avec cette photo » et « Ton diagnostic gratuit n'est pas utilisé » ; 2e photo : score, confiance et ce que Bob a vu, puis l'analyse complète à débloquer comme avant.</t>
+        </is>
+      </c>
+      <c r="F57" s="4" t="inlineStr">
+        <is>
+          <t>Non connecté</t>
+        </is>
+      </c>
+      <c r="G57" s="6" t="inlineStr">
+        <is>
+          <t>À tester</t>
+        </is>
+      </c>
+      <c r="H57" s="6" t="inlineStr">
+        <is>
+          <t>Sur STA le 18/10/2026.</t>
+        </is>
+      </c>
+      <c r="I57" s="6" t="n"/>
+    </row>
+    <row r="58">
+      <c r="A58" s="4" t="n">
+        <v>54</v>
+      </c>
+      <c r="B58" s="5" t="inlineStr">
+        <is>
+          <t>Alignement PROD / STA</t>
+        </is>
+      </c>
+      <c r="C58" s="4" t="inlineStr">
+        <is>
+          <t>Git</t>
+        </is>
+      </c>
+      <c r="D58" s="4" t="inlineStr">
+        <is>
+          <t>Après la fusion : git diff --quiet origin/main origin/Staging.</t>
+        </is>
+      </c>
+      <c r="E58" s="4" t="inlineStr">
+        <is>
+          <t>Aucune différence.</t>
+        </is>
+      </c>
+      <c r="F58" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G58" s="6" t="inlineStr">
+        <is>
+          <t>À tester</t>
+        </is>
+      </c>
+      <c r="H58" s="6" t="n"/>
+      <c r="I58" s="6" t="n"/>
+    </row>
+    <row r="59">
+      <c r="A59" s="4" t="n">
+        <v>55</v>
+      </c>
+      <c r="B59" s="5" t="inlineStr">
+        <is>
+          <t>Base de données PROD</t>
+        </is>
+      </c>
+      <c r="C59" s="4" t="inlineStr">
+        <is>
+          <t>Supabase PROD</t>
+        </is>
+      </c>
+      <c r="D59" s="4" t="inlineStr">
+        <is>
+          <t>Vérifier les tables codes et parrainages.</t>
+        </is>
+      </c>
+      <c r="E59" s="4" t="inlineStr">
+        <is>
+          <t>Tables présentes (créées le 05/10 sur les deux projets).</t>
+        </is>
+      </c>
+      <c r="F59" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G59" s="6" t="inlineStr">
+        <is>
+          <t>À tester</t>
+        </is>
+      </c>
+      <c r="H59" s="6" t="n"/>
+      <c r="I59" s="6" t="n"/>
+    </row>
+    <row r="60">
+      <c r="A60" s="4" t="n">
+        <v>56</v>
+      </c>
+      <c r="B60" s="5" t="inlineStr">
+        <is>
           <t>Règle de travail de décembre</t>
         </is>
       </c>
-      <c r="C57" s="4" t="inlineStr">
+      <c r="C60" s="4" t="inlineStr">
         <is>
           <t>CLAUDE.md</t>
         </is>
       </c>
-      <c r="D57" s="4" t="inlineStr">
+      <c r="D60" s="4" t="inlineStr">
         <is>
           <t>Après la mise en prod : retirer le paragraphe « Jusqu'à décembre 2026 ».</t>
         </is>
       </c>
-      <c r="E57" s="4" t="inlineStr">
+      <c r="E60" s="4" t="inlineStr">
         <is>
           <t>STA redevient identique à la PROD.</t>
         </is>
       </c>
-      <c r="F57" s="4" t="inlineStr">
+      <c r="F60" s="4" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G57" s="6" t="inlineStr">
-        <is>
-          <t>À tester</t>
-        </is>
-      </c>
-      <c r="H57" s="6" t="n"/>
-      <c r="I57" s="6" t="n"/>
+      <c r="G60" s="6" t="inlineStr">
+        <is>
+          <t>À tester</t>
+        </is>
+      </c>
+      <c r="H60" s="6" t="n"/>
+      <c r="I60" s="6" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A2:I2"/>
   </mergeCells>
-  <conditionalFormatting sqref="G5:G57">
+  <conditionalFormatting sqref="G5:G60">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"OK"</formula>
     </cfRule>
@@ -2642,7 +2765,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="G5:G57" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="G5:G60" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"À tester,OK,KO,Non testable"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Diagnostic de suivi : photo proposée après un regarnissage, une scarification, un anti-mousse ou un désherbage, comparée avant / après (STA)
Au bout du délai de l'action (30 jours ; 21 pour un désherbage, src/lib/suiviDiagnostic.json, tirés de la base de
connaissances), l'onglet Diagnostic propose pendant 7 jours une photo du même endroit, et la tâche du matin envoie une
notification une fois par action (api/suiviDiagnostic.cjs, même règle que l'app). Le résultat compare au diagnostic fait
dans les 45 jours avant l'action : photos, écart de score, problèmes réglés, encore là ou nouveaux. Historique des
diagnostics : doublons de l'appareil retirés (même photo). Consignes de Bob ; recette de décembre n° 54 à 56.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AUzY5Y8Bt2KRzzte5cJgH8
</commit_message>
<xml_diff>
--- a/docs/recette/Recette_prod_decembre_2026.xlsx
+++ b/docs/recette/Recette_prod_decembre_2026.xlsx
@@ -505,7 +505,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I60"/>
+  <dimension ref="A1:I63"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -2647,27 +2647,27 @@
       </c>
       <c r="B58" s="5" t="inlineStr">
         <is>
-          <t>Alignement PROD / STA</t>
+          <t>Diagnostic de suivi — proposition</t>
         </is>
       </c>
       <c r="C58" s="4" t="inlineStr">
         <is>
-          <t>Git</t>
+          <t>Diagnostic (accueil)</t>
         </is>
       </c>
       <c r="D58" s="4" t="inlineStr">
         <is>
-          <t>Après la fusion : git diff --quiet origin/main origin/Staging.</t>
+          <t>Compte de test : faire un diagnostic, puis valider « Regarnissage » dans Aujourd'hui ; 30 jours plus tard (ou en antidatant l'action et le diagnostic dans la base de STA), ouvrir l'onglet Diagnostic.</t>
         </is>
       </c>
       <c r="E58" s="4" t="inlineStr">
         <is>
-          <t>Aucune différence.</t>
+          <t>Carte « 📸 C'est le moment du diagnostic de suivi » avec la photo d'avant, la date de l'action, « a 30 jours » et le score d'avant ; carte affichée 7 jours, puis plus après une nouvelle photo. Désherbage : à 21 jours.</t>
         </is>
       </c>
       <c r="F58" s="4" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Premium</t>
         </is>
       </c>
       <c r="G58" s="6" t="inlineStr">
@@ -2675,7 +2675,11 @@
           <t>À tester</t>
         </is>
       </c>
-      <c r="H58" s="6" t="n"/>
+      <c r="H58" s="6" t="inlineStr">
+        <is>
+          <t>Sur STA le 18/10/2026. Délais : base de connaissances (levée J21-J45, anti-mousse 30 j, désherbage 21 j) ; scarification 30 j à valider par Jordan.</t>
+        </is>
+      </c>
       <c r="I58" s="6" t="n"/>
     </row>
     <row r="59">
@@ -2684,27 +2688,27 @@
       </c>
       <c r="B59" s="5" t="inlineStr">
         <is>
-          <t>Base de données PROD</t>
+          <t>Diagnostic de suivi — avant / après</t>
         </is>
       </c>
       <c r="C59" s="4" t="inlineStr">
         <is>
-          <t>Supabase PROD</t>
+          <t>Diagnostic (résultat)</t>
         </is>
       </c>
       <c r="D59" s="4" t="inlineStr">
         <is>
-          <t>Vérifier les tables codes et parrainages.</t>
+          <t>Pendant la période de suivi, faire le diagnostic du même endroit.</t>
         </is>
       </c>
       <c r="E59" s="4" t="inlineStr">
         <is>
-          <t>Tables présentes (créées le 05/10 sur les deux projets).</t>
+          <t>Carte « 📈 Depuis ton regarnissage du … » : photos avant / aujourd'hui avec leurs scores, écart en points (vert si +5 ou plus, rouge si -5 ou moins), problèmes réglés, encore là ou nouveaux.</t>
         </is>
       </c>
       <c r="F59" s="4" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Premium</t>
         </is>
       </c>
       <c r="G59" s="6" t="inlineStr">
@@ -2712,7 +2716,11 @@
           <t>À tester</t>
         </is>
       </c>
-      <c r="H59" s="6" t="n"/>
+      <c r="H59" s="6" t="inlineStr">
+        <is>
+          <t>Sur STA le 18/10/2026.</t>
+        </is>
+      </c>
       <c r="I59" s="6" t="n"/>
     </row>
     <row r="60">
@@ -2721,42 +2729,157 @@
       </c>
       <c r="B60" s="5" t="inlineStr">
         <is>
+          <t>Diagnostic de suivi — notification</t>
+        </is>
+      </c>
+      <c r="C60" s="4" t="inlineStr">
+        <is>
+          <t>Notification du matin (PROD uniquement)</t>
+        </is>
+      </c>
+      <c r="D60" s="4" t="inlineStr">
+        <is>
+          <t>Le jour où le suivi arrive à échéance, avec les notifications ou les conseils par email activés.</t>
+        </is>
+      </c>
+      <c r="E60" s="4" t="inlineStr">
+        <is>
+          <t>Notification « 📸 Ton regarnissage a 30 jours » qui ouvre l'onglet Diagnostic ; une seule fois par action.</t>
+        </is>
+      </c>
+      <c r="F60" s="4" t="inlineStr">
+        <is>
+          <t>Premium avec notifications</t>
+        </is>
+      </c>
+      <c r="G60" s="6" t="inlineStr">
+        <is>
+          <t>Non testable</t>
+        </is>
+      </c>
+      <c r="H60" s="6" t="inlineStr">
+        <is>
+          <t>Non testable sur STA : tâches du matin en prod uniquement.</t>
+        </is>
+      </c>
+      <c r="I60" s="6" t="n"/>
+    </row>
+    <row r="61">
+      <c r="A61" s="4" t="n">
+        <v>57</v>
+      </c>
+      <c r="B61" s="5" t="inlineStr">
+        <is>
+          <t>Alignement PROD / STA</t>
+        </is>
+      </c>
+      <c r="C61" s="4" t="inlineStr">
+        <is>
+          <t>Git</t>
+        </is>
+      </c>
+      <c r="D61" s="4" t="inlineStr">
+        <is>
+          <t>Après la fusion : git diff --quiet origin/main origin/Staging.</t>
+        </is>
+      </c>
+      <c r="E61" s="4" t="inlineStr">
+        <is>
+          <t>Aucune différence.</t>
+        </is>
+      </c>
+      <c r="F61" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G61" s="6" t="inlineStr">
+        <is>
+          <t>À tester</t>
+        </is>
+      </c>
+      <c r="H61" s="6" t="n"/>
+      <c r="I61" s="6" t="n"/>
+    </row>
+    <row r="62">
+      <c r="A62" s="4" t="n">
+        <v>58</v>
+      </c>
+      <c r="B62" s="5" t="inlineStr">
+        <is>
+          <t>Base de données PROD</t>
+        </is>
+      </c>
+      <c r="C62" s="4" t="inlineStr">
+        <is>
+          <t>Supabase PROD</t>
+        </is>
+      </c>
+      <c r="D62" s="4" t="inlineStr">
+        <is>
+          <t>Vérifier les tables codes et parrainages.</t>
+        </is>
+      </c>
+      <c r="E62" s="4" t="inlineStr">
+        <is>
+          <t>Tables présentes (créées le 05/10 sur les deux projets).</t>
+        </is>
+      </c>
+      <c r="F62" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G62" s="6" t="inlineStr">
+        <is>
+          <t>À tester</t>
+        </is>
+      </c>
+      <c r="H62" s="6" t="n"/>
+      <c r="I62" s="6" t="n"/>
+    </row>
+    <row r="63">
+      <c r="A63" s="4" t="n">
+        <v>59</v>
+      </c>
+      <c r="B63" s="5" t="inlineStr">
+        <is>
           <t>Règle de travail de décembre</t>
         </is>
       </c>
-      <c r="C60" s="4" t="inlineStr">
+      <c r="C63" s="4" t="inlineStr">
         <is>
           <t>CLAUDE.md</t>
         </is>
       </c>
-      <c r="D60" s="4" t="inlineStr">
+      <c r="D63" s="4" t="inlineStr">
         <is>
           <t>Après la mise en prod : retirer le paragraphe « Jusqu'à décembre 2026 ».</t>
         </is>
       </c>
-      <c r="E60" s="4" t="inlineStr">
+      <c r="E63" s="4" t="inlineStr">
         <is>
           <t>STA redevient identique à la PROD.</t>
         </is>
       </c>
-      <c r="F60" s="4" t="inlineStr">
+      <c r="F63" s="4" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G60" s="6" t="inlineStr">
-        <is>
-          <t>À tester</t>
-        </is>
-      </c>
-      <c r="H60" s="6" t="n"/>
-      <c r="I60" s="6" t="n"/>
+      <c r="G63" s="6" t="inlineStr">
+        <is>
+          <t>À tester</t>
+        </is>
+      </c>
+      <c r="H63" s="6" t="n"/>
+      <c r="I63" s="6" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A2:I2"/>
   </mergeCells>
-  <conditionalFormatting sqref="G5:G60">
+  <conditionalFormatting sqref="G5:G63">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"OK"</formula>
     </cfRule>
@@ -2765,7 +2888,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="G5:G60" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="G5:G63" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"À tester,OK,KO,Non testable"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Pilotage : comptes de test exclus, offre annuelle à 19,99 € comptée au vrai prix, jours à l'heure de Paris, carte et emails corrigés (STA)
Les 5 écarts relevés le 08/10 : comptes de test exclus comme les admins (adresses « + » des emails admin, ou
{"compteTest": true} dans Clerk) des inscrits, actifs, rétention, sources et de la carte ; abonnés annuels au montant de
la dernière facture payée (offre saisonnière) dans le MRR, l'ARR et « Produits et charges » ; inscriptions, actifs et
visiteurs du jour à l'heure de Paris ; emails de démarrage et de relance séparés des conseils par email. Les actifs par
jour viennent des jours d'utilisation (la vue dau_by_day ne sert plus). Recette de décembre n° 57 à 62.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AUzY5Y8Bt2KRzzte5cJgH8
</commit_message>
<xml_diff>
--- a/docs/recette/Recette_prod_decembre_2026.xlsx
+++ b/docs/recette/Recette_prod_decembre_2026.xlsx
@@ -505,7 +505,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I63"/>
+  <dimension ref="A1:I69"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -2770,27 +2770,27 @@
       </c>
       <c r="B61" s="5" t="inlineStr">
         <is>
-          <t>Alignement PROD / STA</t>
+          <t>Pilotage — comptes de test exclus</t>
         </is>
       </c>
       <c r="C61" s="4" t="inlineStr">
         <is>
-          <t>Git</t>
+          <t>Pilotage → Activité</t>
         </is>
       </c>
       <c r="D61" s="4" t="inlineStr">
         <is>
-          <t>Après la fusion : git diff --quiet origin/main origin/Staging.</t>
+          <t>Créer un compte avec une adresse jordankrebs1+essai@gmail.com (ou marquer un compte {"compteTest": true} dans Clerk : Users → le compte → Metadata → Public), l'utiliser un jour, puis ouvrir Pilotage.</t>
         </is>
       </c>
       <c r="E61" s="4" t="inlineStr">
         <is>
-          <t>Aucune différence.</t>
+          <t>Le compte n'est compté ni dans les inscrits, ni dans les actifs, la rétention, les sources ou la carte ; une adresse « + » d'un vrai utilisateur (autre que l'admin) reste comptée.</t>
         </is>
       </c>
       <c r="F61" s="4" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Admin</t>
         </is>
       </c>
       <c r="G61" s="6" t="inlineStr">
@@ -2798,7 +2798,11 @@
           <t>À tester</t>
         </is>
       </c>
-      <c r="H61" s="6" t="n"/>
+      <c r="H61" s="6" t="inlineStr">
+        <is>
+          <t>Sur STA le 18/10/2026 (écarts relevés le 08/10).</t>
+        </is>
+      </c>
       <c r="I61" s="6" t="n"/>
     </row>
     <row r="62">
@@ -2807,27 +2811,27 @@
       </c>
       <c r="B62" s="5" t="inlineStr">
         <is>
-          <t>Base de données PROD</t>
+          <t>Pilotage — offre annuelle à 19,99 €</t>
         </is>
       </c>
       <c r="C62" s="4" t="inlineStr">
         <is>
-          <t>Supabase PROD</t>
+          <t>Pilotage → Finances (MRR, ARR, Produits et charges)</t>
         </is>
       </c>
       <c r="D62" s="4" t="inlineStr">
         <is>
-          <t>Vérifier les tables codes et parrainages.</t>
+          <t>Avec un abonné annuel pris pendant l'offre saisonnière (à partir du 1/12) : ouvrir Finances.</t>
         </is>
       </c>
       <c r="E62" s="4" t="inlineStr">
         <is>
-          <t>Tables présentes (créées le 05/10 sur les deux projets).</t>
+          <t>L'abonné compte pour 19,99 €/an la 1re année (MRR, ARR et Produits et charges) ; ligne « Abonnements annuels » : « dont 1 à 19,99 € la 1re année ». Les autres annuels restent à 39,99 €.</t>
         </is>
       </c>
       <c r="F62" s="4" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Admin</t>
         </is>
       </c>
       <c r="G62" s="6" t="inlineStr">
@@ -2835,7 +2839,11 @@
           <t>À tester</t>
         </is>
       </c>
-      <c r="H62" s="6" t="n"/>
+      <c r="H62" s="6" t="inlineStr">
+        <is>
+          <t>Sur STA le 18/10/2026. Testable au premier abonné de l'offre.</t>
+        </is>
+      </c>
       <c r="I62" s="6" t="n"/>
     </row>
     <row r="63">
@@ -2844,42 +2852,280 @@
       </c>
       <c r="B63" s="5" t="inlineStr">
         <is>
+          <t>Pilotage — jours à l'heure de Paris</t>
+        </is>
+      </c>
+      <c r="C63" s="4" t="inlineStr">
+        <is>
+          <t>Pilotage → Activité</t>
+        </is>
+      </c>
+      <c r="D63" s="4" t="inlineStr">
+        <is>
+          <t>Après une inscription ou une visite entre minuit et 2 h (heure de Paris) : regarder « Nouveaux aujourd'hui », le graphique sur 30 jours, les mois et « Visiteurs site (auj.) ».</t>
+        </is>
+      </c>
+      <c r="E63" s="4" t="inlineStr">
+        <is>
+          <t>L'inscription et la visite comptent pour le jour même, pas pour la veille.</t>
+        </is>
+      </c>
+      <c r="F63" s="4" t="inlineStr">
+        <is>
+          <t>Admin</t>
+        </is>
+      </c>
+      <c r="G63" s="6" t="inlineStr">
+        <is>
+          <t>Non testable</t>
+        </is>
+      </c>
+      <c r="H63" s="6" t="inlineStr">
+        <is>
+          <t>Sur STA le 18/10/2026 ; vérifié par un test automatique, à constater au premier cas réel.</t>
+        </is>
+      </c>
+      <c r="I63" s="6" t="n"/>
+    </row>
+    <row r="64">
+      <c r="A64" s="4" t="n">
+        <v>60</v>
+      </c>
+      <c r="B64" s="5" t="inlineStr">
+        <is>
+          <t>Pilotage — carte des inscrits</t>
+        </is>
+      </c>
+      <c r="C64" s="4" t="inlineStr">
+        <is>
+          <t>Pilotage → Activité (carte)</t>
+        </is>
+      </c>
+      <c r="D64" s="4" t="inlineStr">
+        <is>
+          <t>Ouvrir la carte des inscrits.</t>
+        </is>
+      </c>
+      <c r="E64" s="4" t="inlineStr">
+        <is>
+          <t>La ville de l'admin et celles des comptes de test ne sont plus comptées (sauf vrai inscrit dans la même ville).</t>
+        </is>
+      </c>
+      <c r="F64" s="4" t="inlineStr">
+        <is>
+          <t>Admin</t>
+        </is>
+      </c>
+      <c r="G64" s="6" t="inlineStr">
+        <is>
+          <t>À tester</t>
+        </is>
+      </c>
+      <c r="H64" s="6" t="inlineStr">
+        <is>
+          <t>Sur STA le 18/10/2026.</t>
+        </is>
+      </c>
+      <c r="I64" s="6" t="n"/>
+    </row>
+    <row r="65">
+      <c r="A65" s="4" t="n">
+        <v>61</v>
+      </c>
+      <c r="B65" s="5" t="inlineStr">
+        <is>
+          <t>Pilotage — emails envoyés</t>
+        </is>
+      </c>
+      <c r="C65" s="4" t="inlineStr">
+        <is>
+          <t>Pilotage → Activité (notifications)</t>
+        </is>
+      </c>
+      <c r="D65" s="4" t="inlineStr">
+        <is>
+          <t>Lire la ligne sous « Notifications ».</t>
+        </is>
+      </c>
+      <c r="E65" s="4" t="inlineStr">
+        <is>
+          <t>« N notifications · N ouvertes · N conseils par email · N emails de démarrage et relances » : les emails de démarrage et de relance ne sont plus comptés comme conseils.</t>
+        </is>
+      </c>
+      <c r="F65" s="4" t="inlineStr">
+        <is>
+          <t>Admin</t>
+        </is>
+      </c>
+      <c r="G65" s="6" t="inlineStr">
+        <is>
+          <t>À tester</t>
+        </is>
+      </c>
+      <c r="H65" s="6" t="inlineStr">
+        <is>
+          <t>Sur STA le 18/10/2026.</t>
+        </is>
+      </c>
+      <c r="I65" s="6" t="n"/>
+    </row>
+    <row r="66">
+      <c r="A66" s="4" t="n">
+        <v>62</v>
+      </c>
+      <c r="B66" s="5" t="inlineStr">
+        <is>
+          <t>Base de données — vue dau_by_day</t>
+        </is>
+      </c>
+      <c r="C66" s="4" t="inlineStr">
+        <is>
+          <t>Supabase STA et PROD</t>
+        </is>
+      </c>
+      <c r="D66" s="4" t="inlineStr">
+        <is>
+          <t>Après la mise en prod : vérifier que plus rien n'utilise la vue dau_by_day (les actifs viennent de daily_active_users), puis la supprimer sur les deux projets.</t>
+        </is>
+      </c>
+      <c r="E66" s="4" t="inlineStr">
+        <is>
+          <t>Vue supprimée ; Pilotage → Activité affiche toujours les actifs par jour.</t>
+        </is>
+      </c>
+      <c r="F66" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G66" s="6" t="inlineStr">
+        <is>
+          <t>À tester</t>
+        </is>
+      </c>
+      <c r="H66" s="6" t="inlineStr">
+        <is>
+          <t>Les actifs par jour sont calculés depuis le 18/10/2026 (STA) à partir des jours d'utilisation, pour exclure les comptes de test.</t>
+        </is>
+      </c>
+      <c r="I66" s="6" t="n"/>
+    </row>
+    <row r="67">
+      <c r="A67" s="4" t="n">
+        <v>63</v>
+      </c>
+      <c r="B67" s="5" t="inlineStr">
+        <is>
+          <t>Alignement PROD / STA</t>
+        </is>
+      </c>
+      <c r="C67" s="4" t="inlineStr">
+        <is>
+          <t>Git</t>
+        </is>
+      </c>
+      <c r="D67" s="4" t="inlineStr">
+        <is>
+          <t>Après la fusion : git diff --quiet origin/main origin/Staging.</t>
+        </is>
+      </c>
+      <c r="E67" s="4" t="inlineStr">
+        <is>
+          <t>Aucune différence.</t>
+        </is>
+      </c>
+      <c r="F67" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G67" s="6" t="inlineStr">
+        <is>
+          <t>À tester</t>
+        </is>
+      </c>
+      <c r="H67" s="6" t="n"/>
+      <c r="I67" s="6" t="n"/>
+    </row>
+    <row r="68">
+      <c r="A68" s="4" t="n">
+        <v>64</v>
+      </c>
+      <c r="B68" s="5" t="inlineStr">
+        <is>
+          <t>Base de données PROD</t>
+        </is>
+      </c>
+      <c r="C68" s="4" t="inlineStr">
+        <is>
+          <t>Supabase PROD</t>
+        </is>
+      </c>
+      <c r="D68" s="4" t="inlineStr">
+        <is>
+          <t>Vérifier les tables codes et parrainages.</t>
+        </is>
+      </c>
+      <c r="E68" s="4" t="inlineStr">
+        <is>
+          <t>Tables présentes (créées le 05/10 sur les deux projets).</t>
+        </is>
+      </c>
+      <c r="F68" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G68" s="6" t="inlineStr">
+        <is>
+          <t>À tester</t>
+        </is>
+      </c>
+      <c r="H68" s="6" t="n"/>
+      <c r="I68" s="6" t="n"/>
+    </row>
+    <row r="69">
+      <c r="A69" s="4" t="n">
+        <v>65</v>
+      </c>
+      <c r="B69" s="5" t="inlineStr">
+        <is>
           <t>Règle de travail de décembre</t>
         </is>
       </c>
-      <c r="C63" s="4" t="inlineStr">
+      <c r="C69" s="4" t="inlineStr">
         <is>
           <t>CLAUDE.md</t>
         </is>
       </c>
-      <c r="D63" s="4" t="inlineStr">
+      <c r="D69" s="4" t="inlineStr">
         <is>
           <t>Après la mise en prod : retirer le paragraphe « Jusqu'à décembre 2026 ».</t>
         </is>
       </c>
-      <c r="E63" s="4" t="inlineStr">
+      <c r="E69" s="4" t="inlineStr">
         <is>
           <t>STA redevient identique à la PROD.</t>
         </is>
       </c>
-      <c r="F63" s="4" t="inlineStr">
+      <c r="F69" s="4" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G63" s="6" t="inlineStr">
-        <is>
-          <t>À tester</t>
-        </is>
-      </c>
-      <c r="H63" s="6" t="n"/>
-      <c r="I63" s="6" t="n"/>
+      <c r="G69" s="6" t="inlineStr">
+        <is>
+          <t>À tester</t>
+        </is>
+      </c>
+      <c r="H69" s="6" t="n"/>
+      <c r="I69" s="6" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A2:I2"/>
   </mergeCells>
-  <conditionalFormatting sqref="G5:G63">
+  <conditionalFormatting sqref="G5:G69">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"OK"</formula>
     </cfRule>
@@ -2888,7 +3134,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="G5:G63" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="G5:G69" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"À tester,OK,KO,Non testable"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Notifications : proposées après la première aide (diagnostic, parcours) plutôt qu'à l'inscription (STA)
Plan trafic ×10, action 9 en version allégée : plus de demande d'autorisation du téléphone à l'inscription (la case
« conseils de Bob » active les rappels, les conseils partent par email). Carte « Activer les notifications » sous le
résultat du diagnostic et dans un parcours lancé ou en attente de la fenêtre de semis, masquée si déjà actives,
refusées ou impossibles, et 14 jours après « Plus tard » ; même activation que la tuile de l'accueil
(useActiverNotifications). Bob ; recette de décembre n° 63 à 65.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AUzY5Y8Bt2KRzzte5cJgH8
</commit_message>
<xml_diff>
--- a/docs/recette/Recette_prod_decembre_2026.xlsx
+++ b/docs/recette/Recette_prod_decembre_2026.xlsx
@@ -505,7 +505,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I69"/>
+  <dimension ref="A1:I72"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -3016,27 +3016,27 @@
       </c>
       <c r="B67" s="5" t="inlineStr">
         <is>
-          <t>Alignement PROD / STA</t>
+          <t>Notifications — plus de demande à l'inscription</t>
         </is>
       </c>
       <c r="C67" s="4" t="inlineStr">
         <is>
-          <t>Git</t>
+          <t>Inscription (consentements)</t>
         </is>
       </c>
       <c r="D67" s="4" t="inlineStr">
         <is>
-          <t>Après la fusion : git diff --quiet origin/main origin/Staging.</t>
+          <t>Créer un compte en laissant « Recevoir les conseils de Bob » coché, puis valider.</t>
         </is>
       </c>
       <c r="E67" s="4" t="inlineStr">
         <is>
-          <t>Aucune différence.</t>
+          <t>Le téléphone ne demande pas l'autorisation des notifications à l'inscription ; texte de la case : « par email ou par notification (Bob te proposera de les activer après ta première aide) » ; les conseils partent par email en attendant.</t>
         </is>
       </c>
       <c r="F67" s="4" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Nouveau compte</t>
         </is>
       </c>
       <c r="G67" s="6" t="inlineStr">
@@ -3044,7 +3044,11 @@
           <t>À tester</t>
         </is>
       </c>
-      <c r="H67" s="6" t="n"/>
+      <c r="H67" s="6" t="inlineStr">
+        <is>
+          <t>Sur STA le 18/10/2026 (plan trafic ×10, action 9 en version allégée).</t>
+        </is>
+      </c>
       <c r="I67" s="6" t="n"/>
     </row>
     <row r="68">
@@ -3053,27 +3057,27 @@
       </c>
       <c r="B68" s="5" t="inlineStr">
         <is>
-          <t>Base de données PROD</t>
+          <t>Notifications — proposées après la première aide</t>
         </is>
       </c>
       <c r="C68" s="4" t="inlineStr">
         <is>
-          <t>Supabase PROD</t>
+          <t>Diagnostic (résultat) ; parcours lancé ou en attente de la fenêtre</t>
         </is>
       </c>
       <c r="D68" s="4" t="inlineStr">
         <is>
-          <t>Vérifier les tables codes et parrainages.</t>
+          <t>Nouveau compte sans notifications : faire un diagnostic, puis ouvrir un parcours ; toucher « Activer les notifications » et accepter l'autorisation du téléphone.</t>
         </is>
       </c>
       <c r="E68" s="4" t="inlineStr">
         <is>
-          <t>Tables présentes (créées le 05/10 sur les deux projets).</t>
+          <t>Carte « 🔔 Bob te prévient au bon moment » sous le résultat (et « Ne rate aucun arrosage » / « Sois prévenu dès que la fenêtre s'ouvre » dans le parcours) ; après activation : notification de test reçue, carte disparue, tuile de l'accueil disparue.</t>
         </is>
       </c>
       <c r="F68" s="4" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Nouveau compte</t>
         </is>
       </c>
       <c r="G68" s="6" t="inlineStr">
@@ -3081,7 +3085,11 @@
           <t>À tester</t>
         </is>
       </c>
-      <c r="H68" s="6" t="n"/>
+      <c r="H68" s="6" t="inlineStr">
+        <is>
+          <t>Sur STA le 18/10/2026.</t>
+        </is>
+      </c>
       <c r="I68" s="6" t="n"/>
     </row>
     <row r="69">
@@ -3090,42 +3098,157 @@
       </c>
       <c r="B69" s="5" t="inlineStr">
         <is>
+          <t>Notifications — « Plus tard »</t>
+        </is>
+      </c>
+      <c r="C69" s="4" t="inlineStr">
+        <is>
+          <t>Diagnostic (résultat)</t>
+        </is>
+      </c>
+      <c r="D69" s="4" t="inlineStr">
+        <is>
+          <t>Toucher « Plus tard » sur la carte, puis refaire un diagnostic le même jour.</t>
+        </is>
+      </c>
+      <c r="E69" s="4" t="inlineStr">
+        <is>
+          <t>La carte ne revient pas pendant 14 jours ; la tuile « Activez les alertes » de l'accueil reste disponible.</t>
+        </is>
+      </c>
+      <c r="F69" s="4" t="inlineStr">
+        <is>
+          <t>Nouveau compte</t>
+        </is>
+      </c>
+      <c r="G69" s="6" t="inlineStr">
+        <is>
+          <t>À tester</t>
+        </is>
+      </c>
+      <c r="H69" s="6" t="inlineStr">
+        <is>
+          <t>Sur STA le 18/10/2026.</t>
+        </is>
+      </c>
+      <c r="I69" s="6" t="n"/>
+    </row>
+    <row r="70">
+      <c r="A70" s="4" t="n">
+        <v>66</v>
+      </c>
+      <c r="B70" s="5" t="inlineStr">
+        <is>
+          <t>Alignement PROD / STA</t>
+        </is>
+      </c>
+      <c r="C70" s="4" t="inlineStr">
+        <is>
+          <t>Git</t>
+        </is>
+      </c>
+      <c r="D70" s="4" t="inlineStr">
+        <is>
+          <t>Après la fusion : git diff --quiet origin/main origin/Staging.</t>
+        </is>
+      </c>
+      <c r="E70" s="4" t="inlineStr">
+        <is>
+          <t>Aucune différence.</t>
+        </is>
+      </c>
+      <c r="F70" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G70" s="6" t="inlineStr">
+        <is>
+          <t>À tester</t>
+        </is>
+      </c>
+      <c r="H70" s="6" t="n"/>
+      <c r="I70" s="6" t="n"/>
+    </row>
+    <row r="71">
+      <c r="A71" s="4" t="n">
+        <v>67</v>
+      </c>
+      <c r="B71" s="5" t="inlineStr">
+        <is>
+          <t>Base de données PROD</t>
+        </is>
+      </c>
+      <c r="C71" s="4" t="inlineStr">
+        <is>
+          <t>Supabase PROD</t>
+        </is>
+      </c>
+      <c r="D71" s="4" t="inlineStr">
+        <is>
+          <t>Vérifier les tables codes et parrainages.</t>
+        </is>
+      </c>
+      <c r="E71" s="4" t="inlineStr">
+        <is>
+          <t>Tables présentes (créées le 05/10 sur les deux projets).</t>
+        </is>
+      </c>
+      <c r="F71" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G71" s="6" t="inlineStr">
+        <is>
+          <t>À tester</t>
+        </is>
+      </c>
+      <c r="H71" s="6" t="n"/>
+      <c r="I71" s="6" t="n"/>
+    </row>
+    <row r="72">
+      <c r="A72" s="4" t="n">
+        <v>68</v>
+      </c>
+      <c r="B72" s="5" t="inlineStr">
+        <is>
           <t>Règle de travail de décembre</t>
         </is>
       </c>
-      <c r="C69" s="4" t="inlineStr">
+      <c r="C72" s="4" t="inlineStr">
         <is>
           <t>CLAUDE.md</t>
         </is>
       </c>
-      <c r="D69" s="4" t="inlineStr">
+      <c r="D72" s="4" t="inlineStr">
         <is>
           <t>Après la mise en prod : retirer le paragraphe « Jusqu'à décembre 2026 ».</t>
         </is>
       </c>
-      <c r="E69" s="4" t="inlineStr">
+      <c r="E72" s="4" t="inlineStr">
         <is>
           <t>STA redevient identique à la PROD.</t>
         </is>
       </c>
-      <c r="F69" s="4" t="inlineStr">
+      <c r="F72" s="4" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G69" s="6" t="inlineStr">
-        <is>
-          <t>À tester</t>
-        </is>
-      </c>
-      <c r="H69" s="6" t="n"/>
-      <c r="I69" s="6" t="n"/>
+      <c r="G72" s="6" t="inlineStr">
+        <is>
+          <t>À tester</t>
+        </is>
+      </c>
+      <c r="H72" s="6" t="n"/>
+      <c r="I72" s="6" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A2:I2"/>
   </mergeCells>
-  <conditionalFormatting sqref="G5:G69">
+  <conditionalFormatting sqref="G5:G72">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"OK"</formula>
     </cfRule>
@@ -3134,7 +3257,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="G5:G69" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="G5:G72" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"À tester,OK,KO,Non testable"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Équipements : choix de la marque avant les explications, erreur du fabricant signalée au retour de connexion (STA)
- Mes équipements : chaque carte (station, robot, arrosage) demande d'abord la marque, puis
  n'affiche que les explications, les champs et le bouton de la marque choisie ; au retour
  d'une connexion chez le fabricant, sa marque est déjà choisie (remarque de Jordan : le texte
  Ecowitt sous le bouton Netatmo prêtait à confusion).
- Retour OAuth sans code : refus de l'utilisateur (access_denied) → « Connexion annulée » ;
  toute autre erreur du fabricant → « La connexion … a échoué » et alerte avec sa raison
  (Pilotage → Bugs), pour diagnostiquer la connexion Netatmo.
- Recette de décembre n° 66 et 67, journal.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AUzY5Y8Bt2KRzzte5cJgH8
</commit_message>
<xml_diff>
--- a/docs/recette/Recette_prod_decembre_2026.xlsx
+++ b/docs/recette/Recette_prod_decembre_2026.xlsx
@@ -505,7 +505,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I72"/>
+  <dimension ref="A1:I74"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -533,7 +533,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -3140,27 +3139,27 @@
       </c>
       <c r="B70" s="5" t="inlineStr">
         <is>
-          <t>Alignement PROD / STA</t>
+          <t>Équipements — choix de la marque</t>
         </is>
       </c>
       <c r="C70" s="4" t="inlineStr">
         <is>
-          <t>Git</t>
+          <t>Mes équipements (station, robot, arrosage)</t>
         </is>
       </c>
       <c r="D70" s="4" t="inlineStr">
         <is>
-          <t>Après la fusion : git diff --quiet origin/main origin/Staging.</t>
+          <t>Ouvrir Mes équipements sans rien de connecté ; dans chaque carte, toucher une marque, puis une autre.</t>
         </is>
       </c>
       <c r="E70" s="4" t="inlineStr">
         <is>
-          <t>Aucune différence.</t>
+          <t>Chaque carte demande d'abord la marque (station : Netatmo, Ecowitt, Davis, Autre marque ; robot : Husqvarna Automower, Gardena SILENO, Mammotion ; arrosage : Gardena, Rachio) ; seules les explications, les champs et le bouton de la marque choisie s'affichent ; au retour d'une connexion chez le fabricant, sa marque est déjà choisie.</t>
         </is>
       </c>
       <c r="F70" s="4" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Premium</t>
         </is>
       </c>
       <c r="G70" s="6" t="inlineStr">
@@ -3168,7 +3167,11 @@
           <t>À tester</t>
         </is>
       </c>
-      <c r="H70" s="6" t="n"/>
+      <c r="H70" s="6" t="inlineStr">
+        <is>
+          <t>Sur STA le 19/10/2026 (remarque de Jordan : le texte Ecowitt sous le bouton Netatmo prêtait à confusion).</t>
+        </is>
+      </c>
       <c r="I70" s="6" t="n"/>
     </row>
     <row r="71">
@@ -3177,27 +3180,27 @@
       </c>
       <c r="B71" s="5" t="inlineStr">
         <is>
-          <t>Base de données PROD</t>
+          <t>Équipements — erreur renvoyée par le fabricant</t>
         </is>
       </c>
       <c r="C71" s="4" t="inlineStr">
         <is>
-          <t>Supabase PROD</t>
+          <t>Mes équipements ; Pilotage → Bugs</t>
         </is>
       </c>
       <c r="D71" s="4" t="inlineStr">
         <is>
-          <t>Vérifier les tables codes et parrainages.</t>
+          <t>Connexion Netatmo, Husqvarna ou Gardena : refuser l'accès sur le site du fabricant ; puis, si possible, provoquer une erreur du fabricant.</t>
         </is>
       </c>
       <c r="E71" s="4" t="inlineStr">
         <is>
-          <t>Tables présentes (créées le 05/10 sur les deux projets).</t>
+          <t>Refus : « Connexion annulée : rien n'a été enregistré », sans alerte ; autre erreur du fabricant : « La connexion … a échoué » et une alerte « Connexion … refusée par le fabricant » avec la raison donnée par le fabricant.</t>
         </is>
       </c>
       <c r="F71" s="4" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Admin</t>
         </is>
       </c>
       <c r="G71" s="6" t="inlineStr">
@@ -3205,7 +3208,11 @@
           <t>À tester</t>
         </is>
       </c>
-      <c r="H71" s="6" t="n"/>
+      <c r="H71" s="6" t="inlineStr">
+        <is>
+          <t>Sur STA le 19/10/2026.</t>
+        </is>
+      </c>
       <c r="I71" s="6" t="n"/>
     </row>
     <row r="72">
@@ -3214,22 +3221,22 @@
       </c>
       <c r="B72" s="5" t="inlineStr">
         <is>
-          <t>Règle de travail de décembre</t>
+          <t>Alignement PROD / STA</t>
         </is>
       </c>
       <c r="C72" s="4" t="inlineStr">
         <is>
-          <t>CLAUDE.md</t>
+          <t>Git</t>
         </is>
       </c>
       <c r="D72" s="4" t="inlineStr">
         <is>
-          <t>Après la mise en prod : retirer le paragraphe « Jusqu'à décembre 2026 ».</t>
+          <t>Après la fusion : git diff --quiet origin/main origin/Staging.</t>
         </is>
       </c>
       <c r="E72" s="4" t="inlineStr">
         <is>
-          <t>STA redevient identique à la PROD.</t>
+          <t>Aucune différence.</t>
         </is>
       </c>
       <c r="F72" s="4" t="inlineStr">
@@ -3244,12 +3251,86 @@
       </c>
       <c r="H72" s="6" t="n"/>
       <c r="I72" s="6" t="n"/>
+    </row>
+    <row r="73">
+      <c r="A73" s="4" t="n">
+        <v>69</v>
+      </c>
+      <c r="B73" s="5" t="inlineStr">
+        <is>
+          <t>Base de données PROD</t>
+        </is>
+      </c>
+      <c r="C73" s="4" t="inlineStr">
+        <is>
+          <t>Supabase PROD</t>
+        </is>
+      </c>
+      <c r="D73" s="4" t="inlineStr">
+        <is>
+          <t>Vérifier les tables codes et parrainages.</t>
+        </is>
+      </c>
+      <c r="E73" s="4" t="inlineStr">
+        <is>
+          <t>Tables présentes (créées le 05/10 sur les deux projets).</t>
+        </is>
+      </c>
+      <c r="F73" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G73" s="6" t="inlineStr">
+        <is>
+          <t>À tester</t>
+        </is>
+      </c>
+      <c r="H73" s="6" t="n"/>
+      <c r="I73" s="6" t="n"/>
+    </row>
+    <row r="74">
+      <c r="A74" s="4" t="n">
+        <v>70</v>
+      </c>
+      <c r="B74" s="5" t="inlineStr">
+        <is>
+          <t>Règle de travail de décembre</t>
+        </is>
+      </c>
+      <c r="C74" s="4" t="inlineStr">
+        <is>
+          <t>CLAUDE.md</t>
+        </is>
+      </c>
+      <c r="D74" s="4" t="inlineStr">
+        <is>
+          <t>Après la mise en prod : retirer le paragraphe « Jusqu'à décembre 2026 ».</t>
+        </is>
+      </c>
+      <c r="E74" s="4" t="inlineStr">
+        <is>
+          <t>STA redevient identique à la PROD.</t>
+        </is>
+      </c>
+      <c r="F74" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G74" s="6" t="inlineStr">
+        <is>
+          <t>À tester</t>
+        </is>
+      </c>
+      <c r="H74" s="6" t="n"/>
+      <c r="I74" s="6" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A2:I2"/>
   </mergeCells>
-  <conditionalFormatting sqref="G5:G72">
+  <conditionalFormatting sqref="G5:G74">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"OK"</formula>
     </cfRule>
@@ -3258,7 +3339,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="G5:G72" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="G5:G74" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"À tester,OK,KO,Non testable"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Équipements : liste déroulante des marques, puis seulement les éléments à renseigner (STA)
Demande de Jordan : une liste déroulante de marques par carte (station, robot, arrosage) au lieu
de boutons ; « Autre marque » renvoie au formulaire « Ton équipement n'est pas dans la liste ? ».
Recette n° 66 et journal mis à jour.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AUzY5Y8Bt2KRzzte5cJgH8
</commit_message>
<xml_diff>
--- a/docs/recette/Recette_prod_decembre_2026.xlsx
+++ b/docs/recette/Recette_prod_decembre_2026.xlsx
@@ -533,6 +533,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -3149,12 +3150,12 @@
       </c>
       <c r="D70" s="4" t="inlineStr">
         <is>
-          <t>Ouvrir Mes équipements sans rien de connecté ; dans chaque carte, toucher une marque, puis une autre.</t>
+          <t>Ouvrir Mes équipements sans rien de connecté ; dans chaque carte, choisir une marque dans la liste déroulante, puis une autre, puis « Choisis la marque… ».</t>
         </is>
       </c>
       <c r="E70" s="4" t="inlineStr">
         <is>
-          <t>Chaque carte demande d'abord la marque (station : Netatmo, Ecowitt, Davis, Autre marque ; robot : Husqvarna Automower, Gardena SILENO, Mammotion ; arrosage : Gardena, Rachio) ; seules les explications, les champs et le bouton de la marque choisie s'affichent ; au retour d'une connexion chez le fabricant, sa marque est déjà choisie.</t>
+          <t>Une liste déroulante par carte (station : Netatmo, Ecowitt, Davis, Autre marque ; robot : Husqvarna Automower, Gardena SILENO, Mammotion, Autre marque ; arrosage : Gardena, Rachio, Autre marque) ; seuls les éléments à renseigner et le bouton de la marque choisie s'affichent ; « Autre marque » renvoie au formulaire « Ton équipement n'est pas dans la liste ? » ; au retour d'une connexion chez le fabricant, sa marque est déjà choisie.</t>
         </is>
       </c>
       <c r="F70" s="4" t="inlineStr">
@@ -3169,7 +3170,7 @@
       </c>
       <c r="H70" s="6" t="inlineStr">
         <is>
-          <t>Sur STA le 19/10/2026 (remarque de Jordan : le texte Ecowitt sous le bouton Netatmo prêtait à confusion).</t>
+          <t>Sur STA le 19/10/2026 (demande de Jordan : une liste déroulante de marques, puis seulement les éléments à renseigner).</t>
         </is>
       </c>
       <c r="I70" s="6" t="n"/>

</xml_diff>

<commit_message>
Suivi : connexion Netatmo validée sur STA sans station, recette n° 31, 35 et 67 (journal)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AUzY5Y8Bt2KRzzte5cJgH8
</commit_message>
<xml_diff>
--- a/docs/recette/Recette_prod_decembre_2026.xlsx
+++ b/docs/recette/Recette_prod_decembre_2026.xlsx
@@ -1769,7 +1769,11 @@
           <t>À tester</t>
         </is>
       </c>
-      <c r="H35" s="6" t="n"/>
+      <c r="H35" s="6" t="inlineStr">
+        <is>
+          <t>Chaîne de connexion validée sur STA le 19/10/2026 par Jordan, sans station (« Aucune station météo trouvée sur ce compte Netatmo ») ; reste le test avec une vraie station.</t>
+        </is>
+      </c>
       <c r="I35" s="6" t="n"/>
     </row>
     <row r="36">
@@ -1917,7 +1921,11 @@
           <t>À tester</t>
         </is>
       </c>
-      <c r="H39" s="6" t="n"/>
+      <c r="H39" s="6" t="inlineStr">
+        <is>
+          <t>Sur STA, l'adresse déclarée chez Netatmo est celle du lien Staging (…vercel.app/api/objets, 19/10/2026) : la remplacer à la mise en prod, Netatmo n'accepte qu'une adresse ; description de l'application en français (19/10/2026).</t>
+        </is>
+      </c>
       <c r="I39" s="6" t="n"/>
     </row>
     <row r="40">
@@ -3211,7 +3219,7 @@
       </c>
       <c r="H71" s="6" t="inlineStr">
         <is>
-          <t>Sur STA le 19/10/2026.</t>
+          <t>Sur STA le 19/10/2026. Vérifié sur STA le 19/10/2026 : erreur « redirect_uri_mismatch » de Netatmo remontée dans Pilotage → Bugs avec sa raison et l'adresse de retour.</t>
         </is>
       </c>
       <c r="I71" s="6" t="n"/>

</xml_diff>

<commit_message>
Suivi : tâche planifiée CRON_SECRET vérifiée en prod (matin et soir), recette « Déjà en prod » n° 27 OK (journal)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AUzY5Y8Bt2KRzzte5cJgH8
</commit_message>
<xml_diff>
--- a/docs/recette/Recette_prod_decembre_2026.xlsx
+++ b/docs/recette/Recette_prod_decembre_2026.xlsx
@@ -533,7 +533,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -3390,6 +3389,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -4544,12 +4544,12 @@
       </c>
       <c r="G31" s="6" t="inlineStr">
         <is>
-          <t>À tester</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="H31" s="6" t="inlineStr">
         <is>
-          <t>En prod le 18/10/2026 (go prod de Jordan) ; clé remplacée par Jordan en prod et sur STA (l'ancienne figurait dans l'historique public du dépôt). Appels sans clé ou avec une mauvaise clé refusés : vérifié le 18/10/2026.</t>
+          <t>En prod le 18/10/2026 (go prod de Jordan) ; clé remplacée par Jordan en prod et sur STA (l'ancienne figurait dans l'historique public du dépôt). Appels sans clé ou avec une mauvaise clé refusés : vérifié le 18/10/2026. Vérifié le 19/10/2026 : tâche du matin (10 conseils vers 8 h 17) et tâche du soir (5 conseils vers 17 h 30, heure de Paris) passées avec la nouvelle clé ; aucune « Tâche planifiée refusée » ni erreur serveur ; publications pg_cron toutes en 200.</t>
         </is>
       </c>
       <c r="I31" s="8" t="n"/>

</xml_diff>

<commit_message>
Équipements : connexion Weather Underground retirée (usage commercial payant) (STA)
Décision de Jordan du 19/10 : les conditions de The Weather Company (section 18) réservent la clé
gratuite des stations à un usage non commercial, l'usage commercial est payant. Connexion retirée
du serveur (api/equipements.cjs, api/objets.js), de Mes équipements (« Autre marque » renvoie au
formulaire « Ton équipement n'est pas dans la liste ? »), des consignes de Bob, de la politique de
confidentialité (6.3, mise à jour du 19 octobre) et de CLAUDE.md. Aucune donnée en base. Recette
n° 43 et 48, journal.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AUzY5Y8Bt2KRzzte5cJgH8
</commit_message>
<xml_diff>
--- a/docs/recette/Recette_prod_decembre_2026.xlsx
+++ b/docs/recette/Recette_prod_decembre_2026.xlsx
@@ -533,6 +533,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -2219,7 +2220,7 @@
       </c>
       <c r="E47" s="4" t="inlineStr">
         <is>
-          <t>Davis et Mammotion cités dans l'article 6.3 (date du 17 octobre) ; Bob cite Netatmo, Ecowitt, Davis, Husqvarna, Gardena, Mammotion et Rachio, sans autre marque.</t>
+          <t>Netatmo, Ecowitt, Davis et Mammotion cités dans l'article 6.3, sans Weather Underground (date du 19 octobre) ; Bob cite Netatmo, Ecowitt, Davis, Husqvarna, Gardena, Mammotion et Rachio, sans autre marque.</t>
         </is>
       </c>
       <c r="F47" s="4" t="inlineStr">
@@ -2234,7 +2235,7 @@
       </c>
       <c r="H47" s="6" t="inlineStr">
         <is>
-          <t>Sur STA le 17/10/2026.</t>
+          <t>Sur STA le 17/10/2026 ; Weather Underground retiré le 19/10/2026.</t>
         </is>
       </c>
       <c r="I47" s="6" t="n"/>
@@ -2409,27 +2410,27 @@
       </c>
       <c r="B52" s="5" t="inlineStr">
         <is>
-          <t>Station Weather Underground — connexion et mesures</t>
+          <t>Station Weather Underground — retirée</t>
         </is>
       </c>
       <c r="C52" s="4" t="inlineStr">
         <is>
-          <t>Mes équipements → Station météo ; Aujourd'hui ; Bob</t>
+          <t>Mes équipements → Station météo</t>
         </is>
       </c>
       <c r="D52" s="4" t="inlineStr">
         <is>
-          <t>Avec une station qui publie sur Weather Underground (Froggit, Bresser, Ambient Weather…) : créer une clé sur wunderground.com (API Keys), saisir l'identifiant de la station et la clé, connecter ; puis ouvrir « Aujourd'hui ».</t>
+          <t>Ouvrir la liste des marques de station, puis choisir « Autre marque ».</t>
         </is>
       </c>
       <c r="E52" s="4" t="inlineStr">
         <is>
-          <t>Station « ✓ connectée » avec son nom (quartier déclaré) ; température en °C, pluie du jour en mm, vent en km/h ; pluie mesurée prise en compte pour l'arrosage ; identifiant faux : message clair.</t>
+          <t>Liste : Netatmo, Ecowitt, Davis, Autre marque, sans Weather Underground ; « Autre marque » renvoie au formulaire « Ton équipement n'est pas dans la liste ? ».</t>
         </is>
       </c>
       <c r="F52" s="4" t="inlineStr">
         <is>
-          <t>Compte avec station publiant sur Weather Underground</t>
+          <t>Premium</t>
         </is>
       </c>
       <c r="G52" s="6" t="inlineStr">
@@ -2439,7 +2440,7 @@
       </c>
       <c r="H52" s="6" t="inlineStr">
         <is>
-          <t>Sur STA le 18/10/2026.</t>
+          <t>Connexion Weather Underground développée sur STA le 18/10/2026 puis retirée le 19/10/2026 (décision de Jordan) : les conditions de The Weather Company (section 18) réservent la clé gratuite à un usage non commercial, l'usage commercial est payant.</t>
         </is>
       </c>
       <c r="I52" s="6" t="n"/>
@@ -3389,7 +3390,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Recette : article Semer au printemps et renvois (une question = un article) dans les évolutions déjà en prod
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AUzY5Y8Bt2KRzzte5cJgH8
</commit_message>
<xml_diff>
--- a/docs/recette/Recette_prod_decembre_2026.xlsx
+++ b/docs/recette/Recette_prod_decembre_2026.xlsx
@@ -3361,7 +3361,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I32"/>
+  <dimension ref="A1:I33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -4596,6 +4596,49 @@
         <v>46313</v>
       </c>
     </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>29</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="inlineStr">
+        <is>
+          <t>Articles Conseils : une question = un article pour le semis (« Semer au printemps » devient la méthode, renvois avec « Quand semer » et « Préparer sa pelouse au printemps »)</t>
+        </is>
+      </c>
+      <c r="C33" s="4" t="inlineStr">
+        <is>
+          <t>Site (/conseils/semer-gazon-printemps, /conseils/quand-semer-gazon, /conseils/preparer-pelouse-printemps)</t>
+        </is>
+      </c>
+      <c r="D33" s="4" t="inlineStr">
+        <is>
+          <t>Ouvrir les 3 articles sur téléphone ; dans la Search Console, inspecter les 3 adresses et demander une indexation.</t>
+        </is>
+      </c>
+      <c r="E33" s="4" t="inlineStr">
+        <is>
+          <t>« Semer du gazon au printemps : la méthode pas à pas », sans tableau des dates (lien vers « Quand semer »), « Mis à jour le 22 octobre 2026 » ; dans « Quand semer », intertitre « Après le semis : les grandes étapes » et question « mai ou juin » ; à l'étape 6 de « Préparer sa pelouse au printemps », renvoi vers la méthode du semis.</t>
+        </is>
+      </c>
+      <c r="F33" s="4" t="inlineStr">
+        <is>
+          <t>Visiteur</t>
+        </is>
+      </c>
+      <c r="G33" s="6" t="inlineStr">
+        <is>
+          <t>À tester</t>
+        </is>
+      </c>
+      <c r="H33" s="6" t="inlineStr">
+        <is>
+          <t>En prod le 22/10/2026 (exception articles Conseils, go de Jordan) ; pages vérifiées en ligne le 22/10 : titre, intertitre, renvois et plan du site à jour.</t>
+        </is>
+      </c>
+      <c r="I33" s="8" t="n"/>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A2:I2"/>
@@ -4609,7 +4652,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="G5:G32" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="G5:G33" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"À tester,OK,KO,Non testable"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Journal et recette : suivi du nouvel inscrit et correctifs du 23/10 (consentements à l'inscription, clics des emails)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AUzY5Y8Bt2KRzzte5cJgH8
</commit_message>
<xml_diff>
--- a/docs/recette/Recette_prod_decembre_2026.xlsx
+++ b/docs/recette/Recette_prod_decembre_2026.xlsx
@@ -3361,7 +3361,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I33"/>
+  <dimension ref="A1:I35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -4639,6 +4639,92 @@
       </c>
       <c r="I33" s="8" t="n"/>
     </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="inlineStr">
+        <is>
+          <t>Inscription : choix « conseils de Bob » conservé (correctif urgent)</t>
+        </is>
+      </c>
+      <c r="C34" s="4" t="inlineStr">
+        <is>
+          <t>Écran d'inscription (/register) ; Pilotage → Activité</t>
+        </is>
+      </c>
+      <c r="D34" s="4" t="inlineStr">
+        <is>
+          <t>Créer un compte de test sur mongazon360.fr, laisser « Recevoir les conseils de Bob » cochée, refuser l'autorisation des notifications si le navigateur la demande ; puis regarder ses consentements (Paramètres → Mes données).</t>
+        </is>
+      </c>
+      <c r="E34" s="4" t="inlineStr">
+        <is>
+          <t>« Conseils de Bob » activés, rappels activés ; avec la case décochée : conseils désactivés. Le compte de test est ensuite marqué compte de test ou supprimé.</t>
+        </is>
+      </c>
+      <c r="F34" s="4" t="inlineStr">
+        <is>
+          <t>Nouveau compte de test</t>
+        </is>
+      </c>
+      <c r="G34" s="6" t="inlineStr">
+        <is>
+          <t>À tester</t>
+        </is>
+      </c>
+      <c r="H34" s="6" t="inlineStr">
+        <is>
+          <t>En prod le 23/10/2026 (go de Jordan). Bug reproduit en test avant correction (choix enregistré « non » quand l'enregistrement est plus lent que la lecture), corrigé et vérifié en test.</t>
+        </is>
+      </c>
+      <c r="I34" s="8" t="n"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>31</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="inlineStr">
+        <is>
+          <t>Emails : clics mesurés (bienvenue, démarrage, relances, conseils)</t>
+        </is>
+      </c>
+      <c r="C35" s="4" t="inlineStr">
+        <is>
+          <t>Emails reçus ; reminders.notif_log (PROD)</t>
+        </is>
+      </c>
+      <c r="D35" s="4" t="inlineStr">
+        <is>
+          <t>Ouvrir un email de démarrage ou de bienvenue reçu après le 23/10 et toucher son bouton ; vérifier que l'adresse ouverte n'affiche plus le paramètre m.</t>
+        </is>
+      </c>
+      <c r="E35" s="4" t="inlineStr">
+        <is>
+          <t>L'app s'ouvre sur la bonne page ; l'envoi est marqué « clic » dans reminders.notif_log ; l'email de bienvenue y est tracé.</t>
+        </is>
+      </c>
+      <c r="F35" s="4" t="inlineStr">
+        <is>
+          <t>Nouveau compte de test</t>
+        </is>
+      </c>
+      <c r="G35" s="6" t="inlineStr">
+        <is>
+          <t>À tester</t>
+        </is>
+      </c>
+      <c r="H35" s="6" t="inlineStr">
+        <is>
+          <t>En prod le 23/10/2026 (go de Jordan) ; testé de bout en bout en test (liens, jeton, enregistrement du clic, jeton falsifié refusé).</t>
+        </is>
+      </c>
+      <c r="I35" s="8" t="n"/>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A2:I2"/>
@@ -4652,7 +4738,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="G5:G33" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="G5:G35" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"À tester,OK,KO,Non testable"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Journal et recette : correctif de l'engrais d'hiver et du chaulage (go prod de Jordan du 24/10)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AUzY5Y8Bt2KRzzte5cJgH8
</commit_message>
<xml_diff>
--- a/docs/recette/Recette_prod_decembre_2026.xlsx
+++ b/docs/recette/Recette_prod_decembre_2026.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Recette décembre" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Déjà en prod (exceptions)" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Recette décembre" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Déjà en prod (exceptions)" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -3361,7 +3361,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I35"/>
+  <dimension ref="A1:I36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -4725,6 +4725,49 @@
       </c>
       <c r="I35" s="8" t="n"/>
     </row>
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>32</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="inlineStr">
+        <is>
+          <t>Engrais d'hiver riche en potassium et chaulage aux doses de la base (correctif urgent)</t>
+        </is>
+      </c>
+      <c r="C36" s="4" t="inlineStr">
+        <is>
+          <t>Aujourd'hui et Ma pelouse (carte « Engrais Hiver »), Plan annuel (novembre), onglet Produits, articles « Chauler sa pelouse » et « Mousse dans la pelouse »</t>
+        </is>
+      </c>
+      <c r="D36" s="4" t="inlineStr">
+        <is>
+          <t>À partir du 1er novembre, avec un compte de test : ouvrir Aujourd'hui (quand l'engrais d'hiver est proposé), le Plan annuel au mois de novembre et l'onglet Produits ; ouvrir les articles « Chauler sa pelouse » et « Mousse dans la pelouse : que faire ? ».</t>
+        </is>
+      </c>
+      <c r="E36" s="4" t="inlineStr">
+        <is>
+          <t>Carte « Engrais Hiver » : « Riche en potassium (résistance au gel), pauvre en azote » (organique en objectif Naturel), sans produit de chaux. Plan annuel de novembre : « Engrais d'hiver » et « Chaulage si sol acide » aux doses de la base (40-60 g/m² entre pH 5 et 6, 80-100 g/m² sous 5), pas de chaulage en sol calcaire. Kit de saison sans chaux. Produits et articles : « Chaulage (sol acide) », 2 sacs pour 300 m².</t>
+        </is>
+      </c>
+      <c r="F36" s="4" t="inlineStr">
+        <is>
+          <t>Compte de test</t>
+        </is>
+      </c>
+      <c r="G36" s="6" t="inlineStr">
+        <is>
+          <t>À tester</t>
+        </is>
+      </c>
+      <c r="H36" s="6" t="inlineStr">
+        <is>
+          <t>En prod le 24/10/2026 (go de Jordan). Vérifié avant la mise en prod : build, Plan annuel de novembre (4 profils), carte, kit et quantités. Aucun engrais d'hiver dans le catalogue : produit à choisir.</t>
+        </is>
+      </c>
+      <c r="I36" s="8" t="n"/>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A2:I2"/>
@@ -4738,7 +4781,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="G5:G35" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="G5:G36" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"À tester,OK,KO,Non testable"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Recette de décembre : plantage d'écran (traduction, extension) et alerte unique par plantage (n° 68 et 69)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AUzY5Y8Bt2KRzzte5cJgH8
</commit_message>
<xml_diff>
--- a/docs/recette/Recette_prod_decembre_2026.xlsx
+++ b/docs/recette/Recette_prod_decembre_2026.xlsx
@@ -505,7 +505,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I74"/>
+  <dimension ref="A1:I76"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -3224,101 +3224,115 @@
       <c r="I71" s="6" t="n"/>
     </row>
     <row r="72">
-      <c r="A72" s="4" t="n">
-        <v>68</v>
+      <c r="A72" s="4" t="inlineStr">
+        <is>
+          <t>68</t>
+        </is>
       </c>
       <c r="B72" s="5" t="inlineStr">
         <is>
+          <t>Plantage d'écran — traduction automatique ou extension du navigateur</t>
+        </is>
+      </c>
+      <c r="C72" s="4" t="inlineStr">
+        <is>
+          <t>Démo (/demo), puis le reste de l'app, sur Chrome (ordinateur)</t>
+        </is>
+      </c>
+      <c r="D72" s="4" t="inlineStr">
+        <is>
+          <t>Ouvrir /demo, clic droit → « Traduire en anglais », puis changer d'onglet plusieurs fois et toucher « S'inscrire » ; refaire sur Aujourd'hui avec un compte connecté.</t>
+        </is>
+      </c>
+      <c r="E72" s="4" t="inlineStr">
+        <is>
+          <t>Aucun écran « Erreur de chargement » ; la page reste utilisable, même si une partie du texte reste traduite.</t>
+        </is>
+      </c>
+      <c r="F72" s="4" t="inlineStr">
+        <is>
+          <t>Visiteur et compte connecté</t>
+        </is>
+      </c>
+      <c r="G72" s="6" t="inlineStr">
+        <is>
+          <t>À tester</t>
+        </is>
+      </c>
+      <c r="H72" s="6" t="inlineStr">
+        <is>
+          <t>Sur STA le 26/10/2026 (alerte du 26/10 sur /demo : « removeChild »). Plantage reproduit sur un banc (traduction simulée), plus de plantage avec le correctif.</t>
+        </is>
+      </c>
+      <c r="I72" s="6" t="n"/>
+    </row>
+    <row r="73">
+      <c r="A73" s="4" t="inlineStr">
+        <is>
+          <t>69</t>
+        </is>
+      </c>
+      <c r="B73" s="5" t="inlineStr">
+        <is>
+          <t>Alertes — un seul email par plantage</t>
+        </is>
+      </c>
+      <c r="C73" s="4" t="inlineStr">
+        <is>
+          <t>Emails d'alerte ; Pilotage → Bugs</t>
+        </is>
+      </c>
+      <c r="D73" s="4" t="inlineStr">
+        <is>
+          <t>À la prochaine alerte « Plantage d'écran » : compter les emails reçus et les lignes du même plantage dans Pilotage → Bugs.</t>
+        </is>
+      </c>
+      <c r="E73" s="4" t="inlineStr">
+        <is>
+          <t>Un seul email et une seule ligne pour un même plantage (le 26/10 : 3 emails pour 1 plantage).</t>
+        </is>
+      </c>
+      <c r="F73" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G73" s="6" t="inlineStr">
+        <is>
+          <t>À tester</t>
+        </is>
+      </c>
+      <c r="H73" s="6" t="inlineStr">
+        <is>
+          <t>Sur STA le 26/10/2026. Test : 3 signalements du même plantage → 1 envoi (3 avant le correctif).</t>
+        </is>
+      </c>
+      <c r="I73" s="6" t="n"/>
+    </row>
+    <row r="74">
+      <c r="A74" s="4" t="inlineStr">
+        <is>
+          <t>70</t>
+        </is>
+      </c>
+      <c r="B74" s="5" t="inlineStr">
+        <is>
           <t>Alignement PROD / STA</t>
         </is>
       </c>
-      <c r="C72" s="4" t="inlineStr">
+      <c r="C74" s="4" t="inlineStr">
         <is>
           <t>Git</t>
         </is>
       </c>
-      <c r="D72" s="4" t="inlineStr">
+      <c r="D74" s="4" t="inlineStr">
         <is>
           <t>Après la fusion : git diff --quiet origin/main origin/Staging.</t>
         </is>
       </c>
-      <c r="E72" s="4" t="inlineStr">
+      <c r="E74" s="4" t="inlineStr">
         <is>
           <t>Aucune différence.</t>
-        </is>
-      </c>
-      <c r="F72" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G72" s="6" t="inlineStr">
-        <is>
-          <t>À tester</t>
-        </is>
-      </c>
-      <c r="H72" s="6" t="n"/>
-      <c r="I72" s="6" t="n"/>
-    </row>
-    <row r="73">
-      <c r="A73" s="4" t="n">
-        <v>69</v>
-      </c>
-      <c r="B73" s="5" t="inlineStr">
-        <is>
-          <t>Base de données PROD</t>
-        </is>
-      </c>
-      <c r="C73" s="4" t="inlineStr">
-        <is>
-          <t>Supabase PROD</t>
-        </is>
-      </c>
-      <c r="D73" s="4" t="inlineStr">
-        <is>
-          <t>Vérifier les tables codes et parrainages.</t>
-        </is>
-      </c>
-      <c r="E73" s="4" t="inlineStr">
-        <is>
-          <t>Tables présentes (créées le 05/10 sur les deux projets).</t>
-        </is>
-      </c>
-      <c r="F73" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G73" s="6" t="inlineStr">
-        <is>
-          <t>À tester</t>
-        </is>
-      </c>
-      <c r="H73" s="6" t="n"/>
-      <c r="I73" s="6" t="n"/>
-    </row>
-    <row r="74">
-      <c r="A74" s="4" t="n">
-        <v>70</v>
-      </c>
-      <c r="B74" s="5" t="inlineStr">
-        <is>
-          <t>Règle de travail de décembre</t>
-        </is>
-      </c>
-      <c r="C74" s="4" t="inlineStr">
-        <is>
-          <t>CLAUDE.md</t>
-        </is>
-      </c>
-      <c r="D74" s="4" t="inlineStr">
-        <is>
-          <t>Après la mise en prod : retirer le paragraphe « Jusqu'à décembre 2026 ».</t>
-        </is>
-      </c>
-      <c r="E74" s="4" t="inlineStr">
-        <is>
-          <t>STA redevient identique à la PROD.</t>
         </is>
       </c>
       <c r="F74" s="4" t="inlineStr">
@@ -3333,6 +3347,84 @@
       </c>
       <c r="H74" s="6" t="n"/>
       <c r="I74" s="6" t="n"/>
+    </row>
+    <row r="75">
+      <c r="A75" s="4" t="inlineStr">
+        <is>
+          <t>71</t>
+        </is>
+      </c>
+      <c r="B75" s="5" t="inlineStr">
+        <is>
+          <t>Base de données PROD</t>
+        </is>
+      </c>
+      <c r="C75" s="4" t="inlineStr">
+        <is>
+          <t>Supabase PROD</t>
+        </is>
+      </c>
+      <c r="D75" s="4" t="inlineStr">
+        <is>
+          <t>Vérifier les tables codes et parrainages.</t>
+        </is>
+      </c>
+      <c r="E75" s="4" t="inlineStr">
+        <is>
+          <t>Tables présentes (créées le 05/10 sur les deux projets).</t>
+        </is>
+      </c>
+      <c r="F75" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G75" s="6" t="inlineStr">
+        <is>
+          <t>À tester</t>
+        </is>
+      </c>
+      <c r="H75" s="6" t="n"/>
+      <c r="I75" s="6" t="n"/>
+    </row>
+    <row r="76">
+      <c r="A76" s="4" t="inlineStr">
+        <is>
+          <t>72</t>
+        </is>
+      </c>
+      <c r="B76" s="5" t="inlineStr">
+        <is>
+          <t>Règle de travail de décembre</t>
+        </is>
+      </c>
+      <c r="C76" s="4" t="inlineStr">
+        <is>
+          <t>CLAUDE.md</t>
+        </is>
+      </c>
+      <c r="D76" s="4" t="inlineStr">
+        <is>
+          <t>Après la mise en prod : retirer le paragraphe « Jusqu'à décembre 2026 ».</t>
+        </is>
+      </c>
+      <c r="E76" s="4" t="inlineStr">
+        <is>
+          <t>STA redevient identique à la PROD.</t>
+        </is>
+      </c>
+      <c r="F76" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G76" s="6" t="inlineStr">
+        <is>
+          <t>À tester</t>
+        </is>
+      </c>
+      <c r="H76" s="6" t="n"/>
+      <c r="I76" s="6" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -3347,7 +3439,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="G5:G74" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="G5:G76" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"À tester,OK,KO,Non testable"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Journal et recette : correctif du plantage d'écran en prod (go de Jordan du 26/10), n° 33 et 34
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AUzY5Y8Bt2KRzzte5cJgH8
</commit_message>
<xml_diff>
--- a/docs/recette/Recette_prod_decembre_2026.xlsx
+++ b/docs/recette/Recette_prod_decembre_2026.xlsx
@@ -505,7 +505,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I76"/>
+  <dimension ref="A1:I74"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -3231,27 +3231,27 @@
       </c>
       <c r="B72" s="5" t="inlineStr">
         <is>
-          <t>Plantage d'écran — traduction automatique ou extension du navigateur</t>
+          <t>Alignement PROD / STA</t>
         </is>
       </c>
       <c r="C72" s="4" t="inlineStr">
         <is>
-          <t>Démo (/demo), puis le reste de l'app, sur Chrome (ordinateur)</t>
+          <t>Git</t>
         </is>
       </c>
       <c r="D72" s="4" t="inlineStr">
         <is>
-          <t>Ouvrir /demo, clic droit → « Traduire en anglais », puis changer d'onglet plusieurs fois et toucher « S'inscrire » ; refaire sur Aujourd'hui avec un compte connecté.</t>
+          <t>Après la fusion : git diff --quiet origin/main origin/Staging.</t>
         </is>
       </c>
       <c r="E72" s="4" t="inlineStr">
         <is>
-          <t>Aucun écran « Erreur de chargement » ; la page reste utilisable, même si une partie du texte reste traduite.</t>
+          <t>Aucune différence.</t>
         </is>
       </c>
       <c r="F72" s="4" t="inlineStr">
         <is>
-          <t>Visiteur et compte connecté</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G72" s="6" t="inlineStr">
@@ -3259,11 +3259,7 @@
           <t>À tester</t>
         </is>
       </c>
-      <c r="H72" s="6" t="inlineStr">
-        <is>
-          <t>Sur STA le 26/10/2026 (alerte du 26/10 sur /demo : « removeChild »). Plantage reproduit sur un banc (traduction simulée), plus de plantage avec le correctif.</t>
-        </is>
-      </c>
+      <c r="H72" s="6" t="n"/>
       <c r="I72" s="6" t="n"/>
     </row>
     <row r="73">
@@ -3274,22 +3270,22 @@
       </c>
       <c r="B73" s="5" t="inlineStr">
         <is>
-          <t>Alertes — un seul email par plantage</t>
+          <t>Base de données PROD</t>
         </is>
       </c>
       <c r="C73" s="4" t="inlineStr">
         <is>
-          <t>Emails d'alerte ; Pilotage → Bugs</t>
+          <t>Supabase PROD</t>
         </is>
       </c>
       <c r="D73" s="4" t="inlineStr">
         <is>
-          <t>À la prochaine alerte « Plantage d'écran » : compter les emails reçus et les lignes du même plantage dans Pilotage → Bugs.</t>
+          <t>Vérifier les tables codes et parrainages.</t>
         </is>
       </c>
       <c r="E73" s="4" t="inlineStr">
         <is>
-          <t>Un seul email et une seule ligne pour un même plantage (le 26/10 : 3 emails pour 1 plantage).</t>
+          <t>Tables présentes (créées le 05/10 sur les deux projets).</t>
         </is>
       </c>
       <c r="F73" s="4" t="inlineStr">
@@ -3302,11 +3298,7 @@
           <t>À tester</t>
         </is>
       </c>
-      <c r="H73" s="6" t="inlineStr">
-        <is>
-          <t>Sur STA le 26/10/2026. Test : 3 signalements du même plantage → 1 envoi (3 avant le correctif).</t>
-        </is>
-      </c>
+      <c r="H73" s="6" t="n"/>
       <c r="I73" s="6" t="n"/>
     </row>
     <row r="74">
@@ -3317,22 +3309,22 @@
       </c>
       <c r="B74" s="5" t="inlineStr">
         <is>
-          <t>Alignement PROD / STA</t>
+          <t>Règle de travail de décembre</t>
         </is>
       </c>
       <c r="C74" s="4" t="inlineStr">
         <is>
-          <t>Git</t>
+          <t>CLAUDE.md</t>
         </is>
       </c>
       <c r="D74" s="4" t="inlineStr">
         <is>
-          <t>Après la fusion : git diff --quiet origin/main origin/Staging.</t>
+          <t>Après la mise en prod : retirer le paragraphe « Jusqu'à décembre 2026 ».</t>
         </is>
       </c>
       <c r="E74" s="4" t="inlineStr">
         <is>
-          <t>Aucune différence.</t>
+          <t>STA redevient identique à la PROD.</t>
         </is>
       </c>
       <c r="F74" s="4" t="inlineStr">
@@ -3347,84 +3339,6 @@
       </c>
       <c r="H74" s="6" t="n"/>
       <c r="I74" s="6" t="n"/>
-    </row>
-    <row r="75">
-      <c r="A75" s="4" t="inlineStr">
-        <is>
-          <t>71</t>
-        </is>
-      </c>
-      <c r="B75" s="5" t="inlineStr">
-        <is>
-          <t>Base de données PROD</t>
-        </is>
-      </c>
-      <c r="C75" s="4" t="inlineStr">
-        <is>
-          <t>Supabase PROD</t>
-        </is>
-      </c>
-      <c r="D75" s="4" t="inlineStr">
-        <is>
-          <t>Vérifier les tables codes et parrainages.</t>
-        </is>
-      </c>
-      <c r="E75" s="4" t="inlineStr">
-        <is>
-          <t>Tables présentes (créées le 05/10 sur les deux projets).</t>
-        </is>
-      </c>
-      <c r="F75" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G75" s="6" t="inlineStr">
-        <is>
-          <t>À tester</t>
-        </is>
-      </c>
-      <c r="H75" s="6" t="n"/>
-      <c r="I75" s="6" t="n"/>
-    </row>
-    <row r="76">
-      <c r="A76" s="4" t="inlineStr">
-        <is>
-          <t>72</t>
-        </is>
-      </c>
-      <c r="B76" s="5" t="inlineStr">
-        <is>
-          <t>Règle de travail de décembre</t>
-        </is>
-      </c>
-      <c r="C76" s="4" t="inlineStr">
-        <is>
-          <t>CLAUDE.md</t>
-        </is>
-      </c>
-      <c r="D76" s="4" t="inlineStr">
-        <is>
-          <t>Après la mise en prod : retirer le paragraphe « Jusqu'à décembre 2026 ».</t>
-        </is>
-      </c>
-      <c r="E76" s="4" t="inlineStr">
-        <is>
-          <t>STA redevient identique à la PROD.</t>
-        </is>
-      </c>
-      <c r="F76" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G76" s="6" t="inlineStr">
-        <is>
-          <t>À tester</t>
-        </is>
-      </c>
-      <c r="H76" s="6" t="n"/>
-      <c r="I76" s="6" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -3439,7 +3353,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="G5:G76" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="G5:G74" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"À tester,OK,KO,Non testable"</formula1>
     </dataValidation>
   </dataValidations>
@@ -3453,7 +3367,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I36"/>
+  <dimension ref="A1:I38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -4860,6 +4774,92 @@
       </c>
       <c r="I36" s="8" t="n"/>
     </row>
+    <row r="37">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>33</t>
+        </is>
+      </c>
+      <c r="B37" s="5" t="inlineStr">
+        <is>
+          <t>Plantage d'écran — traduction automatique ou extension du navigateur</t>
+        </is>
+      </c>
+      <c r="C37" s="4" t="inlineStr">
+        <is>
+          <t>Démo (/demo), puis le reste de l'app, sur Chrome (ordinateur)</t>
+        </is>
+      </c>
+      <c r="D37" s="4" t="inlineStr">
+        <is>
+          <t>Ouvrir /demo, clic droit → « Traduire en anglais », puis changer d'onglet plusieurs fois et toucher « S'inscrire » ; refaire sur Aujourd'hui avec un compte connecté.</t>
+        </is>
+      </c>
+      <c r="E37" s="4" t="inlineStr">
+        <is>
+          <t>Aucun écran « Erreur de chargement » ; la page reste utilisable, même si une partie du texte reste traduite.</t>
+        </is>
+      </c>
+      <c r="F37" s="4" t="inlineStr">
+        <is>
+          <t>Visiteur et compte connecté</t>
+        </is>
+      </c>
+      <c r="G37" s="6" t="inlineStr">
+        <is>
+          <t>À tester</t>
+        </is>
+      </c>
+      <c r="H37" s="6" t="inlineStr">
+        <is>
+          <t>En prod le 26/10/2026 (go de Jordan, correctif urgent) (alerte du 26/10 sur /demo : « removeChild »). Plantage reproduit sur un banc (traduction simulée), plus de plantage avec le correctif.</t>
+        </is>
+      </c>
+      <c r="I37" s="8" t="n"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>34</t>
+        </is>
+      </c>
+      <c r="B38" s="5" t="inlineStr">
+        <is>
+          <t>Alertes — un seul email par plantage</t>
+        </is>
+      </c>
+      <c r="C38" s="4" t="inlineStr">
+        <is>
+          <t>Emails d'alerte ; Pilotage → Bugs</t>
+        </is>
+      </c>
+      <c r="D38" s="4" t="inlineStr">
+        <is>
+          <t>À la prochaine alerte « Plantage d'écran » : compter les emails reçus et les lignes du même plantage dans Pilotage → Bugs.</t>
+        </is>
+      </c>
+      <c r="E38" s="4" t="inlineStr">
+        <is>
+          <t>Un seul email et une seule ligne pour un même plantage (le 26/10 : 3 emails pour 1 plantage).</t>
+        </is>
+      </c>
+      <c r="F38" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G38" s="6" t="inlineStr">
+        <is>
+          <t>À tester</t>
+        </is>
+      </c>
+      <c r="H38" s="6" t="inlineStr">
+        <is>
+          <t>En prod le 26/10/2026 (go de Jordan, correctif urgent). Test : 3 signalements du même plantage → 1 envoi (3 avant le correctif).</t>
+        </is>
+      </c>
+      <c r="I38" s="8" t="n"/>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A2:I2"/>
@@ -4873,7 +4873,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="G5:G36" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="G5:G38" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"À tester,OK,KO,Non testable"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Journal et recette : ligue d'hiver en prod (go de Jordan du 26/10), n° 35 à 42
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AUzY5Y8Bt2KRzzte5cJgH8
</commit_message>
<xml_diff>
--- a/docs/recette/Recette_prod_decembre_2026.xlsx
+++ b/docs/recette/Recette_prod_decembre_2026.xlsx
@@ -3367,7 +3367,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I38"/>
+  <dimension ref="A1:I46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -4860,6 +4860,350 @@
       </c>
       <c r="I38" s="8" t="n"/>
     </row>
+    <row r="39">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>35</t>
+        </is>
+      </c>
+      <c r="B39" s="5" t="inlineStr">
+        <is>
+          <t>Ligue d'hiver — annonce du départ</t>
+        </is>
+      </c>
+      <c r="C39" s="4" t="inlineStr">
+        <is>
+          <t>Accueil (visiteur), Aujourd'hui, Classement</t>
+        </is>
+      </c>
+      <c r="D39" s="4" t="inlineStr">
+        <is>
+          <t>Du 26 au 31/10 : ouvrir l'accueil sans compte, puis Aujourd'hui et Classement avec un compte.</t>
+        </is>
+      </c>
+      <c r="E39" s="4" t="inlineStr">
+        <is>
+          <t>Bandeau « Ligue d'hiver : 1 an de Premium à gagner » sur l'accueil ; carte d'annonce « démarre le dimanche 1er novembre » dans Aujourd'hui et Classement.</t>
+        </is>
+      </c>
+      <c r="F39" s="4" t="inlineStr">
+        <is>
+          <t>Visiteur et compte connecté</t>
+        </is>
+      </c>
+      <c r="G39" s="6" t="inlineStr">
+        <is>
+          <t>À tester</t>
+        </is>
+      </c>
+      <c r="H39" s="6" t="inlineStr">
+        <is>
+          <t>En prod le 26/10/2026 (go de Jordan, exception : la ligue part seule ; départ le 1/11). Bandeau de l'accueil vérifié en ligne le 26/10.</t>
+        </is>
+      </c>
+      <c r="I39" s="8" t="n"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>36</t>
+        </is>
+      </c>
+      <c r="B40" s="5" t="inlineStr">
+        <is>
+          <t>Ligue d'hiver — onglet « Quiz » et semaine 1</t>
+        </is>
+      </c>
+      <c r="C40" s="4" t="inlineStr">
+        <is>
+          <t>Barre du bas, onglet Quiz, Aujourd'hui</t>
+        </is>
+      </c>
+      <c r="D40" s="4" t="inlineStr">
+        <is>
+          <t>Le dimanche 1/11 : regarder la barre du bas, ouvrir l'onglet, puis la carte de la ligue dans Aujourd'hui.</t>
+        </is>
+      </c>
+      <c r="E40" s="4" t="inlineStr">
+        <is>
+          <t>L'onglet Classement s'appelle « Quiz » (🧠) ; semaine 1 sur 13 (dernière tonte) avec le défi et le quiz ; carte « Ligue d'hiver · semaine 1/13 » dans Aujourd'hui.</t>
+        </is>
+      </c>
+      <c r="F40" s="4" t="inlineStr">
+        <is>
+          <t>Compte de test</t>
+        </is>
+      </c>
+      <c r="G40" s="6" t="inlineStr">
+        <is>
+          <t>À tester</t>
+        </is>
+      </c>
+      <c r="H40" s="6" t="inlineStr">
+        <is>
+          <t>En prod le 26/10/2026 (go de Jordan, exception : la ligue part seule ; départ le 1/11).</t>
+        </is>
+      </c>
+      <c r="I40" s="8" t="n"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="4" t="inlineStr">
+        <is>
+          <t>37</t>
+        </is>
+      </c>
+      <c r="B41" s="5" t="inlineStr">
+        <is>
+          <t>Ligue d'hiver — défi de la semaine</t>
+        </is>
+      </c>
+      <c r="C41" s="4" t="inlineStr">
+        <is>
+          <t>Onglet Quiz</t>
+        </is>
+      </c>
+      <c r="D41" s="4" t="inlineStr">
+        <is>
+          <t>Toucher « C'est fait » sur le défi, puis recharger la page.</t>
+        </is>
+      </c>
+      <c r="E41" s="4" t="inlineStr">
+        <is>
+          <t>Défi « ✅ Fait », +50 GreenPoints une seule fois, 1 point d'assiduité.</t>
+        </is>
+      </c>
+      <c r="F41" s="4" t="inlineStr">
+        <is>
+          <t>Compte de test</t>
+        </is>
+      </c>
+      <c r="G41" s="6" t="inlineStr">
+        <is>
+          <t>À tester</t>
+        </is>
+      </c>
+      <c r="H41" s="6" t="inlineStr">
+        <is>
+          <t>En prod le 26/10/2026 (go de Jordan, exception : la ligue part seule ; départ le 1/11).</t>
+        </is>
+      </c>
+      <c r="I41" s="8" t="n"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="4" t="inlineStr">
+        <is>
+          <t>38</t>
+        </is>
+      </c>
+      <c r="B42" s="5" t="inlineStr">
+        <is>
+          <t>Ligue d'hiver — quiz chronométré</t>
+        </is>
+      </c>
+      <c r="C42" s="4" t="inlineStr">
+        <is>
+          <t>Onglet Quiz</t>
+        </is>
+      </c>
+      <c r="D42" s="4" t="inlineStr">
+        <is>
+          <t>Toucher « Commencer le quiz », répondre à 2 questions, recharger la page pendant le chrono, puis laisser la minute finir.</t>
+        </is>
+      </c>
+      <c r="E42" s="4" t="inlineStr">
+        <is>
+          <t>Le temps continue après le rechargement ; envoi automatique à la fin ; correction avec « ta réponse », « bonne réponse », « pas de réponse » ; +30 GreenPoints ; le quiz ne peut plus être recommencé.</t>
+        </is>
+      </c>
+      <c r="F42" s="4" t="inlineStr">
+        <is>
+          <t>Compte de test</t>
+        </is>
+      </c>
+      <c r="G42" s="6" t="inlineStr">
+        <is>
+          <t>À tester</t>
+        </is>
+      </c>
+      <c r="H42" s="6" t="inlineStr">
+        <is>
+          <t>En prod le 26/10/2026 (go de Jordan, exception : la ligue part seule ; départ le 1/11). Testé par Jordan sur STA le 26/10 (envoi à 60,5 s, 1/3 bien enregistré).</t>
+        </is>
+      </c>
+      <c r="I42" s="8" t="n"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="4" t="inlineStr">
+        <is>
+          <t>39</t>
+        </is>
+      </c>
+      <c r="B43" s="5" t="inlineStr">
+        <is>
+          <t>Ligue d'hiver — notifications</t>
+        </is>
+      </c>
+      <c r="C43" s="4" t="inlineStr">
+        <is>
+          <t>Notifications et emails du matin</t>
+        </is>
+      </c>
+      <c r="D43" s="4" t="inlineStr">
+        <is>
+          <t>Le dimanche 1/11 au matin, puis le mercredi 4/11 si le défi n'est pas fait.</t>
+        </is>
+      </c>
+      <c r="E43" s="4" t="inlineStr">
+        <is>
+          <t>Dimanche : « 🧠 Quiz du dimanche » (1re question, 3 questions en 1 minute) ; mercredi : « 🎯 Défi de la semaine » ; une fois par semaine chacun, une notification le matin au plus.</t>
+        </is>
+      </c>
+      <c r="F43" s="4" t="inlineStr">
+        <is>
+          <t>Compte de test</t>
+        </is>
+      </c>
+      <c r="G43" s="6" t="inlineStr">
+        <is>
+          <t>À tester</t>
+        </is>
+      </c>
+      <c r="H43" s="6" t="inlineStr">
+        <is>
+          <t>En prod le 26/10/2026 (go de Jordan, exception : la ligue part seule ; départ le 1/11).</t>
+        </is>
+      </c>
+      <c r="I43" s="8" t="n"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="4" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
+      </c>
+      <c r="B44" s="5" t="inlineStr">
+        <is>
+          <t>Ligue d'hiver — suivi dans Pilotage</t>
+        </is>
+      </c>
+      <c r="C44" s="4" t="inlineStr">
+        <is>
+          <t>Pilotage → Activité, carte « Ligue d'hiver »</t>
+        </is>
+      </c>
+      <c r="D44" s="4" t="inlineStr">
+        <is>
+          <t>Après les premières participations : ouvrir la carte.</t>
+        </is>
+      </c>
+      <c r="E44" s="4" t="inlineStr">
+        <is>
+          <t>Participation par semaine (défis, quiz, bonnes réponses moyennes) et plus assidus dans l'ordre du règlement, sans les comptes de test ni les admins.</t>
+        </is>
+      </c>
+      <c r="F44" s="4" t="inlineStr">
+        <is>
+          <t>Admin</t>
+        </is>
+      </c>
+      <c r="G44" s="6" t="inlineStr">
+        <is>
+          <t>À tester</t>
+        </is>
+      </c>
+      <c r="H44" s="6" t="inlineStr">
+        <is>
+          <t>En prod le 26/10/2026 (go de Jordan, exception : la ligue part seule ; départ le 1/11).</t>
+        </is>
+      </c>
+      <c r="I44" s="8" t="n"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="4" t="inlineStr">
+        <is>
+          <t>41</t>
+        </is>
+      </c>
+      <c r="B45" s="5" t="inlineStr">
+        <is>
+          <t>Ligue d'hiver — règlement et confidentialité</t>
+        </is>
+      </c>
+      <c r="C45" s="4" t="inlineStr">
+        <is>
+          <t>CGU (article 6 g), politique de confidentialité</t>
+        </is>
+      </c>
+      <c r="D45" s="4" t="inlineStr">
+        <is>
+          <t>Ouvrir les CGU puis la politique de confidentialité.</t>
+        </is>
+      </c>
+      <c r="E45" s="4" t="inlineStr">
+        <is>
+          <t>CGU à jour du 26 octobre 2026, article 6 g avec la règle du quiz (1 minute, une seule tentative) ; ligue d'hiver dans la politique de confidentialité (données et durée de conservation).</t>
+        </is>
+      </c>
+      <c r="F45" s="4" t="inlineStr">
+        <is>
+          <t>Visiteur</t>
+        </is>
+      </c>
+      <c r="G45" s="6" t="inlineStr">
+        <is>
+          <t>À tester</t>
+        </is>
+      </c>
+      <c r="H45" s="6" t="inlineStr">
+        <is>
+          <t>En prod le 26/10/2026 (go de Jordan, exception : la ligue part seule ; départ le 1/11).</t>
+        </is>
+      </c>
+      <c r="I45" s="8" t="n"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="4" t="inlineStr">
+        <is>
+          <t>42</t>
+        </is>
+      </c>
+      <c r="B46" s="5" t="inlineStr">
+        <is>
+          <t>Réseaux — quiz du dimanche 1/11</t>
+        </is>
+      </c>
+      <c r="C46" s="4" t="inlineStr">
+        <is>
+          <t>Pilotage → Réseaux ; page Facebook et Instagram</t>
+        </is>
+      </c>
+      <c r="D46" s="4" t="inlineStr">
+        <is>
+          <t>Valider le lot du 1er au 7/11 (quiz compris) avant le 1/11, puis regarder la page le 1/11 après 8 h.</t>
+        </is>
+      </c>
+      <c r="E46" s="4" t="inlineStr">
+        <is>
+          <t>« Quiz du dimanche » publié à 8 h sur Facebook et Instagram avec son visuel ; lien suivi « ligue-hiver » dans Pilotage → Activité.</t>
+        </is>
+      </c>
+      <c r="F46" s="4" t="inlineStr">
+        <is>
+          <t>Admin</t>
+        </is>
+      </c>
+      <c r="G46" s="6" t="inlineStr">
+        <is>
+          <t>À tester</t>
+        </is>
+      </c>
+      <c r="H46" s="6" t="inlineStr">
+        <is>
+          <t>En prod le 26/10/2026 (go de Jordan, exception : la ligue part seule ; départ le 1/11).</t>
+        </is>
+      </c>
+      <c r="I46" s="8" t="n"/>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A2:I2"/>
@@ -4873,7 +5217,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="G5:G38" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="G5:G46" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"À tester,OK,KO,Non testable"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Recette et journal : refonte sur STA (lignes 68 à 80, contrôles finaux en 81 à 83)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AUzY5Y8Bt2KRzzte5cJgH8
</commit_message>
<xml_diff>
--- a/docs/recette/Recette_prod_decembre_2026.xlsx
+++ b/docs/recette/Recette_prod_decembre_2026.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Recette décembre" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Déjà en prod (exceptions)" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Recette décembre" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Déjà en prod (exceptions)" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -505,7 +505,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I74"/>
+  <dimension ref="A1:I87"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -3231,27 +3231,27 @@
       </c>
       <c r="B72" s="5" t="inlineStr">
         <is>
-          <t>Alignement PROD / STA</t>
+          <t>Refonte — barre du bas</t>
         </is>
       </c>
       <c r="C72" s="4" t="inlineStr">
         <is>
-          <t>Git</t>
+          <t>Toute l'app (connecté)</t>
         </is>
       </c>
       <c r="D72" s="4" t="inlineStr">
         <is>
-          <t>Après la fusion : git diff --quiet origin/main origin/Staging.</t>
+          <t>Se connecter et regarder la barre du bas pendant la ligue d'hiver, puis après le 30/01.</t>
         </is>
       </c>
       <c r="E72" s="4" t="inlineStr">
         <is>
-          <t>Aucune différence.</t>
+          <t>4 onglets : Accueil, Aujourd'hui, Diagnostic, Mon gazon, plus « Quiz » jusqu'au 30/01 ; plus d'onglets Produits ni Classement (Produits reste ouvert depuis Mon gazon).</t>
         </is>
       </c>
       <c r="F72" s="4" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Gratuit et Premium</t>
         </is>
       </c>
       <c r="G72" s="6" t="inlineStr">
@@ -3259,7 +3259,11 @@
           <t>À tester</t>
         </is>
       </c>
-      <c r="H72" s="6" t="n"/>
+      <c r="H72" s="6" t="inlineStr">
+        <is>
+          <t>Sur STA le 26/10/2026 (décisions de Jordan du 26/10).</t>
+        </is>
+      </c>
       <c r="I72" s="6" t="n"/>
     </row>
     <row r="73">
@@ -3270,27 +3274,27 @@
       </c>
       <c r="B73" s="5" t="inlineStr">
         <is>
-          <t>Base de données PROD</t>
+          <t>Refonte — accueil : résumé du jour</t>
         </is>
       </c>
       <c r="C73" s="4" t="inlineStr">
         <is>
-          <t>Supabase PROD</t>
+          <t>Accueil</t>
         </is>
       </c>
       <c r="D73" s="4" t="inlineStr">
         <is>
-          <t>Vérifier les tables codes et parrainages.</t>
+          <t>Comparer la carte « Aujourd'hui » de l'accueil avec l'onglet Aujourd'hui, un jour avec des actions puis un jour sans ; toucher la carte.</t>
         </is>
       </c>
       <c r="E73" s="4" t="inlineStr">
         <is>
-          <t>Tables présentes (créées le 05/10 sur les deux projets).</t>
+          <t>Mêmes actions que l'onglet Aujourd'hui ; sans action : « Rien à faire aujourd'hui » et la prochaine action ; la carte ouvre Aujourd'hui.</t>
         </is>
       </c>
       <c r="F73" s="4" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Tous</t>
         </is>
       </c>
       <c r="G73" s="6" t="inlineStr">
@@ -3298,7 +3302,11 @@
           <t>À tester</t>
         </is>
       </c>
-      <c r="H73" s="6" t="n"/>
+      <c r="H73" s="6" t="inlineStr">
+        <is>
+          <t>Sur STA le 26/10/2026 (décisions de Jordan du 26/10).</t>
+        </is>
+      </c>
       <c r="I73" s="6" t="n"/>
     </row>
     <row r="74">
@@ -3309,42 +3317,593 @@
       </c>
       <c r="B74" s="5" t="inlineStr">
         <is>
+          <t>Refonte — série et GreenPoints</t>
+        </is>
+      </c>
+      <c r="C74" s="4" t="inlineStr">
+        <is>
+          <t>Accueil, Mon gazon</t>
+        </is>
+      </c>
+      <c r="D74" s="4" t="inlineStr">
+        <is>
+          <t>Ouvrir l'app un nouveau jour en restant sur l'accueil ; toucher la carte série et GreenPoints.</t>
+        </is>
+      </c>
+      <c r="E74" s="4" t="inlineStr">
+        <is>
+          <t>Série et GreenPoints de connexion comptés dès l'accueil, une fois par jour ; la carte ouvre Mon gazon directement sur « Mes progrès ».</t>
+        </is>
+      </c>
+      <c r="F74" s="4" t="inlineStr">
+        <is>
+          <t>Tous</t>
+        </is>
+      </c>
+      <c r="G74" s="6" t="inlineStr">
+        <is>
+          <t>À tester</t>
+        </is>
+      </c>
+      <c r="H74" s="6" t="inlineStr">
+        <is>
+          <t>Sur STA le 26/10/2026 (décisions de Jordan du 26/10).</t>
+        </is>
+      </c>
+      <c r="I74" s="6" t="n"/>
+    </row>
+    <row r="75">
+      <c r="A75" s="4" t="inlineStr">
+        <is>
+          <t>71</t>
+        </is>
+      </c>
+      <c r="B75" s="5" t="inlineStr">
+        <is>
+          <t>Refonte — Mon gazon</t>
+        </is>
+      </c>
+      <c r="C75" s="4" t="inlineStr">
+        <is>
+          <t>Mon gazon</t>
+        </is>
+      </c>
+      <c r="D75" s="4" t="inlineStr">
+        <is>
+          <t>Parcourir Mon gazon ; retirer une action notée par erreur ; ouvrir l'ancienne adresse /history.</t>
+        </is>
+      </c>
+      <c r="E75" s="4" t="inlineStr">
+        <is>
+          <t>Évolution du score et actions de l'année, « Mes actions » (5 dernières, « Voir tout », retrait), « Mes progrès » (série, GreenPoints, classement ou renvoi vers le Quiz pendant la ligue), badges ; /history n'existe plus.</t>
+        </is>
+      </c>
+      <c r="F75" s="4" t="inlineStr">
+        <is>
+          <t>Tous</t>
+        </is>
+      </c>
+      <c r="G75" s="6" t="inlineStr">
+        <is>
+          <t>À tester</t>
+        </is>
+      </c>
+      <c r="H75" s="6" t="inlineStr">
+        <is>
+          <t>Sur STA le 26/10/2026 (décisions de Jordan du 26/10).</t>
+        </is>
+      </c>
+      <c r="I75" s="6" t="n"/>
+    </row>
+    <row r="76">
+      <c r="A76" s="4" t="inlineStr">
+        <is>
+          <t>72</t>
+        </is>
+      </c>
+      <c r="B76" s="5" t="inlineStr">
+        <is>
+          <t>Refonte — Premium sur l'accueil et le diagnostic</t>
+        </is>
+      </c>
+      <c r="C76" s="4" t="inlineStr">
+        <is>
+          <t>Accueil, Diagnostic</t>
+        </is>
+      </c>
+      <c r="D76" s="4" t="inlineStr">
+        <is>
+          <t>Regarder l'accueil et l'onglet Diagnostic avec un compte gratuit, puis Premium, puis dans l'app Android.</t>
+        </is>
+      </c>
+      <c r="E76" s="4" t="inlineStr">
+        <is>
+          <t>Gratuit : carte « Avec Premium » (sans paysagistes, prix ou offre en cours) ; Premium : raccourcis « Mes équipements » et « Mon plan annuel » ; app Android : pas de carte d'achat.</t>
+        </is>
+      </c>
+      <c r="F76" s="4" t="inlineStr">
+        <is>
+          <t>Gratuit, Premium, app Android</t>
+        </is>
+      </c>
+      <c r="G76" s="6" t="inlineStr">
+        <is>
+          <t>À tester</t>
+        </is>
+      </c>
+      <c r="H76" s="6" t="inlineStr">
+        <is>
+          <t>Sur STA le 26/10/2026 (décisions de Jordan du 26/10).</t>
+        </is>
+      </c>
+      <c r="I76" s="6" t="n"/>
+    </row>
+    <row r="77">
+      <c r="A77" s="4" t="inlineStr">
+        <is>
+          <t>73</t>
+        </is>
+      </c>
+      <c r="B77" s="5" t="inlineStr">
+        <is>
+          <t>Refonte — Choisir son niveau</t>
+        </is>
+      </c>
+      <c r="C77" s="4" t="inlineStr">
+        <is>
+          <t>/subscribe</t>
+        </is>
+      </c>
+      <c r="D77" s="4" t="inlineStr">
+        <is>
+          <t>Ouvrir la page avec un compte gratuit, un compte en essai, puis un abonné ; aller jusqu'au paiement Stripe sans payer.</t>
+        </is>
+      </c>
+      <c r="E77" s="4" t="inlineStr">
+        <is>
+          <t>3 niveaux (Visiteur, Gratuit, Premium) ; « Ton niveau » ou « Ton essai : encore N jours » ; abonné : « Tu es déjà Premium » ; formules, mentions légales et paiement inchangés.</t>
+        </is>
+      </c>
+      <c r="F77" s="4" t="inlineStr">
+        <is>
+          <t>Gratuit, essai, Premium</t>
+        </is>
+      </c>
+      <c r="G77" s="6" t="inlineStr">
+        <is>
+          <t>À tester</t>
+        </is>
+      </c>
+      <c r="H77" s="6" t="inlineStr">
+        <is>
+          <t>Sur STA le 26/10/2026 (décisions de Jordan du 26/10).</t>
+        </is>
+      </c>
+      <c r="I77" s="6" t="n"/>
+    </row>
+    <row r="78">
+      <c r="A78" s="4" t="inlineStr">
+        <is>
+          <t>74</t>
+        </is>
+      </c>
+      <c r="B78" s="5" t="inlineStr">
+        <is>
+          <t>Refonte — plan annuel inclus dans Premium</t>
+        </is>
+      </c>
+      <c r="C78" s="4" t="inlineStr">
+        <is>
+          <t>Mon gazon → Mon plan gazon ; CGV 7 bis</t>
+        </is>
+      </c>
+      <c r="D78" s="4" t="inlineStr">
+        <is>
+          <t>Ouvrir le plan avec un compte gratuit, un compte Premium et un compte ayant acheté un plan à 0,99 €.</t>
+        </is>
+      </c>
+      <c r="E78" s="4" t="inlineStr">
+        <is>
+          <t>Gratuit : aperçu d'un mois et « Inclus dans Premium », aucune vente ; Premium et plans déjà achetés : les 12 mois et le PDF ; CGV 7 bis réécrit.</t>
+        </is>
+      </c>
+      <c r="F78" s="4" t="inlineStr">
+        <is>
+          <t>Gratuit, Premium, acheteur</t>
+        </is>
+      </c>
+      <c r="G78" s="6" t="inlineStr">
+        <is>
+          <t>À tester</t>
+        </is>
+      </c>
+      <c r="H78" s="6" t="inlineStr">
+        <is>
+          <t>Sur STA le 26/10/2026 (décisions de Jordan du 26/10).</t>
+        </is>
+      </c>
+      <c r="I78" s="6" t="n"/>
+    </row>
+    <row r="79">
+      <c r="A79" s="4" t="inlineStr">
+        <is>
+          <t>75</t>
+        </is>
+      </c>
+      <c r="B79" s="5" t="inlineStr">
+        <is>
+          <t>Refonte — accueil visiteur</t>
+        </is>
+      </c>
+      <c r="C79" s="4" t="inlineStr">
+        <is>
+          <t>mongazon360.fr (non connecté)</t>
+        </is>
+      </c>
+      <c r="D79" s="4" t="inlineStr">
+        <is>
+          <t>Saisir une commune (puis une commune homonyme), essayer « Utiliser ma position », ouvrir un article, « Prendre une photo », « Créer mon compte gratuit » ; revenir le lendemain.</t>
+        </is>
+      </c>
+      <c r="E79" s="4" t="inlineStr">
+        <is>
+          <t>Météo du jour de la commune (température, ciel) ; conseil de Bob du jour ; 3 articles de la saison ; barre Accueil, Conseils, Diagnostic, Compte (aussi sur l'essai du diagnostic) ; commune retrouvée à la visite suivante.</t>
+        </is>
+      </c>
+      <c r="F79" s="4" t="inlineStr">
+        <is>
+          <t>Non connecté</t>
+        </is>
+      </c>
+      <c r="G79" s="6" t="inlineStr">
+        <is>
+          <t>À tester</t>
+        </is>
+      </c>
+      <c r="H79" s="6" t="inlineStr">
+        <is>
+          <t>Sur STA le 26/10/2026 (décisions de Jordan du 26/10).</t>
+        </is>
+      </c>
+      <c r="I79" s="6" t="n"/>
+    </row>
+    <row r="80">
+      <c r="A80" s="4" t="inlineStr">
+        <is>
+          <t>76</t>
+        </is>
+      </c>
+      <c r="B80" s="5" t="inlineStr">
+        <is>
+          <t>Refonte — démo retirée</t>
+        </is>
+      </c>
+      <c r="C80" s="4" t="inlineStr">
+        <is>
+          <t>mongazon360.fr/demo ; plan du site</t>
+        </is>
+      </c>
+      <c r="D80" s="4" t="inlineStr">
+        <is>
+          <t>Ouvrir l'ancienne adresse /demo ; lire sitemap.xml.</t>
+        </is>
+      </c>
+      <c r="E80" s="4" t="inlineStr">
+        <is>
+          <t>Redirection vers l'accueil ; /demo absente du plan du site.</t>
+        </is>
+      </c>
+      <c r="F80" s="4" t="inlineStr">
+        <is>
+          <t>Non connecté</t>
+        </is>
+      </c>
+      <c r="G80" s="6" t="inlineStr">
+        <is>
+          <t>À tester</t>
+        </is>
+      </c>
+      <c r="H80" s="6" t="inlineStr">
+        <is>
+          <t>Sur STA le 26/10/2026 (décisions de Jordan du 26/10).</t>
+        </is>
+      </c>
+      <c r="I80" s="6" t="n"/>
+    </row>
+    <row r="81">
+      <c r="A81" s="4" t="inlineStr">
+        <is>
+          <t>77</t>
+        </is>
+      </c>
+      <c r="B81" s="5" t="inlineStr">
+        <is>
+          <t>Refonte — carte Nouveautés</t>
+        </is>
+      </c>
+      <c r="C81" s="4" t="inlineStr">
+        <is>
+          <t>Accueil ; src/components/CarteNouveautes.jsx</t>
+        </is>
+      </c>
+      <c r="D81" s="4" t="inlineStr">
+        <is>
+          <t>Le jour de la mise en prod : régler MISE_EN_PROD sur cette date (commit), puis ouvrir l'app avec un ancien compte et un compte créé ensuite.</t>
+        </is>
+      </c>
+      <c r="E81" s="4" t="inlineStr">
+        <is>
+          <t>Carte « Mongazon360 fait peau neuve » pour l'ancien compte, fermée pour de bon par « J'ai compris » ; rien pour le nouveau compte.</t>
+        </is>
+      </c>
+      <c r="F81" s="4" t="inlineStr">
+        <is>
+          <t>Ancien et nouveau compte</t>
+        </is>
+      </c>
+      <c r="G81" s="6" t="inlineStr">
+        <is>
+          <t>À tester</t>
+        </is>
+      </c>
+      <c r="H81" s="6" t="inlineStr">
+        <is>
+          <t>Sur STA le 26/10/2026 (décisions de Jordan du 26/10).</t>
+        </is>
+      </c>
+      <c r="I81" s="6" t="n"/>
+    </row>
+    <row r="82">
+      <c r="A82" s="4" t="inlineStr">
+        <is>
+          <t>78</t>
+        </is>
+      </c>
+      <c r="B82" s="5" t="inlineStr">
+        <is>
+          <t>Refonte — visiteurs distincts</t>
+        </is>
+      </c>
+      <c r="C82" s="4" t="inlineStr">
+        <is>
+          <t>Pilotage → Activité ; Supabase PROD</t>
+        </is>
+      </c>
+      <c r="D82" s="4" t="inlineStr">
+        <is>
+          <t>Après quelques visites : regarder l'entonnoir ; vérifier la colonne visite des nouvelles lignes de funnel_events.</t>
+        </is>
+      </c>
+      <c r="E82" s="4" t="inlineStr">
+        <is>
+          <t>« Visiteurs distincts (30 j) » affichés par étape ; colonne visite remplie (créée le 26/10 en STA et en PROD) ; pages Cookies et Confidentialité mentionnent l'identifiant de visite.</t>
+        </is>
+      </c>
+      <c r="F82" s="4" t="inlineStr">
+        <is>
+          <t>Admin</t>
+        </is>
+      </c>
+      <c r="G82" s="6" t="inlineStr">
+        <is>
+          <t>À tester</t>
+        </is>
+      </c>
+      <c r="H82" s="6" t="inlineStr">
+        <is>
+          <t>Sur STA le 26/10/2026 (décisions de Jordan du 26/10).</t>
+        </is>
+      </c>
+      <c r="I82" s="6" t="n"/>
+    </row>
+    <row r="83">
+      <c r="A83" s="4" t="inlineStr">
+        <is>
+          <t>79</t>
+        </is>
+      </c>
+      <c r="B83" s="5" t="inlineStr">
+        <is>
+          <t>Refonte — Bob</t>
+        </is>
+      </c>
+      <c r="C83" s="4" t="inlineStr">
+        <is>
+          <t>Bob</t>
+        </is>
+      </c>
+      <c r="D83" s="4" t="inlineStr">
+        <is>
+          <t>Demander « Combien coûte Premium ? », « Où est le classement ? », « Le plan annuel est payant ? ».</t>
+        </is>
+      </c>
+      <c r="E83" s="4" t="inlineStr">
+        <is>
+          <t>Prix 2,99 € et 24,99 €, offre de saison et essai de 7 jours ; classement dans Mon gazon → Mes progrès ; plan annuel inclus dans Premium.</t>
+        </is>
+      </c>
+      <c r="F83" s="4" t="inlineStr">
+        <is>
+          <t>Gratuit</t>
+        </is>
+      </c>
+      <c r="G83" s="6" t="inlineStr">
+        <is>
+          <t>À tester</t>
+        </is>
+      </c>
+      <c r="H83" s="6" t="inlineStr">
+        <is>
+          <t>Sur STA le 26/10/2026 (décisions de Jordan du 26/10).</t>
+        </is>
+      </c>
+      <c r="I83" s="6" t="n"/>
+    </row>
+    <row r="84">
+      <c r="A84" s="4" t="inlineStr">
+        <is>
+          <t>80</t>
+        </is>
+      </c>
+      <c r="B84" s="5" t="inlineStr">
+        <is>
+          <t>Refonte — dates des pages légales</t>
+        </is>
+      </c>
+      <c r="C84" s="4" t="inlineStr">
+        <is>
+          <t>CGV, politique de cookies, politique de confidentialité</t>
+        </is>
+      </c>
+      <c r="D84" s="4" t="inlineStr">
+        <is>
+          <t>Le jour de la mise en prod : mettre la date du jour dans « Mise à jour » de ces 3 pages (commit).</t>
+        </is>
+      </c>
+      <c r="E84" s="4" t="inlineStr">
+        <is>
+          <t>Date de mise à jour = jour de la mise en prod.</t>
+        </is>
+      </c>
+      <c r="F84" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G84" s="6" t="inlineStr">
+        <is>
+          <t>À tester</t>
+        </is>
+      </c>
+      <c r="H84" s="6" t="inlineStr">
+        <is>
+          <t>Sur STA le 26/10/2026 (décisions de Jordan du 26/10).</t>
+        </is>
+      </c>
+      <c r="I84" s="6" t="n"/>
+    </row>
+    <row r="85">
+      <c r="A85" s="4" t="inlineStr">
+        <is>
+          <t>81</t>
+        </is>
+      </c>
+      <c r="B85" s="5" t="inlineStr">
+        <is>
+          <t>Alignement PROD / STA</t>
+        </is>
+      </c>
+      <c r="C85" s="4" t="inlineStr">
+        <is>
+          <t>Git</t>
+        </is>
+      </c>
+      <c r="D85" s="4" t="inlineStr">
+        <is>
+          <t>Après la fusion : git diff --quiet origin/main origin/Staging.</t>
+        </is>
+      </c>
+      <c r="E85" s="4" t="inlineStr">
+        <is>
+          <t>Aucune différence.</t>
+        </is>
+      </c>
+      <c r="F85" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G85" s="6" t="inlineStr">
+        <is>
+          <t>À tester</t>
+        </is>
+      </c>
+      <c r="H85" s="6" t="n"/>
+      <c r="I85" s="6" t="n"/>
+    </row>
+    <row r="86">
+      <c r="A86" s="4" t="inlineStr">
+        <is>
+          <t>82</t>
+        </is>
+      </c>
+      <c r="B86" s="5" t="inlineStr">
+        <is>
+          <t>Base de données PROD</t>
+        </is>
+      </c>
+      <c r="C86" s="4" t="inlineStr">
+        <is>
+          <t>Supabase PROD</t>
+        </is>
+      </c>
+      <c r="D86" s="4" t="inlineStr">
+        <is>
+          <t>Vérifier les tables codes et parrainages.</t>
+        </is>
+      </c>
+      <c r="E86" s="4" t="inlineStr">
+        <is>
+          <t>Tables présentes (créées le 05/10 sur les deux projets).</t>
+        </is>
+      </c>
+      <c r="F86" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G86" s="6" t="inlineStr">
+        <is>
+          <t>À tester</t>
+        </is>
+      </c>
+      <c r="H86" s="6" t="n"/>
+      <c r="I86" s="6" t="n"/>
+    </row>
+    <row r="87">
+      <c r="A87" s="4" t="inlineStr">
+        <is>
+          <t>83</t>
+        </is>
+      </c>
+      <c r="B87" s="5" t="inlineStr">
+        <is>
           <t>Règle de travail de décembre</t>
         </is>
       </c>
-      <c r="C74" s="4" t="inlineStr">
+      <c r="C87" s="4" t="inlineStr">
         <is>
           <t>CLAUDE.md</t>
         </is>
       </c>
-      <c r="D74" s="4" t="inlineStr">
+      <c r="D87" s="4" t="inlineStr">
         <is>
           <t>Après la mise en prod : retirer le paragraphe « Jusqu'à décembre 2026 ».</t>
         </is>
       </c>
-      <c r="E74" s="4" t="inlineStr">
+      <c r="E87" s="4" t="inlineStr">
         <is>
           <t>STA redevient identique à la PROD.</t>
         </is>
       </c>
-      <c r="F74" s="4" t="inlineStr">
+      <c r="F87" s="4" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G74" s="6" t="inlineStr">
-        <is>
-          <t>À tester</t>
-        </is>
-      </c>
-      <c r="H74" s="6" t="n"/>
-      <c r="I74" s="6" t="n"/>
+      <c r="G87" s="6" t="inlineStr">
+        <is>
+          <t>À tester</t>
+        </is>
+      </c>
+      <c r="H87" s="6" t="n"/>
+      <c r="I87" s="6" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A2:I2"/>
   </mergeCells>
-  <conditionalFormatting sqref="G5:G74">
+  <conditionalFormatting sqref="G5:G87">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"OK"</formula>
     </cfRule>
@@ -3353,7 +3912,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="G5:G74" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="G5:G87" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"À tester,OK,KO,Non testable"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Pilotage : graphiques agrandis en plein écran au toucher et petits graphiques plus lisibles (STA)
Chaque graphique de Pilotage (ou son lien « ⤢ Agrandir ») s'ouvre en plein écran : barres plus grandes, ouvertes sur
les jours les plus récents, détail des valeurs du plus récent au plus ancien ; position Google plus grande avec le
détail du mois touché ; carte des inscrits agrandie. Fermeture par ✕, le fond, Échap ou le bouton retour du
téléphone. Petits graphiques : valeur de la plus haute barre visible, dates espacées. Recette de décembre n° 81.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AUzY5Y8Bt2KRzzte5cJgH8
</commit_message>
<xml_diff>
--- a/docs/recette/Recette_prod_decembre_2026.xlsx
+++ b/docs/recette/Recette_prod_decembre_2026.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Recette décembre" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Déjà en prod (exceptions)" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Recette décembre" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Déjà en prod (exceptions)" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -505,7 +505,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I87"/>
+  <dimension ref="A1:I88"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -3790,27 +3790,27 @@
       </c>
       <c r="B85" s="5" t="inlineStr">
         <is>
-          <t>Alignement PROD / STA</t>
+          <t>Pilotage — graphiques agrandis</t>
         </is>
       </c>
       <c r="C85" s="4" t="inlineStr">
         <is>
-          <t>Git</t>
+          <t>Pilotage (Activité, Finances, Réseaux)</t>
         </is>
       </c>
       <c r="D85" s="4" t="inlineStr">
         <is>
-          <t>Après la fusion : git diff --quiet origin/main origin/Staging.</t>
+          <t>Toucher chaque graphique ou « ⤢ Agrandir » (nouveaux inscrits, actifs, visiteurs, position Google, inscriptions, revenus, followers, carte des inscrits), en portrait puis en paysage ; dans la position Google, toucher un mois ; fermer par ✕, en touchant le fond, puis avec le bouton retour du téléphone.</t>
         </is>
       </c>
       <c r="E85" s="4" t="inlineStr">
         <is>
-          <t>Aucune différence.</t>
+          <t>Graphique en plein écran et en grand, ouvert sur les jours les plus récents, avec le détail des valeurs du plus récent au plus ancien ; détail du mois touché ; carte agrandie à faire glisser ; le retour ferme la fenêtre sans quitter Pilotage. Petits graphiques : valeur de la plus haute barre visible, dates qui ne se chevauchent pas.</t>
         </is>
       </c>
       <c r="F85" s="4" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Admin</t>
         </is>
       </c>
       <c r="G85" s="6" t="inlineStr">
@@ -3818,7 +3818,11 @@
           <t>À tester</t>
         </is>
       </c>
-      <c r="H85" s="6" t="n"/>
+      <c r="H85" s="6" t="inlineStr">
+        <is>
+          <t>Sur STA le 28/10/2026 (demande de Jordan du 28/10).</t>
+        </is>
+      </c>
       <c r="I85" s="6" t="n"/>
     </row>
     <row r="86">
@@ -3829,22 +3833,22 @@
       </c>
       <c r="B86" s="5" t="inlineStr">
         <is>
-          <t>Base de données PROD</t>
+          <t>Alignement PROD / STA</t>
         </is>
       </c>
       <c r="C86" s="4" t="inlineStr">
         <is>
-          <t>Supabase PROD</t>
+          <t>Git</t>
         </is>
       </c>
       <c r="D86" s="4" t="inlineStr">
         <is>
-          <t>Vérifier les tables codes et parrainages.</t>
+          <t>Après la fusion : git diff --quiet origin/main origin/Staging.</t>
         </is>
       </c>
       <c r="E86" s="4" t="inlineStr">
         <is>
-          <t>Tables présentes (créées le 05/10 sur les deux projets).</t>
+          <t>Aucune différence.</t>
         </is>
       </c>
       <c r="F86" s="4" t="inlineStr">
@@ -3868,22 +3872,22 @@
       </c>
       <c r="B87" s="5" t="inlineStr">
         <is>
-          <t>Règle de travail de décembre</t>
+          <t>Base de données PROD</t>
         </is>
       </c>
       <c r="C87" s="4" t="inlineStr">
         <is>
-          <t>CLAUDE.md</t>
+          <t>Supabase PROD</t>
         </is>
       </c>
       <c r="D87" s="4" t="inlineStr">
         <is>
-          <t>Après la mise en prod : retirer le paragraphe « Jusqu'à décembre 2026 ».</t>
+          <t>Vérifier les tables codes et parrainages.</t>
         </is>
       </c>
       <c r="E87" s="4" t="inlineStr">
         <is>
-          <t>STA redevient identique à la PROD.</t>
+          <t>Tables présentes (créées le 05/10 sur les deux projets).</t>
         </is>
       </c>
       <c r="F87" s="4" t="inlineStr">
@@ -3898,12 +3902,51 @@
       </c>
       <c r="H87" s="6" t="n"/>
       <c r="I87" s="6" t="n"/>
+    </row>
+    <row r="88">
+      <c r="A88" s="4" t="inlineStr">
+        <is>
+          <t>84</t>
+        </is>
+      </c>
+      <c r="B88" s="5" t="inlineStr">
+        <is>
+          <t>Règle de travail de décembre</t>
+        </is>
+      </c>
+      <c r="C88" s="4" t="inlineStr">
+        <is>
+          <t>CLAUDE.md</t>
+        </is>
+      </c>
+      <c r="D88" s="4" t="inlineStr">
+        <is>
+          <t>Après la mise en prod : retirer le paragraphe « Jusqu'à décembre 2026 ».</t>
+        </is>
+      </c>
+      <c r="E88" s="4" t="inlineStr">
+        <is>
+          <t>STA redevient identique à la PROD.</t>
+        </is>
+      </c>
+      <c r="F88" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G88" s="6" t="inlineStr">
+        <is>
+          <t>À tester</t>
+        </is>
+      </c>
+      <c r="H88" s="6" t="n"/>
+      <c r="I88" s="6" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A2:I2"/>
   </mergeCells>
-  <conditionalFormatting sqref="G5:G87">
+  <conditionalFormatting sqref="G5:G88">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"OK"</formula>
     </cfRule>
@@ -3912,7 +3955,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="G5:G87" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="G5:G88" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"À tester,OK,KO,Non testable"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Recette : graphiques agrandis de Pilotage passés en prod le 28/10 (exception, n° 43)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AUzY5Y8Bt2KRzzte5cJgH8
</commit_message>
<xml_diff>
--- a/docs/recette/Recette_prod_decembre_2026.xlsx
+++ b/docs/recette/Recette_prod_decembre_2026.xlsx
@@ -505,7 +505,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I88"/>
+  <dimension ref="A1:I87"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -3790,27 +3790,27 @@
       </c>
       <c r="B85" s="5" t="inlineStr">
         <is>
-          <t>Pilotage — graphiques agrandis</t>
+          <t>Alignement PROD / STA</t>
         </is>
       </c>
       <c r="C85" s="4" t="inlineStr">
         <is>
-          <t>Pilotage (Activité, Finances, Réseaux)</t>
+          <t>Git</t>
         </is>
       </c>
       <c r="D85" s="4" t="inlineStr">
         <is>
-          <t>Toucher chaque graphique ou « ⤢ Agrandir » (nouveaux inscrits, actifs, visiteurs, position Google, inscriptions, revenus, followers, carte des inscrits), en portrait puis en paysage ; dans la position Google, toucher un mois ; fermer par ✕, en touchant le fond, puis avec le bouton retour du téléphone.</t>
+          <t>Après la fusion : git diff --quiet origin/main origin/Staging.</t>
         </is>
       </c>
       <c r="E85" s="4" t="inlineStr">
         <is>
-          <t>Graphique en plein écran et en grand, ouvert sur les jours les plus récents, avec le détail des valeurs du plus récent au plus ancien ; détail du mois touché ; carte agrandie à faire glisser ; le retour ferme la fenêtre sans quitter Pilotage. Petits graphiques : valeur de la plus haute barre visible, dates qui ne se chevauchent pas.</t>
+          <t>Aucune différence.</t>
         </is>
       </c>
       <c r="F85" s="4" t="inlineStr">
         <is>
-          <t>Admin</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G85" s="6" t="inlineStr">
@@ -3818,11 +3818,7 @@
           <t>À tester</t>
         </is>
       </c>
-      <c r="H85" s="6" t="inlineStr">
-        <is>
-          <t>Sur STA le 28/10/2026 (demande de Jordan du 28/10).</t>
-        </is>
-      </c>
+      <c r="H85" s="6" t="n"/>
       <c r="I85" s="6" t="n"/>
     </row>
     <row r="86">
@@ -3833,22 +3829,22 @@
       </c>
       <c r="B86" s="5" t="inlineStr">
         <is>
-          <t>Alignement PROD / STA</t>
+          <t>Base de données PROD</t>
         </is>
       </c>
       <c r="C86" s="4" t="inlineStr">
         <is>
-          <t>Git</t>
+          <t>Supabase PROD</t>
         </is>
       </c>
       <c r="D86" s="4" t="inlineStr">
         <is>
-          <t>Après la fusion : git diff --quiet origin/main origin/Staging.</t>
+          <t>Vérifier les tables codes et parrainages.</t>
         </is>
       </c>
       <c r="E86" s="4" t="inlineStr">
         <is>
-          <t>Aucune différence.</t>
+          <t>Tables présentes (créées le 05/10 sur les deux projets).</t>
         </is>
       </c>
       <c r="F86" s="4" t="inlineStr">
@@ -3872,22 +3868,22 @@
       </c>
       <c r="B87" s="5" t="inlineStr">
         <is>
-          <t>Base de données PROD</t>
+          <t>Règle de travail de décembre</t>
         </is>
       </c>
       <c r="C87" s="4" t="inlineStr">
         <is>
-          <t>Supabase PROD</t>
+          <t>CLAUDE.md</t>
         </is>
       </c>
       <c r="D87" s="4" t="inlineStr">
         <is>
-          <t>Vérifier les tables codes et parrainages.</t>
+          <t>Après la mise en prod : retirer le paragraphe « Jusqu'à décembre 2026 ».</t>
         </is>
       </c>
       <c r="E87" s="4" t="inlineStr">
         <is>
-          <t>Tables présentes (créées le 05/10 sur les deux projets).</t>
+          <t>STA redevient identique à la PROD.</t>
         </is>
       </c>
       <c r="F87" s="4" t="inlineStr">
@@ -3902,51 +3898,12 @@
       </c>
       <c r="H87" s="6" t="n"/>
       <c r="I87" s="6" t="n"/>
-    </row>
-    <row r="88">
-      <c r="A88" s="4" t="inlineStr">
-        <is>
-          <t>84</t>
-        </is>
-      </c>
-      <c r="B88" s="5" t="inlineStr">
-        <is>
-          <t>Règle de travail de décembre</t>
-        </is>
-      </c>
-      <c r="C88" s="4" t="inlineStr">
-        <is>
-          <t>CLAUDE.md</t>
-        </is>
-      </c>
-      <c r="D88" s="4" t="inlineStr">
-        <is>
-          <t>Après la mise en prod : retirer le paragraphe « Jusqu'à décembre 2026 ».</t>
-        </is>
-      </c>
-      <c r="E88" s="4" t="inlineStr">
-        <is>
-          <t>STA redevient identique à la PROD.</t>
-        </is>
-      </c>
-      <c r="F88" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G88" s="6" t="inlineStr">
-        <is>
-          <t>À tester</t>
-        </is>
-      </c>
-      <c r="H88" s="6" t="n"/>
-      <c r="I88" s="6" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A2:I2"/>
   </mergeCells>
-  <conditionalFormatting sqref="G5:G88">
+  <conditionalFormatting sqref="G5:G87">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"OK"</formula>
     </cfRule>
@@ -3955,7 +3912,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="G5:G88" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="G5:G87" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"À tester,OK,KO,Non testable"</formula1>
     </dataValidation>
   </dataValidations>
@@ -3969,7 +3926,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I46"/>
+  <dimension ref="A1:I47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -5806,11 +5763,54 @@
       </c>
       <c r="I46" s="8" t="n"/>
     </row>
+    <row r="47">
+      <c r="A47" s="4" t="inlineStr">
+        <is>
+          <t>43</t>
+        </is>
+      </c>
+      <c r="B47" s="5" t="inlineStr">
+        <is>
+          <t>Pilotage — graphiques agrandis</t>
+        </is>
+      </c>
+      <c r="C47" s="4" t="inlineStr">
+        <is>
+          <t>Pilotage (Activité, Finances, Réseaux)</t>
+        </is>
+      </c>
+      <c r="D47" s="4" t="inlineStr">
+        <is>
+          <t>Toucher chaque graphique ou « ⤢ Agrandir » (nouveaux inscrits, actifs, visiteurs, position Google, inscriptions, revenus, followers, carte des inscrits), en portrait puis en paysage ; dans la position Google, toucher un mois ; fermer par ✕, en touchant le fond, puis avec le bouton retour du téléphone.</t>
+        </is>
+      </c>
+      <c r="E47" s="4" t="inlineStr">
+        <is>
+          <t>Graphique en plein écran et en grand, ouvert sur les jours les plus récents, avec le détail des valeurs du plus récent au plus ancien ; détail du mois touché ; carte agrandie à faire glisser ; le retour ferme la fenêtre sans quitter Pilotage. Petits graphiques : valeur de la plus haute barre visible, dates qui ne se chevauchent pas.</t>
+        </is>
+      </c>
+      <c r="F47" s="4" t="inlineStr">
+        <is>
+          <t>Admin</t>
+        </is>
+      </c>
+      <c r="G47" s="6" t="inlineStr">
+        <is>
+          <t>À tester</t>
+        </is>
+      </c>
+      <c r="H47" s="6" t="inlineStr">
+        <is>
+          <t>En prod le 28/10/2026 (go de Jordan du 28/10 ; page réservée à l'admin).</t>
+        </is>
+      </c>
+      <c r="I47" s="8" t="n"/>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A2:I2"/>
   </mergeCells>
-  <conditionalFormatting sqref="G5:G30">
+  <conditionalFormatting sqref="G5:G47">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"OK"</formula>
     </cfRule>
@@ -5819,7 +5819,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="G5:G46" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="G5:G47" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"À tester,OK,KO,Non testable"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Offre d'hiver dès le 1er novembre chaque année, jusqu'au 25 février (décision de Jordan du 28/10)
L'offre d'été (1/07 → 15/08) ne change pas. Consignes de Bob tirées des périodes de src/lib/offreSaison.json (plus de
dates écrites en dur). Recette de décembre n° 81 ; n° 58 au nouveau prix de l'offre (12,99 €, à partir du 1/11).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AUzY5Y8Bt2KRzzte5cJgH8
</commit_message>
<xml_diff>
--- a/docs/recette/Recette_prod_decembre_2026.xlsx
+++ b/docs/recette/Recette_prod_decembre_2026.xlsx
@@ -505,7 +505,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I87"/>
+  <dimension ref="A1:I88"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -2819,7 +2819,7 @@
       </c>
       <c r="B62" s="5" t="inlineStr">
         <is>
-          <t>Pilotage — offre annuelle à 19,99 €</t>
+          <t>Pilotage — offre annuelle à 12,99 €</t>
         </is>
       </c>
       <c r="C62" s="4" t="inlineStr">
@@ -2829,12 +2829,12 @@
       </c>
       <c r="D62" s="4" t="inlineStr">
         <is>
-          <t>Avec un abonné annuel pris pendant l'offre saisonnière (à partir du 1/12) : ouvrir Finances.</t>
+          <t>Avec un abonné annuel pris pendant l'offre saisonnière (à partir du 1/11) : ouvrir Finances.</t>
         </is>
       </c>
       <c r="E62" s="4" t="inlineStr">
         <is>
-          <t>L'abonné compte pour 19,99 €/an la 1re année (MRR, ARR et Produits et charges) ; ligne « Abonnements annuels » : « dont 1 à 19,99 € la 1re année ». Les autres annuels restent à 39,99 €.</t>
+          <t>L'abonné compte pour 12,99 €/an la 1re année (MRR, ARR et Produits et charges) ; ligne « Abonnements annuels » : « dont 1 à 12,99 € la 1re année ». Les autres annuels restent à 39,99 €.</t>
         </is>
       </c>
       <c r="F62" s="4" t="inlineStr">
@@ -3790,27 +3790,27 @@
       </c>
       <c r="B85" s="5" t="inlineStr">
         <is>
-          <t>Alignement PROD / STA</t>
+          <t>Offre d'hiver dès le 1er novembre</t>
         </is>
       </c>
       <c r="C85" s="4" t="inlineStr">
         <is>
-          <t>Git</t>
+          <t>Choisir son niveau, accueil, Bob, email de lancement</t>
         </is>
       </c>
       <c r="D85" s="4" t="inlineStr">
         <is>
-          <t>Après la fusion : git diff --quiet origin/main origin/Staging.</t>
+          <t>À partir du 1/11 : ouvrir « Choisir son niveau » et l'accueil avec un compte gratuit ; demander à Bob « Quand est l'offre de saison ? » ; le matin du 1er jour d'offre, regarder l'email reçu par un compte gratuit qui accepte les offres.</t>
         </is>
       </c>
       <c r="E85" s="4" t="inlineStr">
         <is>
-          <t>Aucune différence.</t>
+          <t>Offre d'hiver : Premium 1 an à 12,99 € au lieu de 24,99 €, jusqu'au 25/02 (badge -48 %) ; Bob cite « du 1er novembre au 25 février et du 1er juillet au 15 août » ; email « ❄️ Premium 1 an à 12,99 € — jusqu'au 25/02 ». Avant le 1/11 : pas d'offre.</t>
         </is>
       </c>
       <c r="F85" s="4" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Gratuit</t>
         </is>
       </c>
       <c r="G85" s="6" t="inlineStr">
@@ -3818,7 +3818,11 @@
           <t>À tester</t>
         </is>
       </c>
-      <c r="H85" s="6" t="n"/>
+      <c r="H85" s="6" t="inlineStr">
+        <is>
+          <t>Sur STA le 28/10/2026 (décision de Jordan du 28/10 : l'offre d'hiver commence le 1/11 chaque année).</t>
+        </is>
+      </c>
       <c r="I85" s="6" t="n"/>
     </row>
     <row r="86">
@@ -3829,22 +3833,22 @@
       </c>
       <c r="B86" s="5" t="inlineStr">
         <is>
-          <t>Base de données PROD</t>
+          <t>Alignement PROD / STA</t>
         </is>
       </c>
       <c r="C86" s="4" t="inlineStr">
         <is>
-          <t>Supabase PROD</t>
+          <t>Git</t>
         </is>
       </c>
       <c r="D86" s="4" t="inlineStr">
         <is>
-          <t>Vérifier les tables codes et parrainages.</t>
+          <t>Après la fusion : git diff --quiet origin/main origin/Staging.</t>
         </is>
       </c>
       <c r="E86" s="4" t="inlineStr">
         <is>
-          <t>Tables présentes (créées le 05/10 sur les deux projets).</t>
+          <t>Aucune différence.</t>
         </is>
       </c>
       <c r="F86" s="4" t="inlineStr">
@@ -3868,22 +3872,22 @@
       </c>
       <c r="B87" s="5" t="inlineStr">
         <is>
-          <t>Règle de travail de décembre</t>
+          <t>Base de données PROD</t>
         </is>
       </c>
       <c r="C87" s="4" t="inlineStr">
         <is>
-          <t>CLAUDE.md</t>
+          <t>Supabase PROD</t>
         </is>
       </c>
       <c r="D87" s="4" t="inlineStr">
         <is>
-          <t>Après la mise en prod : retirer le paragraphe « Jusqu'à décembre 2026 ».</t>
+          <t>Vérifier les tables codes et parrainages.</t>
         </is>
       </c>
       <c r="E87" s="4" t="inlineStr">
         <is>
-          <t>STA redevient identique à la PROD.</t>
+          <t>Tables présentes (créées le 05/10 sur les deux projets).</t>
         </is>
       </c>
       <c r="F87" s="4" t="inlineStr">
@@ -3898,12 +3902,51 @@
       </c>
       <c r="H87" s="6" t="n"/>
       <c r="I87" s="6" t="n"/>
+    </row>
+    <row r="88">
+      <c r="A88" s="4" t="inlineStr">
+        <is>
+          <t>84</t>
+        </is>
+      </c>
+      <c r="B88" s="5" t="inlineStr">
+        <is>
+          <t>Règle de travail de décembre</t>
+        </is>
+      </c>
+      <c r="C88" s="4" t="inlineStr">
+        <is>
+          <t>CLAUDE.md</t>
+        </is>
+      </c>
+      <c r="D88" s="4" t="inlineStr">
+        <is>
+          <t>Après la mise en prod : retirer le paragraphe « Jusqu'à décembre 2026 ».</t>
+        </is>
+      </c>
+      <c r="E88" s="4" t="inlineStr">
+        <is>
+          <t>STA redevient identique à la PROD.</t>
+        </is>
+      </c>
+      <c r="F88" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G88" s="6" t="inlineStr">
+        <is>
+          <t>À tester</t>
+        </is>
+      </c>
+      <c r="H88" s="6" t="n"/>
+      <c r="I88" s="6" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A2:I2"/>
   </mergeCells>
-  <conditionalFormatting sqref="G5:G87">
+  <conditionalFormatting sqref="G5:G88">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"OK"</formula>
     </cfRule>
@@ -3912,7 +3955,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="G5:G87" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="G5:G88" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"À tester,OK,KO,Non testable"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Mesure de la refonte : abonnements payants comptés, indicateurs du point du lundi, gel de 3 semaines (décisions de Jordan du 28/10)
Webhook Stripe : une ligne anonyme premium_souscrit (formule, offre) dans funnel_events à chaque abonnement pris, sans
jamais bloquer l'activation de Premium. CLAUDE.md : indicateurs (visites → entrées dans l'app → inscriptions gratuites →
abonnements Premium, avant et après le 1/11), point chaque lundi matin, gel du 31/10 au 21/11 inclus, retour arrière.
Recette de décembre n° 82.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AUzY5Y8Bt2KRzzte5cJgH8
</commit_message>
<xml_diff>
--- a/docs/recette/Recette_prod_decembre_2026.xlsx
+++ b/docs/recette/Recette_prod_decembre_2026.xlsx
@@ -505,7 +505,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I88"/>
+  <dimension ref="A1:I89"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -3833,27 +3833,27 @@
       </c>
       <c r="B86" s="5" t="inlineStr">
         <is>
-          <t>Alignement PROD / STA</t>
+          <t>Mesure — abonnements Premium comptés</t>
         </is>
       </c>
       <c r="C86" s="4" t="inlineStr">
         <is>
-          <t>Git</t>
+          <t>Supabase PROD (funnel_events) ; point KPI du lundi</t>
         </is>
       </c>
       <c r="D86" s="4" t="inlineStr">
         <is>
-          <t>Après la fusion : git diff --quiet origin/main origin/Staging.</t>
+          <t>Après le premier abonnement payant pris en prod (mensuel ou annuel) : regarder funnel_events, étape premium_souscrit.</t>
         </is>
       </c>
       <c r="E86" s="4" t="inlineStr">
         <is>
-          <t>Aucune différence.</t>
+          <t>Une ligne par abonnement pris, sans identifiant d'utilisateur, avec la formule (mensuel ou annuel) et l'offre (saison-hiver pendant l'offre) ; Premium activé même si la mesure échoue (alerte « Mesure — abonnement Premium non compté »).</t>
         </is>
       </c>
       <c r="F86" s="4" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Admin</t>
         </is>
       </c>
       <c r="G86" s="6" t="inlineStr">
@@ -3861,7 +3861,11 @@
           <t>À tester</t>
         </is>
       </c>
-      <c r="H86" s="6" t="n"/>
+      <c r="H86" s="6" t="inlineStr">
+        <is>
+          <t>Sur STA le 28/10/2026 (décision de Jordan du 28/10 : point KPI du lundi).</t>
+        </is>
+      </c>
       <c r="I86" s="6" t="n"/>
     </row>
     <row r="87">
@@ -3872,22 +3876,22 @@
       </c>
       <c r="B87" s="5" t="inlineStr">
         <is>
-          <t>Base de données PROD</t>
+          <t>Alignement PROD / STA</t>
         </is>
       </c>
       <c r="C87" s="4" t="inlineStr">
         <is>
-          <t>Supabase PROD</t>
+          <t>Git</t>
         </is>
       </c>
       <c r="D87" s="4" t="inlineStr">
         <is>
-          <t>Vérifier les tables codes et parrainages.</t>
+          <t>Après la fusion : git diff --quiet origin/main origin/Staging.</t>
         </is>
       </c>
       <c r="E87" s="4" t="inlineStr">
         <is>
-          <t>Tables présentes (créées le 05/10 sur les deux projets).</t>
+          <t>Aucune différence.</t>
         </is>
       </c>
       <c r="F87" s="4" t="inlineStr">
@@ -3911,22 +3915,22 @@
       </c>
       <c r="B88" s="5" t="inlineStr">
         <is>
-          <t>Règle de travail de décembre</t>
+          <t>Base de données PROD</t>
         </is>
       </c>
       <c r="C88" s="4" t="inlineStr">
         <is>
-          <t>CLAUDE.md</t>
+          <t>Supabase PROD</t>
         </is>
       </c>
       <c r="D88" s="4" t="inlineStr">
         <is>
-          <t>Après la mise en prod : retirer le paragraphe « Jusqu'à décembre 2026 ».</t>
+          <t>Vérifier les tables codes et parrainages.</t>
         </is>
       </c>
       <c r="E88" s="4" t="inlineStr">
         <is>
-          <t>STA redevient identique à la PROD.</t>
+          <t>Tables présentes (créées le 05/10 sur les deux projets).</t>
         </is>
       </c>
       <c r="F88" s="4" t="inlineStr">
@@ -3941,12 +3945,51 @@
       </c>
       <c r="H88" s="6" t="n"/>
       <c r="I88" s="6" t="n"/>
+    </row>
+    <row r="89">
+      <c r="A89" s="4" t="inlineStr">
+        <is>
+          <t>85</t>
+        </is>
+      </c>
+      <c r="B89" s="5" t="inlineStr">
+        <is>
+          <t>Règle de travail de décembre</t>
+        </is>
+      </c>
+      <c r="C89" s="4" t="inlineStr">
+        <is>
+          <t>CLAUDE.md</t>
+        </is>
+      </c>
+      <c r="D89" s="4" t="inlineStr">
+        <is>
+          <t>Après la mise en prod : retirer le paragraphe « Jusqu'à décembre 2026 ».</t>
+        </is>
+      </c>
+      <c r="E89" s="4" t="inlineStr">
+        <is>
+          <t>STA redevient identique à la PROD.</t>
+        </is>
+      </c>
+      <c r="F89" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G89" s="6" t="inlineStr">
+        <is>
+          <t>À tester</t>
+        </is>
+      </c>
+      <c r="H89" s="6" t="n"/>
+      <c r="I89" s="6" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A2:I2"/>
   </mergeCells>
-  <conditionalFormatting sqref="G5:G88">
+  <conditionalFormatting sqref="G5:G89">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"OK"</formula>
     </cfRule>
@@ -3955,7 +3998,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="G5:G88" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="G5:G89" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"À tester,OK,KO,Non testable"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Mesure : chaque page Conseils lue reliée à l'entrée dans l'app au cours de la même visite (conseils_vue)
Les pages Conseils écrivent une ligne conseils_vue (page, origine) dans funnel_events, une fois par page et par onglet,
avec l'identifiant de visite de l'app : on saura quels articles mènent à l'app. Invisible pour les visiteurs (autorisé
pendant le gel). Analyse de la hausse des visites du 25 au 28/10 notée au journal ; recette de décembre n° 83.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AUzY5Y8Bt2KRzzte5cJgH8
</commit_message>
<xml_diff>
--- a/docs/recette/Recette_prod_decembre_2026.xlsx
+++ b/docs/recette/Recette_prod_decembre_2026.xlsx
@@ -505,7 +505,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I89"/>
+  <dimension ref="A1:I90"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -3876,27 +3876,27 @@
       </c>
       <c r="B87" s="5" t="inlineStr">
         <is>
-          <t>Alignement PROD / STA</t>
+          <t>Mesure — articles qui mènent à l'app</t>
         </is>
       </c>
       <c r="C87" s="4" t="inlineStr">
         <is>
-          <t>Git</t>
+          <t>Pages Conseils ; Supabase PROD (funnel_events)</t>
         </is>
       </c>
       <c r="D87" s="4" t="inlineStr">
         <is>
-          <t>Après la fusion : git diff --quiet origin/main origin/Staging.</t>
+          <t>Sans être connecté, sur téléphone : ouvrir un article depuis un lien suivi (ex. groupe Facebook), puis toucher « Diagnostic gratuit » dans le même onglet ; regarder funnel_events.</t>
         </is>
       </c>
       <c r="E87" s="4" t="inlineStr">
         <is>
-          <t>Aucune différence.</t>
+          <t>Une ligne conseils_vue (page = article, source = origine) puis la page_view de /essai avec le même identifiant de visite ; un rechargement ne recompte pas l'article ; rien pour un compte connecté.</t>
         </is>
       </c>
       <c r="F87" s="4" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Admin</t>
         </is>
       </c>
       <c r="G87" s="6" t="inlineStr">
@@ -3904,7 +3904,11 @@
           <t>À tester</t>
         </is>
       </c>
-      <c r="H87" s="6" t="n"/>
+      <c r="H87" s="6" t="inlineStr">
+        <is>
+          <t>Sur STA le 28/10/2026 (demande de Jordan du 28/10 : faire atterrir le flux du site dans l'app).</t>
+        </is>
+      </c>
       <c r="I87" s="6" t="n"/>
     </row>
     <row r="88">
@@ -3915,22 +3919,22 @@
       </c>
       <c r="B88" s="5" t="inlineStr">
         <is>
-          <t>Base de données PROD</t>
+          <t>Alignement PROD / STA</t>
         </is>
       </c>
       <c r="C88" s="4" t="inlineStr">
         <is>
-          <t>Supabase PROD</t>
+          <t>Git</t>
         </is>
       </c>
       <c r="D88" s="4" t="inlineStr">
         <is>
-          <t>Vérifier les tables codes et parrainages.</t>
+          <t>Après la fusion : git diff --quiet origin/main origin/Staging.</t>
         </is>
       </c>
       <c r="E88" s="4" t="inlineStr">
         <is>
-          <t>Tables présentes (créées le 05/10 sur les deux projets).</t>
+          <t>Aucune différence.</t>
         </is>
       </c>
       <c r="F88" s="4" t="inlineStr">
@@ -3954,22 +3958,22 @@
       </c>
       <c r="B89" s="5" t="inlineStr">
         <is>
-          <t>Règle de travail de décembre</t>
+          <t>Base de données PROD</t>
         </is>
       </c>
       <c r="C89" s="4" t="inlineStr">
         <is>
-          <t>CLAUDE.md</t>
+          <t>Supabase PROD</t>
         </is>
       </c>
       <c r="D89" s="4" t="inlineStr">
         <is>
-          <t>Après la mise en prod : retirer le paragraphe « Jusqu'à décembre 2026 ».</t>
+          <t>Vérifier les tables codes et parrainages.</t>
         </is>
       </c>
       <c r="E89" s="4" t="inlineStr">
         <is>
-          <t>STA redevient identique à la PROD.</t>
+          <t>Tables présentes (créées le 05/10 sur les deux projets).</t>
         </is>
       </c>
       <c r="F89" s="4" t="inlineStr">
@@ -3984,12 +3988,51 @@
       </c>
       <c r="H89" s="6" t="n"/>
       <c r="I89" s="6" t="n"/>
+    </row>
+    <row r="90">
+      <c r="A90" s="4" t="inlineStr">
+        <is>
+          <t>86</t>
+        </is>
+      </c>
+      <c r="B90" s="5" t="inlineStr">
+        <is>
+          <t>Règle de travail de décembre</t>
+        </is>
+      </c>
+      <c r="C90" s="4" t="inlineStr">
+        <is>
+          <t>CLAUDE.md</t>
+        </is>
+      </c>
+      <c r="D90" s="4" t="inlineStr">
+        <is>
+          <t>Après la mise en prod : retirer le paragraphe « Jusqu'à décembre 2026 ».</t>
+        </is>
+      </c>
+      <c r="E90" s="4" t="inlineStr">
+        <is>
+          <t>STA redevient identique à la PROD.</t>
+        </is>
+      </c>
+      <c r="F90" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G90" s="6" t="inlineStr">
+        <is>
+          <t>À tester</t>
+        </is>
+      </c>
+      <c r="H90" s="6" t="n"/>
+      <c r="I90" s="6" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A2:I2"/>
   </mergeCells>
-  <conditionalFormatting sqref="G5:G89">
+  <conditionalFormatting sqref="G5:G90">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"OK"</formula>
     </cfRule>
@@ -3998,7 +4041,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="G5:G89" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="G5:G90" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"À tester,OK,KO,Non testable"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Mammotion (STA) : modèles pris en charge et autorisation d'usage commercial selon leur réponse du 29/10
Écran Mes équipements, consignes de Bob, CLAUDE.md et recette n° 40 : seul le LUBA 3 AWD est entièrement pris en charge,
rien d'avant 2025 ; usage commercial soumis à l'autorisation écrite préalable de Mammotion, sans laquelle le connecteur
ne part pas en prod. Journal : réponse aux 4 questions et suite.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AUzY5Y8Bt2KRzzte5cJgH8
</commit_message>
<xml_diff>
--- a/docs/recette/Recette_prod_decembre_2026.xlsx
+++ b/docs/recette/Recette_prod_decembre_2026.xlsx
@@ -2091,7 +2091,7 @@
       </c>
       <c r="D44" s="4" t="inlineStr">
         <is>
-          <t>Sur developer.mammotion.com, créer des identifiants (« Create Credentials ») avec un compte Mammotion qui a un robot sorti à partir de 2025, les coller puis « Connecter mon robot Mammotion » ; recommencer avec un compte sans robot compatible.</t>
+          <t>Sur developer.mammotion.com, créer des identifiants (« Create Credentials ») avec un compte Mammotion qui a un LUBA 3 AWD (seul modèle entièrement pris en charge au 29/10/2026), les coller puis « Connecter mon robot Mammotion » ; recommencer avec un compte sans robot compatible.</t>
         </is>
       </c>
       <c r="E44" s="4" t="inlineStr">
@@ -2111,7 +2111,7 @@
       </c>
       <c r="H44" s="6" t="inlineStr">
         <is>
-          <t>Sur STA le 17/10/2026. Avant la prod : accord écrit de Mammotion pour une app payante (ou connexion OAuth fournie par Mammotion).</t>
+          <t>Sur STA le 17/10/2026. Avant la prod : autorisation écrite de Mammotion pour une app payante (réponse du 29/10/2026 : usage commercial soumis à leur autorisation écrite préalable, demandée) ; sans elle, Mammotion masqué en prod (liste des marques, Bob, confidentialité 6.3).</t>
         </is>
       </c>
       <c r="I44" s="6" t="n"/>

</xml_diff>

<commit_message>
Recette et journal : abonnement de test réussi sur STA (paiement, webhook, Premium, comptage), /demo vérifiée
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AUzY5Y8Bt2KRzzte5cJgH8
</commit_message>
<xml_diff>
--- a/docs/recette/Recette_prod_decembre_2026.xlsx
+++ b/docs/recette/Recette_prod_decembre_2026.xlsx
@@ -533,6 +533,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -3476,7 +3477,7 @@
       </c>
       <c r="H77" s="6" t="inlineStr">
         <is>
-          <t>Sur STA le 26/10/2026 (décisions de Jordan du 26/10).</t>
+          <t>Sur STA le 26/10/2026 (décisions de Jordan du 26/10). Paiement de test réussi sur STA le 29/10 (mensuel à 2,99 €, bac à sable Stripe).</t>
         </is>
       </c>
       <c r="I77" s="6" t="n"/>
@@ -3605,7 +3606,7 @@
       </c>
       <c r="H80" s="6" t="inlineStr">
         <is>
-          <t>Sur STA le 26/10/2026 (décisions de Jordan du 26/10).</t>
+          <t>Sur STA le 26/10/2026 (décisions de Jordan du 26/10). Vérifié sur STA le 29/10 : /demo redirigée vers l'accueil (308), absente du plan du site.</t>
         </is>
       </c>
       <c r="I80" s="6" t="n"/>
@@ -3863,7 +3864,7 @@
       </c>
       <c r="H86" s="6" t="inlineStr">
         <is>
-          <t>Sur STA le 28/10/2026 (décision de Jordan du 28/10 : point KPI du lundi).</t>
+          <t>Sur STA le 28/10/2026 (décision de Jordan du 28/10 : point KPI du lundi). Vérifié sur STA le 29/10 : abonnement de test mensuel compté (premium_souscrit, offre vide avant le 1/11).</t>
         </is>
       </c>
       <c r="I86" s="6" t="n"/>

</xml_diff>

<commit_message>
Bob : classement en pause de novembre à janvier, remplacé par la ligue d'hiver ; test de la refonte sur STA noté
Recette (n° 68 à 74 et 79) et journal : résultats du test de Jordan sur STA ; Mon gazon à épurer (chantier à part).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AUzY5Y8Bt2KRzzte5cJgH8
</commit_message>
<xml_diff>
--- a/docs/recette/Recette_prod_decembre_2026.xlsx
+++ b/docs/recette/Recette_prod_decembre_2026.xlsx
@@ -3262,7 +3262,7 @@
       </c>
       <c r="H72" s="6" t="inlineStr">
         <is>
-          <t>Sur STA le 26/10/2026 (décisions de Jordan du 26/10).</t>
+          <t>Sur STA le 26/10/2026 (décisions de Jordan du 26/10). Testé par Jordan sur STA le 29/10 : OK.</t>
         </is>
       </c>
       <c r="I72" s="6" t="n"/>
@@ -3305,7 +3305,7 @@
       </c>
       <c r="H73" s="6" t="inlineStr">
         <is>
-          <t>Sur STA le 26/10/2026 (décisions de Jordan du 26/10).</t>
+          <t>Sur STA le 26/10/2026 (décisions de Jordan du 26/10). Testé par Jordan sur STA le 29/10 : OK.</t>
         </is>
       </c>
       <c r="I73" s="6" t="n"/>
@@ -3348,7 +3348,7 @@
       </c>
       <c r="H74" s="6" t="inlineStr">
         <is>
-          <t>Sur STA le 26/10/2026 (décisions de Jordan du 26/10).</t>
+          <t>Sur STA le 26/10/2026 (décisions de Jordan du 26/10). Testé par Jordan sur STA le 29/10 : OK.</t>
         </is>
       </c>
       <c r="I74" s="6" t="n"/>
@@ -3391,7 +3391,7 @@
       </c>
       <c r="H75" s="6" t="inlineStr">
         <is>
-          <t>Sur STA le 26/10/2026 (décisions de Jordan du 26/10).</t>
+          <t>Sur STA le 26/10/2026 (décisions de Jordan du 26/10). Testé par Jordan sur STA le 29/10 : OK, mais page jugée trop chargée (à épurer ensemble, chantier à part).</t>
         </is>
       </c>
       <c r="I75" s="6" t="n"/>
@@ -3434,7 +3434,7 @@
       </c>
       <c r="H76" s="6" t="inlineStr">
         <is>
-          <t>Sur STA le 26/10/2026 (décisions de Jordan du 26/10).</t>
+          <t>Sur STA le 26/10/2026 (décisions de Jordan du 26/10). Testé par Jordan sur STA le 29/10 : raccourcis Premium OK (compte gratuit et app Android à voir).</t>
         </is>
       </c>
       <c r="I76" s="6" t="n"/>
@@ -3477,7 +3477,7 @@
       </c>
       <c r="H77" s="6" t="inlineStr">
         <is>
-          <t>Sur STA le 26/10/2026 (décisions de Jordan du 26/10). Paiement de test réussi sur STA le 29/10 (mensuel à 2,99 €, bac à sable Stripe).</t>
+          <t>Sur STA le 26/10/2026 (décisions de Jordan du 26/10). Paiement de test réussi sur STA le 29/10 (mensuel à 2,99 €, bac à sable Stripe). Abonné : aucun lien vers la page (voulu) ; « Tu es déjà Premium » à vérifier par l'adresse /subscribe.</t>
         </is>
       </c>
       <c r="I77" s="6" t="n"/>
@@ -3520,7 +3520,7 @@
       </c>
       <c r="H78" s="6" t="inlineStr">
         <is>
-          <t>Sur STA le 26/10/2026 (décisions de Jordan du 26/10).</t>
+          <t>Sur STA le 26/10/2026 (décisions de Jordan du 26/10). Testé par Jordan sur STA le 29/10 : plan Premium OK (compte gratuit à voir).</t>
         </is>
       </c>
       <c r="I78" s="6" t="n"/>
@@ -3735,7 +3735,7 @@
       </c>
       <c r="H83" s="6" t="inlineStr">
         <is>
-          <t>Sur STA le 26/10/2026 (décisions de Jordan du 26/10).</t>
+          <t>Sur STA le 26/10/2026 (décisions de Jordan du 26/10). Testé par Jordan sur STA le 29/10 : OK ; consigne du classement précisée (en pause de novembre à janvier).</t>
         </is>
       </c>
       <c r="I83" s="6" t="n"/>

</xml_diff>

<commit_message>
Mon gazon épuré : 19 blocs → 7 (score et évolution compacts, outils, profil), courbe d'évolution réparée
Décision de Jordan du 29/10 : score santé compact avec « Pourquoi ce score ? » (4 critères et problèmes prioritaires)
et « Partager » ; évolution du score compacte ; « Mes actions » ; « Mes progrès » et badges en une ligne ; « Mes outils »
(plan gazon, équipements, semer ou regarnir, produits et dépenses, parrainage) ; « Mon profil » (complétude fusionnée,
débit de l'arroseur en Premium) ; carte « Avec Premium » pour les comptes gratuits. Retirés : conseil du mois, plan du
mois, produits recommandés, calibrage en grand bloc et ancien bloc Premium, avec leur code. La courbe de l'évolution du
score ne s'affichait pas (points de polyline en %) : tracée en coordonnées étirées. Consignes de Bob, recette n° 71 et
journal à jour.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AUzY5Y8Bt2KRzzte5cJgH8
</commit_message>
<xml_diff>
--- a/docs/recette/Recette_prod_decembre_2026.xlsx
+++ b/docs/recette/Recette_prod_decembre_2026.xlsx
@@ -3361,7 +3361,7 @@
       </c>
       <c r="B75" s="5" t="inlineStr">
         <is>
-          <t>Refonte — Mon gazon</t>
+          <t>Refonte — Mon gazon épuré</t>
         </is>
       </c>
       <c r="C75" s="4" t="inlineStr">
@@ -3371,12 +3371,12 @@
       </c>
       <c r="D75" s="4" t="inlineStr">
         <is>
-          <t>Parcourir Mon gazon ; retirer une action notée par erreur ; ouvrir l'ancienne adresse /history.</t>
+          <t>Parcourir Mon gazon avec un compte gratuit puis Premium ; déplier « Pourquoi ce score ? », « Partager », les badges et, en Premium, le débit de l'arroseur ; retirer une action notée par erreur ; toucher chaque outil ; ouvrir l'ancienne adresse /history.</t>
         </is>
       </c>
       <c r="E75" s="4" t="inlineStr">
         <is>
-          <t>Évolution du score et actions de l'année, « Mes actions » (5 dernières, « Voir tout », retrait), « Mes progrès » (série, GreenPoints, classement ou renvoi vers le Quiz pendant la ligue), badges ; /history n'existe plus.</t>
+          <t>Dans l'ordre : score santé compact (« Pourquoi ce score ? » : 4 critères et problèmes prioritaires ; « Partager »), évolution du score compacte (courbe, actions de l'année en une ligne, bilan de saison), « Mes actions » (5 dernières, « Voir tout », retrait), « Mes progrès » (série, GreenPoints, classement ou renvoi vers le Quiz pendant la ligue), badges en une ligne (« Voir tout »), « Mes outils » (plan gazon, équipements, semer ou regarnir, produits et dépenses ; parrainage avec la mise en prod de décembre), « Mon profil » (complétude, infos, débit de l'arroseur en Premium), « Avec Premium » pour un compte gratuit ; plus de conseil du mois, plan du mois, produits recommandés ni bloc de calibrage ; /history n'existe plus.</t>
         </is>
       </c>
       <c r="F75" s="4" t="inlineStr">
@@ -3391,7 +3391,7 @@
       </c>
       <c r="H75" s="6" t="inlineStr">
         <is>
-          <t>Sur STA le 26/10/2026 (décisions de Jordan du 26/10). Testé par Jordan sur STA le 29/10 : OK, mais page jugée trop chargée (à épurer ensemble, chantier à part).</t>
+          <t>Sur STA le 26/10/2026 (décisions de Jordan du 26/10). Testé par Jordan sur STA le 29/10 : OK, mais page jugée trop chargée (à épurer ensemble, chantier à part). Épurée le 29/10 (décision de Jordan) : 19 blocs → 7, à valider sur STA le 30/10.</t>
         </is>
       </c>
       <c r="I75" s="6" t="n"/>

</xml_diff>

<commit_message>
Choisir son niveau : un compte déjà Premium est renvoyé à l'accueil, sans voir la page
Décision de Jordan du 29/10 : abonné, Premium offert ou admin n'arrivent jamais sur la page (adresse tapée ou ancien lien
d'email) ; l'essai de 7 jours garde la page pour s'abonner. Le message « Tu es déjà Premium », devenu inaccessible, est
retiré. Recette n° 73 et journal à jour.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AUzY5Y8Bt2KRzzte5cJgH8
</commit_message>
<xml_diff>
--- a/docs/recette/Recette_prod_decembre_2026.xlsx
+++ b/docs/recette/Recette_prod_decembre_2026.xlsx
@@ -3457,12 +3457,12 @@
       </c>
       <c r="D77" s="4" t="inlineStr">
         <is>
-          <t>Ouvrir la page avec un compte gratuit, un compte en essai, puis un abonné ; aller jusqu'au paiement Stripe sans payer.</t>
+          <t>Ouvrir la page avec un compte gratuit, puis un compte en essai ; aller jusqu'au paiement Stripe sans payer ; ouvrir l'adresse /subscribe avec un compte abonné, Premium offert ou admin.</t>
         </is>
       </c>
       <c r="E77" s="4" t="inlineStr">
         <is>
-          <t>3 niveaux (Visiteur, Gratuit, Premium) ; « Ton niveau » ou « Ton essai : encore N jours » ; abonné : « Tu es déjà Premium » ; formules, mentions légales et paiement inchangés.</t>
+          <t>3 niveaux (Visiteur, Gratuit, Premium) ; « Ton niveau » ou « Ton essai : encore N jours » ; compte déjà Premium (abonné, Premium offert, admin) : renvoyé à l'accueil, la page ne s'affiche jamais ; formules, mentions légales et paiement inchangés.</t>
         </is>
       </c>
       <c r="F77" s="4" t="inlineStr">
@@ -3477,7 +3477,7 @@
       </c>
       <c r="H77" s="6" t="inlineStr">
         <is>
-          <t>Sur STA le 26/10/2026 (décisions de Jordan du 26/10). Paiement de test réussi sur STA le 29/10 (mensuel à 2,99 €, bac à sable Stripe). Abonné : aucun lien vers la page (voulu). Test de Jordan le 29/10 avec son compte admin : offres affichées au lieu de « Tu es déjà Premium » (compte admin non reconnu comme Premium sur cette page) ; corrigé le 29/10 (STA et version de prod), à revérifier.</t>
+          <t>Sur STA le 26/10/2026 (décisions de Jordan du 26/10). Paiement de test réussi sur STA le 29/10 (mensuel à 2,99 €, bac à sable Stripe). Abonné : aucun lien vers la page (voulu). Test de Jordan le 29/10 avec son compte admin : offres affichées au lieu de « Tu es déjà Premium » (compte admin non reconnu comme Premium sur cette page) ; corrigé le 29/10, puis décision de Jordan le soir même : un compte déjà Premium n'arrive jamais sur la page (renvoi à l'accueil), STA et version de prod.</t>
         </is>
       </c>
       <c r="I77" s="6" t="n"/>

</xml_diff>

<commit_message>
CLAUDE.md, recette n° 72 et journal : équipements connectés réservés à Premium
Complète le commit précédent (la mise à jour de ces fichiers n'y était pas partie).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AUzY5Y8Bt2KRzzte5cJgH8
</commit_message>
<xml_diff>
--- a/docs/recette/Recette_prod_decembre_2026.xlsx
+++ b/docs/recette/Recette_prod_decembre_2026.xlsx
@@ -3404,22 +3404,22 @@
       </c>
       <c r="B76" s="5" t="inlineStr">
         <is>
-          <t>Refonte — Premium sur l'accueil et le diagnostic</t>
+          <t>Refonte — Premium sur l'accueil, le diagnostic et les équipements</t>
         </is>
       </c>
       <c r="C76" s="4" t="inlineStr">
         <is>
-          <t>Accueil, Diagnostic</t>
+          <t>Accueil, Diagnostic, Mes équipements</t>
         </is>
       </c>
       <c r="D76" s="4" t="inlineStr">
         <is>
-          <t>Regarder l'accueil et l'onglet Diagnostic avec un compte gratuit, puis Premium, puis dans l'app Android.</t>
+          <t>Regarder l'accueil et l'onglet Diagnostic avec un compte gratuit, puis Premium, puis dans l'app Android ; ouvrir Mes équipements avec un compte gratuit (avec et sans équipement déjà connecté), puis Premium.</t>
         </is>
       </c>
       <c r="E76" s="4" t="inlineStr">
         <is>
-          <t>Gratuit : carte « Avec Premium » (sans paysagistes, prix ou offre en cours) ; Premium : raccourcis « Mes équipements » et « Mon plan annuel » ; app Android : pas de carte d'achat.</t>
+          <t>Gratuit : carte « Avec Premium » (sans paysagistes, prix ou offre en cours) ; Premium : raccourcis « Mes équipements » et « Mon plan annuel » ; app Android : pas de carte d'achat ; Mes équipements en gratuit : « Inclus dans Premium » et « Découvrir Premium » (pas dans l'app Android), aucune connexion possible, équipement déjà connecté seulement déconnectable ; le serveur refuse aussi connexions et commandes sans Premium ; Premium : connexions inchangées.</t>
         </is>
       </c>
       <c r="F76" s="4" t="inlineStr">
@@ -3434,7 +3434,7 @@
       </c>
       <c r="H76" s="6" t="inlineStr">
         <is>
-          <t>Sur STA le 26/10/2026 (décisions de Jordan du 26/10). Testé par Jordan sur STA le 29/10 : raccourcis Premium OK (compte gratuit et app Android à voir).</t>
+          <t>Sur STA le 26/10/2026 (décisions de Jordan du 26/10). Testé par Jordan sur STA le 29/10 : raccourcis Premium OK (compte gratuit et app Android à voir). Mes équipements ouverts aux comptes gratuits (constat de Jordan le 29/10) : verrou Premium ajouté le 29/10 (STA et version de prod).</t>
         </is>
       </c>
       <c r="I76" s="6" t="n"/>

</xml_diff>

<commit_message>
Pages Compte dans l'app (barre du bas du visiteur) et demande d'équipement non listé réservée à Premium
- Création de compte et connexion : barre du bas du visiteur (Accueil, Conseils, Diagnostic, Compte), onglet Compte en
  surbrillance (demande de Jordan du 29/10).
- Mes équipements d'un compte gratuit : plus de formulaire « Ton équipement n'est pas dans la liste ? », gardé pour
  Premium (décision de Jordan du 29/10).
- Consignes de Bob, CLAUDE.md, recette n° 49, 72 et 75, journal.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AUzY5Y8Bt2KRzzte5cJgH8
</commit_message>
<xml_diff>
--- a/docs/recette/Recette_prod_decembre_2026.xlsx
+++ b/docs/recette/Recette_prod_decembre_2026.xlsx
@@ -533,7 +533,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -2461,17 +2460,17 @@
       </c>
       <c r="D53" s="4" t="inlineStr">
         <is>
-          <t>Dans « Ton équipement n'est pas dans la liste ? » : choisir un type, saisir une marque (et un modèle), toucher « Envoyer ».</t>
+          <t>Avec un compte Premium, dans « Ton équipement n'est pas dans la liste ? » : choisir un type, saisir une marque (et un modèle), toucher « Envoyer » ; puis ouvrir Mes équipements avec un compte gratuit.</t>
         </is>
       </c>
       <c r="E53" s="4" t="inlineStr">
         <is>
-          <t>« ✅ Merci, c'est noté » ; bouton grisé sans marque ; rien de personnel enregistré (demande anonyme).</t>
+          <t>« ✅ Merci, c'est noté » ; bouton grisé sans marque ; rien de personnel enregistré (demande anonyme) ; compte gratuit : formulaire absent.</t>
         </is>
       </c>
       <c r="F53" s="4" t="inlineStr">
         <is>
-          <t>Tous</t>
+          <t>Premium, gratuit</t>
         </is>
       </c>
       <c r="G53" s="6" t="inlineStr">
@@ -2481,7 +2480,7 @@
       </c>
       <c r="H53" s="6" t="inlineStr">
         <is>
-          <t>Sur STA le 18/10/2026.</t>
+          <t>Sur STA le 18/10/2026. Réservé aux comptes Premium depuis le 29/10/2026 (décision de Jordan).</t>
         </is>
       </c>
       <c r="I53" s="6" t="n"/>
@@ -3419,7 +3418,7 @@
       </c>
       <c r="E76" s="4" t="inlineStr">
         <is>
-          <t>Gratuit : carte « Avec Premium » (sans paysagistes, prix ou offre en cours) ; Premium : raccourcis « Mes équipements » et « Mon plan annuel » ; app Android : pas de carte d'achat ; Mes équipements en gratuit : « Inclus dans Premium » et « Découvrir Premium » (pas dans l'app Android), aucune connexion possible, équipement déjà connecté seulement déconnectable ; le serveur refuse aussi connexions et commandes sans Premium ; Premium : connexions inchangées.</t>
+          <t>Gratuit : carte « Avec Premium » (sans paysagistes, prix ou offre en cours) ; Premium : raccourcis « Mes équipements » et « Mon plan annuel » ; app Android : pas de carte d'achat ; Mes équipements en gratuit : « Inclus dans Premium » et « Découvrir Premium » (pas dans l'app Android), aucune connexion ni demande d'équipement non listé, équipement déjà connecté seulement déconnectable ; le serveur refuse aussi connexions et commandes sans Premium ; Premium : connexions inchangées.</t>
         </is>
       </c>
       <c r="F76" s="4" t="inlineStr">
@@ -3434,7 +3433,7 @@
       </c>
       <c r="H76" s="6" t="inlineStr">
         <is>
-          <t>Sur STA le 26/10/2026 (décisions de Jordan du 26/10). Testé par Jordan sur STA le 29/10 : raccourcis Premium OK (compte gratuit et app Android à voir). Mes équipements ouverts aux comptes gratuits (constat de Jordan le 29/10) : verrou Premium ajouté le 29/10 (STA et version de prod).</t>
+          <t>Sur STA le 26/10/2026 (décisions de Jordan du 26/10). Testé par Jordan sur STA le 29/10 : raccourcis Premium OK (compte gratuit et app Android à voir). Mes équipements ouverts aux comptes gratuits (constat de Jordan le 29/10) : verrou Premium ajouté le 29/10 (STA et version de prod), vérifié par Jordan sur STA le 29/10 ; demande d'équipement non listé retirée de la page d'un compte gratuit le 29/10 (décision de Jordan).</t>
         </is>
       </c>
       <c r="I76" s="6" t="n"/>
@@ -3543,12 +3542,12 @@
       </c>
       <c r="D79" s="4" t="inlineStr">
         <is>
-          <t>Saisir une commune (puis une commune homonyme), essayer « Utiliser ma position », ouvrir un article, « Prendre une photo », « Créer mon compte gratuit » ; revenir le lendemain.</t>
+          <t>Saisir une commune (puis une commune homonyme), essayer « Utiliser ma position », ouvrir un article, « Prendre une photo », « Créer mon compte gratuit », puis le lien de connexion ; revenir le lendemain.</t>
         </is>
       </c>
       <c r="E79" s="4" t="inlineStr">
         <is>
-          <t>Météo du jour de la commune (température, ciel) ; conseil de Bob du jour ; 3 articles de la saison ; barre Accueil, Conseils, Diagnostic, Compte (aussi sur l'essai du diagnostic) ; commune retrouvée à la visite suivante.</t>
+          <t>Météo du jour de la commune (température, ciel) ; conseil de Bob du jour ; 3 articles de la saison ; barre Accueil, Conseils, Diagnostic, Compte (aussi sur l'essai du diagnostic, la création de compte et la connexion, onglet Compte en surbrillance) ; commune retrouvée à la visite suivante.</t>
         </is>
       </c>
       <c r="F79" s="4" t="inlineStr">
@@ -3563,7 +3562,7 @@
       </c>
       <c r="H79" s="6" t="inlineStr">
         <is>
-          <t>Sur STA le 26/10/2026 (décisions de Jordan du 26/10).</t>
+          <t>Sur STA le 26/10/2026 (décisions de Jordan du 26/10). Testé par Jordan sur STA le 29/10 : OK ; barre du bas ajoutée le 29/10 à la création de compte et à la connexion (demande de Jordan), à revoir.</t>
         </is>
       </c>
       <c r="I79" s="6" t="n"/>

</xml_diff>

<commit_message>
Recette n° 49, 72, 74 et 75 et journal : tests de Jordan sur STA du 30/10 (compte gratuit, pages Compte)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AUzY5Y8Bt2KRzzte5cJgH8
</commit_message>
<xml_diff>
--- a/docs/recette/Recette_prod_decembre_2026.xlsx
+++ b/docs/recette/Recette_prod_decembre_2026.xlsx
@@ -2480,7 +2480,7 @@
       </c>
       <c r="H53" s="6" t="inlineStr">
         <is>
-          <t>Sur STA le 18/10/2026. Réservé aux comptes Premium depuis le 29/10/2026 (décision de Jordan).</t>
+          <t>Sur STA le 18/10/2026. Réservé aux comptes Premium depuis le 29/10/2026 (décision de Jordan). Vérifié par Jordan sur STA le 30/10 : formulaire absent pour un compte gratuit.</t>
         </is>
       </c>
       <c r="I53" s="6" t="n"/>
@@ -3418,7 +3418,7 @@
       </c>
       <c r="E76" s="4" t="inlineStr">
         <is>
-          <t>Gratuit : carte « Avec Premium » (sans paysagistes, prix ou offre en cours) ; Premium : raccourcis « Mes équipements » et « Mon plan annuel » ; app Android : pas de carte d'achat ; Mes équipements en gratuit : « Inclus dans Premium » et « Découvrir Premium » (pas dans l'app Android), aucune connexion ni demande d'équipement non listé, équipement déjà connecté seulement déconnectable ; le serveur refuse aussi connexions et commandes sans Premium ; Premium : connexions inchangées.</t>
+          <t>Gratuit : carte « Avec Premium » (avantages de Premium sans les paysagistes, puis le prix ou, pendant sa période, l'offre de saison) ; Premium : raccourcis « Mes équipements » et « Mon plan annuel » ; app Android : pas de carte d'achat ; Mes équipements en gratuit : « Inclus dans Premium » et « Découvrir Premium » (pas dans l'app Android), aucune connexion ni demande d'équipement non listé, équipement déjà connecté seulement déconnectable ; le serveur refuse aussi connexions et commandes sans Premium ; Premium : connexions inchangées.</t>
         </is>
       </c>
       <c r="F76" s="4" t="inlineStr">
@@ -3433,7 +3433,7 @@
       </c>
       <c r="H76" s="6" t="inlineStr">
         <is>
-          <t>Sur STA le 26/10/2026 (décisions de Jordan du 26/10). Testé par Jordan sur STA le 29/10 : raccourcis Premium OK (compte gratuit et app Android à voir). Mes équipements ouverts aux comptes gratuits (constat de Jordan le 29/10) : verrou Premium ajouté le 29/10 (STA et version de prod), vérifié par Jordan sur STA le 29/10 ; demande d'équipement non listé retirée de la page d'un compte gratuit le 29/10 (décision de Jordan).</t>
+          <t>Sur STA le 26/10/2026 (décisions de Jordan du 26/10). Testé par Jordan sur STA le 29/10 : raccourcis Premium OK (compte gratuit et app Android à voir). Mes équipements ouverts aux comptes gratuits (constat de Jordan le 29/10) : verrou Premium ajouté le 29/10 (STA et version de prod), vérifié par Jordan sur STA le 29/10 ; demande d'équipement non listé retirée de la page d'un compte gratuit le 29/10 (décision de Jordan). Compte gratuit testé par Jordan sur STA le 30/10 : OK (carte « Avec Premium » de l'accueil, du diagnostic et de Mon gazon ; Mes équipements verrouillé, sans formulaire). App Android : à vérifier après la mise en prod.</t>
         </is>
       </c>
       <c r="I76" s="6" t="n"/>
@@ -3519,7 +3519,7 @@
       </c>
       <c r="H78" s="6" t="inlineStr">
         <is>
-          <t>Sur STA le 26/10/2026 (décisions de Jordan du 26/10). Testé par Jordan sur STA le 29/10 : plan Premium OK (compte gratuit à voir).</t>
+          <t>Sur STA le 26/10/2026 (décisions de Jordan du 26/10). Testé par Jordan sur STA le 29/10 : plan Premium OK (compte gratuit à voir). Compte gratuit testé par Jordan sur STA le 30/10 : OK.</t>
         </is>
       </c>
       <c r="I78" s="6" t="n"/>
@@ -3562,7 +3562,7 @@
       </c>
       <c r="H79" s="6" t="inlineStr">
         <is>
-          <t>Sur STA le 26/10/2026 (décisions de Jordan du 26/10). Testé par Jordan sur STA le 29/10 : OK ; barre du bas ajoutée le 29/10 à la création de compte et à la connexion (demande de Jordan), à revoir.</t>
+          <t>Sur STA le 26/10/2026 (décisions de Jordan du 26/10). Testé par Jordan sur STA le 29/10 : OK ; barre du bas ajoutée le 29/10 à la création de compte et à la connexion (demande de Jordan), vérifiée par Jordan sur STA le 30/10 : OK.</t>
         </is>
       </c>
       <c r="I79" s="6" t="n"/>

</xml_diff>

<commit_message>
Recette n° 13 et journal : bandeau de Bob à 3/3 questions validé par Jordan sur STA (30/10)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AUzY5Y8Bt2KRzzte5cJgH8
</commit_message>
<xml_diff>
--- a/docs/recette/Recette_prod_decembre_2026.xlsx
+++ b/docs/recette/Recette_prod_decembre_2026.xlsx
@@ -1066,7 +1066,11 @@
           <t>À tester</t>
         </is>
       </c>
-      <c r="H17" s="6" t="n"/>
+      <c r="H17" s="6" t="inlineStr">
+        <is>
+          <t>Testé par Jordan sur STA le 30/10 : bandeau OK (« Passe Premium » pour 20 questions par jour, « Parraine un ami ») ; prix de l'offre saisonnière à revoir à partir du 1/11.</t>
+        </is>
+      </c>
       <c r="I17" s="6" t="n"/>
     </row>
     <row r="18">

</xml_diff>

<commit_message>
Bob : compteur de questions écrit en toutes lettres (« 1 question restante sur 3 ce mois-ci »)
« 0/3 questions ce mois-ci » se lisait comme « 0 utilisée » (demande de Jordan du 30/10) ; recette n° 13 et journal.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AUzY5Y8Bt2KRzzte5cJgH8
</commit_message>
<xml_diff>
--- a/docs/recette/Recette_prod_decembre_2026.xlsx
+++ b/docs/recette/Recette_prod_decembre_2026.xlsx
@@ -1053,7 +1053,7 @@
       </c>
       <c r="E17" s="4" t="inlineStr">
         <is>
-          <t>Bandeau : « Passe Premium » (+ prix 1re année pendant l'offre saisonnière) et « 🎁 Parraine un ami » ; saisie bloquée.</t>
+          <t>Bandeau : « Passe Premium » (+ prix 1re année pendant l'offre saisonnière) et « 🎁 Parraine un ami » ; saisie bloquée ; en-tête : « 2 questions restantes sur 3 ce mois-ci », puis « plus de question ce mois-ci ».</t>
         </is>
       </c>
       <c r="F17" s="4" t="inlineStr">
@@ -1068,7 +1068,7 @@
       </c>
       <c r="H17" s="6" t="inlineStr">
         <is>
-          <t>Testé par Jordan sur STA le 30/10 : bandeau OK (« Passe Premium » pour 20 questions par jour, « Parraine un ami ») ; prix de l'offre saisonnière à revoir à partir du 1/11.</t>
+          <t>Testé par Jordan sur STA le 30/10 : bandeau OK (« Passe Premium » pour 20 questions par jour, « Parraine un ami ») ; prix de l'offre saisonnière à revoir à partir du 1/11. Compteur de l'en-tête écrit en toutes lettres sur STA le 30/10 (demande de Jordan : « 0/3 » se lisait à l'envers).</t>
         </is>
       </c>
       <c r="I17" s="6" t="n"/>

</xml_diff>

<commit_message>
Conseils : l'app dans les articles (bandeau, 3 encarts, bouton fixe sur téléphone, grille « Ce que fait l'app »)
Chantier du 22/11 (décisions de Jordan des 28 et 30/10), sur STA :
- catalogue unique des 10 arguments de l'app (src/lib/argumentsApp.json), fonctions en prod seulement ;
- dans chaque article : bandeau sous le titre (2 versions à départager), encarts après « En bref », au milieu et à la
  fin, bouton fixe sur téléphone ; thèmes par l'en-tête « app » ou par mots-clés ;
- grille « Ce que fait l'app » sur la rubrique et Qui sommes-nous ;
- liens balisés « encart » (thème-position), enregistrés avec la page_view de l'app ;
- tableaux des articles défilants sur téléphone (ils élargissaient la page).
CLAUDE.md, recette n° 84 et journal.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AUzY5Y8Bt2KRzzte5cJgH8
</commit_message>
<xml_diff>
--- a/docs/recette/Recette_prod_decembre_2026.xlsx
+++ b/docs/recette/Recette_prod_decembre_2026.xlsx
@@ -505,7 +505,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I90"/>
+  <dimension ref="A1:I91"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -3923,27 +3923,27 @@
       </c>
       <c r="B88" s="5" t="inlineStr">
         <is>
-          <t>Alignement PROD / STA</t>
+          <t>Conseils — l'app dans les articles (prod le 22/11)</t>
         </is>
       </c>
       <c r="C88" s="4" t="inlineStr">
         <is>
-          <t>Git</t>
+          <t>Pages Conseils (article, rubrique, Qui sommes-nous) ; Supabase PROD (funnel_events)</t>
         </is>
       </c>
       <c r="D88" s="4" t="inlineStr">
         <is>
-          <t>Après la fusion : git diff --quiet origin/main origin/Staging.</t>
+          <t>Sans être connecté, sur un téléphone Android puis sur ordinateur : ouvrir un article ; regarder le bandeau sous le titre, les 3 encarts et le bouton fixe ; toucher un encart ; ouvrir la rubrique et Qui sommes-nous.</t>
         </is>
       </c>
       <c r="E88" s="4" t="inlineStr">
         <is>
-          <t>Aucune différence.</t>
+          <t>Bandeau sous le titre sans cacher le texte (« Télécharger sur Google Play » seulement dans le navigateur d'un téléphone Android) ; encarts après « En bref », au milieu et à la fin, thèmes variés selon l'article (src/lib/argumentsApp.json) ; bouton fixe « Ouvrir l'app gratuite » sur téléphone seulement ; grille « Ce que fait l'app » ; l'encart touché ouvre l'app et sa page_view porte encart = thème-position ; aucune page plus large que l'écran.</t>
         </is>
       </c>
       <c r="F88" s="4" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Non connecté</t>
         </is>
       </c>
       <c r="G88" s="6" t="inlineStr">
@@ -3951,7 +3951,11 @@
           <t>À tester</t>
         </is>
       </c>
-      <c r="H88" s="6" t="n"/>
+      <c r="H88" s="6" t="inlineStr">
+        <is>
+          <t>Sur STA le 30/10/2026 (décisions de Jordan des 28 et 30/10) ; bandeau en 2 versions à départager sur les visuels.</t>
+        </is>
+      </c>
       <c r="I88" s="6" t="n"/>
     </row>
     <row r="89">
@@ -3962,22 +3966,22 @@
       </c>
       <c r="B89" s="5" t="inlineStr">
         <is>
-          <t>Base de données PROD</t>
+          <t>Alignement PROD / STA</t>
         </is>
       </c>
       <c r="C89" s="4" t="inlineStr">
         <is>
-          <t>Supabase PROD</t>
+          <t>Git</t>
         </is>
       </c>
       <c r="D89" s="4" t="inlineStr">
         <is>
-          <t>Vérifier les tables codes et parrainages.</t>
+          <t>Après la fusion : git diff --quiet origin/main origin/Staging.</t>
         </is>
       </c>
       <c r="E89" s="4" t="inlineStr">
         <is>
-          <t>Tables présentes (créées le 05/10 sur les deux projets).</t>
+          <t>Aucune différence.</t>
         </is>
       </c>
       <c r="F89" s="4" t="inlineStr">
@@ -4001,22 +4005,22 @@
       </c>
       <c r="B90" s="5" t="inlineStr">
         <is>
-          <t>Règle de travail de décembre</t>
+          <t>Base de données PROD</t>
         </is>
       </c>
       <c r="C90" s="4" t="inlineStr">
         <is>
-          <t>CLAUDE.md</t>
+          <t>Supabase PROD</t>
         </is>
       </c>
       <c r="D90" s="4" t="inlineStr">
         <is>
-          <t>Après la mise en prod : retirer le paragraphe « Jusqu'à décembre 2026 ».</t>
+          <t>Vérifier les tables codes et parrainages.</t>
         </is>
       </c>
       <c r="E90" s="4" t="inlineStr">
         <is>
-          <t>STA redevient identique à la PROD.</t>
+          <t>Tables présentes (créées le 05/10 sur les deux projets).</t>
         </is>
       </c>
       <c r="F90" s="4" t="inlineStr">
@@ -4031,12 +4035,51 @@
       </c>
       <c r="H90" s="6" t="n"/>
       <c r="I90" s="6" t="n"/>
+    </row>
+    <row r="91">
+      <c r="A91" s="4" t="inlineStr">
+        <is>
+          <t>87</t>
+        </is>
+      </c>
+      <c r="B91" s="5" t="inlineStr">
+        <is>
+          <t>Règle de travail de décembre</t>
+        </is>
+      </c>
+      <c r="C91" s="4" t="inlineStr">
+        <is>
+          <t>CLAUDE.md</t>
+        </is>
+      </c>
+      <c r="D91" s="4" t="inlineStr">
+        <is>
+          <t>Après la mise en prod : retirer le paragraphe « Jusqu'à décembre 2026 ».</t>
+        </is>
+      </c>
+      <c r="E91" s="4" t="inlineStr">
+        <is>
+          <t>STA redevient identique à la PROD.</t>
+        </is>
+      </c>
+      <c r="F91" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G91" s="6" t="inlineStr">
+        <is>
+          <t>À tester</t>
+        </is>
+      </c>
+      <c r="H91" s="6" t="n"/>
+      <c r="I91" s="6" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A2:I2"/>
   </mergeCells>
-  <conditionalFormatting sqref="G5:G90">
+  <conditionalFormatting sqref="G5:G91">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"OK"</formula>
     </cfRule>
@@ -4045,7 +4088,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="G5:G90" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="G5:G91" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"À tester,OK,KO,Non testable"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Recette et journal : refonte en prod le 31/10 (24 lignes dans « Déjà en prod », décembre renuméroté)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AUzY5Y8Bt2KRzzte5cJgH8
</commit_message>
<xml_diff>
--- a/docs/recette/Recette_prod_decembre_2026.xlsx
+++ b/docs/recette/Recette_prod_decembre_2026.xlsx
@@ -505,7 +505,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I91"/>
+  <dimension ref="A1:I67"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -1157,27 +1157,27 @@
       </c>
       <c r="B20" s="5" t="inlineStr">
         <is>
-          <t>Météo gratuite — Dashboard</t>
+          <t>Titre du site et de l'app</t>
         </is>
       </c>
       <c r="C20" s="4" t="inlineStr">
         <is>
-          <t>Dashboard</t>
+          <t>Onglet du navigateur, Google, écran d'accueil</t>
         </is>
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
-          <t>Compte gratuit : regarder la carte météo à côté du score.</t>
+          <t>Regarder le titre de l'onglet et le nom de l'app installée.</t>
         </is>
       </c>
       <c r="E20" s="4" t="inlineStr">
         <is>
-          <t>Ville, icône, température et temps du jour ; « 🔒 Vent, pluie, alertes » + bouton Premium.</t>
+          <t>« Mongazon360® – Votre expert gazon » ; descriptions sans « IA » (Google met quelques jours à se mettre à jour).</t>
         </is>
       </c>
       <c r="F20" s="4" t="inlineStr">
         <is>
-          <t>Gratuit (essai terminé)</t>
+          <t>Tous</t>
         </is>
       </c>
       <c r="G20" s="6" t="inlineStr">
@@ -1185,11 +1185,7 @@
           <t>À tester</t>
         </is>
       </c>
-      <c r="H20" s="6" t="inlineStr">
-        <is>
-          <t>Validé sur STA le 09/10/2026 par Jordan ; à revérifier en prod.</t>
-        </is>
-      </c>
+      <c r="H20" s="6" t="n"/>
       <c r="I20" s="6" t="n"/>
     </row>
     <row r="21">
@@ -1198,27 +1194,27 @@
       </c>
       <c r="B21" s="5" t="inlineStr">
         <is>
-          <t>Météo gratuite — Aujourd'hui</t>
+          <t>Mention légale de Bob conservée</t>
         </is>
       </c>
       <c r="C21" s="4" t="inlineStr">
         <is>
-          <t>Aujourd'hui</t>
+          <t>Bob</t>
         </is>
       </c>
       <c r="D21" s="4" t="inlineStr">
         <is>
-          <t>Compte gratuit : bloc météo en haut de page.</t>
+          <t>Ouvrir Bob.</t>
         </is>
       </c>
       <c r="E21" s="4" t="inlineStr">
         <is>
-          <t>Température et temps du jour ; « 🔒 Pluie, humidité et vent : Premium » ; mention Open-Meteo.</t>
+          <t>Bandeau « Bob est une IA… » et message d'accueil toujours présents (obligation légale).</t>
         </is>
       </c>
       <c r="F21" s="4" t="inlineStr">
         <is>
-          <t>Gratuit (essai terminé)</t>
+          <t>Tous</t>
         </is>
       </c>
       <c r="G21" s="6" t="inlineStr">
@@ -1226,11 +1222,7 @@
           <t>À tester</t>
         </is>
       </c>
-      <c r="H21" s="6" t="inlineStr">
-        <is>
-          <t>Validé sur STA le 09/10/2026 par Jordan ; à revérifier en prod.</t>
-        </is>
-      </c>
+      <c r="H21" s="6" t="n"/>
       <c r="I21" s="6" t="n"/>
     </row>
     <row r="22">
@@ -1239,27 +1231,27 @@
       </c>
       <c r="B22" s="5" t="inlineStr">
         <is>
-          <t>Météo Premium inchangée</t>
+          <t>Robot Gardena SILENO — connexion</t>
         </is>
       </c>
       <c r="C22" s="4" t="inlineStr">
         <is>
-          <t>Dashboard, Aujourd'hui</t>
+          <t>Mes équipements → Robot tondeuse</t>
         </is>
       </c>
       <c r="D22" s="4" t="inlineStr">
         <is>
-          <t>Compte Premium : mêmes écrans.</t>
+          <t>« Connecter mon robot Gardena » avec un compte GARDENA smart system qui a un SILENO.</t>
         </is>
       </c>
       <c r="E22" s="4" t="inlineStr">
         <is>
-          <t>Météo complète (vent, pluie, humidité, station si connectée).</t>
+          <t>Retour sur Mes équipements avec « Robot Gardena connecté » ; carte robot (nom, état, batterie) ; libellé « Gardena SILENO ». Si le compte a aussi un arrosage Gardena : les deux sont connectés.</t>
         </is>
       </c>
       <c r="F22" s="4" t="inlineStr">
         <is>
-          <t>Premium</t>
+          <t>Compte avec SILENO (testeur à trouver)</t>
         </is>
       </c>
       <c r="G22" s="6" t="inlineStr">
@@ -1267,11 +1259,7 @@
           <t>À tester</t>
         </is>
       </c>
-      <c r="H22" s="6" t="inlineStr">
-        <is>
-          <t>Validé sur STA le 09/10/2026 par Jordan ; à revérifier en prod.</t>
-        </is>
-      </c>
+      <c r="H22" s="6" t="n"/>
       <c r="I22" s="6" t="n"/>
     </row>
     <row r="23">
@@ -1280,27 +1268,27 @@
       </c>
       <c r="B23" s="5" t="inlineStr">
         <is>
-          <t>Plus de « IA » — Diagnostic</t>
+          <t>Robot Gardena SILENO — sans robot</t>
         </is>
       </c>
       <c r="C23" s="4" t="inlineStr">
         <is>
-          <t>Diagnostic</t>
+          <t>Mes équipements → Robot tondeuse</t>
         </is>
       </c>
       <c r="D23" s="4" t="inlineStr">
         <is>
-          <t>Lire l'en-tête, l'écran Premium, le bouton et les étapes.</t>
+          <t>Même bouton avec un compte Gardena sans robot.</t>
         </is>
       </c>
       <c r="E23" s="4" t="inlineStr">
         <is>
-          <t>« Bob diagnostique votre gazon », « Ce que Bob fait pour vous », « Lancer le diagnostic de Bob » ; aucun « IA ».</t>
+          <t>Message « Aucun robot Gardena trouvé sur ce compte » ; rien n'est enregistré.</t>
         </is>
       </c>
       <c r="F23" s="4" t="inlineStr">
         <is>
-          <t>Gratuit et Premium</t>
+          <t>Compte Gardena sans robot</t>
         </is>
       </c>
       <c r="G23" s="6" t="inlineStr">
@@ -1308,11 +1296,7 @@
           <t>À tester</t>
         </is>
       </c>
-      <c r="H23" s="6" t="inlineStr">
-        <is>
-          <t>Validé sur STA le 09/10/2026 par Jordan ; à revérifier en prod.</t>
-        </is>
-      </c>
+      <c r="H23" s="6" t="n"/>
       <c r="I23" s="6" t="n"/>
     </row>
     <row r="24">
@@ -1321,27 +1305,27 @@
       </c>
       <c r="B24" s="5" t="inlineStr">
         <is>
-          <t>Plus de « IA » — Comparatif et Abonnement</t>
+          <t>Robot Gardena SILENO — proposition</t>
         </is>
       </c>
       <c r="C24" s="4" t="inlineStr">
         <is>
-          <t>Comparatif, Subscribe, SubscribeSuccess</t>
+          <t>Aujourd'hui</t>
         </is>
       </c>
       <c r="D24" s="4" t="inlineStr">
         <is>
-          <t>Lire les listes d'avantages.</t>
+          <t>Jour de pluie / gel : valider « Mettre au repos jusqu'à demain matin », puis un jour sans contrainte : « Relancer son planning ».</t>
         </is>
       </c>
       <c r="E24" s="4" t="inlineStr">
         <is>
-          <t>« Bob, votre assistant gazon 24/7 », « Diagnostic photo par Bob », « Recommandations personnalisées de Bob », « Calcul d'arrosage précis ».</t>
+          <t>Le robot rentre et reste garé (app Gardena : garé jusqu'à nouvel ordre) ; la relance remet son planning. Rien n'est envoyé sans validation.</t>
         </is>
       </c>
       <c r="F24" s="4" t="inlineStr">
         <is>
-          <t>Gratuit</t>
+          <t>Compte avec SILENO</t>
         </is>
       </c>
       <c r="G24" s="6" t="inlineStr">
@@ -1349,11 +1333,7 @@
           <t>À tester</t>
         </is>
       </c>
-      <c r="H24" s="6" t="inlineStr">
-        <is>
-          <t>Validé sur STA le 09/10/2026 par Jordan ; à revérifier en prod.</t>
-        </is>
-      </c>
+      <c r="H24" s="6" t="n"/>
       <c r="I24" s="6" t="n"/>
     </row>
     <row r="25">
@@ -1362,27 +1342,27 @@
       </c>
       <c r="B25" s="5" t="inlineStr">
         <is>
-          <t>Plus de « IA » — Aujourd'hui</t>
+          <t>Robot Gardena SILENO — reprise du matin</t>
         </is>
       </c>
       <c r="C25" s="4" t="inlineStr">
         <is>
-          <t>Aujourd'hui</t>
+          <t>Tâche du matin (PROD)</t>
         </is>
       </c>
       <c r="D25" s="4" t="inlineStr">
         <is>
-          <t>Bloc des recommandations.</t>
+          <t>Le lendemain d'un « repos jusqu'à demain matin », regarder le robot après 8 h.</t>
         </is>
       </c>
       <c r="E25" s="4" t="inlineStr">
         <is>
-          <t>Titre « 🤖 Recommandation Bob » ; messages « recommandation de Bob », « Impossible de contacter Bob ».</t>
+          <t>Planning relancé automatiquement (journal de la tâche : robotsRelances ≥ 1). Non testable sur STA (tâches planifiées en PROD seulement).</t>
         </is>
       </c>
       <c r="F25" s="4" t="inlineStr">
         <is>
-          <t>Gratuit et Premium</t>
+          <t>Compte avec SILENO</t>
         </is>
       </c>
       <c r="G25" s="6" t="inlineStr">
@@ -1390,11 +1370,7 @@
           <t>À tester</t>
         </is>
       </c>
-      <c r="H25" s="6" t="inlineStr">
-        <is>
-          <t>Validé sur STA le 09/10/2026 par Jordan ; à revérifier en prod.</t>
-        </is>
-      </c>
+      <c r="H25" s="6" t="n"/>
       <c r="I25" s="6" t="n"/>
     </row>
     <row r="26">
@@ -1403,27 +1379,27 @@
       </c>
       <c r="B26" s="5" t="inlineStr">
         <is>
-          <t>Plus de « IA » — autres écrans</t>
+          <t>Robot Gardena SILENO — déconnexion</t>
         </is>
       </c>
       <c r="C26" s="4" t="inlineStr">
         <is>
-          <t>Onboarding, Accueil, Démo, Badges, Score</t>
+          <t>Mes équipements</t>
         </is>
       </c>
       <c r="D26" s="4" t="inlineStr">
         <is>
-          <t>Parcourir l'onboarding, la page d'accueil, la démo, la galerie de badges, la fenêtre du score.</t>
+          <t>Avec arrosage ET robot Gardena : déconnecter le robot, puis vérifier l'arrosage.</t>
         </is>
       </c>
       <c r="E26" s="4" t="inlineStr">
         <is>
-          <t>« Planning personnalisé », « Bob, votre assistant gazon », « Arrosage au bon moment », « Diagnostic photo par Bob » ; aucun « IA » ni « intelligent ».</t>
+          <t>L'arrosage reste connecté et fonctionne (la connexion commune n'est révoquée qu'avec le dernier équipement Gardena).</t>
         </is>
       </c>
       <c r="F26" s="4" t="inlineStr">
         <is>
-          <t>Divers</t>
+          <t>Compte avec SILENO + arrosage Gardena</t>
         </is>
       </c>
       <c r="G26" s="6" t="inlineStr">
@@ -1431,11 +1407,7 @@
           <t>À tester</t>
         </is>
       </c>
-      <c r="H26" s="6" t="inlineStr">
-        <is>
-          <t>Validé sur STA le 09/10/2026 par Jordan ; à revérifier en prod.</t>
-        </is>
-      </c>
+      <c r="H26" s="6" t="n"/>
       <c r="I26" s="6" t="n"/>
     </row>
     <row r="27">
@@ -1444,27 +1416,27 @@
       </c>
       <c r="B27" s="5" t="inlineStr">
         <is>
-          <t>Plus de « IA » — messages d'erreur</t>
+          <t>Station Netatmo — connexion</t>
         </is>
       </c>
       <c r="C27" s="4" t="inlineStr">
         <is>
-          <t>Diagnostic, recommandations</t>
+          <t>Mes équipements → Station météo</t>
         </is>
       </c>
       <c r="D27" s="4" t="inlineStr">
         <is>
-          <t>Si possible, provoquer une indisponibilité (ou relire les messages).</t>
+          <t>« Connecter ma station Netatmo » avec un compte Netatmo qui a un module extérieur ou un pluviomètre.</t>
         </is>
       </c>
       <c r="E27" s="4" t="inlineStr">
         <is>
-          <t>« Bob est momentanément indisponible » ; « recommandations de Bob ».</t>
+          <t>Retour sur Mes équipements avec « Station Netatmo connectée » ; carte avec température, pluie du jour et vent ; libellé « Netatmo ».</t>
         </is>
       </c>
       <c r="F27" s="4" t="inlineStr">
         <is>
-          <t>Divers</t>
+          <t>Compte avec station Netatmo (testeur à trouver)</t>
         </is>
       </c>
       <c r="G27" s="6" t="inlineStr">
@@ -1474,7 +1446,7 @@
       </c>
       <c r="H27" s="6" t="inlineStr">
         <is>
-          <t>Validé sur STA le 09/10/2026 par Jordan ; à revérifier en prod.</t>
+          <t>Chaîne de connexion validée sur STA le 19/10/2026 par Jordan, sans station (« Aucune station météo trouvée sur ce compte Netatmo ») ; reste le test avec une vraie station.</t>
         </is>
       </c>
       <c r="I27" s="6" t="n"/>
@@ -1485,27 +1457,27 @@
       </c>
       <c r="B28" s="5" t="inlineStr">
         <is>
-          <t>Titre du site et de l'app</t>
+          <t>Station Netatmo — mesures du jardin</t>
         </is>
       </c>
       <c r="C28" s="4" t="inlineStr">
         <is>
-          <t>Onglet du navigateur, Google, écran d'accueil</t>
+          <t>Aujourd'hui, notifications, Bob</t>
         </is>
       </c>
       <c r="D28" s="4" t="inlineStr">
         <is>
-          <t>Regarder le titre de l'onglet et le nom de l'app installée.</t>
+          <t>Un jour de pluie, ouvrir « Aujourd'hui » et poser une question à Bob sur l'arrosage.</t>
         </is>
       </c>
       <c r="E28" s="4" t="inlineStr">
         <is>
-          <t>« Mongazon360® – Votre expert gazon » ; descriptions sans « IA » (Google met quelques jours à se mettre à jour).</t>
+          <t>La pluie mesurée par la station est prise en compte (arrosage, tonte) ; Bob cite la mesure de la station ; relevé de moins de 10 min.</t>
         </is>
       </c>
       <c r="F28" s="4" t="inlineStr">
         <is>
-          <t>Tous</t>
+          <t>Compte avec station Netatmo</t>
         </is>
       </c>
       <c r="G28" s="6" t="inlineStr">
@@ -1522,27 +1494,27 @@
       </c>
       <c r="B29" s="5" t="inlineStr">
         <is>
-          <t>Mention légale de Bob conservée</t>
+          <t>Station Netatmo — connexion annulée</t>
         </is>
       </c>
       <c r="C29" s="4" t="inlineStr">
         <is>
-          <t>Bob</t>
+          <t>Mes équipements</t>
         </is>
       </c>
       <c r="D29" s="4" t="inlineStr">
         <is>
-          <t>Ouvrir Bob.</t>
+          <t>Cliquer « Connecter ma station Netatmo », puis refuser l'accès sur le site de Netatmo.</t>
         </is>
       </c>
       <c r="E29" s="4" t="inlineStr">
         <is>
-          <t>Bandeau « Bob est une IA… » et message d'accueil toujours présents (obligation légale).</t>
+          <t>Message « Connexion annulée : rien n'a été enregistré » (même chose pour Husqvarna et Gardena).</t>
         </is>
       </c>
       <c r="F29" s="4" t="inlineStr">
         <is>
-          <t>Tous</t>
+          <t>Tout compte</t>
         </is>
       </c>
       <c r="G29" s="6" t="inlineStr">
@@ -1559,27 +1531,27 @@
       </c>
       <c r="B30" s="5" t="inlineStr">
         <is>
-          <t>Robot Gardena SILENO — connexion</t>
+          <t>Station Netatmo — déconnexion</t>
         </is>
       </c>
       <c r="C30" s="4" t="inlineStr">
         <is>
-          <t>Mes équipements → Robot tondeuse</t>
+          <t>Mes équipements</t>
         </is>
       </c>
       <c r="D30" s="4" t="inlineStr">
         <is>
-          <t>« Connecter mon robot Gardena » avec un compte GARDENA smart system qui a un SILENO.</t>
+          <t>« Déconnecter la station ».</t>
         </is>
       </c>
       <c r="E30" s="4" t="inlineStr">
         <is>
-          <t>Retour sur Mes équipements avec « Robot Gardena connecté » ; carte robot (nom, état, batterie) ; libellé « Gardena SILENO ». Si le compte a aussi un arrosage Gardena : les deux sont connectés.</t>
+          <t>La station disparaît ; « Aujourd'hui » repart sur les prévisions météo.</t>
         </is>
       </c>
       <c r="F30" s="4" t="inlineStr">
         <is>
-          <t>Compte avec SILENO (testeur à trouver)</t>
+          <t>Compte avec station Netatmo</t>
         </is>
       </c>
       <c r="G30" s="6" t="inlineStr">
@@ -1596,27 +1568,27 @@
       </c>
       <c r="B31" s="5" t="inlineStr">
         <is>
-          <t>Robot Gardena SILENO — sans robot</t>
+          <t>Station Netatmo — réglages PROD</t>
         </is>
       </c>
       <c r="C31" s="4" t="inlineStr">
         <is>
-          <t>Mes équipements → Robot tondeuse</t>
+          <t>Application Netatmo (dev.netatmo.com) et Vercel</t>
         </is>
       </c>
       <c r="D31" s="4" t="inlineStr">
         <is>
-          <t>Même bouton avec un compte Gardena sans robot.</t>
+          <t>Vérifier l'adresse de retour déclarée dans l'application Netatmo et les variables Vercel.</t>
         </is>
       </c>
       <c r="E31" s="4" t="inlineStr">
         <is>
-          <t>Message « Aucun robot Gardena trouvé sur ce compte » ; rien n'est enregistré.</t>
+          <t>Adresse de retour https://mongazon360.fr/api/objets ; NETATMO_CLIENT_ID et NETATMO_CLIENT_SECRET présentes en Production.</t>
         </is>
       </c>
       <c r="F31" s="4" t="inlineStr">
         <is>
-          <t>Compte Gardena sans robot</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G31" s="6" t="inlineStr">
@@ -1624,7 +1596,11 @@
           <t>À tester</t>
         </is>
       </c>
-      <c r="H31" s="6" t="n"/>
+      <c r="H31" s="6" t="inlineStr">
+        <is>
+          <t>Sur STA, l'adresse déclarée chez Netatmo est celle du lien Staging (…vercel.app/api/objets, 19/10/2026) : la remplacer à la mise en prod, Netatmo n'accepte qu'une adresse ; description de l'application en français (19/10/2026).</t>
+        </is>
+      </c>
       <c r="I31" s="6" t="n"/>
     </row>
     <row r="32">
@@ -1633,27 +1609,27 @@
       </c>
       <c r="B32" s="5" t="inlineStr">
         <is>
-          <t>Robot Gardena SILENO — proposition</t>
+          <t>Automower — hauteur en cm</t>
         </is>
       </c>
       <c r="C32" s="4" t="inlineStr">
         <is>
-          <t>Aujourd'hui</t>
+          <t>Mes équipements, Aujourd'hui (carte du robot)</t>
         </is>
       </c>
       <c r="D32" s="4" t="inlineStr">
         <is>
-          <t>Jour de pluie / gel : valider « Mettre au repos jusqu'à demain matin », puis un jour sans contrainte : « Relancer son planning ».</t>
+          <t>Ouvrir la carte d'un Automower à réglage électrique (ex. 430X).</t>
         </is>
       </c>
       <c r="E32" s="4" t="inlineStr">
         <is>
-          <t>Le robot rentre et reste garé (app Gardena : garé jusqu'à nouvel ordre) ; la relance remet son planning. Rien n'est envoyé sans validation.</t>
+          <t>« Réglage actuel du robot : X cm (niveau N) » ; hauteur conseillée de la saison affichée au-dessus.</t>
         </is>
       </c>
       <c r="F32" s="4" t="inlineStr">
         <is>
-          <t>Compte avec SILENO</t>
+          <t>Compte avec Automower (testeur à trouver)</t>
         </is>
       </c>
       <c r="G32" s="6" t="inlineStr">
@@ -1670,27 +1646,27 @@
       </c>
       <c r="B33" s="5" t="inlineStr">
         <is>
-          <t>Robot Gardena SILENO — reprise du matin</t>
+          <t>Automower — proposition de hauteur</t>
         </is>
       </c>
       <c r="C33" s="4" t="inlineStr">
         <is>
-          <t>Tâche du matin (PROD)</t>
+          <t>Aujourd'hui (carte du robot)</t>
         </is>
       </c>
       <c r="D33" s="4" t="inlineStr">
         <is>
-          <t>Le lendemain d'un « repos jusqu'à demain matin », regarder le robot après 8 h.</t>
+          <t>Un jour où la tonte est possible, avec un robot réglé loin de la hauteur de la saison.</t>
         </is>
       </c>
       <c r="E33" s="4" t="inlineStr">
         <is>
-          <t>Planning relancé automatiquement (journal de la tâche : robotsRelances ≥ 1). Non testable sur STA (tâches planifiées en PROD seulement).</t>
+          <t>Proposition « 📏 Régler la coupe sur X cm » avec la raison (hauteur de la saison, réglage actuel, limite du robot) ; rien n'est envoyé sans clic.</t>
         </is>
       </c>
       <c r="F33" s="4" t="inlineStr">
         <is>
-          <t>Compte avec SILENO</t>
+          <t>Compte avec Automower</t>
         </is>
       </c>
       <c r="G33" s="6" t="inlineStr">
@@ -1707,27 +1683,27 @@
       </c>
       <c r="B34" s="5" t="inlineStr">
         <is>
-          <t>Robot Gardena SILENO — déconnexion</t>
+          <t>Automower — réglage envoyé</t>
         </is>
       </c>
       <c r="C34" s="4" t="inlineStr">
         <is>
-          <t>Mes équipements</t>
+          <t>Aujourd'hui → app Automower Connect</t>
         </is>
       </c>
       <c r="D34" s="4" t="inlineStr">
         <is>
-          <t>Avec arrosage ET robot Gardena : déconnecter le robot, puis vérifier l'arrosage.</t>
+          <t>Valider la proposition, puis regarder la hauteur dans l'app Automower Connect.</t>
         </is>
       </c>
       <c r="E34" s="4" t="inlineStr">
         <is>
-          <t>L'arrosage reste connecté et fonctionne (la connexion commune n'est révoquée qu'avec le dernier équipement Gardena).</t>
+          <t>Hauteur changée sur le robot ; la proposition disparaît au rafraîchissement.</t>
         </is>
       </c>
       <c r="F34" s="4" t="inlineStr">
         <is>
-          <t>Compte avec SILENO + arrosage Gardena</t>
+          <t>Compte avec Automower</t>
         </is>
       </c>
       <c r="G34" s="6" t="inlineStr">
@@ -1744,27 +1720,27 @@
       </c>
       <c r="B35" s="5" t="inlineStr">
         <is>
-          <t>Station Netatmo — connexion</t>
+          <t>Automower — priorités et modèles sans réglage</t>
         </is>
       </c>
       <c r="C35" s="4" t="inlineStr">
         <is>
-          <t>Mes équipements → Station météo</t>
+          <t>Aujourd'hui</t>
         </is>
       </c>
       <c r="D35" s="4" t="inlineStr">
         <is>
-          <t>« Connecter ma station Netatmo » avec un compte Netatmo qui a un module extérieur ou un pluviomètre.</t>
+          <t>Un jour de pluie ; puis un robot à réglage manuel (305, Mark II) ou un Gardena SILENO.</t>
         </is>
       </c>
       <c r="E35" s="4" t="inlineStr">
         <is>
-          <t>Retour sur Mes équipements avec « Station Netatmo connectée » ; carte avec température, pluie du jour et vent ; libellé « Netatmo ».</t>
+          <t>Pluie : proposition de repos, pas de hauteur ; réglage manuel ou Gardena : aucune proposition de hauteur.</t>
         </is>
       </c>
       <c r="F35" s="4" t="inlineStr">
         <is>
-          <t>Compte avec station Netatmo (testeur à trouver)</t>
+          <t>Compte avec Automower ou SILENO</t>
         </is>
       </c>
       <c r="G35" s="6" t="inlineStr">
@@ -1772,11 +1748,7 @@
           <t>À tester</t>
         </is>
       </c>
-      <c r="H35" s="6" t="inlineStr">
-        <is>
-          <t>Chaîne de connexion validée sur STA le 19/10/2026 par Jordan, sans station (« Aucune station météo trouvée sur ce compte Netatmo ») ; reste le test avec une vraie station.</t>
-        </is>
-      </c>
+      <c r="H35" s="6" t="n"/>
       <c r="I35" s="6" t="n"/>
     </row>
     <row r="36">
@@ -1785,27 +1757,27 @@
       </c>
       <c r="B36" s="5" t="inlineStr">
         <is>
-          <t>Station Netatmo — mesures du jardin</t>
+          <t>Robot Mammotion — connexion</t>
         </is>
       </c>
       <c r="C36" s="4" t="inlineStr">
         <is>
-          <t>Aujourd'hui, notifications, Bob</t>
+          <t>Mes équipements → Robot tondeuse</t>
         </is>
       </c>
       <c r="D36" s="4" t="inlineStr">
         <is>
-          <t>Un jour de pluie, ouvrir « Aujourd'hui » et poser une question à Bob sur l'arrosage.</t>
+          <t>Sur developer.mammotion.com, créer des identifiants (« Create Credentials ») avec un compte Mammotion qui a un LUBA 3 AWD (seul modèle entièrement pris en charge au 29/10/2026), les coller puis « Connecter mon robot Mammotion » ; recommencer avec un compte sans robot compatible.</t>
         </is>
       </c>
       <c r="E36" s="4" t="inlineStr">
         <is>
-          <t>La pluie mesurée par la station est prise en compte (arrosage, tonte) ; Bob cite la mesure de la station ; relevé de moins de 10 min.</t>
+          <t>Robot « ✓ connecté » avec son nom, son état et sa batterie ; compte sans robot compatible : message « Aucun robot sur ce compte Mammotion » ; faux identifiants : « Identifiants Mammotion refusés ».</t>
         </is>
       </c>
       <c r="F36" s="4" t="inlineStr">
         <is>
-          <t>Compte avec station Netatmo</t>
+          <t>Compte avec robot Mammotion</t>
         </is>
       </c>
       <c r="G36" s="6" t="inlineStr">
@@ -1813,7 +1785,11 @@
           <t>À tester</t>
         </is>
       </c>
-      <c r="H36" s="6" t="n"/>
+      <c r="H36" s="6" t="inlineStr">
+        <is>
+          <t>Sur STA le 17/10/2026. Avant la prod : autorisation écrite de Mammotion pour une app payante (réponse du 29/10/2026 : usage commercial soumis à leur autorisation écrite préalable, demandée) ; sans elle, Mammotion masqué en prod (liste des marques, Bob, confidentialité 6.3).</t>
+        </is>
+      </c>
       <c r="I36" s="6" t="n"/>
     </row>
     <row r="37">
@@ -1822,27 +1798,27 @@
       </c>
       <c r="B37" s="5" t="inlineStr">
         <is>
-          <t>Station Netatmo — connexion annulée</t>
+          <t>Robot Mammotion — propositions</t>
         </is>
       </c>
       <c r="C37" s="4" t="inlineStr">
         <is>
-          <t>Mes équipements</t>
+          <t>Aujourd'hui (carte du robot)</t>
         </is>
       </c>
       <c r="D37" s="4" t="inlineStr">
         <is>
-          <t>Cliquer « Connecter ma station Netatmo », puis refuser l'accès sur le site de Netatmo.</t>
+          <t>Un jour de pluie ou de gel pendant que le robot tond : valider « Le faire rentrer à sa base » ; un jour sans contre-indication avec le robot en pause : « Reprendre la tonte ».</t>
         </is>
       </c>
       <c r="E37" s="4" t="inlineStr">
         <is>
-          <t>Message « Connexion annulée : rien n'a été enregistré » (même chose pour Husqvarna et Gardena).</t>
+          <t>Le robot rentre à sa base, ou reprend la tonte ; hors saison ou pendant un semis, la raison rappelle de suspendre ses tâches programmées dans l'app Mammotion ; aucune proposition quand le robot est à l'arrêt.</t>
         </is>
       </c>
       <c r="F37" s="4" t="inlineStr">
         <is>
-          <t>Tout compte</t>
+          <t>Compte avec robot Mammotion</t>
         </is>
       </c>
       <c r="G37" s="6" t="inlineStr">
@@ -1850,7 +1826,11 @@
           <t>À tester</t>
         </is>
       </c>
-      <c r="H37" s="6" t="n"/>
+      <c r="H37" s="6" t="inlineStr">
+        <is>
+          <t>Sur STA le 17/10/2026.</t>
+        </is>
+      </c>
       <c r="I37" s="6" t="n"/>
     </row>
     <row r="38">
@@ -1859,27 +1839,27 @@
       </c>
       <c r="B38" s="5" t="inlineStr">
         <is>
-          <t>Station Netatmo — déconnexion</t>
+          <t>Station Davis — connexion et mesures</t>
         </is>
       </c>
       <c r="C38" s="4" t="inlineStr">
         <is>
-          <t>Mes équipements</t>
+          <t>Mes équipements → Station météo ; Aujourd'hui ; Bob</t>
         </is>
       </c>
       <c r="D38" s="4" t="inlineStr">
         <is>
-          <t>« Déconnecter la station ».</t>
+          <t>Sur weatherlink.com, « Generate v2 Key », coller l'API Key v2 et l'API Secret, « Trouver ma station Davis » puis la choisir ; un jour de pluie, ouvrir « Aujourd'hui » et demander à Bob s'il faut arroser.</t>
         </is>
       </c>
       <c r="E38" s="4" t="inlineStr">
         <is>
-          <t>La station disparaît ; « Aujourd'hui » repart sur les prévisions météo.</t>
+          <t>Température en °C, pluie du jour en mm, humidité et vent en km/h affichés ; l'arrosage et Bob tiennent compte de la pluie mesurée ; fausses clés : « Clé ou secret WeatherLink refusés ».</t>
         </is>
       </c>
       <c r="F38" s="4" t="inlineStr">
         <is>
-          <t>Compte avec station Netatmo</t>
+          <t>Compte avec station Davis (WeatherLink Live ou console)</t>
         </is>
       </c>
       <c r="G38" s="6" t="inlineStr">
@@ -1887,7 +1867,11 @@
           <t>À tester</t>
         </is>
       </c>
-      <c r="H38" s="6" t="n"/>
+      <c r="H38" s="6" t="inlineStr">
+        <is>
+          <t>Sur STA le 17/10/2026.</t>
+        </is>
+      </c>
       <c r="I38" s="6" t="n"/>
     </row>
     <row r="39">
@@ -1896,27 +1880,27 @@
       </c>
       <c r="B39" s="5" t="inlineStr">
         <is>
-          <t>Station Netatmo — réglages PROD</t>
+          <t>Équipements — textes et Bob</t>
         </is>
       </c>
       <c r="C39" s="4" t="inlineStr">
         <is>
-          <t>Application Netatmo (dev.netatmo.com) et Vercel</t>
+          <t>Politique de confidentialité (6.3) ; Bob</t>
         </is>
       </c>
       <c r="D39" s="4" t="inlineStr">
         <is>
-          <t>Vérifier l'adresse de retour déclarée dans l'application Netatmo et les variables Vercel.</t>
+          <t>Lire l'article 6.3 de la politique de confidentialité ; demander à Bob quelles marques l'app peut connecter.</t>
         </is>
       </c>
       <c r="E39" s="4" t="inlineStr">
         <is>
-          <t>Adresse de retour https://mongazon360.fr/api/objets ; NETATMO_CLIENT_ID et NETATMO_CLIENT_SECRET présentes en Production.</t>
+          <t>Netatmo, Ecowitt, Davis et Mammotion cités dans l'article 6.3, sans Weather Underground (date du 19 octobre) ; Bob cite Netatmo, Ecowitt, Davis, Husqvarna, Gardena, Mammotion et Rachio, sans autre marque.</t>
         </is>
       </c>
       <c r="F39" s="4" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Premium</t>
         </is>
       </c>
       <c r="G39" s="6" t="inlineStr">
@@ -1926,7 +1910,7 @@
       </c>
       <c r="H39" s="6" t="inlineStr">
         <is>
-          <t>Sur STA, l'adresse déclarée chez Netatmo est celle du lien Staging (…vercel.app/api/objets, 19/10/2026) : la remplacer à la mise en prod, Netatmo n'accepte qu'une adresse ; description de l'application en français (19/10/2026).</t>
+          <t>Sur STA le 17/10/2026 ; Weather Underground retiré le 19/10/2026.</t>
         </is>
       </c>
       <c r="I39" s="6" t="n"/>
@@ -1937,27 +1921,27 @@
       </c>
       <c r="B40" s="5" t="inlineStr">
         <is>
-          <t>Automower — hauteur en cm</t>
+          <t>Capteur de sol — sol humide</t>
         </is>
       </c>
       <c r="C40" s="4" t="inlineStr">
         <is>
-          <t>Mes équipements, Aujourd'hui (carte du robot)</t>
+          <t>Aujourd'hui ; notification du soir ; Bob</t>
         </is>
       </c>
       <c r="D40" s="4" t="inlineStr">
         <is>
-          <t>Ouvrir la carte d'un Automower à réglage électrique (ex. 430X).</t>
+          <t>Avec un capteur Ecowitt ou Gardena qui mesure au-dessus du seuil humide de son sol (ex. ≥ 32 % en limoneux), en saison d'arrosage : ouvrir « Aujourd'hui », attendre la notification du soir, demander à Bob s'il faut arroser.</t>
         </is>
       </c>
       <c r="E40" s="4" t="inlineStr">
         <is>
-          <t>« Réglage actuel du robot : X cm (niveau N) » ; hauteur conseillée de la saison affichée au-dessus.</t>
+          <t>Arrosage bloqué « Sol encore humide (X % mesurés) » ; notification « ✓ Pas d'arrosage demain matin » ; Bob dit qu'il est inutile d'arroser, avec le chiffre du capteur.</t>
         </is>
       </c>
       <c r="F40" s="4" t="inlineStr">
         <is>
-          <t>Compte avec Automower (testeur à trouver)</t>
+          <t>Compte avec capteur de sol</t>
         </is>
       </c>
       <c r="G40" s="6" t="inlineStr">
@@ -1965,7 +1949,11 @@
           <t>À tester</t>
         </is>
       </c>
-      <c r="H40" s="6" t="n"/>
+      <c r="H40" s="6" t="inlineStr">
+        <is>
+          <t>Sur STA le 17/10/2026 (règle validée par Jordan, base de connaissances mise à jour).</t>
+        </is>
+      </c>
       <c r="I40" s="6" t="n"/>
     </row>
     <row r="41">
@@ -1974,27 +1962,27 @@
       </c>
       <c r="B41" s="5" t="inlineStr">
         <is>
-          <t>Automower — proposition de hauteur</t>
+          <t>Capteur de sol — sol sec</t>
         </is>
       </c>
       <c r="C41" s="4" t="inlineStr">
         <is>
-          <t>Aujourd'hui (carte du robot)</t>
+          <t>Aujourd'hui ; notification du soir</t>
         </is>
       </c>
       <c r="D41" s="4" t="inlineStr">
         <is>
-          <t>Un jour où la tonte est possible, avec un robot réglé loin de la hauteur de la saison.</t>
+          <t>Capteur sous le seuil sec (ex. &lt; 25 % en limoneux), sans pluie du jour, un lendemain d'arrosage : ouvrir « Aujourd'hui ».</t>
         </is>
       </c>
       <c r="E41" s="4" t="inlineStr">
         <is>
-          <t>Proposition « 📏 Régler la coupe sur X cm » avec la raison (hauteur de la saison, réglage actuel, limite du robot) ; rien n'est envoyé sans clic.</t>
+          <t>Arrosage conseillé à la dose entière avec « Sol sec mesuré (X %) », sans attendre l'intervalle habituel ; notification du soir « Sol sec » ; avec 3 mm de pluie ou plus dans la journée : calcul habituel.</t>
         </is>
       </c>
       <c r="F41" s="4" t="inlineStr">
         <is>
-          <t>Compte avec Automower</t>
+          <t>Compte avec capteur de sol</t>
         </is>
       </c>
       <c r="G41" s="6" t="inlineStr">
@@ -2002,7 +1990,11 @@
           <t>À tester</t>
         </is>
       </c>
-      <c r="H41" s="6" t="n"/>
+      <c r="H41" s="6" t="inlineStr">
+        <is>
+          <t>Sur STA le 17/10/2026 (règle validée par Jordan, base de connaissances mise à jour).</t>
+        </is>
+      </c>
       <c r="I41" s="6" t="n"/>
     </row>
     <row r="42">
@@ -2011,27 +2003,27 @@
       </c>
       <c r="B42" s="5" t="inlineStr">
         <is>
-          <t>Automower — réglage envoyé</t>
+          <t>Capteur de sol — parcours et arrosage connecté</t>
         </is>
       </c>
       <c r="C42" s="4" t="inlineStr">
         <is>
-          <t>Aujourd'hui → app Automower Connect</t>
+          <t>Parcours en cours ; carte de l'arrosage connecté</t>
         </is>
       </c>
       <c r="D42" s="4" t="inlineStr">
         <is>
-          <t>Valider la proposition, puis regarder la hauteur dans l'app Automower Connect.</t>
+          <t>Pendant un parcours de semis (avant consolidation), avec un sol humide ; puis, hors parcours, avec un arrosage Gardena ou Rachio et un sol humide.</t>
         </is>
       </c>
       <c r="E42" s="4" t="inlineStr">
         <is>
-          <t>Hauteur changée sur le robot ; la proposition disparaît au rafraîchissement.</t>
+          <t>Parcours : l'arrosage de germination n'est pas modifié par le capteur. Arrosage connecté : « Sol encore humide : inutile que les programmes arrosent » et bouton de suspension ; pas de reprise proposée tant que le sol reste humide.</t>
         </is>
       </c>
       <c r="F42" s="4" t="inlineStr">
         <is>
-          <t>Compte avec Automower</t>
+          <t>Compte avec capteur de sol et arrosage connecté</t>
         </is>
       </c>
       <c r="G42" s="6" t="inlineStr">
@@ -2039,7 +2031,11 @@
           <t>À tester</t>
         </is>
       </c>
-      <c r="H42" s="6" t="n"/>
+      <c r="H42" s="6" t="inlineStr">
+        <is>
+          <t>Sur STA le 17/10/2026 (règle validée par Jordan, base de connaissances mise à jour).</t>
+        </is>
+      </c>
       <c r="I42" s="6" t="n"/>
     </row>
     <row r="43">
@@ -2048,27 +2044,27 @@
       </c>
       <c r="B43" s="5" t="inlineStr">
         <is>
-          <t>Automower — priorités et modèles sans réglage</t>
+          <t>Capteur Gardena — lecture et température du sol</t>
         </is>
       </c>
       <c r="C43" s="4" t="inlineStr">
         <is>
-          <t>Aujourd'hui</t>
+          <t>Mes équipements, Aujourd'hui (carte de l'arrosage) ; Parcours</t>
         </is>
       </c>
       <c r="D43" s="4" t="inlineStr">
         <is>
-          <t>Un jour de pluie ; puis un robot à réglage manuel (305, Mark II) ou un Gardena SILENO.</t>
+          <t>Compte Gardena avec un smart Sensor : ouvrir la carte de l'arrosage ; lancer une analyse de fenêtre de semis pour aujourd'hui.</t>
         </is>
       </c>
       <c r="E43" s="4" t="inlineStr">
         <is>
-          <t>Pluie : proposition de repos, pas de hauteur ; réglage manuel ou Gardena : aucune proposition de hauteur.</t>
+          <t>La carte affiche « Capteur : sol à X % d'humidité, Y °C » et l'heure du relevé ; la fenêtre de semis du jour utilise la température mesurée (« votre sol est … (Y °C) » si hors fourchette).</t>
         </is>
       </c>
       <c r="F43" s="4" t="inlineStr">
         <is>
-          <t>Compte avec Automower ou SILENO</t>
+          <t>Compte Gardena avec smart Sensor</t>
         </is>
       </c>
       <c r="G43" s="6" t="inlineStr">
@@ -2076,7 +2072,11 @@
           <t>À tester</t>
         </is>
       </c>
-      <c r="H43" s="6" t="n"/>
+      <c r="H43" s="6" t="inlineStr">
+        <is>
+          <t>Sur STA le 17/10/2026 (règle validée par Jordan, base de connaissances mise à jour).</t>
+        </is>
+      </c>
       <c r="I43" s="6" t="n"/>
     </row>
     <row r="44">
@@ -2085,27 +2085,27 @@
       </c>
       <c r="B44" s="5" t="inlineStr">
         <is>
-          <t>Robot Mammotion — connexion</t>
+          <t>Station Weather Underground — retirée</t>
         </is>
       </c>
       <c r="C44" s="4" t="inlineStr">
         <is>
-          <t>Mes équipements → Robot tondeuse</t>
+          <t>Mes équipements → Station météo</t>
         </is>
       </c>
       <c r="D44" s="4" t="inlineStr">
         <is>
-          <t>Sur developer.mammotion.com, créer des identifiants (« Create Credentials ») avec un compte Mammotion qui a un LUBA 3 AWD (seul modèle entièrement pris en charge au 29/10/2026), les coller puis « Connecter mon robot Mammotion » ; recommencer avec un compte sans robot compatible.</t>
+          <t>Ouvrir la liste des marques de station, puis choisir « Autre marque ».</t>
         </is>
       </c>
       <c r="E44" s="4" t="inlineStr">
         <is>
-          <t>Robot « ✓ connecté » avec son nom, son état et sa batterie ; compte sans robot compatible : message « Aucun robot sur ce compte Mammotion » ; faux identifiants : « Identifiants Mammotion refusés ».</t>
+          <t>Liste : Netatmo, Ecowitt, Davis, Autre marque, sans Weather Underground ; « Autre marque » renvoie au formulaire « Ton équipement n'est pas dans la liste ? ».</t>
         </is>
       </c>
       <c r="F44" s="4" t="inlineStr">
         <is>
-          <t>Compte avec robot Mammotion</t>
+          <t>Premium</t>
         </is>
       </c>
       <c r="G44" s="6" t="inlineStr">
@@ -2115,7 +2115,7 @@
       </c>
       <c r="H44" s="6" t="inlineStr">
         <is>
-          <t>Sur STA le 17/10/2026. Avant la prod : autorisation écrite de Mammotion pour une app payante (réponse du 29/10/2026 : usage commercial soumis à leur autorisation écrite préalable, demandée) ; sans elle, Mammotion masqué en prod (liste des marques, Bob, confidentialité 6.3).</t>
+          <t>Connexion Weather Underground développée sur STA le 18/10/2026 puis retirée le 19/10/2026 (décision de Jordan) : les conditions de The Weather Company (section 18) réservent la clé gratuite à un usage non commercial, l'usage commercial est payant.</t>
         </is>
       </c>
       <c r="I44" s="6" t="n"/>
@@ -2126,27 +2126,27 @@
       </c>
       <c r="B45" s="5" t="inlineStr">
         <is>
-          <t>Robot Mammotion — propositions</t>
+          <t>Équipement non listé — envoi</t>
         </is>
       </c>
       <c r="C45" s="4" t="inlineStr">
         <is>
-          <t>Aujourd'hui (carte du robot)</t>
+          <t>Mes équipements (en bas de page)</t>
         </is>
       </c>
       <c r="D45" s="4" t="inlineStr">
         <is>
-          <t>Un jour de pluie ou de gel pendant que le robot tond : valider « Le faire rentrer à sa base » ; un jour sans contre-indication avec le robot en pause : « Reprendre la tonte ».</t>
+          <t>Avec un compte Premium, dans « Ton équipement n'est pas dans la liste ? » : choisir un type, saisir une marque (et un modèle), toucher « Envoyer » ; puis ouvrir Mes équipements avec un compte gratuit.</t>
         </is>
       </c>
       <c r="E45" s="4" t="inlineStr">
         <is>
-          <t>Le robot rentre à sa base, ou reprend la tonte ; hors saison ou pendant un semis, la raison rappelle de suspendre ses tâches programmées dans l'app Mammotion ; aucune proposition quand le robot est à l'arrêt.</t>
+          <t>« ✅ Merci, c'est noté » ; bouton grisé sans marque ; rien de personnel enregistré (demande anonyme) ; compte gratuit : formulaire absent.</t>
         </is>
       </c>
       <c r="F45" s="4" t="inlineStr">
         <is>
-          <t>Compte avec robot Mammotion</t>
+          <t>Premium, gratuit</t>
         </is>
       </c>
       <c r="G45" s="6" t="inlineStr">
@@ -2156,7 +2156,7 @@
       </c>
       <c r="H45" s="6" t="inlineStr">
         <is>
-          <t>Sur STA le 17/10/2026.</t>
+          <t>Sur STA le 18/10/2026. Réservé aux comptes Premium depuis le 29/10/2026 (décision de Jordan). Vérifié par Jordan sur STA le 30/10 : formulaire absent pour un compte gratuit.</t>
         </is>
       </c>
       <c r="I45" s="6" t="n"/>
@@ -2167,27 +2167,27 @@
       </c>
       <c r="B46" s="5" t="inlineStr">
         <is>
-          <t>Station Davis — connexion et mesures</t>
+          <t>Pilotage — équipements demandés</t>
         </is>
       </c>
       <c r="C46" s="4" t="inlineStr">
         <is>
-          <t>Mes équipements → Station météo ; Aujourd'hui ; Bob</t>
+          <t>Pilotage → Activité (carte « Équipements demandés »)</t>
         </is>
       </c>
       <c r="D46" s="4" t="inlineStr">
         <is>
-          <t>Sur weatherlink.com, « Generate v2 Key », coller l'API Key v2 et l'API Secret, « Trouver ma station Davis » puis la choisir ; un jour de pluie, ouvrir « Aujourd'hui » et demander à Bob s'il faut arroser.</t>
+          <t>Après une ou deux demandes de test : ouvrir Pilotage → Activité.</t>
         </is>
       </c>
       <c r="E46" s="4" t="inlineStr">
         <is>
-          <t>Température en °C, pluie du jour en mm, humidité et vent en km/h affichés ; l'arrosage et Bob tiennent compte de la pluie mesurée ; fausses clés : « Clé ou secret WeatherLink refusés ».</t>
+          <t>Demandes regroupées par type et marque (casse ignorée), du plus demandé au moins demandé, avec les modèles cités.</t>
         </is>
       </c>
       <c r="F46" s="4" t="inlineStr">
         <is>
-          <t>Compte avec station Davis (WeatherLink Live ou console)</t>
+          <t>Admin</t>
         </is>
       </c>
       <c r="G46" s="6" t="inlineStr">
@@ -2197,7 +2197,7 @@
       </c>
       <c r="H46" s="6" t="inlineStr">
         <is>
-          <t>Sur STA le 17/10/2026.</t>
+          <t>Sur STA le 18/10/2026.</t>
         </is>
       </c>
       <c r="I46" s="6" t="n"/>
@@ -2208,22 +2208,22 @@
       </c>
       <c r="B47" s="5" t="inlineStr">
         <is>
-          <t>Équipements — textes et Bob</t>
+          <t>Diagnostic — niveau de confiance</t>
         </is>
       </c>
       <c r="C47" s="4" t="inlineStr">
         <is>
-          <t>Politique de confidentialité (6.3) ; Bob</t>
+          <t>Diagnostic (résultat et historique)</t>
         </is>
       </c>
       <c r="D47" s="4" t="inlineStr">
         <is>
-          <t>Lire l'article 6.3 de la politique de confidentialité ; demander à Bob quelles marques l'app peut connecter.</t>
+          <t>Faire un diagnostic avec une photo nette, en plein jour, à 1 m du sol ; puis rouvrir ce diagnostic dans l'historique.</t>
         </is>
       </c>
       <c r="E47" s="4" t="inlineStr">
         <is>
-          <t>Netatmo, Ecowitt, Davis et Mammotion cités dans l'article 6.3, sans Weather Underground (date du 19 octobre) ; Bob cite Netatmo, Ecowitt, Davis, Husqvarna, Gardena, Mammotion et Rachio, sans autre marque.</t>
+          <t>Sous le score : « 🎯 Confiance élevée, moyenne ou faible » avec une phrase d'explication, et « 👀 Ce que Bob a vu » (2 à 4 éléments réellement visibles sur la photo) ; mêmes informations dans l'historique. Confiance faible : conseil pour reprendre la photo et bouton « Reprendre une photo ».</t>
         </is>
       </c>
       <c r="F47" s="4" t="inlineStr">
@@ -2238,7 +2238,7 @@
       </c>
       <c r="H47" s="6" t="inlineStr">
         <is>
-          <t>Sur STA le 17/10/2026 ; Weather Underground retiré le 19/10/2026.</t>
+          <t>Sur STA le 18/10/2026.</t>
         </is>
       </c>
       <c r="I47" s="6" t="n"/>
@@ -2249,27 +2249,27 @@
       </c>
       <c r="B48" s="5" t="inlineStr">
         <is>
-          <t>Capteur de sol — sol humide</t>
+          <t>Diagnostic — photo à reprendre</t>
         </is>
       </c>
       <c r="C48" s="4" t="inlineStr">
         <is>
-          <t>Aujourd'hui ; notification du soir ; Bob</t>
+          <t>Diagnostic</t>
         </is>
       </c>
       <c r="D48" s="4" t="inlineStr">
         <is>
-          <t>Avec un capteur Ecowitt ou Gardena qui mesure au-dessus du seuil humide de son sol (ex. ≥ 32 % en limoneux), en saison d'arrosage : ouvrir « Aujourd'hui », attendre la notification du soir, demander à Bob s'il faut arroser.</t>
+          <t>Lancer un diagnostic avec une photo floue, très sombre ou sans gazon (ex. un mur).</t>
         </is>
       </c>
       <c r="E48" s="4" t="inlineStr">
         <is>
-          <t>Arrosage bloqué « Sol encore humide (X % mesurés) » ; notification « ✓ Pas d'arrosage demain matin » ; Bob dit qu'il est inutile d'arroser, avec le chiffre du capteur.</t>
+          <t>Écran « 📷 Photo à reprendre » : explication de Bob, conseil pour la reprendre et boutons photo ; aucun score, rien dans l'historique ni dans Bob.</t>
         </is>
       </c>
       <c r="F48" s="4" t="inlineStr">
         <is>
-          <t>Compte avec capteur de sol</t>
+          <t>Premium</t>
         </is>
       </c>
       <c r="G48" s="6" t="inlineStr">
@@ -2279,7 +2279,7 @@
       </c>
       <c r="H48" s="6" t="inlineStr">
         <is>
-          <t>Sur STA le 17/10/2026 (règle validée par Jordan, base de connaissances mise à jour).</t>
+          <t>Sur STA le 18/10/2026.</t>
         </is>
       </c>
       <c r="I48" s="6" t="n"/>
@@ -2290,27 +2290,27 @@
       </c>
       <c r="B49" s="5" t="inlineStr">
         <is>
-          <t>Capteur de sol — sol sec</t>
+          <t>Essai sans compte — photo à reprendre</t>
         </is>
       </c>
       <c r="C49" s="4" t="inlineStr">
         <is>
-          <t>Aujourd'hui ; notification du soir</t>
+          <t>Essai du diagnostic (sans compte)</t>
         </is>
       </c>
       <c r="D49" s="4" t="inlineStr">
         <is>
-          <t>Capteur sous le seuil sec (ex. &lt; 25 % en limoneux), sans pluie du jour, un lendemain d'arrosage : ouvrir « Aujourd'hui ».</t>
+          <t>Non connecté : essai du diagnostic avec une photo sans gazon, puis avec une vraie photo de pelouse.</t>
         </is>
       </c>
       <c r="E49" s="4" t="inlineStr">
         <is>
-          <t>Arrosage conseillé à la dose entière avec « Sol sec mesuré (X %) », sans attendre l'intervalle habituel ; notification du soir « Sol sec » ; avec 3 mm de pluie ou plus dans la journée : calcul habituel.</t>
+          <t>1re photo : « Bob ne peut pas conclure avec cette photo » et « Ton diagnostic gratuit n'est pas utilisé » ; 2e photo : score, confiance et ce que Bob a vu, puis l'analyse complète à débloquer comme avant.</t>
         </is>
       </c>
       <c r="F49" s="4" t="inlineStr">
         <is>
-          <t>Compte avec capteur de sol</t>
+          <t>Non connecté</t>
         </is>
       </c>
       <c r="G49" s="6" t="inlineStr">
@@ -2320,7 +2320,7 @@
       </c>
       <c r="H49" s="6" t="inlineStr">
         <is>
-          <t>Sur STA le 17/10/2026 (règle validée par Jordan, base de connaissances mise à jour).</t>
+          <t>Sur STA le 18/10/2026.</t>
         </is>
       </c>
       <c r="I49" s="6" t="n"/>
@@ -2331,27 +2331,27 @@
       </c>
       <c r="B50" s="5" t="inlineStr">
         <is>
-          <t>Capteur de sol — parcours et arrosage connecté</t>
+          <t>Diagnostic de suivi — travaux indiqués</t>
         </is>
       </c>
       <c r="C50" s="4" t="inlineStr">
         <is>
-          <t>Parcours en cours ; carte de l'arrosage connecté</t>
+          <t>Diagnostic (accueil)</t>
         </is>
       </c>
       <c r="D50" s="4" t="inlineStr">
         <is>
-          <t>Pendant un parcours de semis (avant consolidation), avec un sol humide ; puis, hors parcours, avec un arrosage Gardena ou Rachio et un sol humide.</t>
+          <t>Compte Premium (pas en essai) : faire un diagnostic, puis sur l'accueil de l'onglet Diagnostic, carte « 📝 Travaux faits après ton diagnostic du … ? » : choisir Regarnissage (plusieurs choix possibles), garder la date du jour, Enregistrer ; puis Modifier, et tout décocher pour effacer.</t>
         </is>
       </c>
       <c r="E50" s="4" t="inlineStr">
         <is>
-          <t>Parcours : l'arrosage de germination n'est pas modifié par le capteur. Arrosage connecté : « Sol encore humide : inutile que les programmes arrosent » et bouton de suspension ; pas de reprise proposée tant que le sol reste humide.</t>
+          <t>Carte « 📝 Travaux notés » : « Ton regarnissage du … : Bob te proposera ici une photo de suivi du même endroit du … au … » (J+30 à J+37 ; désherbage : J+21 à J+28) ; date des travaux entre le jour du diagnostic et 45 jours après, jamais dans le futur ; rien dans « Aujourd'hui », sur l'accueil ni en notification.</t>
         </is>
       </c>
       <c r="F50" s="4" t="inlineStr">
         <is>
-          <t>Compte avec capteur de sol et arrosage connecté</t>
+          <t>Premium</t>
         </is>
       </c>
       <c r="G50" s="6" t="inlineStr">
@@ -2361,7 +2361,7 @@
       </c>
       <c r="H50" s="6" t="inlineStr">
         <is>
-          <t>Sur STA le 17/10/2026 (règle validée par Jordan, base de connaissances mise à jour).</t>
+          <t>Sur STA le 19/10/2026 (cadrage de Jordan du 18/10 : tout sur la page Diagnostic). Délais : base de connaissances, « Règles complémentaires » n° 18 (regarnissage, scarification et anti-mousse 30 j, désherbage 21 j).</t>
         </is>
       </c>
       <c r="I50" s="6" t="n"/>
@@ -2372,27 +2372,27 @@
       </c>
       <c r="B51" s="5" t="inlineStr">
         <is>
-          <t>Capteur Gardena — lecture et température du sol</t>
+          <t>Diagnostic de suivi — photo de suivi et avant / après</t>
         </is>
       </c>
       <c r="C51" s="4" t="inlineStr">
         <is>
-          <t>Mes équipements, Aujourd'hui (carte de l'arrosage) ; Parcours</t>
+          <t>Diagnostic (accueil et résultat)</t>
         </is>
       </c>
       <c r="D51" s="4" t="inlineStr">
         <is>
-          <t>Compte Gardena avec un smart Sensor : ouvrir la carte de l'arrosage ; lancer une analyse de fenêtre de semis pour aujourd'hui.</t>
+          <t>Au bout du délai (ou en antidatant le diagnostic et la date des travaux dans la base de STA), ouvrir l'onglet Diagnostic, puis faire le diagnostic du même endroit.</t>
         </is>
       </c>
       <c r="E51" s="4" t="inlineStr">
         <is>
-          <t>La carte affiche « Capteur : sol à X % d'humidité, Y °C » et l'heure du relevé ; la fenêtre de semis du jour utilise la température mesurée (« votre sol est … (Y °C) » si hors fourchette).</t>
+          <t>Carte « 📸 C'est le moment du diagnostic de suivi » (photo d'avant, date des travaux, « a 30 jours », score d'avant) pendant 7 jours, plus après la nouvelle photo ; sur le résultat, carte « 📈 Depuis ton regarnissage du … » : photos avant / aujourd'hui avec leurs scores, écart en points (vert si +5 ou plus, rouge si -5 ou moins), problèmes réglés, encore là ou nouveaux.</t>
         </is>
       </c>
       <c r="F51" s="4" t="inlineStr">
         <is>
-          <t>Compte Gardena avec smart Sensor</t>
+          <t>Premium</t>
         </is>
       </c>
       <c r="G51" s="6" t="inlineStr">
@@ -2402,7 +2402,7 @@
       </c>
       <c r="H51" s="6" t="inlineStr">
         <is>
-          <t>Sur STA le 17/10/2026 (règle validée par Jordan, base de connaissances mise à jour).</t>
+          <t>Sur STA le 18/10/2026 ; travaux indiqués sur la page Diagnostic depuis le 19/10/2026.</t>
         </is>
       </c>
       <c r="I51" s="6" t="n"/>
@@ -2413,27 +2413,27 @@
       </c>
       <c r="B52" s="5" t="inlineStr">
         <is>
-          <t>Station Weather Underground — retirée</t>
+          <t>Diagnostic de suivi — essai de 7 jours</t>
         </is>
       </c>
       <c r="C52" s="4" t="inlineStr">
         <is>
-          <t>Mes équipements → Station météo</t>
+          <t>Diagnostic (accueil)</t>
         </is>
       </c>
       <c r="D52" s="4" t="inlineStr">
         <is>
-          <t>Ouvrir la liste des marques de station, puis choisir « Autre marque ».</t>
+          <t>Compte créé il y a moins de 7 jours, sans abonnement (essai Premium) : faire un diagnostic, puis revenir sur l'accueil de l'onglet Diagnostic.</t>
         </is>
       </c>
       <c r="E52" s="4" t="inlineStr">
         <is>
-          <t>Liste : Netatmo, Ecowitt, Davis, Autre marque, sans Weather Underground ; « Autre marque » renvoie au formulaire « Ton équipement n'est pas dans la liste ? ».</t>
+          <t>Aucune carte des travaux ni de diagnostic de suivi (la photo de suivi tomberait après la fin de l'essai) ; le diagnostic fonctionne normalement.</t>
         </is>
       </c>
       <c r="F52" s="4" t="inlineStr">
         <is>
-          <t>Premium</t>
+          <t>Compte en essai</t>
         </is>
       </c>
       <c r="G52" s="6" t="inlineStr">
@@ -2443,7 +2443,7 @@
       </c>
       <c r="H52" s="6" t="inlineStr">
         <is>
-          <t>Connexion Weather Underground développée sur STA le 18/10/2026 puis retirée le 19/10/2026 (décision de Jordan) : les conditions de The Weather Company (section 18) réservent la clé gratuite à un usage non commercial, l'usage commercial est payant.</t>
+          <t>Décision de Jordan du 18/10/2026.</t>
         </is>
       </c>
       <c r="I52" s="6" t="n"/>
@@ -2454,27 +2454,27 @@
       </c>
       <c r="B53" s="5" t="inlineStr">
         <is>
-          <t>Équipement non listé — envoi</t>
+          <t>Pilotage — comptes de test exclus</t>
         </is>
       </c>
       <c r="C53" s="4" t="inlineStr">
         <is>
-          <t>Mes équipements (en bas de page)</t>
+          <t>Pilotage → Activité</t>
         </is>
       </c>
       <c r="D53" s="4" t="inlineStr">
         <is>
-          <t>Avec un compte Premium, dans « Ton équipement n'est pas dans la liste ? » : choisir un type, saisir une marque (et un modèle), toucher « Envoyer » ; puis ouvrir Mes équipements avec un compte gratuit.</t>
+          <t>Créer un compte avec une adresse jordankrebs1+essai@gmail.com (ou marquer un compte {"compteTest": true} dans Clerk : Users → le compte → Metadata → Public), l'utiliser un jour, puis ouvrir Pilotage.</t>
         </is>
       </c>
       <c r="E53" s="4" t="inlineStr">
         <is>
-          <t>« ✅ Merci, c'est noté » ; bouton grisé sans marque ; rien de personnel enregistré (demande anonyme) ; compte gratuit : formulaire absent.</t>
+          <t>Le compte n'est compté ni dans les inscrits, ni dans les actifs, la rétention, les sources ou la carte ; une adresse « + » d'un vrai utilisateur (autre que l'admin) reste comptée.</t>
         </is>
       </c>
       <c r="F53" s="4" t="inlineStr">
         <is>
-          <t>Premium, gratuit</t>
+          <t>Admin</t>
         </is>
       </c>
       <c r="G53" s="6" t="inlineStr">
@@ -2484,7 +2484,7 @@
       </c>
       <c r="H53" s="6" t="inlineStr">
         <is>
-          <t>Sur STA le 18/10/2026. Réservé aux comptes Premium depuis le 29/10/2026 (décision de Jordan). Vérifié par Jordan sur STA le 30/10 : formulaire absent pour un compte gratuit.</t>
+          <t>Sur STA le 18/10/2026 (écarts relevés le 08/10).</t>
         </is>
       </c>
       <c r="I53" s="6" t="n"/>
@@ -2495,22 +2495,22 @@
       </c>
       <c r="B54" s="5" t="inlineStr">
         <is>
-          <t>Pilotage — équipements demandés</t>
+          <t>Pilotage — offre annuelle à 12,99 €</t>
         </is>
       </c>
       <c r="C54" s="4" t="inlineStr">
         <is>
-          <t>Pilotage → Activité (carte « Équipements demandés »)</t>
+          <t>Pilotage → Finances (MRR, ARR, Produits et charges)</t>
         </is>
       </c>
       <c r="D54" s="4" t="inlineStr">
         <is>
-          <t>Après une ou deux demandes de test : ouvrir Pilotage → Activité.</t>
+          <t>Avec un abonné annuel pris pendant l'offre saisonnière (à partir du 1/11) : ouvrir Finances.</t>
         </is>
       </c>
       <c r="E54" s="4" t="inlineStr">
         <is>
-          <t>Demandes regroupées par type et marque (casse ignorée), du plus demandé au moins demandé, avec les modèles cités.</t>
+          <t>L'abonné compte pour 12,99 €/an la 1re année (MRR, ARR et Produits et charges) ; ligne « Abonnements annuels » : « dont 1 à 12,99 € la 1re année ». Les autres annuels restent à 39,99 €.</t>
         </is>
       </c>
       <c r="F54" s="4" t="inlineStr">
@@ -2525,7 +2525,7 @@
       </c>
       <c r="H54" s="6" t="inlineStr">
         <is>
-          <t>Sur STA le 18/10/2026.</t>
+          <t>Sur STA le 18/10/2026. Testable au premier abonné de l'offre.</t>
         </is>
       </c>
       <c r="I54" s="6" t="n"/>
@@ -2536,37 +2536,37 @@
       </c>
       <c r="B55" s="5" t="inlineStr">
         <is>
-          <t>Diagnostic — niveau de confiance</t>
+          <t>Pilotage — jours à l'heure de Paris</t>
         </is>
       </c>
       <c r="C55" s="4" t="inlineStr">
         <is>
-          <t>Diagnostic (résultat et historique)</t>
+          <t>Pilotage → Activité</t>
         </is>
       </c>
       <c r="D55" s="4" t="inlineStr">
         <is>
-          <t>Faire un diagnostic avec une photo nette, en plein jour, à 1 m du sol ; puis rouvrir ce diagnostic dans l'historique.</t>
+          <t>Après une inscription ou une visite entre minuit et 2 h (heure de Paris) : regarder « Nouveaux aujourd'hui », le graphique sur 30 jours, les mois et « Visiteurs site (auj.) ».</t>
         </is>
       </c>
       <c r="E55" s="4" t="inlineStr">
         <is>
-          <t>Sous le score : « 🎯 Confiance élevée, moyenne ou faible » avec une phrase d'explication, et « 👀 Ce que Bob a vu » (2 à 4 éléments réellement visibles sur la photo) ; mêmes informations dans l'historique. Confiance faible : conseil pour reprendre la photo et bouton « Reprendre une photo ».</t>
+          <t>L'inscription et la visite comptent pour le jour même, pas pour la veille.</t>
         </is>
       </c>
       <c r="F55" s="4" t="inlineStr">
         <is>
-          <t>Premium</t>
+          <t>Admin</t>
         </is>
       </c>
       <c r="G55" s="6" t="inlineStr">
         <is>
-          <t>À tester</t>
+          <t>Non testable</t>
         </is>
       </c>
       <c r="H55" s="6" t="inlineStr">
         <is>
-          <t>Sur STA le 18/10/2026.</t>
+          <t>Sur STA le 18/10/2026 ; vérifié par un test automatique, à constater au premier cas réel.</t>
         </is>
       </c>
       <c r="I55" s="6" t="n"/>
@@ -2577,27 +2577,27 @@
       </c>
       <c r="B56" s="5" t="inlineStr">
         <is>
-          <t>Diagnostic — photo à reprendre</t>
+          <t>Pilotage — carte des inscrits</t>
         </is>
       </c>
       <c r="C56" s="4" t="inlineStr">
         <is>
-          <t>Diagnostic</t>
+          <t>Pilotage → Activité (carte)</t>
         </is>
       </c>
       <c r="D56" s="4" t="inlineStr">
         <is>
-          <t>Lancer un diagnostic avec une photo floue, très sombre ou sans gazon (ex. un mur).</t>
+          <t>Ouvrir la carte des inscrits.</t>
         </is>
       </c>
       <c r="E56" s="4" t="inlineStr">
         <is>
-          <t>Écran « 📷 Photo à reprendre » : explication de Bob, conseil pour la reprendre et boutons photo ; aucun score, rien dans l'historique ni dans Bob.</t>
+          <t>La ville de l'admin et celles des comptes de test ne sont plus comptées (sauf vrai inscrit dans la même ville).</t>
         </is>
       </c>
       <c r="F56" s="4" t="inlineStr">
         <is>
-          <t>Premium</t>
+          <t>Admin</t>
         </is>
       </c>
       <c r="G56" s="6" t="inlineStr">
@@ -2618,27 +2618,27 @@
       </c>
       <c r="B57" s="5" t="inlineStr">
         <is>
-          <t>Essai sans compte — photo à reprendre</t>
+          <t>Pilotage — emails envoyés</t>
         </is>
       </c>
       <c r="C57" s="4" t="inlineStr">
         <is>
-          <t>Essai du diagnostic (sans compte)</t>
+          <t>Pilotage → Activité (notifications)</t>
         </is>
       </c>
       <c r="D57" s="4" t="inlineStr">
         <is>
-          <t>Non connecté : essai du diagnostic avec une photo sans gazon, puis avec une vraie photo de pelouse.</t>
+          <t>Lire la ligne sous « Notifications ».</t>
         </is>
       </c>
       <c r="E57" s="4" t="inlineStr">
         <is>
-          <t>1re photo : « Bob ne peut pas conclure avec cette photo » et « Ton diagnostic gratuit n'est pas utilisé » ; 2e photo : score, confiance et ce que Bob a vu, puis l'analyse complète à débloquer comme avant.</t>
+          <t>« N notifications · N ouvertes · N conseils par email · N emails de démarrage et relances » : les emails de démarrage et de relance ne sont plus comptés comme conseils.</t>
         </is>
       </c>
       <c r="F57" s="4" t="inlineStr">
         <is>
-          <t>Non connecté</t>
+          <t>Admin</t>
         </is>
       </c>
       <c r="G57" s="6" t="inlineStr">
@@ -2659,27 +2659,27 @@
       </c>
       <c r="B58" s="5" t="inlineStr">
         <is>
-          <t>Diagnostic de suivi — travaux indiqués</t>
+          <t>Base de données — vue dau_by_day</t>
         </is>
       </c>
       <c r="C58" s="4" t="inlineStr">
         <is>
-          <t>Diagnostic (accueil)</t>
+          <t>Supabase STA et PROD</t>
         </is>
       </c>
       <c r="D58" s="4" t="inlineStr">
         <is>
-          <t>Compte Premium (pas en essai) : faire un diagnostic, puis sur l'accueil de l'onglet Diagnostic, carte « 📝 Travaux faits après ton diagnostic du … ? » : choisir Regarnissage (plusieurs choix possibles), garder la date du jour, Enregistrer ; puis Modifier, et tout décocher pour effacer.</t>
+          <t>Après la mise en prod : vérifier que plus rien n'utilise la vue dau_by_day (les actifs viennent de daily_active_users), puis la supprimer sur les deux projets.</t>
         </is>
       </c>
       <c r="E58" s="4" t="inlineStr">
         <is>
-          <t>Carte « 📝 Travaux notés » : « Ton regarnissage du … : Bob te proposera ici une photo de suivi du même endroit du … au … » (J+30 à J+37 ; désherbage : J+21 à J+28) ; date des travaux entre le jour du diagnostic et 45 jours après, jamais dans le futur ; rien dans « Aujourd'hui », sur l'accueil ni en notification.</t>
+          <t>Vue supprimée ; Pilotage → Activité affiche toujours les actifs par jour.</t>
         </is>
       </c>
       <c r="F58" s="4" t="inlineStr">
         <is>
-          <t>Premium</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G58" s="6" t="inlineStr">
@@ -2689,7 +2689,7 @@
       </c>
       <c r="H58" s="6" t="inlineStr">
         <is>
-          <t>Sur STA le 19/10/2026 (cadrage de Jordan du 18/10 : tout sur la page Diagnostic). Délais : base de connaissances, « Règles complémentaires » n° 18 (regarnissage, scarification et anti-mousse 30 j, désherbage 21 j).</t>
+          <t>Les actifs par jour sont calculés depuis le 18/10/2026 (STA) à partir des jours d'utilisation, pour exclure les comptes de test.</t>
         </is>
       </c>
       <c r="I58" s="6" t="n"/>
@@ -2700,27 +2700,27 @@
       </c>
       <c r="B59" s="5" t="inlineStr">
         <is>
-          <t>Diagnostic de suivi — photo de suivi et avant / après</t>
+          <t>Notifications — plus de demande à l'inscription</t>
         </is>
       </c>
       <c r="C59" s="4" t="inlineStr">
         <is>
-          <t>Diagnostic (accueil et résultat)</t>
+          <t>Inscription (consentements)</t>
         </is>
       </c>
       <c r="D59" s="4" t="inlineStr">
         <is>
-          <t>Au bout du délai (ou en antidatant le diagnostic et la date des travaux dans la base de STA), ouvrir l'onglet Diagnostic, puis faire le diagnostic du même endroit.</t>
+          <t>Créer un compte en laissant « Recevoir les conseils de Bob » coché, puis valider.</t>
         </is>
       </c>
       <c r="E59" s="4" t="inlineStr">
         <is>
-          <t>Carte « 📸 C'est le moment du diagnostic de suivi » (photo d'avant, date des travaux, « a 30 jours », score d'avant) pendant 7 jours, plus après la nouvelle photo ; sur le résultat, carte « 📈 Depuis ton regarnissage du … » : photos avant / aujourd'hui avec leurs scores, écart en points (vert si +5 ou plus, rouge si -5 ou moins), problèmes réglés, encore là ou nouveaux.</t>
+          <t>Le téléphone ne demande pas l'autorisation des notifications à l'inscription ; texte de la case : « par email ou par notification (Bob te proposera de les activer après ta première aide) » ; les conseils partent par email en attendant.</t>
         </is>
       </c>
       <c r="F59" s="4" t="inlineStr">
         <is>
-          <t>Premium</t>
+          <t>Nouveau compte</t>
         </is>
       </c>
       <c r="G59" s="6" t="inlineStr">
@@ -2730,7 +2730,7 @@
       </c>
       <c r="H59" s="6" t="inlineStr">
         <is>
-          <t>Sur STA le 18/10/2026 ; travaux indiqués sur la page Diagnostic depuis le 19/10/2026.</t>
+          <t>Sur STA le 18/10/2026 (plan trafic ×10, action 9 en version allégée).</t>
         </is>
       </c>
       <c r="I59" s="6" t="n"/>
@@ -2741,27 +2741,27 @@
       </c>
       <c r="B60" s="5" t="inlineStr">
         <is>
-          <t>Diagnostic de suivi — essai de 7 jours</t>
+          <t>Notifications — proposées après la première aide</t>
         </is>
       </c>
       <c r="C60" s="4" t="inlineStr">
         <is>
-          <t>Diagnostic (accueil)</t>
+          <t>Diagnostic (résultat) ; parcours lancé ou en attente de la fenêtre</t>
         </is>
       </c>
       <c r="D60" s="4" t="inlineStr">
         <is>
-          <t>Compte créé il y a moins de 7 jours, sans abonnement (essai Premium) : faire un diagnostic, puis revenir sur l'accueil de l'onglet Diagnostic.</t>
+          <t>Nouveau compte sans notifications : faire un diagnostic, puis ouvrir un parcours ; toucher « Activer les notifications » et accepter l'autorisation du téléphone.</t>
         </is>
       </c>
       <c r="E60" s="4" t="inlineStr">
         <is>
-          <t>Aucune carte des travaux ni de diagnostic de suivi (la photo de suivi tomberait après la fin de l'essai) ; le diagnostic fonctionne normalement.</t>
+          <t>Carte « 🔔 Bob te prévient au bon moment » sous le résultat (et « Ne rate aucun arrosage » / « Sois prévenu dès que la fenêtre s'ouvre » dans le parcours) ; après activation : notification de test reçue, carte disparue, tuile de l'accueil disparue.</t>
         </is>
       </c>
       <c r="F60" s="4" t="inlineStr">
         <is>
-          <t>Compte en essai</t>
+          <t>Nouveau compte</t>
         </is>
       </c>
       <c r="G60" s="6" t="inlineStr">
@@ -2771,7 +2771,7 @@
       </c>
       <c r="H60" s="6" t="inlineStr">
         <is>
-          <t>Décision de Jordan du 18/10/2026.</t>
+          <t>Sur STA le 18/10/2026.</t>
         </is>
       </c>
       <c r="I60" s="6" t="n"/>
@@ -2782,27 +2782,27 @@
       </c>
       <c r="B61" s="5" t="inlineStr">
         <is>
-          <t>Pilotage — comptes de test exclus</t>
+          <t>Notifications — « Plus tard »</t>
         </is>
       </c>
       <c r="C61" s="4" t="inlineStr">
         <is>
-          <t>Pilotage → Activité</t>
+          <t>Diagnostic (résultat)</t>
         </is>
       </c>
       <c r="D61" s="4" t="inlineStr">
         <is>
-          <t>Créer un compte avec une adresse jordankrebs1+essai@gmail.com (ou marquer un compte {"compteTest": true} dans Clerk : Users → le compte → Metadata → Public), l'utiliser un jour, puis ouvrir Pilotage.</t>
+          <t>Toucher « Plus tard » sur la carte, puis refaire un diagnostic le même jour.</t>
         </is>
       </c>
       <c r="E61" s="4" t="inlineStr">
         <is>
-          <t>Le compte n'est compté ni dans les inscrits, ni dans les actifs, la rétention, les sources ou la carte ; une adresse « + » d'un vrai utilisateur (autre que l'admin) reste comptée.</t>
+          <t>La carte ne revient pas pendant 14 jours ; la tuile « Activez les alertes » de l'accueil reste disponible.</t>
         </is>
       </c>
       <c r="F61" s="4" t="inlineStr">
         <is>
-          <t>Admin</t>
+          <t>Nouveau compte</t>
         </is>
       </c>
       <c r="G61" s="6" t="inlineStr">
@@ -2812,7 +2812,7 @@
       </c>
       <c r="H61" s="6" t="inlineStr">
         <is>
-          <t>Sur STA le 18/10/2026 (écarts relevés le 08/10).</t>
+          <t>Sur STA le 18/10/2026.</t>
         </is>
       </c>
       <c r="I61" s="6" t="n"/>
@@ -2823,27 +2823,27 @@
       </c>
       <c r="B62" s="5" t="inlineStr">
         <is>
-          <t>Pilotage — offre annuelle à 12,99 €</t>
+          <t>Équipements — choix de la marque</t>
         </is>
       </c>
       <c r="C62" s="4" t="inlineStr">
         <is>
-          <t>Pilotage → Finances (MRR, ARR, Produits et charges)</t>
+          <t>Mes équipements (station, robot, arrosage)</t>
         </is>
       </c>
       <c r="D62" s="4" t="inlineStr">
         <is>
-          <t>Avec un abonné annuel pris pendant l'offre saisonnière (à partir du 1/11) : ouvrir Finances.</t>
+          <t>Ouvrir Mes équipements sans rien de connecté ; dans chaque carte, choisir une marque dans la liste déroulante, puis une autre, puis « Choisis la marque… ».</t>
         </is>
       </c>
       <c r="E62" s="4" t="inlineStr">
         <is>
-          <t>L'abonné compte pour 12,99 €/an la 1re année (MRR, ARR et Produits et charges) ; ligne « Abonnements annuels » : « dont 1 à 12,99 € la 1re année ». Les autres annuels restent à 39,99 €.</t>
+          <t>Une liste déroulante par carte (station : Netatmo, Ecowitt, Davis, Autre marque ; robot : Husqvarna Automower, Gardena SILENO, Mammotion, Autre marque ; arrosage : Gardena, Rachio, Autre marque) ; seuls les éléments à renseigner et le bouton de la marque choisie s'affichent ; « Autre marque » renvoie au formulaire « Ton équipement n'est pas dans la liste ? » ; au retour d'une connexion chez le fabricant, sa marque est déjà choisie.</t>
         </is>
       </c>
       <c r="F62" s="4" t="inlineStr">
         <is>
-          <t>Admin</t>
+          <t>Premium</t>
         </is>
       </c>
       <c r="G62" s="6" t="inlineStr">
@@ -2853,7 +2853,7 @@
       </c>
       <c r="H62" s="6" t="inlineStr">
         <is>
-          <t>Sur STA le 18/10/2026. Testable au premier abonné de l'offre.</t>
+          <t>Sur STA le 19/10/2026 (demande de Jordan : une liste déroulante de marques, puis seulement les éléments à renseigner).</t>
         </is>
       </c>
       <c r="I62" s="6" t="n"/>
@@ -2864,22 +2864,22 @@
       </c>
       <c r="B63" s="5" t="inlineStr">
         <is>
-          <t>Pilotage — jours à l'heure de Paris</t>
+          <t>Équipements — erreur renvoyée par le fabricant</t>
         </is>
       </c>
       <c r="C63" s="4" t="inlineStr">
         <is>
-          <t>Pilotage → Activité</t>
+          <t>Mes équipements ; Pilotage → Bugs</t>
         </is>
       </c>
       <c r="D63" s="4" t="inlineStr">
         <is>
-          <t>Après une inscription ou une visite entre minuit et 2 h (heure de Paris) : regarder « Nouveaux aujourd'hui », le graphique sur 30 jours, les mois et « Visiteurs site (auj.) ».</t>
+          <t>Connexion Netatmo, Husqvarna ou Gardena : refuser l'accès sur le site du fabricant ; puis, si possible, provoquer une erreur du fabricant.</t>
         </is>
       </c>
       <c r="E63" s="4" t="inlineStr">
         <is>
-          <t>L'inscription et la visite comptent pour le jour même, pas pour la veille.</t>
+          <t>Refus : « Connexion annulée : rien n'a été enregistré », sans alerte ; autre erreur du fabricant : « La connexion … a échoué » et une alerte « Connexion … refusée par le fabricant » avec la raison donnée par le fabricant.</t>
         </is>
       </c>
       <c r="F63" s="4" t="inlineStr">
@@ -2889,43 +2889,45 @@
       </c>
       <c r="G63" s="6" t="inlineStr">
         <is>
-          <t>Non testable</t>
+          <t>À tester</t>
         </is>
       </c>
       <c r="H63" s="6" t="inlineStr">
         <is>
-          <t>Sur STA le 18/10/2026 ; vérifié par un test automatique, à constater au premier cas réel.</t>
+          <t>Sur STA le 19/10/2026. Vérifié sur STA le 19/10/2026 : erreur « redirect_uri_mismatch » de Netatmo remontée dans Pilotage → Bugs avec sa raison et l'adresse de retour.</t>
         </is>
       </c>
       <c r="I63" s="6" t="n"/>
     </row>
     <row r="64">
-      <c r="A64" s="4" t="n">
-        <v>60</v>
+      <c r="A64" s="4" t="inlineStr">
+        <is>
+          <t>60</t>
+        </is>
       </c>
       <c r="B64" s="5" t="inlineStr">
         <is>
-          <t>Pilotage — carte des inscrits</t>
+          <t>Conseils — l'app dans les articles (prod le 22/11)</t>
         </is>
       </c>
       <c r="C64" s="4" t="inlineStr">
         <is>
-          <t>Pilotage → Activité (carte)</t>
+          <t>Pages Conseils (article, rubrique, Qui sommes-nous) ; Supabase PROD (funnel_events)</t>
         </is>
       </c>
       <c r="D64" s="4" t="inlineStr">
         <is>
-          <t>Ouvrir la carte des inscrits.</t>
+          <t>Sans être connecté, sur un téléphone Android puis sur ordinateur : ouvrir un article ; regarder le bandeau sous le titre, les 3 encarts et le bouton fixe ; toucher un encart ; ouvrir la rubrique et Qui sommes-nous.</t>
         </is>
       </c>
       <c r="E64" s="4" t="inlineStr">
         <is>
-          <t>La ville de l'admin et celles des comptes de test ne sont plus comptées (sauf vrai inscrit dans la même ville).</t>
+          <t>Bandeau sous le titre sans cacher le texte (« Télécharger sur Google Play » seulement dans le navigateur d'un téléphone Android) ; encarts après « En bref », au milieu et à la fin, thèmes variés selon l'article (src/lib/argumentsApp.json) ; bouton fixe « Ouvrir l'app gratuite » sur téléphone seulement ; grille « Ce que fait l'app » ; l'encart touché ouvre l'app et sa page_view porte encart = thème-position ; aucune page plus large que l'écran.</t>
         </is>
       </c>
       <c r="F64" s="4" t="inlineStr">
         <is>
-          <t>Admin</t>
+          <t>Non connecté</t>
         </is>
       </c>
       <c r="G64" s="6" t="inlineStr">
@@ -2935,38 +2937,40 @@
       </c>
       <c r="H64" s="6" t="inlineStr">
         <is>
-          <t>Sur STA le 18/10/2026.</t>
+          <t>Sur STA le 30/10/2026 (décisions de Jordan des 28 et 30/10) ; bandeau en 2 versions à départager sur les visuels.</t>
         </is>
       </c>
       <c r="I64" s="6" t="n"/>
     </row>
     <row r="65">
-      <c r="A65" s="4" t="n">
-        <v>61</v>
+      <c r="A65" s="4" t="inlineStr">
+        <is>
+          <t>61</t>
+        </is>
       </c>
       <c r="B65" s="5" t="inlineStr">
         <is>
-          <t>Pilotage — emails envoyés</t>
+          <t>Alignement PROD / STA</t>
         </is>
       </c>
       <c r="C65" s="4" t="inlineStr">
         <is>
-          <t>Pilotage → Activité (notifications)</t>
+          <t>Git</t>
         </is>
       </c>
       <c r="D65" s="4" t="inlineStr">
         <is>
-          <t>Lire la ligne sous « Notifications ».</t>
+          <t>Après la fusion : git diff --quiet origin/main origin/Staging.</t>
         </is>
       </c>
       <c r="E65" s="4" t="inlineStr">
         <is>
-          <t>« N notifications · N ouvertes · N conseils par email · N emails de démarrage et relances » : les emails de démarrage et de relance ne sont plus comptés comme conseils.</t>
+          <t>Aucune différence.</t>
         </is>
       </c>
       <c r="F65" s="4" t="inlineStr">
         <is>
-          <t>Admin</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G65" s="6" t="inlineStr">
@@ -2974,35 +2978,33 @@
           <t>À tester</t>
         </is>
       </c>
-      <c r="H65" s="6" t="inlineStr">
-        <is>
-          <t>Sur STA le 18/10/2026.</t>
-        </is>
-      </c>
+      <c r="H65" s="6" t="n"/>
       <c r="I65" s="6" t="n"/>
     </row>
     <row r="66">
-      <c r="A66" s="4" t="n">
-        <v>62</v>
+      <c r="A66" s="4" t="inlineStr">
+        <is>
+          <t>62</t>
+        </is>
       </c>
       <c r="B66" s="5" t="inlineStr">
         <is>
-          <t>Base de données — vue dau_by_day</t>
+          <t>Base de données PROD</t>
         </is>
       </c>
       <c r="C66" s="4" t="inlineStr">
         <is>
-          <t>Supabase STA et PROD</t>
+          <t>Supabase PROD</t>
         </is>
       </c>
       <c r="D66" s="4" t="inlineStr">
         <is>
-          <t>Après la mise en prod : vérifier que plus rien n'utilise la vue dau_by_day (les actifs viennent de daily_active_users), puis la supprimer sur les deux projets.</t>
+          <t>Vérifier les tables codes et parrainages.</t>
         </is>
       </c>
       <c r="E66" s="4" t="inlineStr">
         <is>
-          <t>Vue supprimée ; Pilotage → Activité affiche toujours les actifs par jour.</t>
+          <t>Tables présentes (créées le 05/10 sur les deux projets).</t>
         </is>
       </c>
       <c r="F66" s="4" t="inlineStr">
@@ -3015,40 +3017,38 @@
           <t>À tester</t>
         </is>
       </c>
-      <c r="H66" s="6" t="inlineStr">
-        <is>
-          <t>Les actifs par jour sont calculés depuis le 18/10/2026 (STA) à partir des jours d'utilisation, pour exclure les comptes de test.</t>
-        </is>
-      </c>
+      <c r="H66" s="6" t="n"/>
       <c r="I66" s="6" t="n"/>
     </row>
     <row r="67">
-      <c r="A67" s="4" t="n">
-        <v>63</v>
+      <c r="A67" s="4" t="inlineStr">
+        <is>
+          <t>63</t>
+        </is>
       </c>
       <c r="B67" s="5" t="inlineStr">
         <is>
-          <t>Notifications — plus de demande à l'inscription</t>
+          <t>Règle de travail de décembre</t>
         </is>
       </c>
       <c r="C67" s="4" t="inlineStr">
         <is>
-          <t>Inscription (consentements)</t>
+          <t>CLAUDE.md</t>
         </is>
       </c>
       <c r="D67" s="4" t="inlineStr">
         <is>
-          <t>Créer un compte en laissant « Recevoir les conseils de Bob » coché, puis valider.</t>
+          <t>Après la mise en prod : retirer le paragraphe « Jusqu'à décembre 2026 ».</t>
         </is>
       </c>
       <c r="E67" s="4" t="inlineStr">
         <is>
-          <t>Le téléphone ne demande pas l'autorisation des notifications à l'inscription ; texte de la case : « par email ou par notification (Bob te proposera de les activer après ta première aide) » ; les conseils partent par email en attendant.</t>
+          <t>STA redevient identique à la PROD.</t>
         </is>
       </c>
       <c r="F67" s="4" t="inlineStr">
         <is>
-          <t>Nouveau compte</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G67" s="6" t="inlineStr">
@@ -3056,1030 +3056,30 @@
           <t>À tester</t>
         </is>
       </c>
-      <c r="H67" s="6" t="inlineStr">
-        <is>
-          <t>Sur STA le 18/10/2026 (plan trafic ×10, action 9 en version allégée).</t>
-        </is>
-      </c>
+      <c r="H67" s="6" t="n"/>
       <c r="I67" s="6" t="n"/>
     </row>
-    <row r="68">
-      <c r="A68" s="4" t="n">
-        <v>64</v>
-      </c>
-      <c r="B68" s="5" t="inlineStr">
-        <is>
-          <t>Notifications — proposées après la première aide</t>
-        </is>
-      </c>
-      <c r="C68" s="4" t="inlineStr">
-        <is>
-          <t>Diagnostic (résultat) ; parcours lancé ou en attente de la fenêtre</t>
-        </is>
-      </c>
-      <c r="D68" s="4" t="inlineStr">
-        <is>
-          <t>Nouveau compte sans notifications : faire un diagnostic, puis ouvrir un parcours ; toucher « Activer les notifications » et accepter l'autorisation du téléphone.</t>
-        </is>
-      </c>
-      <c r="E68" s="4" t="inlineStr">
-        <is>
-          <t>Carte « 🔔 Bob te prévient au bon moment » sous le résultat (et « Ne rate aucun arrosage » / « Sois prévenu dès que la fenêtre s'ouvre » dans le parcours) ; après activation : notification de test reçue, carte disparue, tuile de l'accueil disparue.</t>
-        </is>
-      </c>
-      <c r="F68" s="4" t="inlineStr">
-        <is>
-          <t>Nouveau compte</t>
-        </is>
-      </c>
-      <c r="G68" s="6" t="inlineStr">
-        <is>
-          <t>À tester</t>
-        </is>
-      </c>
-      <c r="H68" s="6" t="inlineStr">
-        <is>
-          <t>Sur STA le 18/10/2026.</t>
-        </is>
-      </c>
-      <c r="I68" s="6" t="n"/>
-    </row>
-    <row r="69">
-      <c r="A69" s="4" t="n">
-        <v>65</v>
-      </c>
-      <c r="B69" s="5" t="inlineStr">
-        <is>
-          <t>Notifications — « Plus tard »</t>
-        </is>
-      </c>
-      <c r="C69" s="4" t="inlineStr">
-        <is>
-          <t>Diagnostic (résultat)</t>
-        </is>
-      </c>
-      <c r="D69" s="4" t="inlineStr">
-        <is>
-          <t>Toucher « Plus tard » sur la carte, puis refaire un diagnostic le même jour.</t>
-        </is>
-      </c>
-      <c r="E69" s="4" t="inlineStr">
-        <is>
-          <t>La carte ne revient pas pendant 14 jours ; la tuile « Activez les alertes » de l'accueil reste disponible.</t>
-        </is>
-      </c>
-      <c r="F69" s="4" t="inlineStr">
-        <is>
-          <t>Nouveau compte</t>
-        </is>
-      </c>
-      <c r="G69" s="6" t="inlineStr">
-        <is>
-          <t>À tester</t>
-        </is>
-      </c>
-      <c r="H69" s="6" t="inlineStr">
-        <is>
-          <t>Sur STA le 18/10/2026.</t>
-        </is>
-      </c>
-      <c r="I69" s="6" t="n"/>
-    </row>
-    <row r="70">
-      <c r="A70" s="4" t="n">
-        <v>66</v>
-      </c>
-      <c r="B70" s="5" t="inlineStr">
-        <is>
-          <t>Équipements — choix de la marque</t>
-        </is>
-      </c>
-      <c r="C70" s="4" t="inlineStr">
-        <is>
-          <t>Mes équipements (station, robot, arrosage)</t>
-        </is>
-      </c>
-      <c r="D70" s="4" t="inlineStr">
-        <is>
-          <t>Ouvrir Mes équipements sans rien de connecté ; dans chaque carte, choisir une marque dans la liste déroulante, puis une autre, puis « Choisis la marque… ».</t>
-        </is>
-      </c>
-      <c r="E70" s="4" t="inlineStr">
-        <is>
-          <t>Une liste déroulante par carte (station : Netatmo, Ecowitt, Davis, Autre marque ; robot : Husqvarna Automower, Gardena SILENO, Mammotion, Autre marque ; arrosage : Gardena, Rachio, Autre marque) ; seuls les éléments à renseigner et le bouton de la marque choisie s'affichent ; « Autre marque » renvoie au formulaire « Ton équipement n'est pas dans la liste ? » ; au retour d'une connexion chez le fabricant, sa marque est déjà choisie.</t>
-        </is>
-      </c>
-      <c r="F70" s="4" t="inlineStr">
-        <is>
-          <t>Premium</t>
-        </is>
-      </c>
-      <c r="G70" s="6" t="inlineStr">
-        <is>
-          <t>À tester</t>
-        </is>
-      </c>
-      <c r="H70" s="6" t="inlineStr">
-        <is>
-          <t>Sur STA le 19/10/2026 (demande de Jordan : une liste déroulante de marques, puis seulement les éléments à renseigner).</t>
-        </is>
-      </c>
-      <c r="I70" s="6" t="n"/>
-    </row>
-    <row r="71">
-      <c r="A71" s="4" t="n">
-        <v>67</v>
-      </c>
-      <c r="B71" s="5" t="inlineStr">
-        <is>
-          <t>Équipements — erreur renvoyée par le fabricant</t>
-        </is>
-      </c>
-      <c r="C71" s="4" t="inlineStr">
-        <is>
-          <t>Mes équipements ; Pilotage → Bugs</t>
-        </is>
-      </c>
-      <c r="D71" s="4" t="inlineStr">
-        <is>
-          <t>Connexion Netatmo, Husqvarna ou Gardena : refuser l'accès sur le site du fabricant ; puis, si possible, provoquer une erreur du fabricant.</t>
-        </is>
-      </c>
-      <c r="E71" s="4" t="inlineStr">
-        <is>
-          <t>Refus : « Connexion annulée : rien n'a été enregistré », sans alerte ; autre erreur du fabricant : « La connexion … a échoué » et une alerte « Connexion … refusée par le fabricant » avec la raison donnée par le fabricant.</t>
-        </is>
-      </c>
-      <c r="F71" s="4" t="inlineStr">
-        <is>
-          <t>Admin</t>
-        </is>
-      </c>
-      <c r="G71" s="6" t="inlineStr">
-        <is>
-          <t>À tester</t>
-        </is>
-      </c>
-      <c r="H71" s="6" t="inlineStr">
-        <is>
-          <t>Sur STA le 19/10/2026. Vérifié sur STA le 19/10/2026 : erreur « redirect_uri_mismatch » de Netatmo remontée dans Pilotage → Bugs avec sa raison et l'adresse de retour.</t>
-        </is>
-      </c>
-      <c r="I71" s="6" t="n"/>
-    </row>
-    <row r="72">
-      <c r="A72" s="4" t="inlineStr">
-        <is>
-          <t>68</t>
-        </is>
-      </c>
-      <c r="B72" s="5" t="inlineStr">
-        <is>
-          <t>Refonte — barre du bas</t>
-        </is>
-      </c>
-      <c r="C72" s="4" t="inlineStr">
-        <is>
-          <t>Toute l'app (connecté)</t>
-        </is>
-      </c>
-      <c r="D72" s="4" t="inlineStr">
-        <is>
-          <t>Se connecter et regarder la barre du bas pendant la ligue d'hiver, puis après le 30/01.</t>
-        </is>
-      </c>
-      <c r="E72" s="4" t="inlineStr">
-        <is>
-          <t>4 onglets : Accueil, Aujourd'hui, Diagnostic, Mon gazon, plus « Quiz » jusqu'au 30/01 ; plus d'onglets Produits ni Classement (Produits reste ouvert depuis Mon gazon).</t>
-        </is>
-      </c>
-      <c r="F72" s="4" t="inlineStr">
-        <is>
-          <t>Gratuit et Premium</t>
-        </is>
-      </c>
-      <c r="G72" s="6" t="inlineStr">
-        <is>
-          <t>À tester</t>
-        </is>
-      </c>
-      <c r="H72" s="6" t="inlineStr">
-        <is>
-          <t>Sur STA le 26/10/2026 (décisions de Jordan du 26/10). Testé par Jordan sur STA le 29/10 : OK.</t>
-        </is>
-      </c>
-      <c r="I72" s="6" t="n"/>
-    </row>
-    <row r="73">
-      <c r="A73" s="4" t="inlineStr">
-        <is>
-          <t>69</t>
-        </is>
-      </c>
-      <c r="B73" s="5" t="inlineStr">
-        <is>
-          <t>Refonte — accueil : résumé du jour</t>
-        </is>
-      </c>
-      <c r="C73" s="4" t="inlineStr">
-        <is>
-          <t>Accueil</t>
-        </is>
-      </c>
-      <c r="D73" s="4" t="inlineStr">
-        <is>
-          <t>Comparer la carte « Aujourd'hui » de l'accueil avec l'onglet Aujourd'hui, un jour avec des actions puis un jour sans ; toucher la carte.</t>
-        </is>
-      </c>
-      <c r="E73" s="4" t="inlineStr">
-        <is>
-          <t>Mêmes actions que l'onglet Aujourd'hui ; sans action : « Rien à faire aujourd'hui » et la prochaine action ; la carte ouvre Aujourd'hui.</t>
-        </is>
-      </c>
-      <c r="F73" s="4" t="inlineStr">
-        <is>
-          <t>Tous</t>
-        </is>
-      </c>
-      <c r="G73" s="6" t="inlineStr">
-        <is>
-          <t>À tester</t>
-        </is>
-      </c>
-      <c r="H73" s="6" t="inlineStr">
-        <is>
-          <t>Sur STA le 26/10/2026 (décisions de Jordan du 26/10). Testé par Jordan sur STA le 29/10 : OK.</t>
-        </is>
-      </c>
-      <c r="I73" s="6" t="n"/>
-    </row>
-    <row r="74">
-      <c r="A74" s="4" t="inlineStr">
-        <is>
-          <t>70</t>
-        </is>
-      </c>
-      <c r="B74" s="5" t="inlineStr">
-        <is>
-          <t>Refonte — série et GreenPoints</t>
-        </is>
-      </c>
-      <c r="C74" s="4" t="inlineStr">
-        <is>
-          <t>Accueil, Mon gazon</t>
-        </is>
-      </c>
-      <c r="D74" s="4" t="inlineStr">
-        <is>
-          <t>Ouvrir l'app un nouveau jour en restant sur l'accueil ; toucher la carte série et GreenPoints.</t>
-        </is>
-      </c>
-      <c r="E74" s="4" t="inlineStr">
-        <is>
-          <t>Série et GreenPoints de connexion comptés dès l'accueil, une fois par jour ; la carte ouvre Mon gazon directement sur « Mes progrès ».</t>
-        </is>
-      </c>
-      <c r="F74" s="4" t="inlineStr">
-        <is>
-          <t>Tous</t>
-        </is>
-      </c>
-      <c r="G74" s="6" t="inlineStr">
-        <is>
-          <t>À tester</t>
-        </is>
-      </c>
-      <c r="H74" s="6" t="inlineStr">
-        <is>
-          <t>Sur STA le 26/10/2026 (décisions de Jordan du 26/10). Testé par Jordan sur STA le 29/10 : OK.</t>
-        </is>
-      </c>
-      <c r="I74" s="6" t="n"/>
-    </row>
-    <row r="75">
-      <c r="A75" s="4" t="inlineStr">
-        <is>
-          <t>71</t>
-        </is>
-      </c>
-      <c r="B75" s="5" t="inlineStr">
-        <is>
-          <t>Refonte — Mon gazon épuré</t>
-        </is>
-      </c>
-      <c r="C75" s="4" t="inlineStr">
-        <is>
-          <t>Mon gazon</t>
-        </is>
-      </c>
-      <c r="D75" s="4" t="inlineStr">
-        <is>
-          <t>Parcourir Mon gazon avec un compte gratuit puis Premium ; déplier « Pourquoi ce score ? », « Partager », les badges et, en Premium, le débit de l'arroseur ; retirer une action notée par erreur ; toucher chaque outil ; ouvrir l'ancienne adresse /history.</t>
-        </is>
-      </c>
-      <c r="E75" s="4" t="inlineStr">
-        <is>
-          <t>Dans l'ordre : score santé compact (« Pourquoi ce score ? » : 4 critères et problèmes prioritaires ; « Partager »), évolution du score compacte (courbe, actions de l'année en une ligne, bilan de saison), « Mes actions » (5 dernières, « Voir tout », retrait), « Mes progrès » en une carte (série, GreenPoints, classement ou renvoi vers le Quiz pendant la ligue), badges en une ligne (« Voir tout »), « Mes outils » (plan gazon, équipements, semer ou regarnir, produits et dépenses ; parrainage avec la mise en prod de décembre), « Mon profil » (complétude, infos, débit de l'arroseur en Premium), « Avec Premium » pour un compte gratuit ; plus de conseil du mois, plan du mois, produits recommandés ni bloc de calibrage ; /history n'existe plus.</t>
-        </is>
-      </c>
-      <c r="F75" s="4" t="inlineStr">
-        <is>
-          <t>Tous</t>
-        </is>
-      </c>
-      <c r="G75" s="6" t="inlineStr">
-        <is>
-          <t>À tester</t>
-        </is>
-      </c>
-      <c r="H75" s="6" t="inlineStr">
-        <is>
-          <t>Sur STA le 26/10/2026 (décisions de Jordan du 26/10). Testé par Jordan sur STA le 29/10 : OK, mais page jugée trop chargée. Épurée le 29/10 (décision de Jordan) : 19 blocs → 7, « Mes progrès » en une carte ; validée par Jordan sur STA le 29/10.</t>
-        </is>
-      </c>
-      <c r="I75" s="6" t="n"/>
-    </row>
-    <row r="76">
-      <c r="A76" s="4" t="inlineStr">
-        <is>
-          <t>72</t>
-        </is>
-      </c>
-      <c r="B76" s="5" t="inlineStr">
-        <is>
-          <t>Refonte — Premium sur l'accueil, le diagnostic et les équipements</t>
-        </is>
-      </c>
-      <c r="C76" s="4" t="inlineStr">
-        <is>
-          <t>Accueil, Diagnostic, Mes équipements</t>
-        </is>
-      </c>
-      <c r="D76" s="4" t="inlineStr">
-        <is>
-          <t>Regarder l'accueil et l'onglet Diagnostic avec un compte gratuit, puis Premium, puis dans l'app Android ; ouvrir Mes équipements avec un compte gratuit (avec et sans équipement déjà connecté), puis Premium.</t>
-        </is>
-      </c>
-      <c r="E76" s="4" t="inlineStr">
-        <is>
-          <t>Gratuit : carte « Avec Premium » (avantages de Premium sans les paysagistes, puis le prix ou, pendant sa période, l'offre de saison) ; Premium : raccourcis « Mes équipements » et « Mon plan annuel » ; app Android : pas de carte d'achat ; Mes équipements en gratuit : « Inclus dans Premium » et « Découvrir Premium » (pas dans l'app Android), aucune connexion ni demande d'équipement non listé, équipement déjà connecté seulement déconnectable ; le serveur refuse aussi connexions et commandes sans Premium ; Premium : connexions inchangées.</t>
-        </is>
-      </c>
-      <c r="F76" s="4" t="inlineStr">
-        <is>
-          <t>Gratuit, Premium, app Android</t>
-        </is>
-      </c>
-      <c r="G76" s="6" t="inlineStr">
-        <is>
-          <t>À tester</t>
-        </is>
-      </c>
-      <c r="H76" s="6" t="inlineStr">
-        <is>
-          <t>Sur STA le 26/10/2026 (décisions de Jordan du 26/10). Testé par Jordan sur STA le 29/10 : raccourcis Premium OK (compte gratuit et app Android à voir). Mes équipements ouverts aux comptes gratuits (constat de Jordan le 29/10) : verrou Premium ajouté le 29/10 (STA et version de prod), vérifié par Jordan sur STA le 29/10 ; demande d'équipement non listé retirée de la page d'un compte gratuit le 29/10 (décision de Jordan). Compte gratuit testé par Jordan sur STA le 30/10 : OK (carte « Avec Premium » de l'accueil, du diagnostic et de Mon gazon ; Mes équipements verrouillé, sans formulaire). App Android : à vérifier après la mise en prod.</t>
-        </is>
-      </c>
-      <c r="I76" s="6" t="n"/>
-    </row>
-    <row r="77">
-      <c r="A77" s="4" t="inlineStr">
-        <is>
-          <t>73</t>
-        </is>
-      </c>
-      <c r="B77" s="5" t="inlineStr">
-        <is>
-          <t>Refonte — Choisir son niveau</t>
-        </is>
-      </c>
-      <c r="C77" s="4" t="inlineStr">
-        <is>
-          <t>/subscribe</t>
-        </is>
-      </c>
-      <c r="D77" s="4" t="inlineStr">
-        <is>
-          <t>Ouvrir la page avec un compte gratuit, puis un compte en essai ; aller jusqu'au paiement Stripe sans payer ; ouvrir l'adresse /subscribe avec un compte abonné, Premium offert ou admin.</t>
-        </is>
-      </c>
-      <c r="E77" s="4" t="inlineStr">
-        <is>
-          <t>3 niveaux (Visiteur, Gratuit, Premium) ; « Ton niveau » ou « Ton essai : encore N jours » ; compte déjà Premium (abonné, Premium offert, admin) : renvoyé à l'accueil, la page ne s'affiche jamais ; formules, mentions légales et paiement inchangés.</t>
-        </is>
-      </c>
-      <c r="F77" s="4" t="inlineStr">
-        <is>
-          <t>Gratuit, essai, Premium</t>
-        </is>
-      </c>
-      <c r="G77" s="6" t="inlineStr">
-        <is>
-          <t>À tester</t>
-        </is>
-      </c>
-      <c r="H77" s="6" t="inlineStr">
-        <is>
-          <t>Sur STA le 26/10/2026 (décisions de Jordan du 26/10). Paiement de test réussi sur STA le 29/10 (mensuel à 2,99 €, bac à sable Stripe). Abonné : aucun lien vers la page (voulu). Test de Jordan le 29/10 avec son compte admin : offres affichées au lieu de « Tu es déjà Premium » (compte admin non reconnu comme Premium sur cette page) ; corrigé le 29/10, puis décision de Jordan le soir même : un compte déjà Premium n'arrive jamais sur la page (renvoi à l'accueil), STA et version de prod.</t>
-        </is>
-      </c>
-      <c r="I77" s="6" t="n"/>
-    </row>
-    <row r="78">
-      <c r="A78" s="4" t="inlineStr">
-        <is>
-          <t>74</t>
-        </is>
-      </c>
-      <c r="B78" s="5" t="inlineStr">
-        <is>
-          <t>Refonte — plan annuel inclus dans Premium</t>
-        </is>
-      </c>
-      <c r="C78" s="4" t="inlineStr">
-        <is>
-          <t>Mon gazon → Mon plan gazon ; CGV 7 bis</t>
-        </is>
-      </c>
-      <c r="D78" s="4" t="inlineStr">
-        <is>
-          <t>Ouvrir le plan avec un compte gratuit, un compte Premium et un compte ayant acheté un plan à 0,99 €.</t>
-        </is>
-      </c>
-      <c r="E78" s="4" t="inlineStr">
-        <is>
-          <t>Gratuit : aperçu d'un mois et « Inclus dans Premium », aucune vente ; Premium et plans déjà achetés : les 12 mois et le PDF ; CGV 7 bis réécrit.</t>
-        </is>
-      </c>
-      <c r="F78" s="4" t="inlineStr">
-        <is>
-          <t>Gratuit, Premium, acheteur</t>
-        </is>
-      </c>
-      <c r="G78" s="6" t="inlineStr">
-        <is>
-          <t>À tester</t>
-        </is>
-      </c>
-      <c r="H78" s="6" t="inlineStr">
-        <is>
-          <t>Sur STA le 26/10/2026 (décisions de Jordan du 26/10). Testé par Jordan sur STA le 29/10 : plan Premium OK (compte gratuit à voir). Compte gratuit testé par Jordan sur STA le 30/10 : OK.</t>
-        </is>
-      </c>
-      <c r="I78" s="6" t="n"/>
-    </row>
-    <row r="79">
-      <c r="A79" s="4" t="inlineStr">
-        <is>
-          <t>75</t>
-        </is>
-      </c>
-      <c r="B79" s="5" t="inlineStr">
-        <is>
-          <t>Refonte — accueil visiteur</t>
-        </is>
-      </c>
-      <c r="C79" s="4" t="inlineStr">
-        <is>
-          <t>mongazon360.fr (non connecté)</t>
-        </is>
-      </c>
-      <c r="D79" s="4" t="inlineStr">
-        <is>
-          <t>Saisir une commune (puis une commune homonyme), essayer « Utiliser ma position », ouvrir un article, « Prendre une photo », « Créer mon compte gratuit », puis le lien de connexion ; revenir le lendemain.</t>
-        </is>
-      </c>
-      <c r="E79" s="4" t="inlineStr">
-        <is>
-          <t>Météo du jour de la commune (température, ciel) ; conseil de Bob du jour ; 3 articles de la saison ; barre Accueil, Conseils, Diagnostic, Compte (aussi sur l'essai du diagnostic, la création de compte et la connexion, onglet Compte en surbrillance) ; commune retrouvée à la visite suivante.</t>
-        </is>
-      </c>
-      <c r="F79" s="4" t="inlineStr">
-        <is>
-          <t>Non connecté</t>
-        </is>
-      </c>
-      <c r="G79" s="6" t="inlineStr">
-        <is>
-          <t>À tester</t>
-        </is>
-      </c>
-      <c r="H79" s="6" t="inlineStr">
-        <is>
-          <t>Sur STA le 26/10/2026 (décisions de Jordan du 26/10). Testé par Jordan sur STA le 29/10 : OK ; barre du bas ajoutée le 29/10 à la création de compte et à la connexion (demande de Jordan), vérifiée par Jordan sur STA le 30/10 : OK.</t>
-        </is>
-      </c>
-      <c r="I79" s="6" t="n"/>
-    </row>
-    <row r="80">
-      <c r="A80" s="4" t="inlineStr">
-        <is>
-          <t>76</t>
-        </is>
-      </c>
-      <c r="B80" s="5" t="inlineStr">
-        <is>
-          <t>Refonte — démo retirée</t>
-        </is>
-      </c>
-      <c r="C80" s="4" t="inlineStr">
-        <is>
-          <t>mongazon360.fr/demo ; plan du site</t>
-        </is>
-      </c>
-      <c r="D80" s="4" t="inlineStr">
-        <is>
-          <t>Ouvrir l'ancienne adresse /demo ; lire sitemap.xml.</t>
-        </is>
-      </c>
-      <c r="E80" s="4" t="inlineStr">
-        <is>
-          <t>Redirection vers l'accueil ; /demo absente du plan du site.</t>
-        </is>
-      </c>
-      <c r="F80" s="4" t="inlineStr">
-        <is>
-          <t>Non connecté</t>
-        </is>
-      </c>
-      <c r="G80" s="6" t="inlineStr">
-        <is>
-          <t>À tester</t>
-        </is>
-      </c>
-      <c r="H80" s="6" t="inlineStr">
-        <is>
-          <t>Sur STA le 26/10/2026 (décisions de Jordan du 26/10). Vérifié sur STA le 29/10 : /demo redirigée vers l'accueil (308), absente du plan du site.</t>
-        </is>
-      </c>
-      <c r="I80" s="6" t="n"/>
-    </row>
-    <row r="81">
-      <c r="A81" s="4" t="inlineStr">
-        <is>
-          <t>77</t>
-        </is>
-      </c>
-      <c r="B81" s="5" t="inlineStr">
-        <is>
-          <t>Refonte — carte Nouveautés</t>
-        </is>
-      </c>
-      <c r="C81" s="4" t="inlineStr">
-        <is>
-          <t>Accueil ; src/components/CarteNouveautes.jsx</t>
-        </is>
-      </c>
-      <c r="D81" s="4" t="inlineStr">
-        <is>
-          <t>Le jour de la mise en prod : régler MISE_EN_PROD sur cette date (commit), puis ouvrir l'app avec un ancien compte et un compte créé ensuite.</t>
-        </is>
-      </c>
-      <c r="E81" s="4" t="inlineStr">
-        <is>
-          <t>Carte « Mongazon360 fait peau neuve » pour l'ancien compte, fermée pour de bon par « J'ai compris » ; rien pour le nouveau compte.</t>
-        </is>
-      </c>
-      <c r="F81" s="4" t="inlineStr">
-        <is>
-          <t>Ancien et nouveau compte</t>
-        </is>
-      </c>
-      <c r="G81" s="6" t="inlineStr">
-        <is>
-          <t>À tester</t>
-        </is>
-      </c>
-      <c r="H81" s="6" t="inlineStr">
-        <is>
-          <t>Sur STA le 26/10/2026 (décisions de Jordan du 26/10).</t>
-        </is>
-      </c>
-      <c r="I81" s="6" t="n"/>
-    </row>
-    <row r="82">
-      <c r="A82" s="4" t="inlineStr">
-        <is>
-          <t>78</t>
-        </is>
-      </c>
-      <c r="B82" s="5" t="inlineStr">
-        <is>
-          <t>Refonte — visiteurs distincts</t>
-        </is>
-      </c>
-      <c r="C82" s="4" t="inlineStr">
-        <is>
-          <t>Pilotage → Activité ; Supabase PROD</t>
-        </is>
-      </c>
-      <c r="D82" s="4" t="inlineStr">
-        <is>
-          <t>Après quelques visites : regarder l'entonnoir ; vérifier la colonne visite des nouvelles lignes de funnel_events.</t>
-        </is>
-      </c>
-      <c r="E82" s="4" t="inlineStr">
-        <is>
-          <t>« Visiteurs distincts (30 j) » affichés par étape ; colonne visite remplie (créée le 26/10 en STA et en PROD) ; pages Cookies et Confidentialité mentionnent l'identifiant de visite.</t>
-        </is>
-      </c>
-      <c r="F82" s="4" t="inlineStr">
-        <is>
-          <t>Admin</t>
-        </is>
-      </c>
-      <c r="G82" s="6" t="inlineStr">
-        <is>
-          <t>À tester</t>
-        </is>
-      </c>
-      <c r="H82" s="6" t="inlineStr">
-        <is>
-          <t>Sur STA le 26/10/2026 (décisions de Jordan du 26/10).</t>
-        </is>
-      </c>
-      <c r="I82" s="6" t="n"/>
-    </row>
-    <row r="83">
-      <c r="A83" s="4" t="inlineStr">
-        <is>
-          <t>79</t>
-        </is>
-      </c>
-      <c r="B83" s="5" t="inlineStr">
-        <is>
-          <t>Refonte — Bob</t>
-        </is>
-      </c>
-      <c r="C83" s="4" t="inlineStr">
-        <is>
-          <t>Bob</t>
-        </is>
-      </c>
-      <c r="D83" s="4" t="inlineStr">
-        <is>
-          <t>Demander « Combien coûte Premium ? », « Où est le classement ? », « Le plan annuel est payant ? ».</t>
-        </is>
-      </c>
-      <c r="E83" s="4" t="inlineStr">
-        <is>
-          <t>Prix 2,99 € et 24,99 €, offre de saison et essai de 7 jours ; classement dans Mon gazon → Mes progrès ; plan annuel inclus dans Premium.</t>
-        </is>
-      </c>
-      <c r="F83" s="4" t="inlineStr">
-        <is>
-          <t>Gratuit</t>
-        </is>
-      </c>
-      <c r="G83" s="6" t="inlineStr">
-        <is>
-          <t>À tester</t>
-        </is>
-      </c>
-      <c r="H83" s="6" t="inlineStr">
-        <is>
-          <t>Sur STA le 26/10/2026 (décisions de Jordan du 26/10). Testé par Jordan sur STA le 29/10 : OK ; consigne du classement précisée (en pause de novembre à janvier).</t>
-        </is>
-      </c>
-      <c r="I83" s="6" t="n"/>
-    </row>
-    <row r="84">
-      <c r="A84" s="4" t="inlineStr">
-        <is>
-          <t>80</t>
-        </is>
-      </c>
-      <c r="B84" s="5" t="inlineStr">
-        <is>
-          <t>Refonte — dates des pages légales</t>
-        </is>
-      </c>
-      <c r="C84" s="4" t="inlineStr">
-        <is>
-          <t>CGV, politique de cookies, politique de confidentialité</t>
-        </is>
-      </c>
-      <c r="D84" s="4" t="inlineStr">
-        <is>
-          <t>Le jour de la mise en prod : mettre la date du jour dans « Mise à jour » de ces 3 pages (commit).</t>
-        </is>
-      </c>
-      <c r="E84" s="4" t="inlineStr">
-        <is>
-          <t>Date de mise à jour = jour de la mise en prod.</t>
-        </is>
-      </c>
-      <c r="F84" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G84" s="6" t="inlineStr">
-        <is>
-          <t>À tester</t>
-        </is>
-      </c>
-      <c r="H84" s="6" t="inlineStr">
-        <is>
-          <t>Sur STA le 26/10/2026 (décisions de Jordan du 26/10).</t>
-        </is>
-      </c>
-      <c r="I84" s="6" t="n"/>
-    </row>
-    <row r="85">
-      <c r="A85" s="4" t="inlineStr">
-        <is>
-          <t>81</t>
-        </is>
-      </c>
-      <c r="B85" s="5" t="inlineStr">
-        <is>
-          <t>Offre d'hiver dès le 1er novembre</t>
-        </is>
-      </c>
-      <c r="C85" s="4" t="inlineStr">
-        <is>
-          <t>Choisir son niveau, accueil, Bob, email de lancement</t>
-        </is>
-      </c>
-      <c r="D85" s="4" t="inlineStr">
-        <is>
-          <t>À partir du 1/11 : ouvrir « Choisir son niveau » et l'accueil avec un compte gratuit ; demander à Bob « Quand est l'offre de saison ? » ; le matin du 1er jour d'offre, regarder l'email reçu par un compte gratuit qui accepte les offres.</t>
-        </is>
-      </c>
-      <c r="E85" s="4" t="inlineStr">
-        <is>
-          <t>Offre d'hiver : Premium 1 an à 12,99 € au lieu de 24,99 €, jusqu'au 25/02 (badge -48 %) ; Bob cite « du 1er novembre au 25 février et du 1er juillet au 15 août » ; email « ❄️ Premium 1 an à 12,99 € — jusqu'au 25/02 ». Avant le 1/11 : pas d'offre.</t>
-        </is>
-      </c>
-      <c r="F85" s="4" t="inlineStr">
-        <is>
-          <t>Gratuit</t>
-        </is>
-      </c>
-      <c r="G85" s="6" t="inlineStr">
-        <is>
-          <t>À tester</t>
-        </is>
-      </c>
-      <c r="H85" s="6" t="inlineStr">
-        <is>
-          <t>Sur STA le 28/10/2026 (décision de Jordan du 28/10 : l'offre d'hiver commence le 1/11 chaque année).</t>
-        </is>
-      </c>
-      <c r="I85" s="6" t="n"/>
-    </row>
-    <row r="86">
-      <c r="A86" s="4" t="inlineStr">
-        <is>
-          <t>82</t>
-        </is>
-      </c>
-      <c r="B86" s="5" t="inlineStr">
-        <is>
-          <t>Mesure — abonnements Premium comptés</t>
-        </is>
-      </c>
-      <c r="C86" s="4" t="inlineStr">
-        <is>
-          <t>Supabase PROD (funnel_events) ; point KPI du lundi</t>
-        </is>
-      </c>
-      <c r="D86" s="4" t="inlineStr">
-        <is>
-          <t>Après le premier abonnement payant pris en prod (mensuel ou annuel) : regarder funnel_events, étape premium_souscrit.</t>
-        </is>
-      </c>
-      <c r="E86" s="4" t="inlineStr">
-        <is>
-          <t>Une ligne par abonnement pris, sans identifiant d'utilisateur, avec la formule (mensuel ou annuel) et l'offre (saison-hiver pendant l'offre) ; Premium activé même si la mesure échoue (alerte « Mesure — abonnement Premium non compté »).</t>
-        </is>
-      </c>
-      <c r="F86" s="4" t="inlineStr">
-        <is>
-          <t>Admin</t>
-        </is>
-      </c>
-      <c r="G86" s="6" t="inlineStr">
-        <is>
-          <t>À tester</t>
-        </is>
-      </c>
-      <c r="H86" s="6" t="inlineStr">
-        <is>
-          <t>Sur STA le 28/10/2026 (décision de Jordan du 28/10 : point KPI du lundi). Vérifié sur STA le 29/10 : abonnement de test mensuel compté (premium_souscrit, offre vide avant le 1/11). Abonnement de test annuel (24,99 €) réussi par Jordan sur STA le 30/10 : compté (formule annuel), Premium activé, aucune erreur.</t>
-        </is>
-      </c>
-      <c r="I86" s="6" t="n"/>
-    </row>
-    <row r="87">
-      <c r="A87" s="4" t="inlineStr">
-        <is>
-          <t>83</t>
-        </is>
-      </c>
-      <c r="B87" s="5" t="inlineStr">
-        <is>
-          <t>Mesure — articles qui mènent à l'app</t>
-        </is>
-      </c>
-      <c r="C87" s="4" t="inlineStr">
-        <is>
-          <t>Pages Conseils ; Supabase PROD (funnel_events)</t>
-        </is>
-      </c>
-      <c r="D87" s="4" t="inlineStr">
-        <is>
-          <t>Sans être connecté, sur téléphone : ouvrir un article depuis un lien suivi (ex. groupe Facebook), puis toucher « Diagnostic gratuit » dans le même onglet ; regarder funnel_events.</t>
-        </is>
-      </c>
-      <c r="E87" s="4" t="inlineStr">
-        <is>
-          <t>Une ligne conseils_vue (page = article, source = origine) puis la page_view de /essai avec le même identifiant de visite ; un rechargement ne recompte pas l'article ; rien pour un compte connecté.</t>
-        </is>
-      </c>
-      <c r="F87" s="4" t="inlineStr">
-        <is>
-          <t>Admin</t>
-        </is>
-      </c>
-      <c r="G87" s="6" t="inlineStr">
-        <is>
-          <t>À tester</t>
-        </is>
-      </c>
-      <c r="H87" s="6" t="inlineStr">
-        <is>
-          <t>Sur STA le 28/10/2026 (demande de Jordan du 28/10 : faire atterrir le flux du site dans l'app).</t>
-        </is>
-      </c>
-      <c r="I87" s="6" t="n"/>
-    </row>
-    <row r="88">
-      <c r="A88" s="4" t="inlineStr">
-        <is>
-          <t>84</t>
-        </is>
-      </c>
-      <c r="B88" s="5" t="inlineStr">
-        <is>
-          <t>Conseils — l'app dans les articles (prod le 22/11)</t>
-        </is>
-      </c>
-      <c r="C88" s="4" t="inlineStr">
-        <is>
-          <t>Pages Conseils (article, rubrique, Qui sommes-nous) ; Supabase PROD (funnel_events)</t>
-        </is>
-      </c>
-      <c r="D88" s="4" t="inlineStr">
-        <is>
-          <t>Sans être connecté, sur un téléphone Android puis sur ordinateur : ouvrir un article ; regarder le bandeau sous le titre, les 3 encarts et le bouton fixe ; toucher un encart ; ouvrir la rubrique et Qui sommes-nous.</t>
-        </is>
-      </c>
-      <c r="E88" s="4" t="inlineStr">
-        <is>
-          <t>Bandeau sous le titre sans cacher le texte (« Télécharger sur Google Play » seulement dans le navigateur d'un téléphone Android) ; encarts après « En bref », au milieu et à la fin, thèmes variés selon l'article (src/lib/argumentsApp.json) ; bouton fixe « Ouvrir l'app gratuite » sur téléphone seulement ; grille « Ce que fait l'app » ; l'encart touché ouvre l'app et sa page_view porte encart = thème-position ; aucune page plus large que l'écran.</t>
-        </is>
-      </c>
-      <c r="F88" s="4" t="inlineStr">
-        <is>
-          <t>Non connecté</t>
-        </is>
-      </c>
-      <c r="G88" s="6" t="inlineStr">
-        <is>
-          <t>À tester</t>
-        </is>
-      </c>
-      <c r="H88" s="6" t="inlineStr">
-        <is>
-          <t>Sur STA le 30/10/2026 (décisions de Jordan des 28 et 30/10) ; bandeau en 2 versions à départager sur les visuels.</t>
-        </is>
-      </c>
-      <c r="I88" s="6" t="n"/>
-    </row>
-    <row r="89">
-      <c r="A89" s="4" t="inlineStr">
-        <is>
-          <t>85</t>
-        </is>
-      </c>
-      <c r="B89" s="5" t="inlineStr">
-        <is>
-          <t>Alignement PROD / STA</t>
-        </is>
-      </c>
-      <c r="C89" s="4" t="inlineStr">
-        <is>
-          <t>Git</t>
-        </is>
-      </c>
-      <c r="D89" s="4" t="inlineStr">
-        <is>
-          <t>Après la fusion : git diff --quiet origin/main origin/Staging.</t>
-        </is>
-      </c>
-      <c r="E89" s="4" t="inlineStr">
-        <is>
-          <t>Aucune différence.</t>
-        </is>
-      </c>
-      <c r="F89" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G89" s="6" t="inlineStr">
-        <is>
-          <t>À tester</t>
-        </is>
-      </c>
-      <c r="H89" s="6" t="n"/>
-      <c r="I89" s="6" t="n"/>
-    </row>
-    <row r="90">
-      <c r="A90" s="4" t="inlineStr">
-        <is>
-          <t>86</t>
-        </is>
-      </c>
-      <c r="B90" s="5" t="inlineStr">
-        <is>
-          <t>Base de données PROD</t>
-        </is>
-      </c>
-      <c r="C90" s="4" t="inlineStr">
-        <is>
-          <t>Supabase PROD</t>
-        </is>
-      </c>
-      <c r="D90" s="4" t="inlineStr">
-        <is>
-          <t>Vérifier les tables codes et parrainages.</t>
-        </is>
-      </c>
-      <c r="E90" s="4" t="inlineStr">
-        <is>
-          <t>Tables présentes (créées le 05/10 sur les deux projets).</t>
-        </is>
-      </c>
-      <c r="F90" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G90" s="6" t="inlineStr">
-        <is>
-          <t>À tester</t>
-        </is>
-      </c>
-      <c r="H90" s="6" t="n"/>
-      <c r="I90" s="6" t="n"/>
-    </row>
-    <row r="91">
-      <c r="A91" s="4" t="inlineStr">
-        <is>
-          <t>87</t>
-        </is>
-      </c>
-      <c r="B91" s="5" t="inlineStr">
-        <is>
-          <t>Règle de travail de décembre</t>
-        </is>
-      </c>
-      <c r="C91" s="4" t="inlineStr">
-        <is>
-          <t>CLAUDE.md</t>
-        </is>
-      </c>
-      <c r="D91" s="4" t="inlineStr">
-        <is>
-          <t>Après la mise en prod : retirer le paragraphe « Jusqu'à décembre 2026 ».</t>
-        </is>
-      </c>
-      <c r="E91" s="4" t="inlineStr">
-        <is>
-          <t>STA redevient identique à la PROD.</t>
-        </is>
-      </c>
-      <c r="F91" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G91" s="6" t="inlineStr">
-        <is>
-          <t>À tester</t>
-        </is>
-      </c>
-      <c r="H91" s="6" t="n"/>
-      <c r="I91" s="6" t="n"/>
-    </row>
+    <row r="72"/>
+    <row r="73"/>
+    <row r="74"/>
+    <row r="75"/>
+    <row r="76"/>
+    <row r="77"/>
+    <row r="78"/>
+    <row r="79"/>
+    <row r="80"/>
+    <row r="81"/>
+    <row r="82"/>
+    <row r="83"/>
+    <row r="84"/>
+    <row r="85"/>
+    <row r="86"/>
+    <row r="87"/>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A2:I2"/>
   </mergeCells>
-  <conditionalFormatting sqref="G5:G91">
+  <conditionalFormatting sqref="G5:G67">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"OK"</formula>
     </cfRule>
@@ -4088,7 +3088,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="G5:G91" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="G5:G67" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"À tester,OK,KO,Non testable"</formula1>
     </dataValidation>
   </dataValidations>
@@ -4102,7 +3102,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I47"/>
+  <dimension ref="A1:I71"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -5982,11 +4982,995 @@
       </c>
       <c r="I47" s="8" t="n"/>
     </row>
+    <row r="48">
+      <c r="A48" s="4" t="n">
+        <v>44</v>
+      </c>
+      <c r="B48" s="5" t="inlineStr">
+        <is>
+          <t>Météo gratuite — Dashboard</t>
+        </is>
+      </c>
+      <c r="C48" s="4" t="inlineStr">
+        <is>
+          <t>Dashboard</t>
+        </is>
+      </c>
+      <c r="D48" s="4" t="inlineStr">
+        <is>
+          <t>Compte gratuit : regarder la carte météo à côté du score.</t>
+        </is>
+      </c>
+      <c r="E48" s="4" t="inlineStr">
+        <is>
+          <t>Ville, icône, température et temps du jour ; « 🔒 Vent, pluie, alertes » + bouton Premium.</t>
+        </is>
+      </c>
+      <c r="F48" s="4" t="inlineStr">
+        <is>
+          <t>Gratuit (essai terminé)</t>
+        </is>
+      </c>
+      <c r="G48" s="6" t="inlineStr">
+        <is>
+          <t>À tester</t>
+        </is>
+      </c>
+      <c r="H48" s="6" t="inlineStr">
+        <is>
+          <t>Validé sur STA le 09/10/2026 par Jordan ; à revérifier en prod. Passée en prod le 31/10/2026 avec la refonte (décision de Jordan du 28/10).</t>
+        </is>
+      </c>
+      <c r="I48" s="8" t="n"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="4" t="n">
+        <v>45</v>
+      </c>
+      <c r="B49" s="5" t="inlineStr">
+        <is>
+          <t>Météo gratuite — Aujourd'hui</t>
+        </is>
+      </c>
+      <c r="C49" s="4" t="inlineStr">
+        <is>
+          <t>Aujourd'hui</t>
+        </is>
+      </c>
+      <c r="D49" s="4" t="inlineStr">
+        <is>
+          <t>Compte gratuit : bloc météo en haut de page.</t>
+        </is>
+      </c>
+      <c r="E49" s="4" t="inlineStr">
+        <is>
+          <t>Température et temps du jour ; « 🔒 Pluie, humidité et vent : Premium » ; mention Open-Meteo.</t>
+        </is>
+      </c>
+      <c r="F49" s="4" t="inlineStr">
+        <is>
+          <t>Gratuit (essai terminé)</t>
+        </is>
+      </c>
+      <c r="G49" s="6" t="inlineStr">
+        <is>
+          <t>À tester</t>
+        </is>
+      </c>
+      <c r="H49" s="6" t="inlineStr">
+        <is>
+          <t>Validé sur STA le 09/10/2026 par Jordan ; à revérifier en prod. Passée en prod le 31/10/2026 avec la refonte (décision de Jordan du 28/10).</t>
+        </is>
+      </c>
+      <c r="I49" s="8" t="n"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="4" t="n">
+        <v>46</v>
+      </c>
+      <c r="B50" s="5" t="inlineStr">
+        <is>
+          <t>Météo Premium inchangée</t>
+        </is>
+      </c>
+      <c r="C50" s="4" t="inlineStr">
+        <is>
+          <t>Dashboard, Aujourd'hui</t>
+        </is>
+      </c>
+      <c r="D50" s="4" t="inlineStr">
+        <is>
+          <t>Compte Premium : mêmes écrans.</t>
+        </is>
+      </c>
+      <c r="E50" s="4" t="inlineStr">
+        <is>
+          <t>Météo complète (vent, pluie, humidité, station si connectée).</t>
+        </is>
+      </c>
+      <c r="F50" s="4" t="inlineStr">
+        <is>
+          <t>Premium</t>
+        </is>
+      </c>
+      <c r="G50" s="6" t="inlineStr">
+        <is>
+          <t>À tester</t>
+        </is>
+      </c>
+      <c r="H50" s="6" t="inlineStr">
+        <is>
+          <t>Validé sur STA le 09/10/2026 par Jordan ; à revérifier en prod. Passée en prod le 31/10/2026 avec la refonte (décision de Jordan du 28/10).</t>
+        </is>
+      </c>
+      <c r="I50" s="8" t="n"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="4" t="n">
+        <v>47</v>
+      </c>
+      <c r="B51" s="5" t="inlineStr">
+        <is>
+          <t>Plus de « IA » — Diagnostic</t>
+        </is>
+      </c>
+      <c r="C51" s="4" t="inlineStr">
+        <is>
+          <t>Diagnostic</t>
+        </is>
+      </c>
+      <c r="D51" s="4" t="inlineStr">
+        <is>
+          <t>Lire l'en-tête, l'écran Premium, le bouton et les étapes.</t>
+        </is>
+      </c>
+      <c r="E51" s="4" t="inlineStr">
+        <is>
+          <t>« Bob diagnostique votre gazon », « Ce que Bob fait pour vous », « Lancer le diagnostic de Bob » ; aucun « IA ».</t>
+        </is>
+      </c>
+      <c r="F51" s="4" t="inlineStr">
+        <is>
+          <t>Gratuit et Premium</t>
+        </is>
+      </c>
+      <c r="G51" s="6" t="inlineStr">
+        <is>
+          <t>À tester</t>
+        </is>
+      </c>
+      <c r="H51" s="6" t="inlineStr">
+        <is>
+          <t>Validé sur STA le 09/10/2026 par Jordan ; à revérifier en prod. Passée en prod le 31/10/2026 avec la refonte (décision de Jordan du 28/10).</t>
+        </is>
+      </c>
+      <c r="I51" s="8" t="n"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="4" t="n">
+        <v>48</v>
+      </c>
+      <c r="B52" s="5" t="inlineStr">
+        <is>
+          <t>Plus de « IA » — Comparatif et Abonnement</t>
+        </is>
+      </c>
+      <c r="C52" s="4" t="inlineStr">
+        <is>
+          <t>Comparatif, Subscribe, SubscribeSuccess</t>
+        </is>
+      </c>
+      <c r="D52" s="4" t="inlineStr">
+        <is>
+          <t>Lire les listes d'avantages.</t>
+        </is>
+      </c>
+      <c r="E52" s="4" t="inlineStr">
+        <is>
+          <t>« Bob, votre assistant gazon 24/7 », « Diagnostic photo par Bob », « Recommandations personnalisées de Bob », « Calcul d'arrosage précis ».</t>
+        </is>
+      </c>
+      <c r="F52" s="4" t="inlineStr">
+        <is>
+          <t>Gratuit</t>
+        </is>
+      </c>
+      <c r="G52" s="6" t="inlineStr">
+        <is>
+          <t>À tester</t>
+        </is>
+      </c>
+      <c r="H52" s="6" t="inlineStr">
+        <is>
+          <t>Validé sur STA le 09/10/2026 par Jordan ; à revérifier en prod. Passée en prod le 31/10/2026 avec la refonte (décision de Jordan du 28/10).</t>
+        </is>
+      </c>
+      <c r="I52" s="8" t="n"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="4" t="n">
+        <v>49</v>
+      </c>
+      <c r="B53" s="5" t="inlineStr">
+        <is>
+          <t>Plus de « IA » — Aujourd'hui</t>
+        </is>
+      </c>
+      <c r="C53" s="4" t="inlineStr">
+        <is>
+          <t>Aujourd'hui</t>
+        </is>
+      </c>
+      <c r="D53" s="4" t="inlineStr">
+        <is>
+          <t>Bloc des recommandations.</t>
+        </is>
+      </c>
+      <c r="E53" s="4" t="inlineStr">
+        <is>
+          <t>Titre « 🤖 Recommandation Bob » ; messages « recommandation de Bob », « Impossible de contacter Bob ».</t>
+        </is>
+      </c>
+      <c r="F53" s="4" t="inlineStr">
+        <is>
+          <t>Gratuit et Premium</t>
+        </is>
+      </c>
+      <c r="G53" s="6" t="inlineStr">
+        <is>
+          <t>À tester</t>
+        </is>
+      </c>
+      <c r="H53" s="6" t="inlineStr">
+        <is>
+          <t>Validé sur STA le 09/10/2026 par Jordan ; à revérifier en prod. Passée en prod le 31/10/2026 avec la refonte (décision de Jordan du 28/10).</t>
+        </is>
+      </c>
+      <c r="I53" s="8" t="n"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="4" t="n">
+        <v>50</v>
+      </c>
+      <c r="B54" s="5" t="inlineStr">
+        <is>
+          <t>Plus de « IA » — autres écrans</t>
+        </is>
+      </c>
+      <c r="C54" s="4" t="inlineStr">
+        <is>
+          <t>Onboarding, Accueil, Démo, Badges, Score</t>
+        </is>
+      </c>
+      <c r="D54" s="4" t="inlineStr">
+        <is>
+          <t>Parcourir l'onboarding, la page d'accueil, la démo, la galerie de badges, la fenêtre du score.</t>
+        </is>
+      </c>
+      <c r="E54" s="4" t="inlineStr">
+        <is>
+          <t>« Planning personnalisé », « Bob, votre assistant gazon », « Arrosage au bon moment », « Diagnostic photo par Bob » ; aucun « IA » ni « intelligent ».</t>
+        </is>
+      </c>
+      <c r="F54" s="4" t="inlineStr">
+        <is>
+          <t>Divers</t>
+        </is>
+      </c>
+      <c r="G54" s="6" t="inlineStr">
+        <is>
+          <t>À tester</t>
+        </is>
+      </c>
+      <c r="H54" s="6" t="inlineStr">
+        <is>
+          <t>Validé sur STA le 09/10/2026 par Jordan ; à revérifier en prod. Passée en prod le 31/10/2026 avec la refonte (décision de Jordan du 28/10).</t>
+        </is>
+      </c>
+      <c r="I54" s="8" t="n"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="4" t="n">
+        <v>51</v>
+      </c>
+      <c r="B55" s="5" t="inlineStr">
+        <is>
+          <t>Plus de « IA » — messages d'erreur</t>
+        </is>
+      </c>
+      <c r="C55" s="4" t="inlineStr">
+        <is>
+          <t>Diagnostic, recommandations</t>
+        </is>
+      </c>
+      <c r="D55" s="4" t="inlineStr">
+        <is>
+          <t>Si possible, provoquer une indisponibilité (ou relire les messages).</t>
+        </is>
+      </c>
+      <c r="E55" s="4" t="inlineStr">
+        <is>
+          <t>« Bob est momentanément indisponible » ; « recommandations de Bob ».</t>
+        </is>
+      </c>
+      <c r="F55" s="4" t="inlineStr">
+        <is>
+          <t>Divers</t>
+        </is>
+      </c>
+      <c r="G55" s="6" t="inlineStr">
+        <is>
+          <t>À tester</t>
+        </is>
+      </c>
+      <c r="H55" s="6" t="inlineStr">
+        <is>
+          <t>Validé sur STA le 09/10/2026 par Jordan ; à revérifier en prod. Passée en prod le 31/10/2026 avec la refonte (décision de Jordan du 28/10).</t>
+        </is>
+      </c>
+      <c r="I55" s="8" t="n"/>
+    </row>
+    <row r="56">
+      <c r="A56" s="4" t="n">
+        <v>52</v>
+      </c>
+      <c r="B56" s="5" t="inlineStr">
+        <is>
+          <t>Refonte — barre du bas</t>
+        </is>
+      </c>
+      <c r="C56" s="4" t="inlineStr">
+        <is>
+          <t>Toute l'app (connecté)</t>
+        </is>
+      </c>
+      <c r="D56" s="4" t="inlineStr">
+        <is>
+          <t>Se connecter et regarder la barre du bas pendant la ligue d'hiver, puis après le 30/01.</t>
+        </is>
+      </c>
+      <c r="E56" s="4" t="inlineStr">
+        <is>
+          <t>4 onglets : Accueil, Aujourd'hui, Diagnostic, Mon gazon, plus « Quiz » jusqu'au 30/01 ; plus d'onglets Produits ni Classement (Produits reste ouvert depuis Mon gazon).</t>
+        </is>
+      </c>
+      <c r="F56" s="4" t="inlineStr">
+        <is>
+          <t>Gratuit et Premium</t>
+        </is>
+      </c>
+      <c r="G56" s="6" t="inlineStr">
+        <is>
+          <t>À tester</t>
+        </is>
+      </c>
+      <c r="H56" s="6" t="inlineStr">
+        <is>
+          <t>Sur STA le 26/10/2026 (décisions de Jordan du 26/10). Testé par Jordan sur STA le 29/10 : OK. Passée en prod le 31/10/2026 avec la refonte (décision de Jordan du 28/10).</t>
+        </is>
+      </c>
+      <c r="I56" s="8" t="n"/>
+    </row>
+    <row r="57">
+      <c r="A57" s="4" t="n">
+        <v>53</v>
+      </c>
+      <c r="B57" s="5" t="inlineStr">
+        <is>
+          <t>Refonte — accueil : résumé du jour</t>
+        </is>
+      </c>
+      <c r="C57" s="4" t="inlineStr">
+        <is>
+          <t>Accueil</t>
+        </is>
+      </c>
+      <c r="D57" s="4" t="inlineStr">
+        <is>
+          <t>Comparer la carte « Aujourd'hui » de l'accueil avec l'onglet Aujourd'hui, un jour avec des actions puis un jour sans ; toucher la carte.</t>
+        </is>
+      </c>
+      <c r="E57" s="4" t="inlineStr">
+        <is>
+          <t>Mêmes actions que l'onglet Aujourd'hui ; sans action : « Rien à faire aujourd'hui » et la prochaine action ; la carte ouvre Aujourd'hui.</t>
+        </is>
+      </c>
+      <c r="F57" s="4" t="inlineStr">
+        <is>
+          <t>Tous</t>
+        </is>
+      </c>
+      <c r="G57" s="6" t="inlineStr">
+        <is>
+          <t>À tester</t>
+        </is>
+      </c>
+      <c r="H57" s="6" t="inlineStr">
+        <is>
+          <t>Sur STA le 26/10/2026 (décisions de Jordan du 26/10). Testé par Jordan sur STA le 29/10 : OK. Passée en prod le 31/10/2026 avec la refonte (décision de Jordan du 28/10).</t>
+        </is>
+      </c>
+      <c r="I57" s="8" t="n"/>
+    </row>
+    <row r="58">
+      <c r="A58" s="4" t="n">
+        <v>54</v>
+      </c>
+      <c r="B58" s="5" t="inlineStr">
+        <is>
+          <t>Refonte — série et GreenPoints</t>
+        </is>
+      </c>
+      <c r="C58" s="4" t="inlineStr">
+        <is>
+          <t>Accueil, Mon gazon</t>
+        </is>
+      </c>
+      <c r="D58" s="4" t="inlineStr">
+        <is>
+          <t>Ouvrir l'app un nouveau jour en restant sur l'accueil ; toucher la carte série et GreenPoints.</t>
+        </is>
+      </c>
+      <c r="E58" s="4" t="inlineStr">
+        <is>
+          <t>Série et GreenPoints de connexion comptés dès l'accueil, une fois par jour ; la carte ouvre Mon gazon directement sur « Mes progrès ».</t>
+        </is>
+      </c>
+      <c r="F58" s="4" t="inlineStr">
+        <is>
+          <t>Tous</t>
+        </is>
+      </c>
+      <c r="G58" s="6" t="inlineStr">
+        <is>
+          <t>À tester</t>
+        </is>
+      </c>
+      <c r="H58" s="6" t="inlineStr">
+        <is>
+          <t>Sur STA le 26/10/2026 (décisions de Jordan du 26/10). Testé par Jordan sur STA le 29/10 : OK. Passée en prod le 31/10/2026 avec la refonte (décision de Jordan du 28/10).</t>
+        </is>
+      </c>
+      <c r="I58" s="8" t="n"/>
+    </row>
+    <row r="59">
+      <c r="A59" s="4" t="n">
+        <v>55</v>
+      </c>
+      <c r="B59" s="5" t="inlineStr">
+        <is>
+          <t>Refonte — Mon gazon épuré</t>
+        </is>
+      </c>
+      <c r="C59" s="4" t="inlineStr">
+        <is>
+          <t>Mon gazon</t>
+        </is>
+      </c>
+      <c r="D59" s="4" t="inlineStr">
+        <is>
+          <t>Parcourir Mon gazon avec un compte gratuit puis Premium ; déplier « Pourquoi ce score ? », « Partager », les badges et, en Premium, le débit de l'arroseur ; retirer une action notée par erreur ; toucher chaque outil ; ouvrir l'ancienne adresse /history.</t>
+        </is>
+      </c>
+      <c r="E59" s="4" t="inlineStr">
+        <is>
+          <t>Dans l'ordre : score santé compact (« Pourquoi ce score ? » : 4 critères et problèmes prioritaires ; « Partager »), évolution du score compacte (courbe, actions de l'année en une ligne, bilan de saison), « Mes actions » (5 dernières, « Voir tout », retrait), « Mes progrès » en une carte (série, GreenPoints, classement ou renvoi vers le Quiz pendant la ligue), badges en une ligne (« Voir tout »), « Mes outils » (plan gazon, équipements, semer ou regarnir, produits et dépenses ; parrainage avec la mise en prod de décembre), « Mon profil » (complétude, infos, débit de l'arroseur en Premium), « Avec Premium » pour un compte gratuit ; plus de conseil du mois, plan du mois, produits recommandés ni bloc de calibrage ; /history n'existe plus.</t>
+        </is>
+      </c>
+      <c r="F59" s="4" t="inlineStr">
+        <is>
+          <t>Tous</t>
+        </is>
+      </c>
+      <c r="G59" s="6" t="inlineStr">
+        <is>
+          <t>À tester</t>
+        </is>
+      </c>
+      <c r="H59" s="6" t="inlineStr">
+        <is>
+          <t>Sur STA le 26/10/2026 (décisions de Jordan du 26/10). Testé par Jordan sur STA le 29/10 : OK, mais page jugée trop chargée. Épurée le 29/10 (décision de Jordan) : 19 blocs → 7, « Mes progrès » en une carte ; validée par Jordan sur STA le 29/10. Passée en prod le 31/10/2026 avec la refonte (décision de Jordan du 28/10).</t>
+        </is>
+      </c>
+      <c r="I59" s="8" t="n"/>
+    </row>
+    <row r="60">
+      <c r="A60" s="4" t="n">
+        <v>56</v>
+      </c>
+      <c r="B60" s="5" t="inlineStr">
+        <is>
+          <t>Refonte — Premium sur l'accueil, le diagnostic et les équipements</t>
+        </is>
+      </c>
+      <c r="C60" s="4" t="inlineStr">
+        <is>
+          <t>Accueil, Diagnostic, Mes équipements</t>
+        </is>
+      </c>
+      <c r="D60" s="4" t="inlineStr">
+        <is>
+          <t>Regarder l'accueil et l'onglet Diagnostic avec un compte gratuit, puis Premium, puis dans l'app Android ; ouvrir Mes équipements avec un compte gratuit (avec et sans équipement déjà connecté), puis Premium.</t>
+        </is>
+      </c>
+      <c r="E60" s="4" t="inlineStr">
+        <is>
+          <t>Gratuit : carte « Avec Premium » (avantages de Premium sans les paysagistes, puis le prix ou, pendant sa période, l'offre de saison) ; Premium : raccourcis « Mes équipements » et « Mon plan annuel » ; app Android : pas de carte d'achat ; Mes équipements en gratuit : « Inclus dans Premium » et « Découvrir Premium » (pas dans l'app Android), aucune connexion ni demande d'équipement non listé, équipement déjà connecté seulement déconnectable ; le serveur refuse aussi connexions et commandes sans Premium ; Premium : connexions inchangées.</t>
+        </is>
+      </c>
+      <c r="F60" s="4" t="inlineStr">
+        <is>
+          <t>Gratuit, Premium, app Android</t>
+        </is>
+      </c>
+      <c r="G60" s="6" t="inlineStr">
+        <is>
+          <t>À tester</t>
+        </is>
+      </c>
+      <c r="H60" s="6" t="inlineStr">
+        <is>
+          <t>Sur STA le 26/10/2026 (décisions de Jordan du 26/10). Testé par Jordan sur STA le 29/10 : raccourcis Premium OK (compte gratuit et app Android à voir). Mes équipements ouverts aux comptes gratuits (constat de Jordan le 29/10) : verrou Premium ajouté le 29/10 (STA et version de prod), vérifié par Jordan sur STA le 29/10 ; demande d'équipement non listé retirée de la page d'un compte gratuit le 29/10 (décision de Jordan). Compte gratuit testé par Jordan sur STA le 30/10 : OK (carte « Avec Premium » de l'accueil, du diagnostic et de Mon gazon ; Mes équipements verrouillé, sans formulaire). App Android : à vérifier après la mise en prod. Passée en prod le 31/10/2026 avec la refonte (décision de Jordan du 28/10).</t>
+        </is>
+      </c>
+      <c r="I60" s="8" t="n"/>
+    </row>
+    <row r="61">
+      <c r="A61" s="4" t="n">
+        <v>57</v>
+      </c>
+      <c r="B61" s="5" t="inlineStr">
+        <is>
+          <t>Refonte — Choisir son niveau</t>
+        </is>
+      </c>
+      <c r="C61" s="4" t="inlineStr">
+        <is>
+          <t>/subscribe</t>
+        </is>
+      </c>
+      <c r="D61" s="4" t="inlineStr">
+        <is>
+          <t>Ouvrir la page avec un compte gratuit, puis un compte en essai ; aller jusqu'au paiement Stripe sans payer ; ouvrir l'adresse /subscribe avec un compte abonné, Premium offert ou admin.</t>
+        </is>
+      </c>
+      <c r="E61" s="4" t="inlineStr">
+        <is>
+          <t>3 niveaux (Visiteur, Gratuit, Premium) ; « Ton niveau » ou « Ton essai : encore N jours » ; compte déjà Premium (abonné, Premium offert, admin) : renvoyé à l'accueil, la page ne s'affiche jamais ; formules, mentions légales et paiement inchangés.</t>
+        </is>
+      </c>
+      <c r="F61" s="4" t="inlineStr">
+        <is>
+          <t>Gratuit, essai, Premium</t>
+        </is>
+      </c>
+      <c r="G61" s="6" t="inlineStr">
+        <is>
+          <t>À tester</t>
+        </is>
+      </c>
+      <c r="H61" s="6" t="inlineStr">
+        <is>
+          <t>Sur STA le 26/10/2026 (décisions de Jordan du 26/10). Paiement de test réussi sur STA le 29/10 (mensuel à 2,99 €, bac à sable Stripe). Abonné : aucun lien vers la page (voulu). Test de Jordan le 29/10 avec son compte admin : offres affichées au lieu de « Tu es déjà Premium » (compte admin non reconnu comme Premium sur cette page) ; corrigé le 29/10, puis décision de Jordan le soir même : un compte déjà Premium n'arrive jamais sur la page (renvoi à l'accueil), STA et version de prod. Passée en prod le 31/10/2026 avec la refonte (décision de Jordan du 28/10).</t>
+        </is>
+      </c>
+      <c r="I61" s="8" t="n"/>
+    </row>
+    <row r="62">
+      <c r="A62" s="4" t="n">
+        <v>58</v>
+      </c>
+      <c r="B62" s="5" t="inlineStr">
+        <is>
+          <t>Refonte — plan annuel inclus dans Premium</t>
+        </is>
+      </c>
+      <c r="C62" s="4" t="inlineStr">
+        <is>
+          <t>Mon gazon → Mon plan gazon ; CGV 7 bis</t>
+        </is>
+      </c>
+      <c r="D62" s="4" t="inlineStr">
+        <is>
+          <t>Ouvrir le plan avec un compte gratuit, un compte Premium et un compte ayant acheté un plan à 0,99 €.</t>
+        </is>
+      </c>
+      <c r="E62" s="4" t="inlineStr">
+        <is>
+          <t>Gratuit : aperçu d'un mois et « Inclus dans Premium », aucune vente ; Premium et plans déjà achetés : les 12 mois et le PDF ; CGV 7 bis réécrit.</t>
+        </is>
+      </c>
+      <c r="F62" s="4" t="inlineStr">
+        <is>
+          <t>Gratuit, Premium, acheteur</t>
+        </is>
+      </c>
+      <c r="G62" s="6" t="inlineStr">
+        <is>
+          <t>À tester</t>
+        </is>
+      </c>
+      <c r="H62" s="6" t="inlineStr">
+        <is>
+          <t>Sur STA le 26/10/2026 (décisions de Jordan du 26/10). Testé par Jordan sur STA le 29/10 : plan Premium OK (compte gratuit à voir). Compte gratuit testé par Jordan sur STA le 30/10 : OK. Passée en prod le 31/10/2026 avec la refonte (décision de Jordan du 28/10).</t>
+        </is>
+      </c>
+      <c r="I62" s="8" t="n"/>
+    </row>
+    <row r="63">
+      <c r="A63" s="4" t="n">
+        <v>59</v>
+      </c>
+      <c r="B63" s="5" t="inlineStr">
+        <is>
+          <t>Refonte — accueil visiteur</t>
+        </is>
+      </c>
+      <c r="C63" s="4" t="inlineStr">
+        <is>
+          <t>mongazon360.fr (non connecté)</t>
+        </is>
+      </c>
+      <c r="D63" s="4" t="inlineStr">
+        <is>
+          <t>Saisir une commune (puis une commune homonyme), essayer « Utiliser ma position », ouvrir un article, « Prendre une photo », « Créer mon compte gratuit », puis le lien de connexion ; revenir le lendemain.</t>
+        </is>
+      </c>
+      <c r="E63" s="4" t="inlineStr">
+        <is>
+          <t>Météo du jour de la commune (température, ciel) ; conseil de Bob du jour ; 3 articles de la saison ; barre Accueil, Conseils, Diagnostic, Compte (aussi sur l'essai du diagnostic, la création de compte et la connexion, onglet Compte en surbrillance) ; commune retrouvée à la visite suivante.</t>
+        </is>
+      </c>
+      <c r="F63" s="4" t="inlineStr">
+        <is>
+          <t>Non connecté</t>
+        </is>
+      </c>
+      <c r="G63" s="6" t="inlineStr">
+        <is>
+          <t>À tester</t>
+        </is>
+      </c>
+      <c r="H63" s="6" t="inlineStr">
+        <is>
+          <t>Sur STA le 26/10/2026 (décisions de Jordan du 26/10). Testé par Jordan sur STA le 29/10 : OK ; barre du bas ajoutée le 29/10 à la création de compte et à la connexion (demande de Jordan), vérifiée par Jordan sur STA le 30/10 : OK. Passée en prod le 31/10/2026 avec la refonte (décision de Jordan du 28/10).</t>
+        </is>
+      </c>
+      <c r="I63" s="8" t="n"/>
+    </row>
+    <row r="64">
+      <c r="A64" s="4" t="n">
+        <v>60</v>
+      </c>
+      <c r="B64" s="5" t="inlineStr">
+        <is>
+          <t>Refonte — démo retirée</t>
+        </is>
+      </c>
+      <c r="C64" s="4" t="inlineStr">
+        <is>
+          <t>mongazon360.fr/demo ; plan du site</t>
+        </is>
+      </c>
+      <c r="D64" s="4" t="inlineStr">
+        <is>
+          <t>Ouvrir l'ancienne adresse /demo ; lire sitemap.xml.</t>
+        </is>
+      </c>
+      <c r="E64" s="4" t="inlineStr">
+        <is>
+          <t>Redirection vers l'accueil ; /demo absente du plan du site.</t>
+        </is>
+      </c>
+      <c r="F64" s="4" t="inlineStr">
+        <is>
+          <t>Non connecté</t>
+        </is>
+      </c>
+      <c r="G64" s="6" t="inlineStr">
+        <is>
+          <t>À tester</t>
+        </is>
+      </c>
+      <c r="H64" s="6" t="inlineStr">
+        <is>
+          <t>Sur STA le 26/10/2026 (décisions de Jordan du 26/10). Vérifié sur STA le 29/10 : /demo redirigée vers l'accueil (308), absente du plan du site. Passée en prod le 31/10/2026 avec la refonte (décision de Jordan du 28/10).</t>
+        </is>
+      </c>
+      <c r="I64" s="8" t="n"/>
+    </row>
+    <row r="65">
+      <c r="A65" s="4" t="n">
+        <v>61</v>
+      </c>
+      <c r="B65" s="5" t="inlineStr">
+        <is>
+          <t>Refonte — carte Nouveautés</t>
+        </is>
+      </c>
+      <c r="C65" s="4" t="inlineStr">
+        <is>
+          <t>Accueil ; src/components/CarteNouveautes.jsx</t>
+        </is>
+      </c>
+      <c r="D65" s="4" t="inlineStr">
+        <is>
+          <t>Le jour de la mise en prod : régler MISE_EN_PROD sur cette date (commit), puis ouvrir l'app avec un ancien compte et un compte créé ensuite.</t>
+        </is>
+      </c>
+      <c r="E65" s="4" t="inlineStr">
+        <is>
+          <t>Carte « Mongazon360 fait peau neuve » pour l'ancien compte, fermée pour de bon par « J'ai compris » ; rien pour le nouveau compte.</t>
+        </is>
+      </c>
+      <c r="F65" s="4" t="inlineStr">
+        <is>
+          <t>Ancien et nouveau compte</t>
+        </is>
+      </c>
+      <c r="G65" s="6" t="inlineStr">
+        <is>
+          <t>À tester</t>
+        </is>
+      </c>
+      <c r="H65" s="6" t="inlineStr">
+        <is>
+          <t>Sur STA le 26/10/2026 (décisions de Jordan du 26/10). Passée en prod le 31/10/2026 avec la refonte (décision de Jordan du 28/10).</t>
+        </is>
+      </c>
+      <c r="I65" s="8" t="n"/>
+    </row>
+    <row r="66">
+      <c r="A66" s="4" t="n">
+        <v>62</v>
+      </c>
+      <c r="B66" s="5" t="inlineStr">
+        <is>
+          <t>Refonte — visiteurs distincts</t>
+        </is>
+      </c>
+      <c r="C66" s="4" t="inlineStr">
+        <is>
+          <t>Pilotage → Activité ; Supabase PROD</t>
+        </is>
+      </c>
+      <c r="D66" s="4" t="inlineStr">
+        <is>
+          <t>Après quelques visites : regarder l'entonnoir ; vérifier la colonne visite des nouvelles lignes de funnel_events.</t>
+        </is>
+      </c>
+      <c r="E66" s="4" t="inlineStr">
+        <is>
+          <t>« Visiteurs distincts (30 j) » affichés par étape ; colonne visite remplie (créée le 26/10 en STA et en PROD) ; pages Cookies et Confidentialité mentionnent l'identifiant de visite.</t>
+        </is>
+      </c>
+      <c r="F66" s="4" t="inlineStr">
+        <is>
+          <t>Admin</t>
+        </is>
+      </c>
+      <c r="G66" s="6" t="inlineStr">
+        <is>
+          <t>À tester</t>
+        </is>
+      </c>
+      <c r="H66" s="6" t="inlineStr">
+        <is>
+          <t>Sur STA le 26/10/2026 (décisions de Jordan du 26/10). Passée en prod le 31/10/2026 avec la refonte (décision de Jordan du 28/10).</t>
+        </is>
+      </c>
+      <c r="I66" s="8" t="n"/>
+    </row>
+    <row r="67">
+      <c r="A67" s="4" t="n">
+        <v>63</v>
+      </c>
+      <c r="B67" s="5" t="inlineStr">
+        <is>
+          <t>Refonte — Bob</t>
+        </is>
+      </c>
+      <c r="C67" s="4" t="inlineStr">
+        <is>
+          <t>Bob</t>
+        </is>
+      </c>
+      <c r="D67" s="4" t="inlineStr">
+        <is>
+          <t>Demander « Combien coûte Premium ? », « Où est le classement ? », « Le plan annuel est payant ? ».</t>
+        </is>
+      </c>
+      <c r="E67" s="4" t="inlineStr">
+        <is>
+          <t>Prix 2,99 € et 24,99 €, offre de saison et essai de 7 jours ; classement dans Mon gazon → Mes progrès ; plan annuel inclus dans Premium.</t>
+        </is>
+      </c>
+      <c r="F67" s="4" t="inlineStr">
+        <is>
+          <t>Gratuit</t>
+        </is>
+      </c>
+      <c r="G67" s="6" t="inlineStr">
+        <is>
+          <t>À tester</t>
+        </is>
+      </c>
+      <c r="H67" s="6" t="inlineStr">
+        <is>
+          <t>Sur STA le 26/10/2026 (décisions de Jordan du 26/10). Testé par Jordan sur STA le 29/10 : OK ; consigne du classement précisée (en pause de novembre à janvier). Passée en prod le 31/10/2026 avec la refonte (décision de Jordan du 28/10).</t>
+        </is>
+      </c>
+      <c r="I67" s="8" t="n"/>
+    </row>
+    <row r="68">
+      <c r="A68" s="4" t="n">
+        <v>64</v>
+      </c>
+      <c r="B68" s="5" t="inlineStr">
+        <is>
+          <t>Refonte — dates des pages légales</t>
+        </is>
+      </c>
+      <c r="C68" s="4" t="inlineStr">
+        <is>
+          <t>CGV, politique de cookies, politique de confidentialité</t>
+        </is>
+      </c>
+      <c r="D68" s="4" t="inlineStr">
+        <is>
+          <t>Le jour de la mise en prod : mettre la date du jour dans « Mise à jour » de ces 3 pages (commit).</t>
+        </is>
+      </c>
+      <c r="E68" s="4" t="inlineStr">
+        <is>
+          <t>Date de mise à jour = jour de la mise en prod.</t>
+        </is>
+      </c>
+      <c r="F68" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G68" s="6" t="inlineStr">
+        <is>
+          <t>À tester</t>
+        </is>
+      </c>
+      <c r="H68" s="6" t="inlineStr">
+        <is>
+          <t>Sur STA le 26/10/2026 (décisions de Jordan du 26/10). Passée en prod le 31/10/2026 avec la refonte (décision de Jordan du 28/10).</t>
+        </is>
+      </c>
+      <c r="I68" s="8" t="n"/>
+    </row>
+    <row r="69">
+      <c r="A69" s="4" t="n">
+        <v>65</v>
+      </c>
+      <c r="B69" s="5" t="inlineStr">
+        <is>
+          <t>Offre d'hiver dès le 1er novembre</t>
+        </is>
+      </c>
+      <c r="C69" s="4" t="inlineStr">
+        <is>
+          <t>Choisir son niveau, accueil, Bob, email de lancement</t>
+        </is>
+      </c>
+      <c r="D69" s="4" t="inlineStr">
+        <is>
+          <t>À partir du 1/11 : ouvrir « Choisir son niveau » et l'accueil avec un compte gratuit ; demander à Bob « Quand est l'offre de saison ? » ; le matin du 1er jour d'offre, regarder l'email reçu par un compte gratuit qui accepte les offres.</t>
+        </is>
+      </c>
+      <c r="E69" s="4" t="inlineStr">
+        <is>
+          <t>Offre d'hiver : Premium 1 an à 12,99 € au lieu de 24,99 €, jusqu'au 25/02 (badge -48 %) ; Bob cite « du 1er novembre au 25 février et du 1er juillet au 15 août » ; email « ❄️ Premium 1 an à 12,99 € — jusqu'au 25/02 ». Avant le 1/11 : pas d'offre.</t>
+        </is>
+      </c>
+      <c r="F69" s="4" t="inlineStr">
+        <is>
+          <t>Gratuit</t>
+        </is>
+      </c>
+      <c r="G69" s="6" t="inlineStr">
+        <is>
+          <t>À tester</t>
+        </is>
+      </c>
+      <c r="H69" s="6" t="inlineStr">
+        <is>
+          <t>Sur STA le 28/10/2026 (décision de Jordan du 28/10 : l'offre d'hiver commence le 1/11 chaque année). Passée en prod le 31/10/2026 avec la refonte (décision de Jordan du 28/10).</t>
+        </is>
+      </c>
+      <c r="I69" s="8" t="n"/>
+    </row>
+    <row r="70">
+      <c r="A70" s="4" t="n">
+        <v>66</v>
+      </c>
+      <c r="B70" s="5" t="inlineStr">
+        <is>
+          <t>Mesure — abonnements Premium comptés</t>
+        </is>
+      </c>
+      <c r="C70" s="4" t="inlineStr">
+        <is>
+          <t>Supabase PROD (funnel_events) ; point KPI du lundi</t>
+        </is>
+      </c>
+      <c r="D70" s="4" t="inlineStr">
+        <is>
+          <t>Après le premier abonnement payant pris en prod (mensuel ou annuel) : regarder funnel_events, étape premium_souscrit.</t>
+        </is>
+      </c>
+      <c r="E70" s="4" t="inlineStr">
+        <is>
+          <t>Une ligne par abonnement pris, sans identifiant d'utilisateur, avec la formule (mensuel ou annuel) et l'offre (saison-hiver pendant l'offre) ; Premium activé même si la mesure échoue (alerte « Mesure — abonnement Premium non compté »).</t>
+        </is>
+      </c>
+      <c r="F70" s="4" t="inlineStr">
+        <is>
+          <t>Admin</t>
+        </is>
+      </c>
+      <c r="G70" s="6" t="inlineStr">
+        <is>
+          <t>À tester</t>
+        </is>
+      </c>
+      <c r="H70" s="6" t="inlineStr">
+        <is>
+          <t>Sur STA le 28/10/2026 (décision de Jordan du 28/10 : point KPI du lundi). Vérifié sur STA le 29/10 : abonnement de test mensuel compté (premium_souscrit, offre vide avant le 1/11). Abonnement de test annuel (24,99 €) réussi par Jordan sur STA le 30/10 : compté (formule annuel), Premium activé, aucune erreur. Passée en prod le 31/10/2026 avec la refonte (décision de Jordan du 28/10).</t>
+        </is>
+      </c>
+      <c r="I70" s="8" t="n"/>
+    </row>
+    <row r="71">
+      <c r="A71" s="4" t="n">
+        <v>67</v>
+      </c>
+      <c r="B71" s="5" t="inlineStr">
+        <is>
+          <t>Mesure — articles qui mènent à l'app</t>
+        </is>
+      </c>
+      <c r="C71" s="4" t="inlineStr">
+        <is>
+          <t>Pages Conseils ; Supabase PROD (funnel_events)</t>
+        </is>
+      </c>
+      <c r="D71" s="4" t="inlineStr">
+        <is>
+          <t>Sans être connecté, sur téléphone : ouvrir un article depuis un lien suivi (ex. groupe Facebook), puis toucher « Diagnostic gratuit » dans le même onglet ; regarder funnel_events.</t>
+        </is>
+      </c>
+      <c r="E71" s="4" t="inlineStr">
+        <is>
+          <t>Une ligne conseils_vue (page = article, source = origine) puis la page_view de /essai avec le même identifiant de visite ; un rechargement ne recompte pas l'article ; rien pour un compte connecté.</t>
+        </is>
+      </c>
+      <c r="F71" s="4" t="inlineStr">
+        <is>
+          <t>Admin</t>
+        </is>
+      </c>
+      <c r="G71" s="6" t="inlineStr">
+        <is>
+          <t>À tester</t>
+        </is>
+      </c>
+      <c r="H71" s="6" t="inlineStr">
+        <is>
+          <t>Sur STA le 28/10/2026 (demande de Jordan du 28/10 : faire atterrir le flux du site dans l'app). Passée en prod le 31/10/2026 avec la refonte (décision de Jordan du 28/10).</t>
+        </is>
+      </c>
+      <c r="I71" s="8" t="n"/>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A2:I2"/>
   </mergeCells>
-  <conditionalFormatting sqref="G5:G47">
+  <conditionalFormatting sqref="G5:G71">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"OK"</formula>
     </cfRule>
@@ -5995,7 +5979,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="G5:G47" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="G5:G71" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"À tester,OK,KO,Non testable"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Recette « Déjà en prod » et journal : annonce « Mongazon360 fait peau neuve », tests de Jordan en prod, lot du 8 au 14/11
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AUzY5Y8Bt2KRzzte5cJgH8
</commit_message>
<xml_diff>
--- a/docs/recette/Recette_prod_decembre_2026.xlsx
+++ b/docs/recette/Recette_prod_decembre_2026.xlsx
@@ -3059,22 +3059,6 @@
       <c r="H67" s="6" t="n"/>
       <c r="I67" s="6" t="n"/>
     </row>
-    <row r="72"/>
-    <row r="73"/>
-    <row r="74"/>
-    <row r="75"/>
-    <row r="76"/>
-    <row r="77"/>
-    <row r="78"/>
-    <row r="79"/>
-    <row r="80"/>
-    <row r="81"/>
-    <row r="82"/>
-    <row r="83"/>
-    <row r="84"/>
-    <row r="85"/>
-    <row r="86"/>
-    <row r="87"/>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A2:I2"/>
@@ -3102,7 +3086,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I71"/>
+  <dimension ref="A1:I72"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -5966,11 +5950,52 @@
       </c>
       <c r="I71" s="8" t="n"/>
     </row>
+    <row r="72">
+      <c r="A72" s="4" t="n">
+        <v>68</v>
+      </c>
+      <c r="B72" s="5" t="inlineStr">
+        <is>
+          <t>Annonce « Mongazon360 fait peau neuve » (notification unique)</t>
+        </is>
+      </c>
+      <c r="C72" s="4" t="inlineStr">
+        <is>
+          <t>Notification du matin ou conseil par email ; Pilotage → Activité (notifications) ; Supabase PROD (reminders.notif_log)</t>
+        </is>
+      </c>
+      <c r="D72" s="4" t="inlineStr">
+        <is>
+          <t>Entre le 3 et le 8/11 : regarder les notifications reçues par un compte créé avant le 31/10 qui accepte les conseils (gratuit, puis Premium) et par un compte créé après ; compter les envois (notif_log, type annonce_refonte-2026).</t>
+        </is>
+      </c>
+      <c r="E72" s="4" t="inlineStr">
+        <is>
+          <t>Une seule fois par compte créé avant le 31/10, le matin, jamais avant une urgence, un parcours, une action due ou un risque de maladie ; texte avec l'offre d'hiver (Premium 1 an à 12,99 € la 1re année, jusqu'au 25/02) pour un compte sans Premium ; rien pour un compte créé après le 31/10 ; la notification ouvre l'accueil.</t>
+        </is>
+      </c>
+      <c r="F72" s="4" t="inlineStr">
+        <is>
+          <t>Gratuit, Premium, nouveau compte</t>
+        </is>
+      </c>
+      <c r="G72" s="6" t="inlineStr">
+        <is>
+          <t>À tester</t>
+        </is>
+      </c>
+      <c r="H72" s="6" t="inlineStr">
+        <is>
+          <t>En prod le 31/10/2026 (go de Jordan du 31/10, pendant le gel) ; banc d'essai du moteur au vert (14 cas). Annonce à retirer de src/lib/annonces.json après le 8/11.</t>
+        </is>
+      </c>
+      <c r="I72" s="8" t="n"/>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A2:I2"/>
   </mergeCells>
-  <conditionalFormatting sqref="G5:G71">
+  <conditionalFormatting sqref="G5:G72">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"OK"</formula>
     </cfRule>
@@ -5979,7 +6004,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="G5:G71" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="G5:G72" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"À tester,OK,KO,Non testable"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Recette « Déjà en prod » et journal : page de paiement et contrôles de Jordan en prod (31/10)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AUzY5Y8Bt2KRzzte5cJgH8
</commit_message>
<xml_diff>
--- a/docs/recette/Recette_prod_decembre_2026.xlsx
+++ b/docs/recette/Recette_prod_decembre_2026.xlsx
@@ -5494,7 +5494,7 @@
       </c>
       <c r="H60" s="6" t="inlineStr">
         <is>
-          <t>Sur STA le 26/10/2026 (décisions de Jordan du 26/10). Testé par Jordan sur STA le 29/10 : raccourcis Premium OK (compte gratuit et app Android à voir). Mes équipements ouverts aux comptes gratuits (constat de Jordan le 29/10) : verrou Premium ajouté le 29/10 (STA et version de prod), vérifié par Jordan sur STA le 29/10 ; demande d'équipement non listé retirée de la page d'un compte gratuit le 29/10 (décision de Jordan). Compte gratuit testé par Jordan sur STA le 30/10 : OK (carte « Avec Premium » de l'accueil, du diagnostic et de Mon gazon ; Mes équipements verrouillé, sans formulaire). App Android : à vérifier après la mise en prod. Passée en prod le 31/10/2026 avec la refonte (décision de Jordan du 28/10).</t>
+          <t>Sur STA le 26/10/2026 (décisions de Jordan du 26/10). Testé par Jordan sur STA le 29/10 : raccourcis Premium OK (compte gratuit et app Android à voir). Mes équipements ouverts aux comptes gratuits (constat de Jordan le 29/10) : verrou Premium ajouté le 29/10 (STA et version de prod), vérifié par Jordan sur STA le 29/10 ; demande d'équipement non listé retirée de la page d'un compte gratuit le 29/10 (décision de Jordan). Compte gratuit testé par Jordan sur STA le 30/10 : OK (carte « Avec Premium » de l'accueil, du diagnostic et de Mon gazon ; Mes équipements verrouillé, sans formulaire). App Android : à vérifier après la mise en prod. Passée en prod le 31/10/2026 avec la refonte (décision de Jordan du 28/10). Vérifié en prod par Jordan le 31/10 : app Android sans carte d'achat, nouvelle barre du bas.</t>
         </is>
       </c>
       <c r="I60" s="8" t="n"/>
@@ -5535,7 +5535,7 @@
       </c>
       <c r="H61" s="6" t="inlineStr">
         <is>
-          <t>Sur STA le 26/10/2026 (décisions de Jordan du 26/10). Paiement de test réussi sur STA le 29/10 (mensuel à 2,99 €, bac à sable Stripe). Abonné : aucun lien vers la page (voulu). Test de Jordan le 29/10 avec son compte admin : offres affichées au lieu de « Tu es déjà Premium » (compte admin non reconnu comme Premium sur cette page) ; corrigé le 29/10, puis décision de Jordan le soir même : un compte déjà Premium n'arrive jamais sur la page (renvoi à l'accueil), STA et version de prod. Passée en prod le 31/10/2026 avec la refonte (décision de Jordan du 28/10).</t>
+          <t>Sur STA le 26/10/2026 (décisions de Jordan du 26/10). Paiement de test réussi sur STA le 29/10 (mensuel à 2,99 €, bac à sable Stripe). Abonné : aucun lien vers la page (voulu). Test de Jordan le 29/10 avec son compte admin : offres affichées au lieu de « Tu es déjà Premium » (compte admin non reconnu comme Premium sur cette page) ; corrigé le 29/10, puis décision de Jordan le soir même : un compte déjà Premium n'arrive jamais sur la page (renvoi à l'accueil), STA et version de prod. Passée en prod le 31/10/2026 avec la refonte (décision de Jordan du 28/10). Vérifié en prod par Jordan le 31/10 : page de paiement Stripe à 2,99 € par mois et 24,99 € par an, produit « Mongazon360 Premium » (sans payer).</t>
         </is>
       </c>
       <c r="I61" s="8" t="n"/>
@@ -5699,7 +5699,7 @@
       </c>
       <c r="H65" s="6" t="inlineStr">
         <is>
-          <t>Sur STA le 26/10/2026 (décisions de Jordan du 26/10). Passée en prod le 31/10/2026 avec la refonte (décision de Jordan du 28/10).</t>
+          <t>Sur STA le 26/10/2026 (décisions de Jordan du 26/10). Passée en prod le 31/10/2026 avec la refonte (décision de Jordan du 28/10). Vérifié en prod par Jordan le 31/10 : carte affichée sur son compte, fermée par « J'ai compris » (nouveau compte à voir).</t>
         </is>
       </c>
       <c r="I65" s="8" t="n"/>

</xml_diff>

<commit_message>
Conseils : bandeau A retenu par Jordan (version B retirée), visuels du chantier du 22/11 validés le 31/10
Bandeau « Dans l'app, ces conseils deviennent votre plan », 10 accroches, bouton fixe sur téléphone,
forme et couleurs des encarts validés. Recette décembre n° 60, journal et CLAUDE.md mis à jour.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AUzY5Y8Bt2KRzzte5cJgH8
</commit_message>
<xml_diff>
--- a/docs/recette/Recette_prod_decembre_2026.xlsx
+++ b/docs/recette/Recette_prod_decembre_2026.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Recette décembre" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Déjà en prod (exceptions)" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Recette décembre" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Déjà en prod (exceptions)" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -2922,7 +2922,7 @@
       </c>
       <c r="E64" s="4" t="inlineStr">
         <is>
-          <t>Bandeau sous le titre sans cacher le texte (« Télécharger sur Google Play » seulement dans le navigateur d'un téléphone Android) ; encarts après « En bref », au milieu et à la fin, thèmes variés selon l'article (src/lib/argumentsApp.json) ; bouton fixe « Ouvrir l'app gratuite » sur téléphone seulement ; grille « Ce que fait l'app » ; l'encart touché ouvre l'app et sa page_view porte encart = thème-position ; aucune page plus large que l'écran.</t>
+          <t>Bandeau « Dans l'app, ces conseils deviennent votre plan » sous le titre, sans cacher le texte (« Télécharger sur Google Play » seulement dans le navigateur d'un téléphone Android) ; encarts après « En bref », au milieu et à la fin, thèmes variés selon l'article (src/lib/argumentsApp.json) ; bouton fixe « Ouvrir l'app gratuite » sur téléphone seulement ; grille « Ce que fait l'app » ; l'encart touché ouvre l'app et sa page_view porte encart = thème-position ; aucune page plus large que l'écran.</t>
         </is>
       </c>
       <c r="F64" s="4" t="inlineStr">
@@ -2937,7 +2937,7 @@
       </c>
       <c r="H64" s="6" t="inlineStr">
         <is>
-          <t>Sur STA le 30/10/2026 (décisions de Jordan des 28 et 30/10) ; bandeau en 2 versions à départager sur les visuels.</t>
+          <t>Sur STA le 30/10/2026 (décisions de Jordan des 28 et 30/10) ; visuels validés par Jordan le 31/10 : bandeau A (version B retirée), 10 accroches, bouton fixe, forme et couleurs des encarts.</t>
         </is>
       </c>
       <c r="I64" s="6" t="n"/>

</xml_diff>

<commit_message>
Partage du score : message copié avant d'ouvrir Facebook, à coller dans la publication (constat de Jordan du 31/10)
Facebook ignore le texte tout prêt (paramètre quote) et ne garde que le lien : le score n'apparaissait pas. Le
message est maintenant copié, avec une confirmation propre à Facebook, Instagram et Copier. Recette décembre n° 63.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AUzY5Y8Bt2KRzzte5cJgH8
</commit_message>
<xml_diff>
--- a/docs/recette/Recette_prod_decembre_2026.xlsx
+++ b/docs/recette/Recette_prod_decembre_2026.xlsx
@@ -505,7 +505,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I67"/>
+  <dimension ref="A1:I68"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -3028,42 +3028,85 @@
       </c>
       <c r="B67" s="5" t="inlineStr">
         <is>
+          <t>Partage du score sur Facebook : message copié</t>
+        </is>
+      </c>
+      <c r="C67" s="4" t="inlineStr">
+        <is>
+          <t>Mon gazon (Partager)</t>
+        </is>
+      </c>
+      <c r="D67" s="4" t="inlineStr">
+        <is>
+          <t>Sur un téléphone : Mon gazon → Partager → Facebook, puis coller le texte dans la publication Facebook. Refaire avec Instagram et Copier.</t>
+        </is>
+      </c>
+      <c r="E67" s="4" t="inlineStr">
+        <is>
+          <t>En touchant Facebook, le message du score est copié (« ✅ Message copié : collez-le dans votre publication Facebook ») puis Facebook s'ouvre avec le lien ; une fois le texte collé, la publication montre le score et le lien. Instagram et Copier copient aussi le message, avec leur propre confirmation.</t>
+        </is>
+      </c>
+      <c r="F67" s="4" t="inlineStr">
+        <is>
+          <t>Tous</t>
+        </is>
+      </c>
+      <c r="G67" s="6" t="inlineStr">
+        <is>
+          <t>À tester</t>
+        </is>
+      </c>
+      <c r="H67" s="6" t="inlineStr">
+        <is>
+          <t>Constat de Jordan du 31/10/2026 : partage Facebook sans le score (Facebook ignore le texte tout prêt et ne garde que le lien) ; correctif sur STA le 31/10.</t>
+        </is>
+      </c>
+      <c r="I67" s="6" t="n"/>
+    </row>
+    <row r="68">
+      <c r="A68" s="4" t="inlineStr">
+        <is>
+          <t>64</t>
+        </is>
+      </c>
+      <c r="B68" s="5" t="inlineStr">
+        <is>
           <t>Règle de travail de décembre</t>
         </is>
       </c>
-      <c r="C67" s="4" t="inlineStr">
+      <c r="C68" s="4" t="inlineStr">
         <is>
           <t>CLAUDE.md</t>
         </is>
       </c>
-      <c r="D67" s="4" t="inlineStr">
+      <c r="D68" s="4" t="inlineStr">
         <is>
           <t>Après la mise en prod : retirer le paragraphe « Jusqu'à décembre 2026 ».</t>
         </is>
       </c>
-      <c r="E67" s="4" t="inlineStr">
+      <c r="E68" s="4" t="inlineStr">
         <is>
           <t>STA redevient identique à la PROD.</t>
         </is>
       </c>
-      <c r="F67" s="4" t="inlineStr">
+      <c r="F68" s="4" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G67" s="6" t="inlineStr">
-        <is>
-          <t>À tester</t>
-        </is>
-      </c>
-      <c r="H67" s="6" t="n"/>
-      <c r="I67" s="6" t="n"/>
+      <c r="G68" s="6" t="inlineStr">
+        <is>
+          <t>À tester</t>
+        </is>
+      </c>
+      <c r="H68" s="6" t="n"/>
+      <c r="I68" s="6" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A2:I2"/>
   </mergeCells>
-  <conditionalFormatting sqref="G5:G67">
+  <conditionalFormatting sqref="G5:G68">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"OK"</formula>
     </cfRule>
@@ -3072,7 +3115,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="G5:G67" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="G5:G68" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"À tester,OK,KO,Non testable"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Recette « Déjà en prod » et journal : correctif du partage Facebook en prod le 31/10 (go de Jordan)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AUzY5Y8Bt2KRzzte5cJgH8
</commit_message>
<xml_diff>
--- a/docs/recette/Recette_prod_decembre_2026.xlsx
+++ b/docs/recette/Recette_prod_decembre_2026.xlsx
@@ -505,7 +505,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I68"/>
+  <dimension ref="A1:I67"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -3028,27 +3028,27 @@
       </c>
       <c r="B67" s="5" t="inlineStr">
         <is>
-          <t>Partage du score sur Facebook : message copié</t>
+          <t>Règle de travail de décembre</t>
         </is>
       </c>
       <c r="C67" s="4" t="inlineStr">
         <is>
-          <t>Mon gazon (Partager)</t>
+          <t>CLAUDE.md</t>
         </is>
       </c>
       <c r="D67" s="4" t="inlineStr">
         <is>
-          <t>Sur un téléphone : Mon gazon → Partager → Facebook, puis coller le texte dans la publication Facebook. Refaire avec Instagram et Copier.</t>
+          <t>Après la mise en prod : retirer le paragraphe « Jusqu'à décembre 2026 ».</t>
         </is>
       </c>
       <c r="E67" s="4" t="inlineStr">
         <is>
-          <t>En touchant Facebook, le message du score est copié (« ✅ Message copié : collez-le dans votre publication Facebook ») puis Facebook s'ouvre avec le lien ; une fois le texte collé, la publication montre le score et le lien. Instagram et Copier copient aussi le message, avec leur propre confirmation.</t>
+          <t>STA redevient identique à la PROD.</t>
         </is>
       </c>
       <c r="F67" s="4" t="inlineStr">
         <is>
-          <t>Tous</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G67" s="6" t="inlineStr">
@@ -3056,57 +3056,14 @@
           <t>À tester</t>
         </is>
       </c>
-      <c r="H67" s="6" t="inlineStr">
-        <is>
-          <t>Constat de Jordan du 31/10/2026 : partage Facebook sans le score (Facebook ignore le texte tout prêt et ne garde que le lien) ; correctif sur STA le 31/10.</t>
-        </is>
-      </c>
+      <c r="H67" s="6" t="n"/>
       <c r="I67" s="6" t="n"/>
-    </row>
-    <row r="68">
-      <c r="A68" s="4" t="inlineStr">
-        <is>
-          <t>64</t>
-        </is>
-      </c>
-      <c r="B68" s="5" t="inlineStr">
-        <is>
-          <t>Règle de travail de décembre</t>
-        </is>
-      </c>
-      <c r="C68" s="4" t="inlineStr">
-        <is>
-          <t>CLAUDE.md</t>
-        </is>
-      </c>
-      <c r="D68" s="4" t="inlineStr">
-        <is>
-          <t>Après la mise en prod : retirer le paragraphe « Jusqu'à décembre 2026 ».</t>
-        </is>
-      </c>
-      <c r="E68" s="4" t="inlineStr">
-        <is>
-          <t>STA redevient identique à la PROD.</t>
-        </is>
-      </c>
-      <c r="F68" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G68" s="6" t="inlineStr">
-        <is>
-          <t>À tester</t>
-        </is>
-      </c>
-      <c r="H68" s="6" t="n"/>
-      <c r="I68" s="6" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A2:I2"/>
   </mergeCells>
-  <conditionalFormatting sqref="G5:G68">
+  <conditionalFormatting sqref="G5:G67">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"OK"</formula>
     </cfRule>
@@ -3115,7 +3072,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="G5:G68" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="G5:G67" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"À tester,OK,KO,Non testable"</formula1>
     </dataValidation>
   </dataValidations>
@@ -3129,7 +3086,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I72"/>
+  <dimension ref="A1:I73"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -6034,11 +5991,54 @@
       </c>
       <c r="I72" s="8" t="n"/>
     </row>
+    <row r="73">
+      <c r="A73" s="4" t="inlineStr">
+        <is>
+          <t>69</t>
+        </is>
+      </c>
+      <c r="B73" s="5" t="inlineStr">
+        <is>
+          <t>Partage du score sur Facebook : message copié</t>
+        </is>
+      </c>
+      <c r="C73" s="4" t="inlineStr">
+        <is>
+          <t>Mon gazon (Partager)</t>
+        </is>
+      </c>
+      <c r="D73" s="4" t="inlineStr">
+        <is>
+          <t>Sur un téléphone : Mon gazon → Partager → Facebook, puis coller le texte dans la publication Facebook. Refaire avec Instagram et Copier.</t>
+        </is>
+      </c>
+      <c r="E73" s="4" t="inlineStr">
+        <is>
+          <t>En touchant Facebook, le message du score est copié (« ✅ Message copié : collez-le dans votre publication Facebook ») puis Facebook s'ouvre avec le lien ; une fois le texte collé, la publication montre le score et le lien. Instagram et Copier copient aussi le message, avec leur propre confirmation.</t>
+        </is>
+      </c>
+      <c r="F73" s="4" t="inlineStr">
+        <is>
+          <t>Tous</t>
+        </is>
+      </c>
+      <c r="G73" s="6" t="inlineStr">
+        <is>
+          <t>À tester</t>
+        </is>
+      </c>
+      <c r="H73" s="6" t="inlineStr">
+        <is>
+          <t>Constat de Jordan du 31/10/2026 : partage Facebook sans le score (Facebook ignore le texte tout prêt et ne garde que le lien). En prod le 31/10/2026 (correctif, go de Jordan du 31/10).</t>
+        </is>
+      </c>
+      <c r="I73" s="8" t="n"/>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A2:I2"/>
   </mergeCells>
-  <conditionalFormatting sqref="G5:G72">
+  <conditionalFormatting sqref="G5:G73">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"OK"</formula>
     </cfRule>
@@ -6047,7 +6047,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="G5:G72" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="G5:G73" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"À tester,OK,KO,Non testable"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Partage du score en image : carte 1080 × 1350 partagée par le menu du téléphone (décision de Jordan du 31/10, prod le 22/11)
src/lib/carteScore.js dessine la carte (jauge, libellé, notre pelouse, Bob, invitation au diagnostic gratuit) ; dans
Mon gazon → Partager, aperçu et bouton « Partager l'image de mon score » quand le téléphone sait partager une image.
Chaque partage est compté dans funnel_events (partage_score, canal). Recette décembre n° 63, CLAUDE.md, journal.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AUzY5Y8Bt2KRzzte5cJgH8
</commit_message>
<xml_diff>
--- a/docs/recette/Recette_prod_decembre_2026.xlsx
+++ b/docs/recette/Recette_prod_decembre_2026.xlsx
@@ -505,7 +505,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I67"/>
+  <dimension ref="A1:I68"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -3028,42 +3028,85 @@
       </c>
       <c r="B67" s="5" t="inlineStr">
         <is>
+          <t>Partage du score en image (prod le 22/11)</t>
+        </is>
+      </c>
+      <c r="C67" s="4" t="inlineStr">
+        <is>
+          <t>Mon gazon (Partager) ; Supabase PROD (funnel_events)</t>
+        </is>
+      </c>
+      <c r="D67" s="4" t="inlineStr">
+        <is>
+          <t>Sur un téléphone Android (app ou navigateur) : Mon gazon → Partager ; regarder l'aperçu, toucher « Partager l'image de mon score », choisir Facebook, puis recommencer avec WhatsApp. Sur un ordinateur : ouvrir Partager.</t>
+        </is>
+      </c>
+      <c r="E67" s="4" t="inlineStr">
+        <is>
+          <t>Aperçu de l'image (score, libellé, notre pelouse, Bob, « Et la vôtre ? Diagnostic photo gratuit sur mongazon360.fr ») ; le menu de partage du téléphone s'ouvre avec l'image ; Facebook publie l'image (message copié, à coller) ; WhatsApp envoie l'image avec le message. Sur un ordinateur qui ne sait pas partager d'image : pas de bouton, les autres restent. Une ligne partage_score (canal image, whatsapp, facebook…) par bouton touché.</t>
+        </is>
+      </c>
+      <c r="F67" s="4" t="inlineStr">
+        <is>
+          <t>Tous</t>
+        </is>
+      </c>
+      <c r="G67" s="6" t="inlineStr">
+        <is>
+          <t>À tester</t>
+        </is>
+      </c>
+      <c r="H67" s="6" t="inlineStr">
+        <is>
+          <t>Décision de Jordan du 31/10/2026 (proposition 6 pour la visibilité) ; sur STA le 31/10.</t>
+        </is>
+      </c>
+      <c r="I67" s="6" t="n"/>
+    </row>
+    <row r="68">
+      <c r="A68" s="4" t="inlineStr">
+        <is>
+          <t>64</t>
+        </is>
+      </c>
+      <c r="B68" s="5" t="inlineStr">
+        <is>
           <t>Règle de travail de décembre</t>
         </is>
       </c>
-      <c r="C67" s="4" t="inlineStr">
+      <c r="C68" s="4" t="inlineStr">
         <is>
           <t>CLAUDE.md</t>
         </is>
       </c>
-      <c r="D67" s="4" t="inlineStr">
+      <c r="D68" s="4" t="inlineStr">
         <is>
           <t>Après la mise en prod : retirer le paragraphe « Jusqu'à décembre 2026 ».</t>
         </is>
       </c>
-      <c r="E67" s="4" t="inlineStr">
+      <c r="E68" s="4" t="inlineStr">
         <is>
           <t>STA redevient identique à la PROD.</t>
         </is>
       </c>
-      <c r="F67" s="4" t="inlineStr">
+      <c r="F68" s="4" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G67" s="6" t="inlineStr">
-        <is>
-          <t>À tester</t>
-        </is>
-      </c>
-      <c r="H67" s="6" t="n"/>
-      <c r="I67" s="6" t="n"/>
+      <c r="G68" s="6" t="inlineStr">
+        <is>
+          <t>À tester</t>
+        </is>
+      </c>
+      <c r="H68" s="6" t="n"/>
+      <c r="I68" s="6" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A2:I2"/>
   </mergeCells>
-  <conditionalFormatting sqref="G5:G67">
+  <conditionalFormatting sqref="G5:G68">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"OK"</formula>
     </cfRule>
@@ -3072,7 +3115,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="G5:G67" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="G5:G68" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"À tester,OK,KO,Non testable"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Partage du résultat du quiz en image (décision de Jordan du 31/10, prod le 22/11)
Après la correction du quiz de la ligue d'hiver, « Partager mon résultat » envoie l'image du résultat (semaine, thème,
bonnes réponses sur 3, jamais les réponses) et le texte partage.resultat de ligueHiver.json, avec le lien de la ligue.
Cartes du score et du quiz réunies dans src/lib/cartesPartage.js (fond commun). Mesure partage_quiz. Recette n° 64.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AUzY5Y8Bt2KRzzte5cJgH8
</commit_message>
<xml_diff>
--- a/docs/recette/Recette_prod_decembre_2026.xlsx
+++ b/docs/recette/Recette_prod_decembre_2026.xlsx
@@ -505,7 +505,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I68"/>
+  <dimension ref="A1:I69"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -3071,42 +3071,85 @@
       </c>
       <c r="B68" s="5" t="inlineStr">
         <is>
+          <t>Partage du résultat du quiz en image (prod le 22/11)</t>
+        </is>
+      </c>
+      <c r="C68" s="4" t="inlineStr">
+        <is>
+          <t>Onglet Quiz (ligue d'hiver) ; Supabase PROD (funnel_events)</t>
+        </is>
+      </c>
+      <c r="D68" s="4" t="inlineStr">
+        <is>
+          <t>Sur un téléphone Android : faire le quiz de la semaine, puis toucher « Partager mon résultat » et choisir Facebook ou WhatsApp.</t>
+        </is>
+      </c>
+      <c r="E68" s="4" t="inlineStr">
+        <is>
+          <t>Le menu de partage du téléphone s'ouvre avec l'image du résultat (ligue d'hiver, semaine, thème, bonnes réponses sur 3 avec une pastille par question, « Et toi ? Quiz gratuit… mongazon360.fr ») et le texte « J'ai eu x/3 au quiz gazon de la semaine… » avec le lien de la ligue ; aucune réponse du quiz n'apparaît. Sans partage d'image : texte et lien seulement. Une ligne partage_quiz (canal, semaine, bonnes) par partage.</t>
+        </is>
+      </c>
+      <c r="F68" s="4" t="inlineStr">
+        <is>
+          <t>Tous</t>
+        </is>
+      </c>
+      <c r="G68" s="6" t="inlineStr">
+        <is>
+          <t>À tester</t>
+        </is>
+      </c>
+      <c r="H68" s="6" t="inlineStr">
+        <is>
+          <t>Décision de Jordan du 31/10/2026 (proposition 7 pour la visibilité) ; sur STA le 31/10.</t>
+        </is>
+      </c>
+      <c r="I68" s="6" t="n"/>
+    </row>
+    <row r="69">
+      <c r="A69" s="4" t="inlineStr">
+        <is>
+          <t>65</t>
+        </is>
+      </c>
+      <c r="B69" s="5" t="inlineStr">
+        <is>
           <t>Règle de travail de décembre</t>
         </is>
       </c>
-      <c r="C68" s="4" t="inlineStr">
+      <c r="C69" s="4" t="inlineStr">
         <is>
           <t>CLAUDE.md</t>
         </is>
       </c>
-      <c r="D68" s="4" t="inlineStr">
+      <c r="D69" s="4" t="inlineStr">
         <is>
           <t>Après la mise en prod : retirer le paragraphe « Jusqu'à décembre 2026 ».</t>
         </is>
       </c>
-      <c r="E68" s="4" t="inlineStr">
+      <c r="E69" s="4" t="inlineStr">
         <is>
           <t>STA redevient identique à la PROD.</t>
         </is>
       </c>
-      <c r="F68" s="4" t="inlineStr">
+      <c r="F69" s="4" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G68" s="6" t="inlineStr">
-        <is>
-          <t>À tester</t>
-        </is>
-      </c>
-      <c r="H68" s="6" t="n"/>
-      <c r="I68" s="6" t="n"/>
+      <c r="G69" s="6" t="inlineStr">
+        <is>
+          <t>À tester</t>
+        </is>
+      </c>
+      <c r="H69" s="6" t="n"/>
+      <c r="I69" s="6" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A2:I2"/>
   </mergeCells>
-  <conditionalFormatting sqref="G5:G68">
+  <conditionalFormatting sqref="G5:G69">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"OK"</formula>
     </cfRule>
@@ -3115,7 +3158,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="G5:G68" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="G5:G69" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"À tester,OK,KO,Non testable"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Code de parrainage dans les partages du score et du quiz (décision de Jordan du 31/10, décembre avec le parrainage)
src/lib/useMonCode.js lit le code de l'utilisateur (api/parrainage.cjs) : lien ?p=CODE, texte « 1 mois de Premium
offert grâce à mon code » et image avec le code, pour le score, le résultat du quiz et le défi « partage ». Sans code :
lien simple comme avant. Recette décembre n° 65, CLAUDE.md, journal (propositions 3, 4, 7 et 8).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AUzY5Y8Bt2KRzzte5cJgH8
</commit_message>
<xml_diff>
--- a/docs/recette/Recette_prod_decembre_2026.xlsx
+++ b/docs/recette/Recette_prod_decembre_2026.xlsx
@@ -505,7 +505,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I69"/>
+  <dimension ref="A1:I70"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -3114,42 +3114,85 @@
       </c>
       <c r="B69" s="5" t="inlineStr">
         <is>
+          <t>Code de parrainage dans les partages</t>
+        </is>
+      </c>
+      <c r="C69" s="4" t="inlineStr">
+        <is>
+          <t>Mon gazon (Partager) ; onglet Quiz (Partager mon résultat, défi « partage »)</t>
+        </is>
+      </c>
+      <c r="D69" s="4" t="inlineStr">
+        <is>
+          <t>Avec un compte qui a un code de parrainage : partager le score, puis le résultat du quiz, par WhatsApp ; ouvrir le lien reçu sur un autre appareil, non connecté.</t>
+        </is>
+      </c>
+      <c r="E69" s="4" t="inlineStr">
+        <is>
+          <t>Texte avec « 1 mois de Premium offert grâce à mon code CODE » et lien https://mongazon360.fr/?p=CODE (quiz : lien de la ligue suivi de &amp;p=CODE) ; image avec « Code CODE : 1 mois de Premium offert sur mongazon360.fr » ; à l'ouverture du lien, bandeau du code et champ prérempli à l'inscription. Sans code disponible : lien simple, comme avant.</t>
+        </is>
+      </c>
+      <c r="F69" s="4" t="inlineStr">
+        <is>
+          <t>Tous</t>
+        </is>
+      </c>
+      <c r="G69" s="6" t="inlineStr">
+        <is>
+          <t>À tester</t>
+        </is>
+      </c>
+      <c r="H69" s="6" t="inlineStr">
+        <is>
+          <t>Décision de Jordan du 31/10/2026 (proposition 8 pour la visibilité) ; sur STA le 31/10, en prod avec le parrainage en décembre.</t>
+        </is>
+      </c>
+      <c r="I69" s="6" t="n"/>
+    </row>
+    <row r="70">
+      <c r="A70" s="4" t="inlineStr">
+        <is>
+          <t>66</t>
+        </is>
+      </c>
+      <c r="B70" s="5" t="inlineStr">
+        <is>
           <t>Règle de travail de décembre</t>
         </is>
       </c>
-      <c r="C69" s="4" t="inlineStr">
+      <c r="C70" s="4" t="inlineStr">
         <is>
           <t>CLAUDE.md</t>
         </is>
       </c>
-      <c r="D69" s="4" t="inlineStr">
+      <c r="D70" s="4" t="inlineStr">
         <is>
           <t>Après la mise en prod : retirer le paragraphe « Jusqu'à décembre 2026 ».</t>
         </is>
       </c>
-      <c r="E69" s="4" t="inlineStr">
+      <c r="E70" s="4" t="inlineStr">
         <is>
           <t>STA redevient identique à la PROD.</t>
         </is>
       </c>
-      <c r="F69" s="4" t="inlineStr">
+      <c r="F70" s="4" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G69" s="6" t="inlineStr">
-        <is>
-          <t>À tester</t>
-        </is>
-      </c>
-      <c r="H69" s="6" t="n"/>
-      <c r="I69" s="6" t="n"/>
+      <c r="G70" s="6" t="inlineStr">
+        <is>
+          <t>À tester</t>
+        </is>
+      </c>
+      <c r="H70" s="6" t="n"/>
+      <c r="I70" s="6" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A2:I2"/>
   </mergeCells>
-  <conditionalFormatting sqref="G5:G69">
+  <conditionalFormatting sqref="G5:G70">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"OK"</formula>
     </cfRule>
@@ -3158,7 +3201,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="G5:G69" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="G5:G70" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"À tester,OK,KO,Non testable"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>